<commit_message>
Verify the My Work drawer repair: MW-15 to MW-21 all fixed
Re-checked 0a57743 and 89ed015 in a signed-in browser at 1440 and 390, writes
blocked:
- MW-20: title, empty space, status, Log update, Add manually - 5/5 keep the
  drawer open on both viewports
- MW-16: Log update opens a visible form on a phone
- MW-15: 44px close in the header at 390; tapping the scrim strip closes
- MW-17: one close control; focus lands on it
- MW-21: View details -> Delete task -> confirm step, no DELETE on first tap
- MW-18: /finance and /team capped at 1400 at 1920, /my-work full width
- MW-19: Department lists departments with work; Completed is under Status

Findings marked Fixed with verification notes; coverage T-116, T-117,
T-119..T-125 flipped to PASS. Plan areas B-H ticked.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_UI_Bug_Report.xlsx
+++ b/docs/DecisionOS_UI_Bug_Report.xlsx
@@ -1672,9 +1672,9 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1722,7 +1722,11 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED FIXED 2026-09-13 (0a57743): clicking the title, empty space, status, Log update and Add manually leaves the drawer open - 5 of 5 at 1440 and 5 of 5 at 390.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="82" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1755,9 +1759,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1805,7 +1809,11 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED FIXED 2026-09-13 (0a57743): 'View details' at the foot of the drawer opens the detail dialog; Delete task is there and asks for confirmation before any DELETE is sent (1440 and 390).</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="82" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -1838,9 +1846,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1890,7 +1898,7 @@
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>RE-CHECKED 2026-09-13 on the newest code (78d01df): close tab still at x=-43 and stock close still under the title. Tapping inside the drawer now closes it, but only because of MW-20; once MW-20 is fixed this dead end returns, so fix both together.</t>
+          <t>VERIFIED FIXED 2026-09-13 (0a57743, 89ed015): at 390px the close sits in the drawer header, 44x44 and tappable; the drawer is 92% wide so tapping the strip beside it closes it; Escape still closes.</t>
         </is>
       </c>
     </row>
@@ -1925,9 +1933,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1977,7 +1985,7 @@
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>RE-CHECKED 2026-09-13 on the newest code: tapping Log update now closes the drawer outright (MW-20) and no form mounts. The hidden-body cause below still applies once MW-20 is fixed.</t>
+          <t>VERIFIED FIXED 2026-09-13 (0a57743): on a phone, Log update opens a visible update form inside the drawer.</t>
         </is>
       </c>
     </row>
@@ -2012,9 +2020,9 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -2062,7 +2070,11 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED FIXED 2026-09-13 (0a57743): one close control ('Close task') at 1440 and 390, and focus lands on it when the drawer opens.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="82" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -2095,9 +2107,9 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -2145,7 +2157,11 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED FIXED 2026-09-13 (0a57743): at 1920 /finance and /team are capped at 1400px again; /my-work keeps the full 1920.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="82" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -2178,9 +2194,9 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -2228,7 +2244,11 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED FIXED 2026-09-13 (0a57743): Department lists only departments holding work ('All 25', 'Logistics 1'); Completed moved to the Status filter.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="82" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -10464,14 +10484,14 @@
           <t>Usability</t>
         </is>
       </c>
-      <c r="H57" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Lists 'Completed' as a department and six 0-count options; picking one is silently undone</t>
+          <t>Was: Completed listed as a department + six 0-count options (MW-19). Re-checked after 0a57743: All 25 / Logistics 1; Completed is under Status</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -10516,14 +10536,14 @@
           <t>Functional</t>
         </is>
       </c>
-      <c r="H58" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Opens (672px, whole card and Enter both work, checkbox does not open it) - but on the newest code any click inside closes it</t>
+          <t>Was: any click inside closed it (MW-20). Re-checked after 0a57743: stays open for all 5 inside clicks</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -10620,14 +10640,14 @@
           <t>Regression</t>
         </is>
       </c>
-      <c r="H60" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Passed on 2a17592 (form visible, no crash); after 78d01df the click closes the drawer and no form appears</t>
+          <t>Re-checked after 0a57743: form visible, drawer stays open</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -10672,14 +10692,14 @@
           <t>Navigation</t>
         </is>
       </c>
-      <c r="H61" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Close tab at x=-43 off-screen, stock close under the title, no scrim, Back leaves the page</t>
+          <t>Was: no reachable close (MW-15). Re-checked after 0a57743 + 89ed015: 44px close in the header, scrim strip tap closes, Escape closes</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -10724,14 +10744,14 @@
           <t>Regression</t>
         </is>
       </c>
-      <c r="H62" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Form mounts inside the display:none desktop body</t>
+          <t>Was: form inside a hidden body (MW-16). Re-checked after 0a57743: form visible</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -10776,14 +10796,14 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="H63" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Two close buttons; initial focus on the stock one hidden under the title</t>
+          <t>Was: two closes, focus hidden (MW-17). Re-checked after 0a57743: one close, focus on it</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -10828,14 +10848,14 @@
           <t>Layout</t>
         </is>
       </c>
-      <c r="H64" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Cap removed in shared Layout; Finance tiles and Team cards stretch to ~610px</t>
+          <t>Was: cap removed globally (MW-18). Re-checked after 0a57743: Finance and Team 1400px, My Work 1920px</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -10880,14 +10900,14 @@
           <t>Functional</t>
         </is>
       </c>
-      <c r="H65" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>10 of 10 clicks closed the drawer across 1440 and 390</t>
+          <t>Was: 10 of 10 closed it (MW-20). Re-checked after 0a57743: 10 of 10 stay open</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -10932,14 +10952,14 @@
           <t>Functional</t>
         </is>
       </c>
-      <c r="H66" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>No Delete / View details control anywhere; the detail dialog has no opener</t>
+          <t>Was: unreachable (MW-21). Re-checked after 0a57743: View details -&gt; Delete task -&gt; confirm step</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -27955,7 +27975,7 @@
       </c>
       <c r="B46" s="22" t="inlineStr">
         <is>
-          <t>270 (175 pass, 93 fail, 0 blocked, 2 not run)</t>
+          <t>270 (184 pass, 84 fail, 0 blocked, 2 not run)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ask section: the three root causes from the full audit
- ASK-20 High: one shared load-error pattern (403 / 404 / network), and no
  empty state unless the query succeeded with zero rows. Closes OP-10, CR-10,
  CR-11, FN-07, FN-09, DD-01, DD-02, DD-03, CL-01.
- ASK-21 High: one permission map read by routes, nav, More tiles, Desk tiles
  and the backend guards, with a role x route test. Closes FN-07, CR-12,
  CR-13, DD-03, GL-02, TM-05.
- ASK-22 High: phone parity - no desktop-only action without a tappable mobile
  equivalent. Closes FN-08, CR-04, CR-05, CR-09, DD-04, GL-02, MW-22.

Notes: the ASK numbering clash with commit labels continues (ASK-18..21);
match by content, not number.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_UI_Bug_Report.xlsx
+++ b/docs/DecisionOS_UI_Bug_Report.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bug Log'!$A$1:$Q$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Coverage'!$A$1:$J$273</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Verified Non-Issues'!$A$1:$E$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Action List'!$A$1:$K$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Action List'!$A$1:$K$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21610,7 +21610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K104"/>
+  <dimension ref="A1:K107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -22749,50 +22749,54 @@
     <row r="21" ht="82" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>MW-08</t>
+          <t>ASK-20</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>UI audit</t>
+          <t>Founder review</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Task card - Update / Escalate</t>
+          <t>One load-error pattern for every page (root cause 1 of 3)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Bug fix</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
+          <t>Change request</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Restyle that one button to the segmented-control treatment the rest of the toolbar moved to in the same commit (kr-pressed / kr-pop, as the priority bands use), or simply restore the two constants. Then stop the class recurring: craco narrows ESLint to react-hooks rules only, which drops eslint-config-react-app's no-undef - the rule that would have failed the build on this exact line.</t>
+          <t>Build ONE shared &lt;QueryError&gt; (message + Retry) and use it wherever a query's data drives the page. It must branch on the failure: 403 -&gt; 'You don't have access to this' (with who to ask), 404 -&gt; 'This no longer exists' (with a way back), network / 5xx -&gt; 'Couldn't load - Retry'. While loading or failed, counts show '-', never 0. Rule for code review: a page may not render its empty state unless the query SUCCEEDED with zero rows.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>The app CRASHES. A ReferenceError is thrown while rendering the form, the form never appears, and the whole React tree unmounts - the page is gone, not just the form. Recovery needs a reload. The work trail, hand-off and escalation flow is therefore completely unusable.</t>
+          <t>The audit found the same fault on every major page: the page reads only data / isLoading, so a failed request falls through to the empty state or an endless skeleton. An owner on a weak connection is told 'Nothing waiting on you' (DD-02), 'No expenses yet' (FN-09), 'You're all caught up' (CL-01), or watches a skeleton that never ends (OP-10, CR-10). A missing decision traps the user with no way out (DD-01). Staff refused by the ledger see fake empty books (FN-07, DD-03). Fixing it once, in one component, closes nine findings.</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:147 (UpdateForm); constants removed in 5fb96f2; lint narrowed at craco.config.js:74</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr"/>
+          <t>pages/Desk.js:284-292, pages/OperatingScore.js:85-92, pages/CRM.js:524-527, pages/Ledger.js:1522-1527, pages/ContactProfile.js:151-160, components/DecisionDialog.js:188-218, pages/Notifications.js, pages/People.js, pages/Journal.js, pages/Calendar.js; pattern to copy: pages/WorkCoach.js:36-57</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>OP-10, CR-10, CR-11, FN-07, FN-09, DD-01, DD-02, DD-03, CL-01</t>
+        </is>
+      </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
           <t>To do</t>
@@ -22802,50 +22806,54 @@
     <row r="22" ht="82" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>MW-20</t>
+          <t>ASK-21</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>UI audit</t>
+          <t>Founder review</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Task drawer - every click inside closes it</t>
+          <t>One permission map for route, nav and API (root cause 2 of 3)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Bug fix</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
+          <t>Change request</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Stop propagation at the drawer boundary: onClick={(e) =&gt; e.stopPropagation()} and onKeyDown={(e) =&gt; e.stopPropagation()} on SheetContent. Or, better, render the Sheet as a SIBLING of the card root rather than a child, so the drawer is outside the clickable element in the component tree. Also guard the root handler with e.currentTarget.contains(e.target) - that is a DOM check, which a portal click fails. Add the five-click test to the verify script.</t>
+          <t>Define each surface's access rule ONCE - e.g. finance: needs 'finance' or 'ledger'; crm: needs 'people'; ops: everyone (self view); team: everyone (read-only without team_manage) - and have App.js routes, Layout.js nav pills, AllAppsPanel.jsx tiles, the Desk's KPI tiles and the backend require_* guards all read from it. Add a test that walks every role x route and fails if the page opens while its data 403s, or if a nav/tile/link points at a page the role is refused. Decide separately whether data_input-only users get a capture-only Finance.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Every click closes it, on both viewports - 10 of 10. The drawer is now the only place a task can be worked (status, progress, Complete, Attach, Log update, hand off), so none of that is usable. On mobile the status pill tap fired its PATCH before the drawer shut, so the action happens but the user is thrown back to the list without seeing it. Likely also (from the code, not testable while the form cannot be opened): pressing Space or Enter in any drawer field hits the card's onKeyDown, which calls preventDefault and toggles the drawer - so a user could not type a space in an update note.</t>
+          <t>The rules have drifted apart in five places. The Finance route admits data_input but its API needs ledger/finance, so Sales and Production open an empty Finance (FN-07). /crm/outstanding checks nothing and serves per-customer money totals to any signed-in user (CR-12). The Desk links non-CRM roles to Access Denied (CR-13) and fetches ledger data it is refused (DD-03). The mobile More panel hides Ops, Team and Settings that the routes allow (GL-02). Every colleague can read every other colleague's access matrix (TM-05). Each fix done alone will drift again.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:1242-1255 (card root onClick / onKeyDown), the &lt;Sheet&gt; rendered inside the same component (~:1360)</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr"/>
+          <t>App.js:187-254 (Protected perms), components/Layout.js:58-84 (nav perms), components/mobile/AllAppsPanel.jsx:54-128 (tile filters), pages/Desk.js:563-661, lib/perms.js, routers/ledger.py:619-625, routers/crm.py:37-38, routers/finance.py</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>FN-07, CR-12, CR-13, DD-03, GL-02, TM-05; ASK-13, ASK-15</t>
+        </is>
+      </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
           <t>To do</t>
@@ -22855,27 +22863,27 @@
     <row r="23" ht="82" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>MW-09</t>
+          <t>ASK-22</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>UI audit</t>
+          <t>Founder review</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Task card - 'Log update or hand off' (mobile)</t>
+          <t>Phone parity: no desktop-only actions (root cause 3 of 3)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Bug fix</t>
+          <t>Change request</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -22885,20 +22893,24 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Wire it to the same handler its desktop counterpart uses so it opens UpdateForm - and fix MW-08 first, or the newly working button will simply crash the page instead of doing nothing.</t>
+          <t>Adopt a rule: any action available on desktop must have a reachable, tappable (24px+) equivalent below lg, or be deliberately marked desktop-only in the code. Audit every 'hidden lg:*' / 'lg:block' control against it. Immediate cases: Add income / expense / asset / inventory on Finance (FN-08), the CRM add menu and filter (CR-04, CR-05), Score with AI on the contact profile (CR-09), Company / You on the Desk (DD-04), Ops / Team / Settings for staff (GL-02), and a 44px bulk-select checkbox that does not open the task on a near-miss (MW-22).</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Nothing happens at all - no form, no navigation, no error. The button is inert. Combined with MW-08 on desktop, there is no working way to log a task update or hand a task off on either viewport.</t>
+          <t>DecisionOS is used from the owner's phone first, yet six findings are actions that exist on desktop and vanish, clip or shrink on a phone - most often because a control was wrapped in 'hidden lg:block' with no mobile placement. A cash expense with no bill cannot be recorded from a phone at all (FN-08).</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:1496-1505 (log-update-m button, no onClick)</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr"/>
+          <t>pages/Ledger.js:1422-1437, :1630; pages/CRM.js (mobile add + filter); pages/mobile/ContactProfileMobile.jsx; pages/Desk.js:426, :470; components/mobile/AllAppsPanel.jsx; pages/MyWork.js (bulk-select checkbox)</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>FN-08, CR-04, CR-05, CR-09, DD-04, GL-02, MW-22</t>
+        </is>
+      </c>
       <c r="K23" s="7" t="inlineStr">
         <is>
           <t>To do</t>
@@ -22908,7 +22920,7 @@
     <row r="24" ht="82" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>MW-10</t>
+          <t>MW-08</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -22918,12 +22930,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Application shell</t>
+          <t>Task card - Update / Escalate</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -22931,24 +22943,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Add an error boundary around the routed page area - it should show a short apology, a Reload action, and report the error - so a single broken component costs one panel rather than the whole product. Worth a second boundary around the app shell as a backstop.</t>
+          <t>Restyle that one button to the segmented-control treatment the rest of the toolbar moved to in the same commit (kr-pressed / kr-pop, as the priority bands use), or simply restore the two constants. Then stop the class recurring: craco narrows ESLint to react-hooks rules only, which drops eslint-config-react-app's no-undef - the rule that would have failed the build on this exact line.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>One component throwing takes down the entire application. After the MW-08 crash the React root is left with no children, so the user is looking at a blank page with no message and no recovery except a manual reload. Any future render error anywhere will behave the same way.</t>
+          <t>The app CRASHES. A ReferenceError is thrown while rendering the form, the form never appears, and the whole React tree unmounts - the page is gone, not just the form. Recovery needs a reload. The work trail, hand-off and escalation flow is therefore completely unusable.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/App.js (route tree) and components/Layout.js (shell)</t>
+          <t>pages/MyWork.js:147 (UpdateForm); constants removed in 5fb96f2; lint narrowed at craco.config.js:74</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr"/>
@@ -22961,7 +22973,7 @@
     <row r="25" ht="82" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>MW-01</t>
+          <t>MW-20</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -22976,7 +22988,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Task card - status control</t>
+          <t>Task drawer - every click inside closes it</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -22984,24 +22996,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Write the PATCH response straight into the cache instead of trusting the refetch: qc.setQueryData(['tasks', mine], rows =&gt; rows.map(r =&gt; r.id === t.id ? data : r)) using the object the PATCH already returns, then invalidate. That is the standard React Query update-from-response pattern and removes the race entirely. If the refetch must stay authoritative, the list read needs read-your-writes consistency instead.</t>
+          <t>Stop propagation at the drawer boundary: onClick={(e) =&gt; e.stopPropagation()} and onKeyDown={(e) =&gt; e.stopPropagation()} on SheetContent. Or, better, render the Sheet as a SIBLING of the card root rather than a child, so the drawer is outside the clickable element in the component tree. Also guard the root handler with e.currentTarget.contains(e.target) - that is a DOM check, which a portal click fails. Add the five-click test to the verify script.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>The save succeeds (PATCH returns 200 with the new status) and a success toast appears, but the card keeps showing the PREVIOUS status. The list refetch that follows returns the pre-change value, which overwrites the UI. The correct status only appears after a full page reload. Reproduced 8 out of 8 attempts; mobile pills stay unpressed the same way. The progress percentage behaves identically: setting 50% stores 50 on the server while the card still reads 0 until reloaded.</t>
+          <t>Every click closes it, on both viewports - 10 of 10. The drawer is now the only place a task can be worked (status, progress, Complete, Attach, Log update, hand off), so none of that is usable. On mobile the status pill tap fired its PATCH before the drawer shut, so the action happens but the user is thrown back to the list without seeing it. Likely also (from the code, not testable while the form cannot be opened): pressing Space or Enter in any drawer field hits the card's onKeyDown, which calls preventDefault and toggles the drawer - so a user could not type a space in an update note.</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:1127 setStatus / 1134 setProgress; refresh() at 2102</t>
+          <t>pages/MyWork.js:1242-1255 (card root onClick / onKeyDown), the &lt;Sheet&gt; rendered inside the same component (~:1360)</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr"/>
@@ -23014,7 +23026,7 @@
     <row r="26" ht="82" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>MW-02</t>
+          <t>MW-09</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -23029,7 +23041,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Task card - detail dialog</t>
+          <t>Task card - 'Log update or hand off' (mobile)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -23044,17 +23056,17 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Give the card a way in: an overflow / more menu on the summary row, or make the title open details, calling setDetailOpen(true). If the detail dialog is genuinely retired, delete the component and move the Delete action onto the inline expanded card instead - either way a task must be deletable.</t>
+          <t>Wire it to the same handler its desktop counterpart uses so it opens UpdateForm - and fix MW-08 first, or the newly working button will simply crash the page instead of doing nothing.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>There is NO delete control anywhere in My Work, on either viewport, and the task detail dialog never opens. The dialog and its Delete button exist in the code but are unreachable, so the proof gallery, the source-reference panel and the AI insight panel are all dead UI too.</t>
+          <t>Nothing happens at all - no form, no navigation, no error. The button is inert. Combined with MW-08 on desktop, there is no working way to log a task update or hand a task off on either viewport.</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:986 (state), 1837 (render), 737-890 (the dialog + delete)</t>
+          <t>pages/MyWork.js:1496-1505 (log-update-m button, no onClick)</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
@@ -23067,7 +23079,7 @@
     <row r="27" ht="82" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>MW-21</t>
+          <t>MW-10</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -23077,12 +23089,12 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Task - Delete</t>
+          <t>Application shell</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -23097,17 +23109,17 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Put 'Delete task' in the drawer - a quiet destructive button at the foot of the drawer, keeping the existing confirm step - or restore a 'View details' entry. Owner-only, as it was.</t>
+          <t>Add an error boundary around the routed page area - it should show a short apology, a Reload action, and report the error - so a single broken component costs one panel rather than the whole product. Worth a second boundary around the app shell as a backstop.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>There is no way to delete a task. The detail dialog still contains 'Delete task' with its confirmation, but nothing opens that dialog any more. Its only entry point was 'View details' in the card's ••• menu, and 98b43f4 removed that menu on the reasoning that 'the drawer already exposes every detail action' - but the drawer has no Delete.</t>
+          <t>One component throwing takes down the entire application. After the MW-08 crash the React root is left with no children, so the user is looking at a blank page with no message and no recovery except a manual reload. Any future render error anywhere will behave the same way.</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:782-940 (TaskDetailDialog + delete), :1074 and :1941 (detailOpen with no opener)</t>
+          <t>frontend/src/App.js (route tree) and components/Layout.js (shell)</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
@@ -23120,7 +23132,7 @@
     <row r="28" ht="82" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>MW-15</t>
+          <t>MW-01</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -23135,7 +23147,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Task drawer - close (mobile)</t>
+          <t>Task card - status control</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -23150,17 +23162,17 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Below sm, put the close INSIDE the drawer header (a 44px X at the right of the sticky title bar, or a back chevron at its left) and keep the protruding tab for sm and up: e.g. 'right-3 top-3 sm:left-0 sm:right-auto sm:-translate-x-full'. Alternatively leave a strip of scrim on phones (w-[92%]) so tapping outside works. Either way, test on a phone width before shipping a change to the drawer frame.</t>
+          <t>Write the PATCH response straight into the cache instead of trusting the refetch: qc.setQueryData(['tasks', mine], rows =&gt; rows.map(r =&gt; r.id === t.id ? data : r)) using the object the PATCH already returns, then invalidate. That is the standard React Query update-from-response pattern and removes the race entirely. If the refetch must stay authoritative, the list read needs read-your-writes consistency instead.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>There is no way to close it. The drawer is w-full, so it covers the whole screen and there is no scrim left to tap. The new left-edge close tab sits at x=-43, entirely off-screen. The stock Radix close is at top-right but the sticky title bar paints over it - only a sliver of its focus ring peeks out. Escape closes it, but phones have no Escape key. Browser Back does not close the drawer either: it leaves My Work for the previous route. A phone user who opens a task is stuck.</t>
+          <t>The save succeeds (PATCH returns 200 with the new status) and a success toast appears, but the card keeps showing the PREVIOUS status. The list refetch that follows returns the pre-change value, which overwrites the UI. The correct status only appears after a full page reload. Reproduced 8 out of 8 attempts; mobile pills stay unpressed the same way. The progress percentage behaves identically: setting 50% stores 50 on the server while the card still reads 0 until reloaded.</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:1427-1441 (SheetContent w-full + SheetClose -translate-x-full)</t>
+          <t>pages/MyWork.js:1127 setStatus / 1134 setProgress; refresh() at 2102</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
@@ -23173,7 +23185,7 @@
     <row r="29" ht="82" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>MW-16</t>
+          <t>MW-02</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -23188,7 +23200,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Task drawer - 'Log update or hand off' (mobile)</t>
+          <t>Task card - detail dialog</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -23203,17 +23215,17 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Render TaskTrail (or at least its UpdateForm) outside the lg-gated body, shared by both layouts, or mount a second instance inside the mobile body. Add the MW-09 check to the verify script so the next drawer change cannot regress it silently.</t>
+          <t>Give the card a way in: an overflow / more menu on the summary row, or make the title open details, calling setDetailOpen(true). If the detail dialog is genuinely retired, delete the component and move the Delete action onto the inline expanded card instead - either way a task must be deletable.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Nothing appears. The button is visible and tappable, and the form IS mounted - but inside the desktop body, which is display:none below lg. This is MW-09 back: the one control that records what happened is inert on phones again. Desktop is unaffected (form opens, no crash).</t>
+          <t>There is NO delete control anywhere in My Work, on either viewport, and the task detail dialog never opens. The dialog and its Delete button exist in the code but are unreachable, so the proof gallery, the source-reference panel and the AI insight panel are all dead UI too.</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:1658-1662 (mobile trigger), :1679 (desktop body 'hidden lg:block'), :1960 (the only &lt;TaskTrail&gt;)</t>
+          <t>pages/MyWork.js:986 (state), 1837 (render), 737-890 (the dialog + delete)</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
@@ -23226,7 +23238,7 @@
     <row r="30" ht="82" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CR-04</t>
+          <t>MW-21</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -23236,12 +23248,12 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Add contact menu (mobile)</t>
+          <t>Task - Delete</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -23256,17 +23268,17 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Give the popover collision-aware placement so it flips and clamps inside the viewport, or on mobile present the same three choices as a bottom sheet -- the pattern the app already uses elsewhere for phone menus.</t>
+          <t>Put 'Delete task' in the drawer - a quiet destructive button at the foot of the drawer, keeping the existing confirm step - or restore a 'View details' entry. Owner-only, as it was.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Four fifths of the menu is off-screen. It opens anchored to the + button and runs off the right edge, so all the user sees is a 55px strip carrying three anonymous icons -- every label is cut off. 'New Buyer', 'New Supplier' and 'Import from spreadsheet' are all invisible, so adding a contact on a phone means guessing which icon to press.</t>
+          <t>There is no way to delete a task. The detail dialog still contains 'Delete task' with its confirmation, but nothing opens that dialog any more. Its only entry point was 'View details' in the card's ••• menu, and 98b43f4 removed that menu on the reasoning that 'the drawer already exposes every detail action' - but the drawer has no Delete.</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:405-480 (crm-add-menu popover)</t>
+          <t>pages/MyWork.js:782-940 (TaskDetailDialog + delete), :1074 and :1941 (detailOpen with no opener)</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
@@ -23279,7 +23291,7 @@
     <row r="31" ht="82" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>CR-05</t>
+          <t>MW-15</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -23289,12 +23301,12 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Filter button (mobile)</t>
+          <t>Task drawer - close (mobile)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -23309,17 +23321,17 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Wire it to a sheet or popover containing the status filter and sort that desktop shows inline. Both controls already exist and only need somewhere to be shown.</t>
+          <t>Below sm, put the close INSIDE the drawer header (a 44px X at the right of the sticky title bar, or a back chevron at its left) and keep the protruding tab for sm and up: e.g. 'right-3 top-3 sm:left-0 sm:right-auto sm:-translate-x-full'. Alternatively leave a strip of scrim on phones (w-[92%]) so tapping outside works. Either way, test on a phone width before shipping a change to the drawer frame.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Nothing happens at all. Not a single thing changes -- same text, same element count, no dialog, no menu, no sheet. Meanwhile the status filter and the sort control both exist in the DOM at zero size, so on a phone there is no way to filter by status or change the sort order.</t>
+          <t>There is no way to close it. The drawer is w-full, so it covers the whole screen and there is no scrim left to tap. The new left-edge close tab sits at x=-43, entirely off-screen. The stock Radix close is at top-right but the sticky title bar paints over it - only a sliver of its focus ring peeks out. Escape closes it, but phones have no Escape key. Browser Back does not close the drawer either: it leaves My Work for the previous route. A phone user who opens a task is stuck.</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:739 (crm-mobile-filter); the controls it should reveal are at :858 (crm-status-filter) and :869 (crm-sort)</t>
+          <t>pages/MyWork.js:1427-1441 (SheetContent w-full + SheetClose -translate-x-full)</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
@@ -23332,7 +23344,7 @@
     <row r="32" ht="82" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>OP-01</t>
+          <t>MW-16</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -23342,12 +23354,12 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Team execution panel</t>
+          <t>Task drawer - 'Log update or hand off' (mobile)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -23362,17 +23374,17 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Decide which is true and make them agree. A rolling window is the more useful of the two -- an operating score should recover when the business recovers -- so filter each query to the last 30 days and keep the caption. If all-time is deliberate, the caption has to say so.</t>
+          <t>Render TaskTrail (or at least its UpdateForm) outside the lg-gated body, shared by both layouts, or mount a second instance inside the mobile body. Add the MW-09 check to the verify script so the next drawer change cannot regress it silently.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>The panel says 'Last 30 days - open anyone to see their full ops'. The service applies no date filter anywhere: tasks, decisions, invoices and the per-employee leaderboard are all queried for the whole tenant with no window at all. So an owner reads a colleague's score believing it reflects the last month, when it carries every task since the workspace opened -- somebody who was slow in August can never recover from it, and somebody who has improved this month does not show it.</t>
+          <t>Nothing appears. The button is visible and tappable, and the form IS mounted - but inside the desktop body, which is display:none below lg. This is MW-09 back: the one control that records what happened is inert on phones again. Desktop is unaffected (form opens, no crash).</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>services/operating_score.py (all queries); the caption is in pages/OperatingScore.js, team-execution section</t>
+          <t>pages/MyWork.js:1658-1662 (mobile trigger), :1679 (desktop body 'hidden lg:block'), :1960 (the only &lt;TaskTrail&gt;)</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
@@ -23385,7 +23397,7 @@
     <row r="33" ht="82" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>OP-02</t>
+          <t>CR-04</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -23395,12 +23407,12 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>'Do these first' on mobile</t>
+          <t>Add contact menu (mobile)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -23415,17 +23427,17 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>On mobile the band should flow with the page rather than being pinned, so the score, the actions and the team list scroll as one column. If it must stay pinned, it needs to collapse to a handle the user can pull up.</t>
+          <t>Give the popover collision-aware placement so it flips and clamps inside the viewport, or on mobile present the same three choices as a bottom sheet -- the pattern the app already uses elsewhere for phone menus.</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>It is 90 per cent hidden. 'Do these first' occupies y=425 to 710, and a fixed black 'Team execution' band is pinned from y=454 to the bottom of the screen -- 374px, 46 per cent of the viewport -- covering 256 of its 285px. Scrolling does not help: the document itself does not scroll (scrollHeight equals clientHeight), and the element that does scroll is the dark band, not the page. So the three actions the page exists to recommend are permanently reduced to one visible line.</t>
+          <t>Four fifths of the menu is off-screen. It opens anchored to the + button and runs off the right edge, so all the user sees is a 55px strip carrying three anonymous icons -- every label is cut off. 'New Buyer', 'New Supplier' and 'Import from spreadsheet' are all invisible, so adding a contact on a phone means guessing which icon to press.</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>pages/OperatingScore.js (kr-dark-band team-execution section)</t>
+          <t>pages/CRM.js:405-480 (crm-add-menu popover)</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
@@ -23438,7 +23450,7 @@
     <row r="34" ht="82" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>OP-03</t>
+          <t>CR-05</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -23448,12 +23460,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Operating score model</t>
+          <t>Filter button (mobile)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -23468,17 +23480,17 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Score each leg as a bounded rate rather than a penalty subtracted from a constant, so the number always has somewhere to move. Where a leg really is at the floor, say 'below floor' rather than printing a 0 that looks like an empty metric. See ASK-19 for the wider redesign.</t>
+          <t>Wire it to a sheet or popover containing the status filter and sort that desktop shows inline. Both controls already exist and only need somewhere to be shown.</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Two of the four legs are pinned at the floor and carry no information. Execution reads 0 and Responsiveness reads 0. Responsiveness actually computes to -296 before clamping (100 - 16 complaints x 12 - 68 overdue x 3), so it would take closing 8 complaints AND clearing 33 overdue tasks before the number moves off zero by a single point. The page's own advice is 'Close 16 open complaints' -- doing all of that would leave the score exactly where it is. The owner gets no gradient at precisely the moment they most need one.</t>
+          <t>Nothing happens at all. Not a single thing changes -- same text, same element count, no dialog, no menu, no sheet. Meanwhile the status filter and the sort control both exist in the DOM at zero size, so on a phone there is no way to filter by status or change the sort order.</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>services/operating_score.py:_score_execution and the responsiveness expression in _company_operating_view</t>
+          <t>pages/CRM.js:739 (crm-mobile-filter); the controls it should reveal are at :858 (crm-status-filter) and :869 (crm-sort)</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
@@ -23491,7 +23503,7 @@
     <row r="35" ht="82" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>OP-10</t>
+          <t>OP-01</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -23506,7 +23518,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Ops page when the request fails</t>
+          <t>Team execution panel</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -23521,17 +23533,17 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Read isError and error from the query and render a message: 403 -&gt; 'Only the owner can view another person's operating page', 404 -&gt; 'This person is no longer on the team', otherwise 'Couldn't load'. Each with a link to /operating-score. WorkCoach.js:36-57 is the pattern to copy. Also set retry: false for 4xx so the error shows at once.</t>
+          <t>Decide which is true and make them agree. A rolling window is the more useful of the two -- an operating score should recover when the business recovers -- so filter each query to the last 30 days and keep the caption. If all-time is deliberate, the caption has to say so.</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>The loading skeleton stays on screen forever, with aria-busy=true and no text at all. The API answered in milliseconds - 404 'Team member not found' for the owner, 403 for the three other roles - but the page never shows it. The user cannot tell a slow page from a broken link or a refused one, and there is no way back except the browser. Any stale shared link (a person who has left, a link forwarded to a teammate) lands here.</t>
+          <t>The panel says 'Last 30 days - open anyone to see their full ops'. The service applies no date filter anywhere: tasks, decisions, invoices and the per-employee leaderboard are all queried for the whole tenant with no window at all. So an owner reads a colleague's score believing it reflects the last month, when it carries every task since the workspace opened -- somebody who was slow in August can never recover from it, and somebody who has improved this month does not show it.</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>pages/OperatingScore.js:85-92 (useQuery + the skeleton fallback); pages/WorkCoach.js:36-57 (the working pattern)</t>
+          <t>services/operating_score.py (all queries); the caption is in pages/OperatingScore.js, team-execution section</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
@@ -23544,7 +23556,7 @@
     <row r="36" ht="82" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>CR-10</t>
+          <t>OP-02</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -23554,12 +23566,12 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Contact list when loading fails</t>
+          <t>'Do these first' on mobile</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -23574,17 +23586,17 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Read isError from the query and render 'Couldn't load your contacts' with a Retry that calls refetch(). Show '-' rather than 0 in the scope chips while loading or failed. Same fix pattern as OP-10 - worth one shared &lt;QueryError&gt; component.</t>
+          <t>On mobile the band should flow with the page rather than being pinned, so the score, the actions and the team list scroll as one column. If it must stay pinned, it needs to collapse to a handle the user can pull up.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>The loading skeleton stays forever. On desktop the chips read 'Buyers 0' and 'Suppliers 0' above six blank placeholder cards, so an owner with a flaky connection sees what looks like a CRM with no customers, still loading. On mobile it is the same skeleton with nothing else. No toast, no message, no retry. The same fault as OP-10 on Ops.</t>
+          <t>It is 90 per cent hidden. 'Do these first' occupies y=425 to 710, and a fixed black 'Team execution' band is pinned from y=454 to the bottom of the screen -- 374px, 46 per cent of the viewport -- covering 256 of its 285px. Scrolling does not help: the document itself does not scroll (scrollHeight equals clientHeight), and the element that does scroll is the dark band, not the page. So the three actions the page exists to recommend are permanently reduced to one visible line.</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:524-527 (contacts useQuery), scope-count chips :819-835</t>
+          <t>pages/OperatingScore.js (kr-dark-band team-execution section)</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
@@ -23597,7 +23609,7 @@
     <row r="37" ht="82" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>FN-01</t>
+          <t>OP-03</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -23607,12 +23619,12 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Every money figure</t>
+          <t>Operating score model</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -23627,17 +23639,17 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Delete the private fmt() and import inr from lib/format. The helper already exists and already does the right thing, so this is an import swap rather than a rewrite. Worth a lint rule banning Intl.NumberFormat with a currency style outside lib/format.js.</t>
+          <t>Score each leg as a bounded rate rather than a penalty subtracted from a constant, so the number always has somewhere to move. Where a leg really is at the floor, say 'below floor' rather than printing a 0 that looks like an empty metric. See ASK-19 for the wider redesign.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Finance renders 2685000 as Rs 2,685,000 -- Western thousands grouping. Indian convention is Rs 26,85,000. Every tile is affected: Asset Value shows Rs 4,085,000 for what an Indian owner reads as Rs 40,85,000. Worse than being consistently wrong, it is inconsistent: the AI panels ON THE SAME PAGE correctly say 'Rs 7.49L' and 'Rs 13.18 L', and CRM cards elsewhere show 'Rs 4,00,000'. And because the locale is left undefined, the grouping follows each viewer's browser -- the same figure renders differently for different people.</t>
+          <t>Two of the four legs are pinned at the floor and carry no information. Execution reads 0 and Responsiveness reads 0. Responsiveness actually computes to -296 before clamping (100 - 16 complaints x 12 - 68 overdue x 3), so it would take closing 8 complaints AND clearing 33 overdue tasks before the number moves off zero by a single point. The page's own advice is 'Close 16 open complaints' -- doing all of that would leave the score exactly where it is. The owner gets no gradient at precisely the moment they most need one.</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:61-64 (private fmt); lib/format.js:19-30 (inr, and the rule it states)</t>
+          <t>services/operating_score.py:_score_execution and the responsiveness expression in _company_operating_view</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
@@ -23650,7 +23662,7 @@
     <row r="38" ht="82" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>FN-02</t>
+          <t>OP-10</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -23660,12 +23672,12 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Net profit hero (mobile)</t>
+          <t>Ops page when the request fails</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -23680,17 +23692,17 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Either compute a monthly net and show that, or drop the chip. The backend already buckets by month for expenses, so half the machinery exists -- it needs the revenue side to match (see FN-03).</t>
+          <t>Read isError and error from the query and render a message: 403 -&gt; 'Only the owner can view another person's operating page', 404 -&gt; 'This person is no longer on the team', otherwise 'Couldn't load'. Each with a link to /operating-score. WorkCoach.js:36-57 is the pattern to copy. Also set retry: false for 4xx so the error shows at once.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>It is the all-time figure. The hero shows Rs 738,034 beneath a chip reading 'This month', and 738034 is exactly net_profit from the API, which is computed with no date filter over records spanning June to August. So an owner glancing at their phone reads a lifetime number as a monthly one -- and on a money screen that is the kind of mistake that gets acted on.</t>
+          <t>The loading skeleton stays on screen forever, with aria-busy=true and no text at all. The API answered in milliseconds - 404 'Team member not found' for the owner, 403 for the three other roles - but the page never shows it. The user cannot tell a slow page from a broken link or a refused one, and there is no way back except the browser. Any stale shared link (a person who has left, a link forwarded to a teammate) lands here.</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1005 (net), :1042 ('This month' chip), :1048 (the value)</t>
+          <t>pages/OperatingScore.js:85-92 (useQuery + the skeleton fallback); pages/WorkCoach.js:36-57 (the working pattern)</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
@@ -23703,7 +23715,7 @@
     <row r="39" ht="82" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>FN-03</t>
+          <t>CR-10</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -23713,12 +23725,12 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Revenue and Net profit trend badges (mobile)</t>
+          <t>Contact list when loading fails</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -23733,17 +23745,17 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Have ledger_summary return revenue and net per month alongside expenses, and bind each trend to its own series. Until then the honest move is to hide the badges rather than show a number that means something else -- and drop the ?? fallback, which is what let this ship silently.</t>
+          <t>Read isError from the query and render 'Couldn't load your contacts' with a Retry that calls refetch(). Show '-' rather than 0 in the scope chips while loading or failed. Same fix pattern as OP-10 - worth one shared &lt;QueryError&gt; component.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Both trend badges are computed from EXPENSES. The Revenue tile reads 'Rs 2,685,000, down 22.1%' -- but that 22.1% is the month-on-month fall in SPENDING, from Rs 10,77,500 in July to Rs 8,39,469 in August. Revenue did not fall; costs did, which is usually good news being reported in red as bad. The Net profit trend is the same number from the same series.</t>
+          <t>The loading skeleton stays forever. On desktop the chips read 'Buyers 0' and 'Suppliers 0' above six blank placeholder cards, so an owner with a flaky connection sees what looks like a CRM with no customers, still loading. On mobile it is the same skeleton with nothing else. No toast, no message, no retry. The same fault as OP-10 on Ops.</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1009-1015 (months, netPoints, netTrend), :1061 (revenue trend); routers/ledger.py:1237-1245 (by_month is expenses only)</t>
+          <t>pages/CRM.js:524-527 (contacts useQuery), scope-count chips :819-835</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
@@ -23756,7 +23768,7 @@
     <row r="40" ht="82" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>FN-06</t>
+          <t>FN-01</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -23771,7 +23783,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Delete on expenses, invoices and payments</t>
+          <t>Every money figure</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -23786,17 +23798,17 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Put a confirm step in del() and delRevenue(): an AlertDialog naming the record and amount ('Delete invoice SBT/25-26/0431 for Rs 2,85,000?'). Alternatively delete optimistically with an Undo toast and commit after a few seconds. Either way, one tap must not be final.</t>
+          <t>Delete the private fmt() and import inr from lib/format. The helper already exists and already does the right thing, so this is an import swap rather than a rewrite. Worth a lint rule banning Intl.NumberFormat with a currency style outside lib/format.js.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>One tap sends the DELETE straight away. No confirmation dialog, no 'are you sure', no undo toast - for all three record types, both viewports, both roles. The trash icon is a 36px target at the end of each row, so a stray tap while scrolling a phone ledger deletes a real invoice or payment and silently changes Revenue, Received and Net profit. (The harness blocked every DELETE, so nothing was removed.)</t>
+          <t>Finance renders 2685000 as Rs 2,685,000 -- Western thousands grouping. Indian convention is Rs 26,85,000. Every tile is affected: Asset Value shows Rs 4,085,000 for what an Indian owner reads as Rs 40,85,000. Worse than being consistently wrong, it is inconsistent: the AI panels ON THE SAME PAGE correctly say 'Rs 7.49L' and 'Rs 13.18 L', and CRM cards elsewhere show 'Rs 4,00,000'. And because the locale is left undefined, the grouping follows each viewer's browser -- the same figure renders differently for different people.</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1541-1549 (del, delRevenue); :886 and :912 (revenue invoice/payment trash); :1264 (expense trash)</t>
+          <t>pages/Ledger.js:61-64 (private fmt); lib/format.js:19-30 (inr, and the rule it states)</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
@@ -23809,7 +23821,7 @@
     <row r="41" ht="82" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>FN-07</t>
+          <t>FN-02</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -23824,7 +23836,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Finance for Sales and Production</t>
+          <t>Net profit hero (mobile)</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -23839,17 +23851,17 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Decide what data_input-only users should get. If it is capture only, show them the capture bar and Inbox with a line such as 'You can upload bills here; totals are visible to Finance and the Owner', and hide the money tabs. If they should not be here at all, drop data_input from the route and nav perms. In both cases handle 403 in the page (see FN-09).</t>
+          <t>Either compute a monthly net and show that, or drop the chip. The backend already buckets by month for expenses, so half the machinery exists -- it needs the revenue side to match (see FN-03).</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Both roles see Finance in the nav and the Money dock and can open it - then every ledger request is refused (6 x 403). The Overview sits on 'Loading...' forever. Revenue, Expenses, Assets and Inventory each show their empty state ('No expenses yet...'), telling the user the company has no money records rather than that they are not allowed to see them. Only the capture bar works. So the page misinforms rather than refuses.</t>
+          <t>It is the all-time figure. The hero shows Rs 738,034 beneath a chip reading 'This month', and 738034 is exactly net_profit from the API, which is computed with no date filter over records spanning June to August. So an owner glancing at their phone reads a lifetime number as a monthly one -- and on a money screen that is the kind of mistake that gets acted on.</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>App.js:237 (route perms); components/Layout.js:79 (nav perms); routers/ledger.py:619-625 (require_ledger); pages/Ledger.js:1522-1527 (queries without isError), :1641-1642 (Loading...)</t>
+          <t>pages/Ledger.js:1005 (net), :1042 ('This month' chip), :1048 (the value)</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
@@ -23862,7 +23874,7 @@
     <row r="42" ht="82" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>FN-08</t>
+          <t>FN-03</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -23877,7 +23889,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Adding records on a phone</t>
+          <t>Revenue and Net profit trend badges (mobile)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -23892,17 +23904,17 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Render the per-tab Add button on mobile too (drop hidden lg:block, or add a mobile placement), and have the tile open AddExpenseDialog directly through state rather than clicking a DOM node by testid.</t>
+          <t>Have ledger_summary return revenue and net per month alongside expenses, and bind each trend to its own series. Until then the honest move is to hide the badges rather than show a number that means something else -- and drop the ?? fallback, which is what let this ship silently.</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>There is no way to add a record manually on a phone. The four Add buttons (Add income / expense / asset / inventory) are rendered but hidden below lg. The 'Add expense' tile in 'Simplify your finances' does nothing on any tab: it looks for an element that does not exist. Upload and scan still work, so a cash expense with no bill cannot be recorded from the phone at all.</t>
+          <t>Both trend badges are computed from EXPENSES. The Revenue tile reads 'Rs 2,685,000, down 22.1%' -- but that 22.1% is the month-on-month fall in SPENDING, from Rs 10,77,500 in July to Rs 8,39,469 in August. Revenue did not fall; costs did, which is usually good news being reported in red as bad. The Net profit trend is the same number from the same series.</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1422-1429 (tile + querySelector), :1630 ('hidden lg:block' addBtn), :1551-1557 (addBtn per tab)</t>
+          <t>pages/Ledger.js:1009-1015 (months, netPoints, netTrend), :1061 (revenue trend); routers/ledger.py:1237-1245 (by_month is expenses only)</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr"/>
@@ -23915,7 +23927,7 @@
     <row r="43" ht="82" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>DD-01</t>
+          <t>FN-06</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -23925,12 +23937,12 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Decision Desk</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>/decisions/:id - missing or not yours</t>
+          <t>Delete on expenses, invoices and payments</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -23945,17 +23957,17 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Give the error branch a 'Back to Decision Desk' button (and the same close control). Branch the copy on status: 403 -&gt; no access, 404 -&gt; 'This decision no longer exists', otherwise 'Couldn't load - Retry'.</t>
+          <t>Put a confirm step in del() and delRevenue(): an AlertDialog naming the record and amount ('Delete invoice SBT/25-26/0431 for Rs 2,85,000?'). Alternatively delete optimistically with an Undo toast and commit after a few seconds. Either way, one tap must not be final.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Full-screen 'Access restricted - You don't have access to this decision.' with no Close, no Back and no link. Escape and outside taps are deliberately ignored on the page variant, so the user is trapped until they find the browser Back button. The message is also wrong for a missing decision (the API said 404 'Not found') and for a network error. Decisions are opened from notifications and pasted links, so this is where stale links land.</t>
+          <t>One tap sends the DELETE straight away. No confirmation dialog, no 'are you sure', no undo toast - for all three record types, both viewports, both roles. The trash icon is a 36px target at the end of each row, so a stray tap while scrolling a phone ledger deletes a real invoice or payment and silently changes Revenue, Received and Net profit. (The harness blocked every DELETE, so nothing was removed.)</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>components/DecisionDialog.js:188-218 (error branch, page variant handlers)</t>
+          <t>pages/Ledger.js:1541-1549 (del, delRevenue); :886 and :912 (revenue invoice/payment trash); :1264 (expense trash)</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
@@ -23968,7 +23980,7 @@
     <row r="44" ht="82" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>DD-02</t>
+          <t>FN-07</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -23978,12 +23990,12 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Decision Desk</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Desk board when loading fails</t>
+          <t>Finance for Sales and Production</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -23998,17 +24010,17 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Check isError on the board queries; render 'Couldn't load your desk - Retry' and keep counts as '-' rather than 0. Same shared &lt;QueryError&gt; as OP-10 / CR-10 / FN-09.</t>
+          <t>Decide what data_input-only users should get. If it is capture only, show them the capture bar and Inbox with a line such as 'You can upload bills here; totals are visible to Finance and the Owner', and hide the money tabs. If they should not be here at all, drop data_input from the route and nav perms. In both cases handle 403 in the page (see FN-09).</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>It says 'Nothing waiting on you' with Needs your decision 0, On fire 0, Due today 0, Important 0. The real counts at the time were 53 decisions and 58 on fire. An owner on a weak connection is told the desk is clear.</t>
+          <t>Both roles see Finance in the nav and the Money dock and can open it - then every ledger request is refused (6 x 403). The Overview sits on 'Loading...' forever. Revenue, Expenses, Assets and Inventory each show their empty state ('No expenses yet...'), telling the user the company has no money records rather than that they are not allowed to see them. Only the capture bar works. So the page misinforms rather than refuses.</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>pages/Desk.js:284-292 (boardQs + zero counters)</t>
+          <t>App.js:237 (route perms); components/Layout.js:79 (nav perms); routers/ledger.py:619-625 (require_ledger); pages/Ledger.js:1522-1527 (queries without isError), :1641-1642 (Loading...)</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
@@ -24021,7 +24033,7 @@
     <row r="45" ht="82" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>MW-03</t>
+          <t>FN-08</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -24031,12 +24043,12 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Header - global search (Cmd+K)</t>
+          <t>Adding records on a phone</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -24044,24 +24056,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Inside CommandDialog, wrap a DialogTitle (and a DialogDescription) in the VisuallyHidden primitive so the dialog is named for assistive tech without changing the visual design.</t>
+          <t>Render the per-tab Add button on mobile too (drop hidden lg:block, or add a mobile placement), and have the tile open AddExpenseDialog directly through state rather than clicking a DOM node by testid.</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>The dialog exposes aria-labelledby pointing at an element id that does not exist, so it is announced with no name. Radix logs an error every time it opens. Reproduces on My Work and on Finance, so it affects every screen.</t>
+          <t>There is no way to add a record manually on a phone. The four Add buttons (Add income / expense / asset / inventory) are rendered but hidden below lg. The 'Add expense' tile in 'Simplify your finances' does nothing on any tab: it looks for an element that does not exist. Upload and scan still work, so a cash expense with no bill cannot be recorded from the phone at all.</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>components/ui/command.jsx:19 (used at components/Layout.js:599)</t>
+          <t>pages/Ledger.js:1422-1429 (tile + querySelector), :1630 ('hidden lg:block' addBtn), :1551-1557 (addBtn per tab)</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
@@ -24074,7 +24086,7 @@
     <row r="46" ht="82" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>MW-04</t>
+          <t>DD-01</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -24084,12 +24096,12 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Decision Desk</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Dex FAB picker (mobile)</t>
+          <t>/decisions/:id - missing or not yours</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -24097,24 +24109,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F46" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Close the picker on Escape - either a keydown listener while picker is open, or render it inside a Radix DismissableLayer / Popover so dismissal, focus trapping and aria come from the same primitive the other sheets already use.</t>
+          <t>Give the error branch a 'Back to Decision Desk' button (and the same close control). Branch the copy on status: 403 -&gt; no access, 404 -&gt; 'This decision no longer exists', otherwise 'Couldn't load - Retry'.</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Escape does nothing - the menu stays open and its full-screen scrim keeps blocking the page underneath. Only a pointer tap outside closes it. There is also no focus trap, so keyboard focus walks behind the open menu.</t>
+          <t>Full-screen 'Access restricted - You don't have access to this decision.' with no Close, no Back and no link. Escape and outside taps are deliberately ignored on the page variant, so the user is trapped until they find the browser Back button. The message is also wrong for a missing decision (the API said 404 'Not found') and for a network error. Decisions are opened from notifications and pasted links, so this is where stale links land.</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>components/mobile/DexFab.jsx:70-82</t>
+          <t>components/DecisionDialog.js:188-218 (error branch, page variant handlers)</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
@@ -24127,7 +24139,7 @@
     <row r="47" ht="82" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>MW-11</t>
+          <t>DD-02</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -24137,12 +24149,12 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Decision Desk</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Toolbar in the Leave / Workflows views</t>
+          <t>Desk board when loading fails</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -24150,24 +24162,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Render the task-scope controls only while view === 'mywork'. Leave the view toggle itself (Workflows / Leave) in place, since that is how you get back. If a scope control must stay, it should not silently change view - that side effect is what makes it feel broken.</t>
+          <t>Check isError on the board queries; render 'Couldn't load your desk - Retry' and keep counts as '-' rather than 0. Same shared &lt;QueryError&gt; as OP-10 / CR-10 / FN-09.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Four task-only controls stay visible in both views - New Task, My Tasks, All Tasks and AI Priority - none of which mean anything for leave or for pipelines. Worse, pressing My Tasks, All Tasks or AI Priority silently throws you back to the task list, losing the view you were in with no warning. In the Leave view 'New Task' is also the largest, darkest button on screen, and it creates a task, not a leave request.</t>
+          <t>It says 'Nothing waiting on you' with Needs your decision 0, On fire 0, Due today 0, Important 0. The real counts at the time were 53 decisions and 58 on fire. An owner on a weak connection is told the desk is clear.</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:2429-2515 (mywork-controls / work-view-toggle); handlers at 2442, 2448, 2463</t>
+          <t>pages/Desk.js:284-292 (boardQs + zero counters)</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr"/>
@@ -24180,7 +24192,7 @@
     <row r="48" ht="82" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>MW-12</t>
+          <t>MW-03</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -24190,12 +24202,12 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Leave and Workflows entry points</t>
+          <t>Header - global search (Cmd+K)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -24210,17 +24222,17 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Pick one home per feature and use it on both viewports. Given Leave already has its own route and its own mobile tile, the cheaper and more consistent direction is to make the standalone page the home on desktop too - see the note on MW-11 about how little of Leave actually belongs in My Work.</t>
+          <t>Inside CommandDialog, wrap a DialogTitle (and a DialogDescription) in the VisuallyHidden primitive so the dialog is named for assistive tech without changing the visual design.</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Neither toggle is reachable on mobile - both are in the DOM but hidden, so from My Work there is no way into Leave or Workflows on a phone. They are reachable, but from somewhere else entirely: the 'More' panel lists them as their own destinations. So the same two features are sub-views of My Work on desktop and separate destinations on mobile.</t>
+          <t>The dialog exposes aria-labelledby pointing at an element id that does not exist, so it is announced with no name. Radix logs an error every time it opens. Reproduces on My Work and on Finance, so it affects every screen.</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:2476 (work-view-toggle); components/mobile/AllAppsPanel.jsx</t>
+          <t>components/ui/command.jsx:19 (used at components/Layout.js:599)</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
@@ -24233,7 +24245,7 @@
     <row r="49" ht="82" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>MW-17</t>
+          <t>MW-04</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -24243,12 +24255,12 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Task drawer - two close buttons, invisible focus</t>
+          <t>Dex FAB picker (mobile)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -24263,17 +24275,17 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Give SheetContent a hideClose prop (default false, so other sheets are unchanged) and pass it here; set onOpenAutoFocus to focus the title or the close tab. That also resolves which close MW-15 should keep.</t>
+          <t>Close the picker on Escape - either a keydown listener while picker is open, or render it inside a Radix DismissableLayer / Popover so dismissal, focus trapping and aria come from the same primitive the other sheets already use.</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Every drawer carries TWO close buttons: the new 'Close task' tab and the stock shadcn 'Close' that SheetContent always renders. The stock one is covered by the sticky title bar, yet Radix focuses it on open - so keyboard focus starts on a control nobody can see, and a screen reader announces 'Close' and 'Close task' as two separate buttons.</t>
+          <t>Escape does nothing - the menu stays open and its full-screen scrim keeps blocking the page underneath. Only a pointer tap outside closes it. There is also no focus trap, so keyboard focus walks behind the open menu.</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>components/ui/sheet.jsx:46-58; pages/MyWork.js:1427-1445</t>
+          <t>components/mobile/DexFab.jsx:70-82</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr"/>
@@ -24286,7 +24298,7 @@
     <row r="50" ht="82" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>MW-18</t>
+          <t>MW-11</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -24296,12 +24308,12 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Application shell at wide widths</t>
+          <t>Toolbar in the Leave / Workflows views</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -24316,17 +24328,17 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Restore the cap in Layout and lift it only where wanted: give My Work its own page-level wrapper (or a data-wide flag the shell reads). If wider is wanted everywhere, cap at ~1600px rather than none, and constrain the Finance tiles and AI brief rows internally.</t>
+          <t>Render the task-scope controls only while view === 'mywork'. Leave the view toggle itself (Workflows / Leave) in place, since that is how you get back. If a scope control must stay, it should not silently change view - that side effect is what makes it feel broken.</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>The cap was removed in the shared Layout, so EVERY page now runs edge-to-edge. On Finance each KPI tile is ~610px wide with its value at the far left and its arrow ~550px away; the Capture bar is 1,856px wide holding three small buttons; AI brief rows put the 'Urgent' tag ~1,700px from the sentence it qualifies. On Team each member card is ~610px wide with the name and '6 permissions' at opposite ends. Nothing overflows - it just reads as sparse and makes the eye travel.</t>
+          <t>Four task-only controls stay visible in both views - New Task, My Tasks, All Tasks and AI Priority - none of which mean anything for leave or for pipelines. Worse, pressing My Tasks, All Tasks or AI Priority silently throws you back to the task list, losing the view you were in with no warning. In the Leave view 'New Task' is also the largest, darkest button on screen, and it creates a task, not a leave request.</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>components/Layout.js:634 (app-shell className)</t>
+          <t>pages/MyWork.js:2429-2515 (mywork-controls / work-view-toggle); handlers at 2442, 2448, 2463</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
@@ -24339,7 +24351,7 @@
     <row r="51" ht="82" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>TM-05</t>
+          <t>MW-12</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -24349,12 +24361,12 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Member profile - ACCESS block</t>
+          <t>Leave and Workflows entry points</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -24369,17 +24381,17 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Gate the whole ACCESS section, not just its button. This is the same change the founder asked for in ASK-13 and ASK-15, so treat them as one piece of work: hide access on the roster, and show the section only to people who hold the permission that governs it.</t>
+          <t>Pick one home per feature and use it on both viewports. Given Leave already has its own route and its own mobile tile, the cheaper and more consistent direction is to make the standalone page the home on desktop too - see the note on MW-11 about how little of Leave actually belongs in My Work.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Every role can read every other member's complete permission matrix. Production and Finance -- who hold neither team_manage nor people -- can open Priya Nair's card and see '6 permissions', then inside: '6 of 14 areas', the granted chips, and the full denial list naming every area she cannot reach. Only the Edit access BUTTON is gated to the owner; viewing is not gated at all.</t>
+          <t>Neither toggle is reachable on mobile - both are in the DOM but hidden, so from My Work there is no way into Leave or Workflows on a phone. They are reachable, but from somewhere else entirely: the 'More' panel lists them as their own destinations. So the same two features are sub-views of My Work on desktop and separate destinations on mobile.</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:411 + :441 (card count), :580-606 (ACCESS block, granted-perms and the denial list)</t>
+          <t>pages/MyWork.js:2476 (work-view-toggle); components/mobile/AllAppsPanel.jsx</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
@@ -24392,7 +24404,7 @@
     <row r="52" ht="82" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>TM-06</t>
+          <t>MW-17</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -24402,12 +24414,12 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Add member - all form fields</t>
+          <t>Task drawer - two close buttons, invisible focus</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -24422,17 +24434,17 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Give all six a real label with htmlFor pointing at the input's id. Keep placeholders for examples ('e.g. 98765 43210'), not for the field name. This is part of the ASK-14 redesign but is worth doing even if that redesign is deferred -- it is a few lines and it is the difference between the form being usable with a screen reader and not.</t>
+          <t>Give SheetContent a hideClose prop (default false, so other sheets are unchanged) and pass it here; set onOpenAutoFocus to focus the title or the close tab. That also resolves which close MW-15 should keep.</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Not one of the six fields has a programmatic label. Name, Email, Temp password and Mobile number are placeholder-only, so the field name disappears the moment anything is typed -- a sighted user who tabs away and back cannot tell which box is which. Role and Reporting Manager LOOK labelled, but their text is not associated with the control, so a screen reader gets nothing from them either.</t>
+          <t>Every drawer carries TWO close buttons: the new 'Close task' tab and the stock shadcn 'Close' that SheetContent always renders. The stock one is covered by the sticky title bar, yet Radix focuses it on open - so keyboard focus starts on a control nobody can see, and a screen reader announces 'Close' and 'Close task' as two separate buttons.</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:120, :121, :129, :132 (placeholder-only), :137-138 and :143-144 (unassociated labels)</t>
+          <t>components/ui/sheet.jsx:46-58; pages/MyWork.js:1427-1445</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
@@ -24445,7 +24457,7 @@
     <row r="53" ht="82" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>CR-02</t>
+          <t>MW-18</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -24455,12 +24467,12 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Add contact dialog - all fields</t>
+          <t>Application shell at wide widths</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -24475,17 +24487,17 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Associate a real label with every field here and in Team's Add member (TM-06). Worth doing as one pass over both dialogs rather than twice, and worth adding a lint rule or a test so the next form starts labelled.</t>
+          <t>Restore the cap in Layout and lift it only where wanted: give My Work its own page-level wrapper (or a data-wide flag the shell reads). If wider is wanted everywhere, cap at ~1600px rather than none, and constrain the Finance tiles and AI brief rows internally.</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>None of the six fields has a label of any kind - the dialog contains no label elements at all. Name, Company, Phone and Email are placeholder-only, and the two selects have nothing naming them. This is the same defect as TM-06 in Team, in a different dialog, which makes it a pattern across the app rather than a one-off.</t>
+          <t>The cap was removed in the shared Layout, so EVERY page now runs edge-to-edge. On Finance each KPI tile is ~610px wide with its value at the far left and its arrow ~550px away; the Capture bar is 1,856px wide holding three small buttons; AI brief rows put the 'Urgent' tag ~1,700px from the sentence it qualifies. On Team each member card is ~610px wide with the name and '6 permissions' at opposite ends. Nothing overflows - it just reads as sparse and makes the eye travel.</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:282 (crm-contact-name), :313 (lifecycle), and the four unlabelled inputs between them</t>
+          <t>components/Layout.js:634 (app-shell className)</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
@@ -24498,7 +24510,7 @@
     <row r="54" ht="82" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>CR-06</t>
+          <t>TM-05</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -24508,12 +24520,12 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Contact cards (mobile)</t>
+          <t>Member profile - ACCESS block</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -24528,17 +24540,17 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Go single column under about 480px, matching Team. If two columns are wanted on larger phones, drop the company line and the touched line to keep the name whole.</t>
+          <t>Gate the whole ACCESS section, not just its button. This is the same change the founder asked for in ASK-13 and ASK-15, so treat them as one piece of work: hide access on the roster, and show the section only to people who hold the permission that governs it.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>The grid stays two columns on a 375px screen, giving each card 161px. Eight text nodes truncate as a result, including the customer names themselves -- 'Krishna Garments Pvt Ltd' needs 144px and gets 114, 'Anand Fabrics' needs 88 and gets 76. Supporting lines like '6 open complaints' and 'Touched 29 days ago' wrap onto two lines, and the card heights go ragged. Team's roster drops to a single column on the same screen and reads cleanly, so the app already has the better answer.</t>
+          <t>Every role can read every other member's complete permission matrix. Production and Finance -- who hold neither team_manage nor people -- can open Priya Nair's card and see '6 permissions', then inside: '6 of 14 areas', the granted chips, and the full denial list naming every area she cannot reach. Only the Edit access BUTTON is gated to the owner; viewing is not gated at all.</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:940-1050 (contact card grid)</t>
+          <t>pages/Team.js:411 + :441 (card count), :580-606 (ACCESS block, granted-perms and the denial list)</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
@@ -24551,7 +24563,7 @@
     <row r="55" ht="82" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>CR-08</t>
+          <t>TM-06</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -24561,12 +24573,12 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Contact profile (mobile) - In progress list</t>
+          <t>Add member - all form fields</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -24581,17 +24593,17 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Guard on the value, not on the humaniser: render the human date when there is one, the raw date only when the value exists but will not parse, and nothing at all when there is no date. Worth grepping for the same `|| \`... ${value}\`` shape elsewhere -- this pattern fails the same way wherever it appears.</t>
+          <t>Give all six a real label with htmlFor pointing at the input's id. Keep placeholders for examples ('e.g. 98765 43210'), not for the field name. This is part of the ASK-14 redesign but is worth doing even if that redesign is deferred -- it is a few lines and it is the difference between the form being usable with a screen reader and not.</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>The literal word 'undefined' is printed to the user: two rows read 'Due undefined - Rs 1' and 'Due undefined - Rs 6,00,000'. It is the kind of thing a customer screenshots.</t>
+          <t>Not one of the six fields has a programmatic label. Name, Email, Temp password and Mobile number are placeholder-only, so the field name disappears the moment anything is typed -- a sighted user who tabs away and back cannot tell which box is which. Role and Reporting Manager LOOK labelled, but their text is not associated with the control, so a screen reader gets nothing from them either.</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>pages/mobile/ContactProfileMobile.jsx:215 (fallback), :24 (humanDate)</t>
+          <t>pages/Team.js:120, :121, :129, :132 (placeholder-only), :137-138 and :143-144 (unassociated labels)</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr"/>
@@ -24604,7 +24616,7 @@
     <row r="56" ht="82" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>OP-04</t>
+          <t>CR-02</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -24614,12 +24626,12 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>'Sales' category</t>
+          <t>Add contact dialog - all fields</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -24634,17 +24646,17 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Rename it to what it measures -- Decision velocity, or Approvals -- which is a genuinely good metric for a decision OS. If a real Sales leg is wanted, invoices already carry the data for revenue this period against last.</t>
+          <t>Associate a real label with every field here and in Team's Add member (TM-06). Worth doing as one pass over both dialogs rather than twice, and worth adding a lint rule or a test so the next form starts labelled.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>It is the share of DECISIONS that have been approved -- approved/total x 100 -- and contains no revenue, no orders, no pipeline and no customer. On live data it reads 22 because 17 of 77 decisions are approved. An owner could sell nothing all month and lift 'Sales' by approving decisions, or have a record month and watch it fall because approvals are backed up. The number is real and useful; the label is the wrong one.</t>
+          <t>None of the six fields has a label of any kind - the dialog contains no label elements at all. Name, Company, Phone and Email are placeholder-only, and the two selects have nothing naming them. This is the same defect as TM-06 in Team, in a different dialog, which makes it a pattern across the app rather than a one-off.</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>services/operating_score.py:_score_sales</t>
+          <t>pages/CRM.js:282 (crm-contact-name), :313 (lifecycle), and the four unlabelled inputs between them</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr"/>
@@ -24657,7 +24669,7 @@
     <row r="57" ht="82" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>OP-05</t>
+          <t>CR-06</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -24667,12 +24679,12 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Operating score model</t>
+          <t>Contact cards (mobile)</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -24687,17 +24699,17 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Pick one home for lateness. Execution is the natural one; Responsiveness should be about complaints and reply time, which is what its name promises.</t>
+          <t>Go single column under about 480px, matching Team. If two columns are wanted on larger phones, drop the company line and the touched line to keep the name whole.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>One overdue task is charged twice: it raises the overdue ratio inside Execution (x40 of the ratio) and is also subtracted directly from Responsiveness (x3 per task). Those two legs are 35 and 20 per cent of the overall score, so lateness quietly drives 55 per cent of it. On the live tenant that is -20.9 on one leg and -204 on the other.</t>
+          <t>The grid stays two columns on a 375px screen, giving each card 161px. Eight text nodes truncate as a result, including the customer names themselves -- 'Krishna Garments Pvt Ltd' needs 144px and gets 114, 'Anand Fabrics' needs 88 and gets 76. Supporting lines like '6 open complaints' and 'Touched 29 days ago' wrap onto two lines, and the card heights go ragged. Team's roster drops to a single column on the same screen and reads cleanly, so the app already has the better answer.</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>services/operating_score.py:_score_execution and _company_operating_view</t>
+          <t>pages/CRM.js:940-1050 (contact card grid)</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr"/>
@@ -24710,7 +24722,7 @@
     <row r="58" ht="82" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>OP-06</t>
+          <t>CR-08</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -24720,12 +24732,12 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Operating score model</t>
+          <t>Contact profile (mobile) - In progress list</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -24740,17 +24752,17 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Express each as a rate against the relevant denominator -- complaints per active customer, overdue as a share of open work, overdue invoices as a share of open invoices -- so the score means the same thing at any size.</t>
+          <t>Guard on the value, not on the humaniser: render the human date when there is one, the raw date only when the value exists but will not parse, and nothing at all when there is no date. Worth grepping for the same `|| \`... ${value}\`` shape elsewhere -- this pattern fails the same way wherever it appears.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Three penalties are absolute rather than proportional: complaints x12, overdue x3, overdue invoices x5. A five-person shop with 9 open complaints scores 0 on Responsiveness; so does a 500-person company with 9. As a tenant grows, the score falls for reasons that have nothing to do with how well it is run, and the metric stops being comparable with its own past.</t>
+          <t>The literal word 'undefined' is printed to the user: two rows read 'Due undefined - Rs 1' and 'Due undefined - Rs 6,00,000'. It is the kind of thing a customer screenshots.</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>services/operating_score.py:_company_operating_view</t>
+          <t>pages/mobile/ContactProfileMobile.jsx:215 (fallback), :24 (humanDate)</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr"/>
@@ -24763,7 +24775,7 @@
     <row r="59" ht="82" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>OP-09</t>
+          <t>OP-04</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -24778,7 +24790,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>'View all' links and the formula panel (mobile)</t>
+          <t>'Sales' category</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -24793,17 +24805,17 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Fixing OP-02 -- letting the page scroll as one column on mobile -- makes the formula panel reachable on its own. The View all links still need to grow to 24px minimum and to sit clear of the Dex button's safe area.</t>
+          <t>Rename it to what it measures -- Decision velocity, or Approvals -- which is a genuinely good metric for a decision OS. If a real Sales leg is wanted, invoices already carry the data for revenue this period against last.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Three problems, all downstream of the page not scrolling on mobile. The two 'View all' links measure 61x20, under the 24px minimum, and the first of them is physically covered by the floating Dex button. The 'How is this calculated' formula panel sits at y=1153 on an 812px screen and cannot be reached at all, so the one place that explains where the score comes from is invisible on a phone -- which matters more than usual here, given two of the four legs read 0.</t>
+          <t>It is the share of DECISIONS that have been approved -- approved/total x 100 -- and contains no revenue, no orders, no pipeline and no customer. On live data it reads 22 because 17 of 77 decisions are approved. An owner could sell nothing all month and lift 'Sales' by approving decisions, or have a record month and watch it fall because approvals are backed up. The number is real and useful; the label is the wrong one.</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>pages/OperatingScore.js (View all links, operating-formula-toggle)</t>
+          <t>services/operating_score.py:_score_sales</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr"/>
@@ -24816,7 +24828,7 @@
     <row r="60" ht="82" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>OP-11</t>
+          <t>OP-05</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -24831,7 +24843,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Personal (self) view - bottom band (mobile)</t>
+          <t>Operating score model</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -24846,17 +24858,17 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Keep KM-33 for the owner view. In the self view, drop the kr-dark-band class (or add a variant that stays in the scroll flow) and show the peer ranking as an ordinary line or card above the open work. If a pinned sheet is wanted here, it needs content worth pinning and bottom padding that clears the dock.</t>
+          <t>Pick one home for lateness. Execution is the natural one; Responsiveness should be about complaints and reply time, which is what its name promises.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>A 176px near-black band is pinned to the bottom of every non-owner's phone screen - over a fifth of the viewport - and it holds ONE sentence: 'Among your sales peers you are ranked 2 of 7.' That sentence sits behind the floating dock, so it is only partly readable, and the band does not move when the page scrolls. It reads as a black rendering fault rather than a panel.</t>
+          <t>One overdue task is charged twice: it raises the overdue ratio inside Execution (x40 of the ratio) and is also subtracted directly from Responsiveness (x3 per task). Those two legs are 35 and 20 per cent of the overall score, so lateness quietly drives 55 per cent of it. On the live tenant that is -20.9 on one leg and -204 on the other.</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>pages/OperatingScore.js (operating-self-band section); index.css:2171-2190 (.kr-dark-band fixed below lg, KM-33)</t>
+          <t>services/operating_score.py:_score_execution and _company_operating_view</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr"/>
@@ -24869,7 +24881,7 @@
     <row r="61" ht="82" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>OP-12</t>
+          <t>OP-06</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -24884,7 +24896,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>AI Work Coach - entry point</t>
+          <t>Operating score model</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -24899,17 +24911,17 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Add 'AI coach' next to 'Back to company' in the view-as banner (owner coaching a teammate), and 'My AI coach' on the self view and in the More panel. If the coach is being retired, remove the route and its endpoints instead of leaving it reachable only by URL.</t>
+          <t>Express each as a rate against the relevant denominator -- complaints per active customer, overdue as a share of open work, overdue invoices as a share of open invoices -- so the score means the same thing at any size.</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Nothing in the app links to the AI Work Coach. It still works - it loads for all four roles, the owner can open a teammate's coach, the permission message is right - but the only way in is typing /coach. On 2026-09-12 the Ops employee card opened the coach (plan item D3); it now opens that person's Ops page instead, which removed the last route in. Two of the four demo seats already have coaching generated on 29 Aug, so this is a feature people used.</t>
+          <t>Three penalties are absolute rather than proportional: complaints x12, overdue x3, overdue invoices x5. A five-person shop with 9 open complaints scores 0 on Responsiveness; so does a 500-person company with 9. As a tenant grows, the score falls for reasons that have nothing to do with how well it is run, and the metric stops being comparable with its own past.</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>App.js:228 (/coach route); pages/OperatingScore.js:931 (employee card link); pages/OperatingScore.js:119-141 (ViewAsBanner)</t>
+          <t>services/operating_score.py:_company_operating_view</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr"/>
@@ -24922,7 +24934,7 @@
     <row r="62" ht="82" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>CR-11</t>
+          <t>OP-09</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -24932,12 +24944,12 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Contact profile when loading fails</t>
+          <t>'View all' links and the formula panel (mobile)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -24952,17 +24964,17 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Split the branch: if error has no response (network) or a 5xx, say 'Couldn't load this contact' with Retry; keep the 'isn't here' copy for a 404 or an empty body.</t>
+          <t>Fixing OP-02 -- letting the page scroll as one column on mobile -- makes the formula panel reachable on its own. The View all links still need to grow to 24px minimum and to sit clear of the Dex button's safe area.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>The page says 'That contact isn't here. It may have been merged or removed.' The customer exists; only the request failed. An owner reading this on a weak phone signal is told a real customer has been deleted or merged.</t>
+          <t>Three problems, all downstream of the page not scrolling on mobile. The two 'View all' links measure 61x20, under the 24px minimum, and the first of them is physically covered by the floating Dex button. The 'How is this calculated' formula panel sits at y=1153 on an 812px screen and cannot be reached at all, so the one place that explains where the score comes from is invisible on a phone -- which matters more than usual here, given two of the four legs read 0.</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>pages/ContactProfile.js:151-160; pages/mobile/ContactProfileMobile.jsx:85-99</t>
+          <t>pages/OperatingScore.js (View all links, operating-formula-toggle)</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr"/>
@@ -24975,7 +24987,7 @@
     <row r="63" ht="82" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>CR-12</t>
+          <t>OP-11</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -24985,12 +24997,12 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>GET /api/crm/outstanding</t>
+          <t>Personal (self) view - bottom band (mobile)</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -25005,17 +25017,17 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Gate it with require_perm('people') (it only feeds the CRM grid) or require_perm('finance') to match the profile endpoint.</t>
+          <t>Keep KM-33 for the owner view. In the self view, drop the kr-dark-band class (or add a variant that stays in the scroll flow) and show the peer ranking as an ordinary line or card above the open work. If a pinned sheet is wanted here, it needs content worth pinning and bottom padding that clears the dock.</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>GET /api/contacts and GET /api/contacts/&lt;id&gt;/profile correctly refuse Sales with 403 - but GET /api/crm/outstanding answers 200 with every customer's receivables, payables, invoice count and days overdue. The keys are contact ids rather than names, so it is not a full leak on its own, but it hands money data to roles the rest of the app deliberately keeps out of finance.</t>
+          <t>A 176px near-black band is pinned to the bottom of every non-owner's phone screen - over a fifth of the viewport - and it holds ONE sentence: 'Among your sales peers you are ranked 2 of 7.' That sentence sits behind the floating dock, so it is only partly readable, and the band does not move when the page scrolls. It reads as a black rendering fault rather than a panel.</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>routers/crm.py:37-38 (outstanding_by_contact, Depends(get_current_user))</t>
+          <t>pages/OperatingScore.js (operating-self-band section); index.css:2171-2190 (.kr-dark-band fixed below lg, KM-33)</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr"/>
@@ -25028,7 +25040,7 @@
     <row r="64" ht="82" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>FN-04</t>
+          <t>OP-12</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -25038,12 +25050,12 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>'Net profit' tile</t>
+          <t>AI Work Coach - entry point</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -25058,17 +25070,17 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Rename to something the formula actually supports -- 'Billed minus spend', or 'Gross margin (billed)' -- or compute a real net that accounts for COGS and inventory. The former is a one-line change and stops the page overclaiming.</t>
+          <t>Add 'AI coach' next to 'Back to company' in the view-as banner (owner coaching a teammate), and 'My AI coach' on the self view and in the More panel. If the coach is being retired, remove the route and its endpoints instead of leaving it reachable only by URL.</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>It is revenue BILLED minus ALL recorded expenses, including expenses not yet paid. It subtracts no cost of goods and no inventory movement, and ignores assets entirely -- Rs 40,85,000 of them. On live data it reports Rs 7,38,034, where the cash-basis figure is Rs 6,44,500, a gap of Rs 93,534. The arithmetic is right; the name is doing more work than the formula can support.</t>
+          <t>Nothing in the app links to the AI Work Coach. It still works - it loads for all four roles, the owner can open a teammate's coach, the permission message is right - but the only way in is typing /coach. On 2026-09-12 the Ops employee card opened the coach (plan item D3); it now opens that person's Ops page instead, which removed the last route in. Two of the four demo seats already have coaching generated on 29 Aug, so this is a feature people used.</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>routers/ledger.py:1257 (net_profit); pages/Ledger.js:566-573 (the tile)</t>
+          <t>App.js:228 (/coach route); pages/OperatingScore.js:931 (employee card link); pages/OperatingScore.js:119-141 (ViewAsBanner)</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr"/>
@@ -25081,7 +25093,7 @@
     <row r="65" ht="82" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>FN-05</t>
+          <t>CR-11</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -25091,12 +25103,12 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>All figures</t>
+          <t>Contact profile when loading fails</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -25111,17 +25123,17 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Accept a period parameter (this month, this quarter, this FY -- the Indian financial year matters here) and filter each query by it, defaulting to the current month. That single change also gives FN-02 and FN-03 the data they are currently faking.</t>
+          <t>Split the branch: if error has no response (network) or a 5xx, say 'Couldn't load this contact' with Retry; keep the 'isn't here' copy for a 404 or an empty body.</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Every figure is all-time and there is no way to change that. Expenses, invoices, payments, assets and inventory are each queried for the whole tenant with no window and capped at 5000 records. So the page can tell an owner what they have billed since the company started, but not what they billed this month -- which is the question a finance screen is opened to answer. It is also why FN-02's 'This month' chip has nothing to bind to.</t>
+          <t>The page says 'That contact isn't here. It may have been merged or removed.' The customer exists; only the request failed. An owner reading this on a weak phone signal is told a real customer has been deleted or merged.</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>routers/ledger.py:1223-1262 (ledger_summary)</t>
+          <t>pages/ContactProfile.js:151-160; pages/mobile/ContactProfileMobile.jsx:85-99</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr"/>
@@ -25134,7 +25146,7 @@
     <row r="66" ht="82" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>FN-09</t>
+          <t>CR-12</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -25144,12 +25156,12 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Finance when a request fails</t>
+          <t>GET /api/crm/outstanding</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -25164,17 +25176,17 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Check isError on each query and render 'Couldn't load &lt;tab&gt;' with Retry (403: 'You don't have access to the ledger'). One shared &lt;QueryError&gt; would serve this, OP-10 and CR-10.</t>
+          <t>Gate it with require_perm('people') (it only feeds the CRM grid) or require_perm('finance') to match the profile endpoint.</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Summary fails: the Overview says 'Loading...' indefinitely. Expenses fails: the Expenses tab shows 'No expenses yet - approved purchase bills and payments show up here automatically, or add one manually', directly under an AI panel that is still analysing those same expenses. An owner on a bad connection is told their books are empty. The same missing branch is behind FN-07.</t>
+          <t>GET /api/contacts and GET /api/contacts/&lt;id&gt;/profile correctly refuse Sales with 403 - but GET /api/crm/outstanding answers 200 with every customer's receivables, payables, invoice count and days overdue. The keys are contact ids rather than names, so it is not a full leak on its own, but it hands money data to roles the rest of the app deliberately keeps out of finance.</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1522-1527, :1641-1642, :1657-1659</t>
+          <t>routers/crm.py:37-38 (outstanding_by_contact, Depends(get_current_user))</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr"/>
@@ -25187,7 +25199,7 @@
     <row r="67" ht="82" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>MW-22</t>
+          <t>FN-04</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -25197,12 +25209,12 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Task card - bulk-select checkbox (mobile)</t>
+          <t>'Net profit' tile</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -25217,17 +25229,17 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Give the checkbox a 44x44 hit area again (a padded label around it, or a transparent ::before), and keep stopPropagation on that area so it never opens the drawer.</t>
+          <t>Rename to something the formula actually supports -- 'Billed minus spend', or 'Gross margin (billed)' -- or compute a real net that accounts for COGS and inventory. The former is a one-line change and stops the page overclaiming.</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>The checkbox is now 16x16 inside a 16x22 label - nothing larger is clickable. A tap 10px off in any direction lands on the card, and since 78d01df the whole card opens the task drawer. So on a phone, trying to select tasks for a bulk action frequently opens a task instead. 12 checkboxes on the first screen, all the same.</t>
+          <t>It is revenue BILLED minus ALL recorded expenses, including expenses not yet paid. It subtracts no cost of goods and no inventory movement, and ignores assets entirely -- Rs 40,85,000 of them. On live data it reports Rs 7,38,034, where the cash-basis figure is Rs 6,44,500, a gap of Rs 93,534. The arithmetic is right; the name is doing more work than the formula can support.</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js (task card summary - bulk-select checkbox, top-left)</t>
+          <t>routers/ledger.py:1257 (net_profit); pages/Ledger.js:566-573 (the tile)</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr"/>
@@ -25240,7 +25252,7 @@
     <row r="68" ht="82" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>GL-01</t>
+          <t>FN-05</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -25250,12 +25262,12 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Desktop header - notification bell</t>
+          <t>All figures</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -25270,17 +25282,17 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Move Bellicon to module scope (a real component that takes notif/unread/bellCount as props), or render the Popover JSX inline rather than through an inner component. The same applies to any other component declared inside Layout.</t>
+          <t>Accept a period parameter (this month, this quarter, this FY -- the Indian financial year matters here) and filter each query by it, defaulting to the current month. That single change also gives FN-02 and FN-03 the data they are currently faking.</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>On Decision Desk, My Work and Team the dropdown opens and then closes on its own about 0.4s later, dropping focus to &lt;body&gt;; nothing was clicked in between. On Finance it stays open. So on the desktop's most-used pages a user clicks the bell, sees a flash, and cannot read or open a notification. (The phone bell works.)</t>
+          <t>Every figure is all-time and there is no way to change that. Expenses, invoices, payments, assets and inventory are each queried for the whole tenant with no window and capped at 5000 records. So the page can tell an owner what they have billed since the company started, but not what they billed this month -- which is the question a finance screen is opened to answer. It is also why FN-02's 'This month' chip has nothing to bind to.</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>components/Layout.js:366-424 (Bellicon inside Layout)</t>
+          <t>routers/ledger.py:1223-1262 (ledger_summary)</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr"/>
@@ -25293,7 +25305,7 @@
     <row r="69" ht="82" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>GL-02</t>
+          <t>FN-09</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -25303,12 +25315,12 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Mobile More panel - non-owners</t>
+          <t>Finance when a request fails</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -25323,17 +25335,17 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Align the tile filters with the routes: show Ops to everyone (it already renders a self view), Team to everyone (read-only for non-managers), and Settings to everyone (profile + security for non-owners).</t>
+          <t>Check isError on each query and render 'Couldn't load &lt;tab&gt;' with Retry (403: 'You don't have access to the ledger'). One shared &lt;QueryError&gt; would serve this, OP-10 and CR-10.</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>On a phone, Sales, Production and Finance see only two tiles: Workflows and Leave. They cannot reach Ops, Team or Settings, although all three routes open for them and the desktop nav shows them Ops and Team. Ops was deliberately opened to every role so staff see their own metrics (App.js:222-226) - on mobile that view is unreachable.</t>
+          <t>Summary fails: the Overview says 'Loading...' indefinitely. Expenses fails: the Expenses tab shows 'No expenses yet - approved purchase bills and payments show up here automatically, or add one manually', directly under an AI panel that is still analysing those same expenses. An owner on a bad connection is told their books are empty. The same missing branch is behind FN-07.</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>components/mobile/AllAppsPanel.jsx:70-83 and :127 (tile filters)</t>
+          <t>pages/Ledger.js:1522-1527, :1641-1642, :1657-1659</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr"/>
@@ -25346,7 +25358,7 @@
     <row r="70" ht="82" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>DD-03</t>
+          <t>MW-22</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -25356,12 +25368,12 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Decision Desk</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Money tiles for Sales / Production</t>
+          <t>Task card - bulk-select checkbox (mobile)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -25376,17 +25388,17 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Render money tiles only when hasPerm(user,'finance') || hasPerm(user,'ledger'); otherwise show the role's own tiles.</t>
+          <t>Give the checkbox a 44x44 hit area again (a padded label around it, or a transparent ::before), and keep stopPropagation on that area so it never opens the drawer.</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>'Net profit' and 'Spend, this month' show '...' forever - their data (ledger summary) is refused with 403 - while 'To collect (overdue) Rs 7.5 L' is shown to these roles, a customer-receivables figure they have no finance permission for. Tapping the money tiles leads to the empty Finance page of FN-07.</t>
+          <t>The checkbox is now 16x16 inside a 16x22 label - nothing larger is clickable. A tap 10px off in any direction lands on the card, and since 78d01df the whole card opens the task drawer. So on a phone, trying to select tasks for a bulk action frequently opens a task instead. 12 checkboxes on the first screen, all the same.</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>pages/Desk.js:563-661 (KPI tiles), pages/desk/useDeskMetrics.js</t>
+          <t>pages/MyWork.js (task card summary - bulk-select checkbox, top-left)</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr"/>
@@ -25399,7 +25411,7 @@
     <row r="71" ht="82" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>CL-01</t>
+          <t>GL-01</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -25414,7 +25426,7 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Notifications, People, Journal, Calendar when loading fails</t>
+          <t>Desktop header - notification bell</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -25429,17 +25441,17 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>One shared &lt;QueryError onRetry&gt; used wherever a query's data drives the page; branch 403 vs other errors. Fixing it once fixes OP-10, CR-10, FN-09, DD-02 and this.</t>
+          <t>Move Bellicon to module scope (a real component that takes notif/unread/bellCount as props), or render the Popover JSX inline rather than through an inner component. The same applies to any other component declared inside Layout.</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Notifications says 'You're all caught up.' People says 'Members 0 - No team members yet.' Calendar shows every filter at 0. Journal shows only its header and nothing below. None says anything failed. With OP-10, CR-10, FN-09 and DD-02 this is the same fault on nine surfaces.</t>
+          <t>On Decision Desk, My Work and Team the dropdown opens and then closes on its own about 0.4s later, dropping focus to &lt;body&gt;; nothing was clicked in between. On Finance it stays open. So on the desktop's most-used pages a user clicks the bell, sees a flash, and cannot read or open a notification. (The phone bell works.)</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>pages/Notifications.js:14, pages/People.js:47-53, pages/Journal.js:185, pages/Calendar.js:62</t>
+          <t>components/Layout.js:366-424 (Bellicon inside Layout)</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr"/>
@@ -25452,7 +25464,7 @@
     <row r="72" ht="82" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>CL-02</t>
+          <t>GL-02</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -25462,12 +25474,12 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Calendar events</t>
+          <t>Mobile More panel - non-owners</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -25482,17 +25494,17 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Wrap each event in a Link to its source (task -&gt; /my-work?task=, decision -&gt; /decisions/, invoice -&gt; /finance?tab=revenue, leave -&gt; /team).</t>
+          <t>Align the tile filters with the routes: show Ops to everyone (it already renders a self view), Team to everyone (read-only for non-managers), and Settings to everyone (profile + security for non-owners).</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Nothing happens. Events are plain &lt;div&gt;s with no link or handler, so the calendar shows 'Vendor Call - Next Monday - Overdue' but the user cannot get from it to the task to act on it.</t>
+          <t>On a phone, Sales, Production and Finance see only two tiles: Workflows and Leave. They cannot reach Ops, Team or Settings, although all three routes open for them and the desktop nav shows them Ops and Team. Ops was deliberately opened to every role so staff see their own metrics (App.js:222-226) - on mobile that view is unreachable.</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>pages/Calendar.js:233 (cal-event)</t>
+          <t>components/mobile/AllAppsPanel.jsx:70-83 and :127 (tile filters)</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr"/>
@@ -25505,7 +25517,7 @@
     <row r="73" ht="82" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>MW-13</t>
+          <t>DD-03</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -25515,12 +25527,12 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Decision Desk</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Workflows view - pipeline cards</t>
+          <t>Money tiles for Sales / Production</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -25528,24 +25540,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F73" s="8" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Give each an aria-label that names its card, e.g. 'Delete card: Dispatch 100 sales items today'. The card title is already to hand where the button is rendered.</t>
+          <t>Render money tiles only when hasPerm(user,'finance') || hasPerm(user,'ledger'); otherwise show the role's own tiles.</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Five separate buttons are all named exactly 'Delete card', and two are both named 'Advance to Delivered'. Sighted users tell them apart by which card they sit on; a screen-reader user hears the same phrase five times with nothing to say which shipment is about to be deleted. Deletion is the most destructive action in the view, which is what lifts this above cosmetic.</t>
+          <t>'Net profit' and 'Spend, this month' show '...' forever - their data (ledger summary) is refused with 403 - while 'To collect (overdue) Rs 7.5 L' is shown to these roles, a customer-receivables figure they have no finance permission for. Tapping the money tiles leads to the empty Finance page of FN-07.</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>pages/Workflows.js (delete-workflow-* and advance-workflow-* buttons)</t>
+          <t>pages/Desk.js:563-661 (KPI tiles), pages/desk/useDeskMetrics.js</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr"/>
@@ -25558,7 +25570,7 @@
     <row r="74" ht="82" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>MW-19</t>
+          <t>CL-01</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -25568,12 +25580,12 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Department filter dropdown</t>
+          <t>Notifications, People, Journal, Calendar when loading fails</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -25581,24 +25593,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F74" s="8" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Filter options to count &gt; 0 (keep All), or render zero-count ones disabled; move Completed into the Status dropdown.</t>
+          <t>One shared &lt;QueryError onRetry&gt; used wherever a query's data drives the page; branch 403 vs other errors. Fixing it once fixes OP-10, CR-10, FN-09, DD-02 and this.</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Three problems. (1) 'Completed 7' is listed as a Department - it is a state, and the Status dropdown beside it is where it belongs. (2) Six of the nine options read 0 (Sales 0, Production 0, Quality Control 0, Inventory 0, Finance 0, HR 0) - the old chip strip hid empty categories on a founder ask (U7-05.9). (3) Picking an empty one is silently undone: the trigger still reads 'Department: All 26' and nothing tells the user why.</t>
+          <t>Notifications says 'You're all caught up.' People says 'Members 0 - No team members yet.' Calendar shows every filter at 0. Journal shows only its header and nothing below. None says anything failed. With OP-10, CR-10, FN-09 and DD-02 this is the same fault on nine surfaces.</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:2042-2075 (FilterDropdown), :2735-2743 (Department options), :2288-2298 (snap-back effect)</t>
+          <t>pages/Notifications.js:14, pages/People.js:47-53, pages/Journal.js:185, pages/Calendar.js:62</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr"/>
@@ -25611,7 +25623,7 @@
     <row r="75" ht="82" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>TM-01</t>
+          <t>CL-02</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -25621,12 +25633,12 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Add member - login method toggle</t>
+          <t>Calendar events</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -25634,24 +25646,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F75" s="8" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Add aria-pressed to both buttons, and wrap them in a role='group' with an accessible label such as 'Login method' - matching the permission grid immediately below it.</t>
+          <t>Wrap each event in a Link to its source (task -&gt; /my-work?task=, decision -&gt; /decisions/, invoice -&gt; /finance?tab=revenue, leave -&gt; /team).</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Neither half carries aria-pressed. The selection is conveyed only by a class swap (kr-pressed against kr-pop), so a sighted user sees which method is active and a screen-reader user hears two identical unlabelled buttons. Choosing between a password and an OTP decides how that person will sign in for good, so it is worth announcing.</t>
+          <t>Nothing happens. Events are plain &lt;div&gt;s with no link or handler, so the calendar shows 'Vendor Call - Next Monday - Overdue' but the user cannot get from it to the task to act on it.</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:122-127 (login-method-toggle); the pattern to copy is at :165</t>
+          <t>pages/Calendar.js:233 (cal-event)</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr"/>
@@ -25664,7 +25676,7 @@
     <row r="76" ht="82" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>TM-07</t>
+          <t>MW-13</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -25674,12 +25686,12 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Member profile dialog - closing</t>
+          <t>Workflows view - pipeline cards</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -25694,17 +25706,17 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Keep the Dialog mounted with open={!!u} and render only its content conditionally, so Radix's own focus return runs; or remember the opening card and focus it in onCloseAutoFocus.</t>
+          <t>Give each an aria-label that names its card, e.g. 'Delete card: Dispatch 100 sales items today'. The card title is already to hand where the button is rendered.</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Focus drops to &lt;body&gt;. A keyboard or screen-reader user who opens the fifth card and closes it is thrown back to the top of the page and has to Tab through the header, search and every earlier card to get back. On a 12-person roster that is a nuisance; on the larger teams the search box is built for, it makes the roster hard to work through.</t>
+          <t>Five separate buttons are all named exactly 'Delete card', and two are both named 'Advance to Delivered'. Sighted users tell them apart by which card they sit on; a screen-reader user hears the same phrase five times with nothing to say which shipment is about to be deleted. Deletion is the most destructive action in the view, which is what lifts this above cosmetic.</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:450 (onOpen sets profileUser), :541-542 (openChange, 'if (!u) return null')</t>
+          <t>pages/Workflows.js (delete-workflow-* and advance-workflow-* buttons)</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr"/>
@@ -25717,7 +25729,7 @@
     <row r="77" ht="82" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>TM-08</t>
+          <t>MW-19</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -25727,12 +25739,12 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Default close button on every dialog</t>
+          <t>Department filter dropdown</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -25747,17 +25759,17 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Give the default close a hit area: 'grid h-8 w-8 place-items-center' around the icon (32px), keeping the icon at 16px. One change fixes every dialog at once.</t>
+          <t>Filter options to count &gt; 0 (keep All), or render zero-count ones disabled; move Completed into the Status dropdown.</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>On desktop the close X is 16x16px - the bare icon with no padding. On mobile the same control measures 44x44, so the fault is desktop-only. It comes from the shared dialog component, so it applies to every dialog that keeps the default close: Add member, Edit access, the invite link modal, and the rest of the app's dialogs that use it. The Team profile dialog avoids it by hiding the default and drawing its own 36px close.</t>
+          <t>Three problems. (1) 'Completed 7' is listed as a Department - it is a state, and the Status dropdown beside it is where it belongs. (2) Six of the nine options read 0 (Sales 0, Production 0, Quality Control 0, Inventory 0, Finance 0, HR 0) - the old chip strip hid empty categories on a founder ask (U7-05.9). (3) Picking an empty one is silently undone: the trigger still reads 'Department: All 26' and nothing tells the user why.</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>components/ui/dialog.jsx:37-41</t>
+          <t>pages/MyWork.js:2042-2075 (FilterDropdown), :2735-2743 (Department options), :2288-2298 (snap-back effect)</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr"/>
@@ -25770,7 +25782,7 @@
     <row r="78" ht="82" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>CR-01</t>
+          <t>TM-01</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -25780,12 +25792,12 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Scope chips (Buyers / Suppliers)</t>
+          <t>Add member - login method toggle</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -25800,17 +25812,17 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Add aria-pressed to the desktop chips, mirroring the mobile pair, and give the row a role='group' with a label. Same family as TM-01.</t>
+          <t>Add aria-pressed to both buttons, and wrap them in a role='group' with an accessible label such as 'Login method' - matching the permission grid immediately below it.</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>The desktop chips carry no aria-pressed at all, while the mobile twins of the same control set it correctly (true on Buyers, false on Suppliers). So the identical control is announced properly on a phone and not on a laptop. The filtering itself is correct - Buyers shows 11, Suppliers shows 6, and switching back restores 11.</t>
+          <t>Neither half carries aria-pressed. The selection is conveyed only by a class swap (kr-pressed against kr-pop), so a sighted user sees which method is active and a screen-reader user hears two identical unlabelled buttons. Choosing between a password and an OTP decides how that person will sign in for good, so it is worth announcing.</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:819-836 (crm-scope-chips, desktop); the correct pattern is at :794-805 (crm-scope-mobile)</t>
+          <t>pages/Team.js:122-127 (login-method-toggle); the pattern to copy is at :165</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr"/>
@@ -25823,7 +25835,7 @@
     <row r="79" ht="82" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>CR-07</t>
+          <t>TM-07</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -25833,12 +25845,12 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Contact profile - Log activity</t>
+          <t>Member profile dialog - closing</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -25853,17 +25865,17 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Repaint Log with the standard primary, and check the contact profile's background against the list it is reached from -- a detail page changing ground colour makes the two feel like separate apps.</t>
+          <t>Keep the Dialog mounted with open={!!u} and render only its content conditionally, so Radix's own focus return runs; or remember the opening card and focus it in onCloseAutoFocus.</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>The Log button on the contact profile is indigo, rgb(55,58,205), while every other primary action in the app -- Add contact, Add member, Complete, Approve -- is the near-black ink colour. Contrast is fine at 7.93:1; the problem is that it reads as a different product for a moment. The contact profile also sits on a strong amber gradient while the CRM list it came from is neutral grey, which compounds the shift.</t>
+          <t>Focus drops to &lt;body&gt;. A keyboard or screen-reader user who opens the fifth card and closes it is thrown back to the top of the page and has to Tab through the header, search and every earlier card to get back. On a 12-person roster that is a nuisance; on the larger teams the search box is built for, it makes the roster hard to work through.</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>pages/ContactProfile.js (Log button and page background)</t>
+          <t>pages/Team.js:450 (onOpen sets profileUser), :541-542 (openChange, 'if (!u) return null')</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr"/>
@@ -25876,7 +25888,7 @@
     <row r="80" ht="82" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>OP-07</t>
+          <t>TM-08</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -25886,12 +25898,12 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Operating score - empty workspace</t>
+          <t>Default close button on every dialog</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -25906,17 +25918,17 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Keep the neutral internal default if it helps the maths, but let the UI show 'not enough data yet' rather than a score, using the enough_data flag that is already computed and sent.</t>
+          <t>Give the default close a hit area: 'grid h-8 w-8 place-items-center' around the icon (32px), keeping the icon at 16px. One change fixes every dialog at once.</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Completion, approval rate and collection rate each fall back to 0.7 when there is nothing to divide by, so a brand-new tenant that has done nothing at all scores about 70 out of 100 and is told it is doing reasonably well. There is an enough_data flag in the payload, so the page can already tell the difference -- the default just makes the number look earned.</t>
+          <t>On desktop the close X is 16x16px - the bare icon with no padding. On mobile the same control measures 44x44, so the fault is desktop-only. It comes from the shared dialog component, so it applies to every dialog that keeps the default close: Add member, Edit access, the invite link modal, and the rest of the app's dialogs that use it. The Team profile dialog avoids it by hiding the default and drawing its own 36px close.</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>services/operating_score.py (the 0.7 defaults, enough_data)</t>
+          <t>components/ui/dialog.jsx:37-41</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr"/>
@@ -25929,7 +25941,7 @@
     <row r="81" ht="82" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>OP-08</t>
+          <t>CR-01</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -25939,12 +25951,12 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Category cards</t>
+          <t>Scope chips (Buyers / Suppliers)</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -25959,17 +25971,17 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Give a floored score its own treatment -- a filled track in the warning colour, or an explicit 'at floor' marker -- so it reads as a measured bad result rather than an absent one.</t>
+          <t>Add aria-pressed to the desktop chips, mirroring the mobile pair, and give the row a role='group' with a label. Same family as TM-01.</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Execution and Responsiveness both render '0 / 100' above a completely empty progress bar, which is pixel-identical to how an unmeasured category would look. Two of the four cards on the page therefore read as 'nothing here' when they actually mean 'this is as bad as it gets'.</t>
+          <t>The desktop chips carry no aria-pressed at all, while the mobile twins of the same control set it correctly (true on Buyers, false on Suppliers). So the identical control is announced properly on a phone and not on a laptop. The filtering itself is correct - Buyers shows 11, Suppliers shows 6, and switching back restores 11.</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>pages/OperatingScore.js (category card progress track)</t>
+          <t>pages/CRM.js:819-836 (crm-scope-chips, desktop); the correct pattern is at :794-805 (crm-scope-mobile)</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr"/>
@@ -25982,7 +25994,7 @@
     <row r="82" ht="82" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>OP-13</t>
+          <t>CR-07</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -25992,12 +26004,12 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>'Back to company' and 'See all' links</t>
+          <t>Contact profile - Log activity</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -26012,17 +26024,17 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Give both links py-1.5 (or min-h-6 with inline-flex items-center) so the hit area reaches 24px without changing the look. Fix with OP-09 in one pass.</t>
+          <t>Repaint Log with the standard primary, and check the contact profile's background against the list it is reached from -- a detail page changing ground colour makes the two feel like separate apps.</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>'Back to company' in the view-as banner is 109x16 on desktop and 117x20 on mobile - and it is the only way out of view-as mode other than the browser. 'See all' above 'Your open work' is 52x16 on desktop and 55x20 on mobile, on every non-owner's page. Same pattern as the 'View all' links in OP-09, on two screens OP-09 did not cover.</t>
+          <t>The Log button on the contact profile is indigo, rgb(55,58,205), while every other primary action in the app -- Add contact, Add member, Complete, Approve -- is the near-black ink colour. Contrast is fine at 7.93:1; the problem is that it reads as a different product for a moment. The contact profile also sits on a strong amber gradient while the CRM list it came from is neutral grey, which compounds the shift.</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>pages/OperatingScore.js:133-139 (Back to company); the 'See all' link in the self view's open-work header</t>
+          <t>pages/ContactProfile.js (Log button and page background)</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr"/>
@@ -26035,7 +26047,7 @@
     <row r="83" ht="82" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>OP-14</t>
+          <t>OP-07</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -26050,7 +26062,7 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>AI Work Coach - error page</t>
+          <t>Operating score - empty workspace</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -26065,17 +26077,17 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Branch the title too: 403 -&gt; 'Not allowed', 404 -&gt; 'Person not found', otherwise 'Couldn't load coaching'.</t>
+          <t>Keep the neutral internal default if it helps the maths, but let the UI show 'not enough data yet' rather than a score, using the enough_data flag that is already computed and sent.</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>The page is titled 'Access denied' while its body says 'Couldn't load coaching - Something went wrong.' Nothing was denied: the owner may view anyone's coach, and the API answered 404 'Employee not found'. The title blames permissions for a missing person.</t>
+          <t>Completion, approval rate and collection rate each fall back to 0.7 when there is nothing to divide by, so a brand-new tenant that has done nothing at all scores about 70 out of 100 and is told it is doing reasonably well. There is an enough_data flag in the payload, so the page can already tell the difference -- the default just makes the number look earned.</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>pages/WorkCoach.js:36-57</t>
+          <t>services/operating_score.py (the 0.7 defaults, enough_data)</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr"/>
@@ -26088,7 +26100,7 @@
     <row r="84" ht="82" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>CR-09</t>
+          <t>OP-08</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -26098,12 +26110,12 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Contact profile (mobile) - Score with AI</t>
+          <t>Category cards</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -26118,17 +26130,17 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Add a 'Score with AI' action to the mobile profile's action row, reusing the same POST /contacts/{id}/rescore mutation - or record that scoring is desktop-only by design.</t>
+          <t>Give a floored score its own treatment -- a filled track in the warning colour, or an explicit 'at floor' marker -- so it reads as a measured bad result rather than an absent one.</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Desktop has 'Score with AI' (and 'Re-score'); its failure path works - 'Could not score right now', label restored. The mobile contact profile has no scoring control at all, only a read-only 'Health nn/100' row, so the score cannot be refreshed from a phone.</t>
+          <t>Execution and Responsiveness both render '0 / 100' above a completely empty progress bar, which is pixel-identical to how an unmeasured category would look. Two of the four cards on the page therefore read as 'nothing here' when they actually mean 'this is as bad as it gets'.</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>pages/ContactProfile.js:134-137 + :250-273 (desktop); pages/mobile/ContactProfileMobile.jsx:254 (Health row only)</t>
+          <t>pages/OperatingScore.js (category card progress track)</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr"/>
@@ -26141,7 +26153,7 @@
     <row r="85" ht="82" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>CR-13</t>
+          <t>OP-13</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -26151,12 +26163,12 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Decision Desk 'Complaints' tile -&gt; /crm</t>
+          <t>'Back to company' and 'See all' links</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -26171,17 +26183,17 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Only set the link when hasPerm(user, 'people'); otherwise render the tile as plain (non-link) or point it at a view the role can open.</t>
+          <t>Give both links py-1.5 (or min-h-6 with inline-flex items-center) so the hit area reaches 24px without changing the look. Fix with OP-09 in one pass.</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>CRM itself is correctly hidden and a direct visit shows Access Denied - but the 'Complaints' KPI tile on Decision Desk links to /crm for all three roles, on desktop and mobile. Tapping the number lands on 'ACCESS DENIED'. It is the most prominent link on their home screen to a page they are not allowed to see.</t>
+          <t>'Back to company' in the view-as banner is 109x16 on desktop and 117x20 on mobile - and it is the only way out of view-as mode other than the browser. 'See all' above 'Your open work' is 52x16 on desktop and 55x20 on mobile, on every non-owner's page. Same pattern as the 'View all' links in OP-09, on two screens OP-09 did not cover.</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>pages/Desk.js:569-572 (mobile tile), :614-617 (desktop tile)</t>
+          <t>pages/OperatingScore.js:133-139 (Back to company); the 'See all' link in the self view's open-work header</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr"/>
@@ -26194,7 +26206,7 @@
     <row r="86" ht="82" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>CR-14</t>
+          <t>OP-14</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -26204,12 +26216,12 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Contact profile - 'Back to CRM' (desktop)</t>
+          <t>AI Work Coach - error page</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -26224,17 +26236,17 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>py-1 or min-h-6 on the back link.</t>
+          <t>Branch the title too: 403 -&gt; 'Not allowed', 404 -&gt; 'Person not found', otherwise 'Couldn't load coaching'.</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>'Back to CRM' is 103x20 - the only other interactive element under 24px on the page. The mobile 'Back to people' is fine.</t>
+          <t>The page is titled 'Access denied' while its body says 'Couldn't load coaching - Something went wrong.' Nothing was denied: the owner may view anyone's coach, and the API answered 404 'Employee not found'. The title blames permissions for a missing person.</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>pages/ContactProfile.js:205 (profile-back)</t>
+          <t>pages/WorkCoach.js:36-57</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr"/>
@@ -26247,7 +26259,7 @@
     <row r="87" ht="82" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>FN-10</t>
+          <t>CR-09</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -26257,12 +26269,12 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Mobile capture card - 'Export' tile</t>
+          <t>Contact profile (mobile) - Score with AI</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -26277,17 +26289,17 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Rename it 'Import - CSV, Excel' with an upload icon. If export is wanted, build it as a separate action.</t>
+          <t>Add a 'Score with AI' action to the mobile profile's action row, reusing the same POST /contacts/{id}/rescore mutation - or record that scoring is desktop-only by design.</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>The fourth tile reads 'Export - CSV, Excel' but is a file picker that UPLOADS a spreadsheet to /ingest/csv. An owner wanting to download their books for the accountant taps it and gets a file-open dialog. Desktop labels the same control correctly as 'CSV / Excel' under Capture. There is no export anywhere on the page.</t>
+          <t>Desktop has 'Score with AI' (and 'Re-score'); its failure path works - 'Could not score right now', label restored. The mobile contact profile has no scoring control at all, only a read-only 'Health nn/100' row, so the score cannot be refreshed from a phone.</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1430-1437</t>
+          <t>pages/ContactProfile.js:134-137 + :250-273 (desktop); pages/mobile/ContactProfileMobile.jsx:254 (Health row only)</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr"/>
@@ -26300,7 +26312,7 @@
     <row r="88" ht="82" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>FN-11</t>
+          <t>CR-13</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -26310,12 +26322,12 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Mobile overview - 'View all 3+ action items'</t>
+          <t>Decision Desk 'Complaints' tile -&gt; /crm</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -26330,17 +26342,17 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>py-1 on the link.</t>
+          <t>Only set the link when hasPerm(user, 'people'); otherwise render the tile as plain (non-link) or point it at a view the role can open.</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>'View all 3+ action items' is 322x20 - wide but under 24px tall. It works (opens the Revenue tab).</t>
+          <t>CRM itself is correctly hidden and a direct visit shows Access Denied - but the 'Complaints' KPI tile on Decision Desk links to /crm for all three roles, on desktop and mobile. Tapping the number lands on 'ACCESS DENIED'. It is the most prominent link on their home screen to a page they are not allowed to see.</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1075 (ledger-mobile-viewall)</t>
+          <t>pages/Desk.js:569-572 (mobile tile), :614-617 (desktop tile)</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr"/>
@@ -26353,7 +26365,7 @@
     <row r="89" ht="82" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>MW-05</t>
+          <t>CR-14</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -26363,12 +26375,12 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Task list - bento grid</t>
+          <t>Contact profile - 'Back to CRM' (desktop)</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -26383,17 +26395,17 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Make the button a column flex container and pin content to the top - add 'flex flex-col justify-start' to its className. Verified live in the browser: all three titles then start at 17px.</t>
+          <t>py-1 or min-h-6 on the back link.</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Titles in one row start at different heights - the spread was 39px, 17px, 11px and 17px across the first four rows. A short title sinks toward the middle of its card while a long one starts at the top, so the row reads as ragged. The checkboxes stay aligned, which makes it more obvious.</t>
+          <t>'Back to CRM' is 103x20 - the only other interactive element under 24px on the page. The mobile 'Back to people' is fine.</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:1181 (the task-summary button className)</t>
+          <t>pages/ContactProfile.js:205 (profile-back)</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr"/>
@@ -26406,7 +26418,7 @@
     <row r="90" ht="82" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>GL-03</t>
+          <t>FN-10</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -26416,12 +26428,12 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>/login while signed in</t>
+          <t>Mobile capture card - 'Export' tile</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -26436,17 +26448,17 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>If the auth context has a user, &lt;Navigate to='/app' replace/&gt; (the same hand-off Home already uses).</t>
+          <t>Rename it 'Import - CSV, Excel' with an upload icon. If export is wanted, build it as a separate action.</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>The sign-in form is shown again. A user following an old bookmark or a 'Sign in' link sees a login screen while already logged in.</t>
+          <t>The fourth tile reads 'Export - CSV, Excel' but is a file picker that UPLOADS a spreadsheet to /ingest/csv. An owner wanting to download their books for the accountant taps it and gets a file-open dialog. Desktop labels the same control correctly as 'CSV / Excel' under Capture. There is no export anywhere on the page.</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>pages/Login.js (component top)</t>
+          <t>pages/Ledger.js:1430-1437</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr"/>
@@ -26459,7 +26471,7 @@
     <row r="91" ht="82" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>DD-04</t>
+          <t>FN-11</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -26469,12 +26481,12 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Decision Desk</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Company / You switch (mobile)</t>
+          <t>Mobile overview - 'View all 3+ action items'</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -26489,17 +26501,17 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Show the joined pill pair above the score below lg.</t>
+          <t>py-1 on the link.</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Both copies of the Company / You pills are in the DOM but invisible at phone width, so the phone only ever shows the company score.</t>
+          <t>'View all 3+ action items' is 322x20 - wide but under 24px tall. It works (opens the Revenue tab).</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>pages/Desk.js:426 and :470 (scope pill placements)</t>
+          <t>pages/Ledger.js:1075 (ledger-mobile-viewall)</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr"/>
@@ -26512,7 +26524,7 @@
     <row r="92" ht="82" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>DD-05</t>
+          <t>MW-05</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -26522,12 +26534,12 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Decision Desk</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Decision review - note mic</t>
+          <t>Task list - bento grid</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -26542,17 +26554,17 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Wire it to the same capture Dex uses, or remove the mic and its helper line until it is.</t>
+          <t>Make the button a column flex container and pin content to the top - add 'flex flex-col justify-start' to its className. Verified live in the browser: all three titles then start at 17px.</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>It only shows a toast: 'Voice capture is available from the Dex panel'. The button and the helper line invite an action the page does not do.</t>
+          <t>Titles in one row start at different heights - the spread was 39px, 17px, 11px and 17px across the first four rows. A short title sinks toward the middle of its card while a long one starts at the top, so the row reads as ragged. The checkboxes stay aligned, which makes it more obvious.</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>components/DecisionDialog.js:421-445</t>
+          <t>pages/MyWork.js:1181 (the task-summary button className)</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr"/>
@@ -26565,7 +26577,7 @@
     <row r="93" ht="82" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>CL-03</t>
+          <t>GL-03</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -26575,12 +26587,12 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Mark all read</t>
+          <t>/login while signed in</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -26595,17 +26607,17 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>toast.error('Couldn't mark notifications read') in onError.</t>
+          <t>If the auth context has a user, &lt;Navigate to='/app' replace/&gt; (the same hand-off Home already uses).</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Nothing happens and nothing is said - no toast, the unread dots stay - so the user cannot tell whether it worked.</t>
+          <t>The sign-in form is shown again. A user following an old bookmark or a 'Sign in' link sees a login screen while already logged in.</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>pages/Notifications.js:17-21</t>
+          <t>pages/Login.js (component top)</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr"/>
@@ -26618,7 +26630,7 @@
     <row r="94" ht="82" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>CL-04</t>
+          <t>DD-04</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -26628,12 +26640,12 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Decision Desk</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Operations tab - add links</t>
+          <t>Company / You switch (mobile)</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -26648,17 +26660,17 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>py-1 / min-h-6 on both.</t>
+          <t>Show the joined pill pair above the score below lg.</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>'Add operational task' (149x20) and 'Add approval rule' (131x20) are under 24px.</t>
+          <t>Both copies of the Company / You pills are in the DOM but invisible at phone width, so the phone only ever shows the company score.</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>pages/Settings.js (OperatingModelEditor add buttons)</t>
+          <t>pages/Desk.js:426 and :470 (scope pill placements)</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr"/>
@@ -26671,7 +26683,7 @@
     <row r="95" ht="82" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>AU-01</t>
+          <t>DD-05</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -26681,12 +26693,12 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Sign-in</t>
+          <t>Decision Desk</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Login, sign-up and admin fields</t>
+          <t>Decision review - note mic</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -26701,17 +26713,17 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Add labels (visually hidden where the design has none). Same fix as TM-06.</t>
+          <t>Wire it to the same capture Dex uses, or remove the mic and its helper line until it is.</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Login email and password, the sign-up company name, and the admin email and password have no associated label or aria-label. The admin screen shows the words EMAIL and PASSWORD but they are not tied to the inputs.</t>
+          <t>It only shows a toast: 'Voice capture is available from the Dex panel'. The button and the helper line invite an action the page does not do.</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>pages/Login.js:298-299, pages/Signup.js (basics), pages/admin/AdminLogin.js:44-57</t>
+          <t>components/DecisionDialog.js:421-445</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr"/>
@@ -26724,7 +26736,7 @@
     <row r="96" ht="82" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>AU-02</t>
+          <t>CL-03</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -26734,12 +26746,12 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Sign-in</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Mobile OTP - phone number</t>
+          <t>Mark all read</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -26754,17 +26766,17 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Require 10 digits (after stripping +91 / spaces) before enabling Send, and say 'Enter a 10-digit mobile number'.</t>
+          <t>toast.error('Couldn't mark notifications read') in onError.</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>The 3-digit number is sent to the server; with no provider reachable the user only sees 'Something went wrong. Please try again.', which does not tell them the number is wrong.</t>
+          <t>Nothing happens and nothing is said - no toast, the unread dots stay - so the user cannot tell whether it worked.</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>pages/Login.js:179-190, :317</t>
+          <t>pages/Notifications.js:17-21</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr"/>
@@ -26777,7 +26789,7 @@
     <row r="97" ht="82" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>AU-03</t>
+          <t>CL-04</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -26787,12 +26799,12 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Sign-in</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Login - header links (desktop)</t>
+          <t>Operations tab - add links</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -26807,17 +26819,17 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>py-1 on both links.</t>
+          <t>py-1 / min-h-6 on both.</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>The 'DecisionOS' logo link is 91x21 and 'Need a workspace? Register' is 194x20.</t>
+          <t>'Add operational task' (149x20) and 'Add approval rule' (131x20) are under 24px.</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>pages/Login.js:241-246</t>
+          <t>pages/Settings.js (OperatingModelEditor add buttons)</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr"/>
@@ -26830,7 +26842,7 @@
     <row r="98" ht="82" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>MW-14</t>
+          <t>AU-01</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -26840,12 +26852,12 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Sign-in</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Page heading in the Leave / Workflows views</t>
+          <t>Login, sign-up and admin fields</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -26853,24 +26865,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F98" s="9" t="inlineStr">
-        <is>
-          <t>Nit</t>
+      <c r="F98" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Swap the heading with the view - 'Leave' or 'Workflows' - or append the view name. Only worth doing if the views stay inside My Work at all; see MW-12.</t>
+          <t>Add labels (visually hidden where the design has none). Same fix as TM-06.</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>The heading stays 'My Work' with the eyebrow 'YOUR DAY, SIMPLIFIED' even when the body is entirely leave requests or delivery pipelines. Nothing above the fold says which of the three views is active except the small toggle pill.</t>
+          <t>Login email and password, the sign-up company name, and the admin email and password have no associated label or aria-label. The admin screen shows the words EMAIL and PASSWORD but they are not tied to the inputs.</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js (page header, above the view switch at 2527)</t>
+          <t>pages/Login.js:298-299, pages/Signup.js (basics), pages/admin/AdminLogin.js:44-57</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr"/>
@@ -26883,7 +26895,7 @@
     <row r="99" ht="82" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>CR-03</t>
+          <t>AU-02</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -26893,12 +26905,12 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Sign-in</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Add contact dialog - dismiss controls</t>
+          <t>Mobile OTP - phone number</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -26906,24 +26918,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F99" s="9" t="inlineStr">
-        <is>
-          <t>Nit</t>
+      <c r="F99" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Pick one convention for the whole app - most products keep the X and drop the Cancel, or keep Cancel on destructive-ish forms only - and apply it to both this dialog and TM-04.</t>
+          <t>Require 10 digits (after stripping +91 / spaces) before enabling Send, and say 'Enter a 10-digit mobile number'.</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Two: a 'Cancel' button beside Add contact, and a separate 'Close' X. Team's profile dialog has the same duplication (TM-04), so it is worth settling once for the app rather than per dialog.</t>
+          <t>The 3-digit number is sent to the server; with no provider reachable the user only sees 'Something went wrong. Please try again.', which does not tell them the number is wrong.</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:242-365 (crm-contact-dialog footer)</t>
+          <t>pages/Login.js:179-190, :317</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr"/>
@@ -26936,7 +26948,7 @@
     <row r="100" ht="82" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>TM-02</t>
+          <t>AU-03</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -26946,12 +26958,12 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Sign-in</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Owner section grid</t>
+          <t>Login - header links (desktop)</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -26959,24 +26971,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F100" s="9" t="inlineStr">
-        <is>
-          <t>Nit</t>
+      <c r="F100" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Either let a single-card group span the row, or give the owner its own treatment at the top of the page - it is a different kind of row from a department, and looks like one.</t>
+          <t>py-1 on both links.</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>The Owner group uses the same three-column grid as every other role but will almost always hold exactly one card, so 874px of a 1336px row is blank. It reads as a rendering fault rather than a deliberate space.</t>
+          <t>The 'DecisionOS' logo link is 91x21 and 'Need a workspace? Register' is 194x20.</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:366 (team-cards-&lt;role&gt; grid)</t>
+          <t>pages/Login.js:241-246</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr"/>
@@ -26989,7 +27001,7 @@
     <row r="101" ht="82" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>TM-03</t>
+          <t>MW-14</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -26999,12 +27011,12 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Member cards</t>
+          <t>Page heading in the Leave / Workflows views</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -27019,17 +27031,17 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Put the reporting line on the card - one line, 'Reports to Sunita Rao' - and consider replacing the bare count with the two or three areas that distinguish this person, keeping the full list in the dialog. Cheapest alternative: soften the eyebrow so it stops promising what the list does not show.</t>
+          <t>Swap the heading with the view - 'Leave' or 'Workflows' - or append the view name. Only worth doing if the views stay inside My Work at all; see MW-12.</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>The cards show name, email, status and a permission COUNT. The reporting line is absent entirely, and access is reduced to a number that says nothing about what the person can reach. Both exist one click deeper - the profile dialog reads 'REPORTS TO Sunita Rao' and '13 of 14 areas' with the areas listed - so the data is there and simply is not surfaced where the page says it will be.</t>
+          <t>The heading stays 'My Work' with the eyebrow 'YOUR DAY, SIMPLIFIED' even when the body is entirely leave requests or delivery pipelines. Nothing above the fold says which of the three views is active except the small toggle pill.</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:417-450 (member card); manager already resolved at :475</t>
+          <t>pages/MyWork.js (page header, above the view switch at 2527)</t>
         </is>
       </c>
       <c r="J101" s="2" t="inlineStr"/>
@@ -27042,7 +27054,7 @@
     <row r="102" ht="82" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>TM-04</t>
+          <t>CR-03</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -27052,12 +27064,12 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Member profile dialog</t>
+          <t>Add contact dialog - dismiss controls</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -27072,17 +27084,17 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Keep one. If the custom 36px control is the intended one, hide the primitive's default close for this dialog.</t>
+          <t>Pick one convention for the whole app - most products keep the X and drop the Cancel, or keep Cancel on destructive-ish forms only - and apply it to both this dialog and TM-04.</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Two separate visible buttons are both named exactly 'Close'. A screen-reader user tabbing the dialog meets the same name twice with nothing to separate them.</t>
+          <t>Two: a 'Cancel' button beside Add contact, and a separate 'Close' X. Team's profile dialog has the same duplication (TM-04), so it is worth settling once for the app rather than per dialog.</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:497-535 (profile dialog header)</t>
+          <t>pages/CRM.js:242-365 (crm-contact-dialog footer)</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr"/>
@@ -27095,7 +27107,7 @@
     <row r="103" ht="82" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>MW-06</t>
+          <t>TM-02</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -27105,12 +27117,12 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Category tab bar</t>
+          <t>Owner section grid</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
@@ -27125,17 +27137,17 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>While the tasks query is loading, render a dash or omit the count, matching the skeleton treatment already used for the cards below.</t>
+          <t>Either let a single-card group span the row, or give the owner its own treatment at the top of the page - it is a different kind of row from a department, and looks like one.</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>The tab reads 'All 0' for the whole fetch, which states a count of zero rather than an unknown one. The card skeletons underneath are correct, so the count is the only misleading element.</t>
+          <t>The Owner group uses the same three-column grid as every other role but will almost always hold exactly one card, so 874px of a 1336px row is blank. It reads as a rendering fault rather than a deliberate space.</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:2556-2566 (work-tabs counts)</t>
+          <t>pages/Team.js:366 (team-cards-&lt;role&gt; grid)</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr"/>
@@ -27148,58 +27160,217 @@
     <row r="104" ht="82" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
+          <t>TM-03</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>UI audit</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Member cards</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>Bug fix</t>
+        </is>
+      </c>
+      <c r="F104" s="9" t="inlineStr">
+        <is>
+          <t>Nit</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>Put the reporting line on the card - one line, 'Reports to Sunita Rao' - and consider replacing the bare count with the two or three areas that distinguish this person, keeping the full list in the dialog. Cheapest alternative: soften the eyebrow so it stops promising what the list does not show.</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>The cards show name, email, status and a permission COUNT. The reporting line is absent entirely, and access is reduced to a number that says nothing about what the person can reach. Both exist one click deeper - the profile dialog reads 'REPORTS TO Sunita Rao' and '13 of 14 areas' with the areas listed - so the data is there and simply is not surfaced where the page says it will be.</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>pages/Team.js:417-450 (member card); manager already resolved at :475</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr"/>
+      <c r="K104" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="82" customHeight="1">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>TM-04</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>UI audit</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>Member profile dialog</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>Bug fix</t>
+        </is>
+      </c>
+      <c r="F105" s="9" t="inlineStr">
+        <is>
+          <t>Nit</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Keep one. If the custom 36px control is the intended one, hide the primitive's default close for this dialog.</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>Two separate visible buttons are both named exactly 'Close'. A screen-reader user tabbing the dialog meets the same name twice with nothing to separate them.</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>pages/Team.js:497-535 (profile dialog header)</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr"/>
+      <c r="K105" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="82" customHeight="1">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>MW-06</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>UI audit</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>My Work</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Category tab bar</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>Bug fix</t>
+        </is>
+      </c>
+      <c r="F106" s="9" t="inlineStr">
+        <is>
+          <t>Nit</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>While the tasks query is loading, render a dash or omit the count, matching the skeleton treatment already used for the cards below.</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>The tab reads 'All 0' for the whole fetch, which states a count of zero rather than an unknown one. The card skeletons underneath are correct, so the count is the only misleading element.</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>pages/MyWork.js:2556-2566 (work-tabs counts)</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr"/>
+      <c r="K106" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="82" customHeight="1">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
           <t>MW-07</t>
         </is>
       </c>
-      <c r="B104" s="2" t="inlineStr">
+      <c r="B107" s="2" t="inlineStr">
         <is>
           <t>UI audit</t>
         </is>
       </c>
-      <c r="C104" s="2" t="inlineStr">
+      <c r="C107" s="2" t="inlineStr">
         <is>
           <t>My Work</t>
         </is>
       </c>
-      <c r="D104" s="2" t="inlineStr">
+      <c r="D107" s="2" t="inlineStr">
         <is>
           <t>Task card - Complete (evidence required)</t>
         </is>
       </c>
-      <c r="E104" s="2" t="inlineStr">
+      <c r="E107" s="2" t="inlineStr">
         <is>
           <t>By design</t>
         </is>
       </c>
-      <c r="F104" s="9" t="inlineStr">
+      <c r="F107" s="9" t="inlineStr">
         <is>
           <t>Nit</t>
         </is>
       </c>
-      <c r="G104" s="2" t="inlineStr">
+      <c r="G107" s="2" t="inlineStr">
         <is>
           <t>Optional polish only: disable Complete while proof is missing and put the reason in a tooltip or helper line, so the constraint is visible before the click rather than after it. Current behaviour is safe and correct.</t>
         </is>
       </c>
-      <c r="H104" s="2" t="inlineStr">
+      <c r="H107" s="2" t="inlineStr">
         <is>
           <t>Completion IS correctly blocked - the task stays in the active list and an explanatory toast appears. The only nit is that the button looks available and only explains itself after it is pressed.</t>
         </is>
       </c>
-      <c r="I104" s="2" t="inlineStr">
+      <c r="I107" s="2" t="inlineStr">
         <is>
           <t>pages/MyWork.js:1107-1119</t>
         </is>
       </c>
-      <c r="J104" s="2" t="inlineStr"/>
-      <c r="K104" s="4" t="inlineStr">
+      <c r="J107" s="2" t="inlineStr"/>
+      <c r="K107" s="4" t="inlineStr">
         <is>
           <t>Not a defect</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K104"/>
+  <autoFilter ref="A1:K107"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27210,7 +27381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B58"/>
+  <dimension ref="A1:B59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -27277,481 +27448,493 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr"/>
-      <c r="B8" s="16" t="inlineStr"/>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="12" t="inlineStr"/>
-      <c r="B9" s="13" t="inlineStr">
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Still happening. Later commits label ASK-18 (Workflows well), ASK-19 (card summary), ASK-20 (My Work scroll) and ASK-21 (New Task dialog) from the other list. In this workbook ASK-18 is the CRM In-progress list, ASK-19 the operating score KPIs, and ASK-20 / ASK-21 / ASK-22 are the three root causes from the full audit (load errors, permission map, phone parity). Match commits to this sheet by content, not by number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr"/>
+      <c r="B9" s="16" t="inlineStr"/>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="12" t="inlineStr"/>
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Leave approvals: who approves, and is the Settings screen needed?</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="12" t="inlineStr"/>
-      <c r="B10" s="14" t="inlineStr">
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="12" t="inlineStr"/>
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>Raised 2026-09-12 by Yogesh - Owner. Status: DEFERRED, Yogesh deciding. Relates to ASK-8. Nothing is to be built from this note until that call is made.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="15" t="inlineStr"/>
-      <c r="B11" s="16" t="inlineStr"/>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="17" t="inlineStr"/>
-      <c r="B12" s="18" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr"/>
+      <c r="B12" s="16" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="17" t="inlineStr"/>
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>THE QUESTION</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="15" t="inlineStr"/>
-      <c r="B13" s="16" t="inlineStr">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="15" t="inlineStr"/>
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>Leave approval is mostly done by either the owner or a manager. The approver is already chosen when a team member is added. So does the 'Leave Approvers by Department' settings screen need to exist at all?</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr"/>
-      <c r="B14" s="16" t="inlineStr"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="17" t="inlineStr"/>
-      <c r="B15" s="18" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr"/>
+      <c r="B15" s="16" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="17" t="inlineStr"/>
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>HOW APPROVAL IS DECIDED TODAY</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="15" t="inlineStr"/>
-      <c r="B16" s="16" t="inlineStr">
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="15" t="inlineStr"/>
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>When someone requests leave the system asks three questions IN ORDER and stops at the first that answers. The code is services/leave.py, _resolve_leave_approver.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>Tier 1</t>
-        </is>
-      </c>
-      <c r="B17" s="16" t="inlineStr">
-        <is>
-          <t>Does this person have a Reporting Manager? If yes, that manager approves. The Reporting Manager is chosen in Team when the member is added or edited (pages/Team.js:144, the member-manager-select dropdown; stored as reporting_manager_id).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Does this person have a Reporting Manager? If yes, that manager approves. The Reporting Manager is chosen in Team when the member is added or edited (pages/Team.js:144, the member-manager-select dropdown; stored as reporting_manager_id).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>Otherwise: is there a department rule for their role? If yes, that person approves. THIS IS THE SETTINGS SCREEN under discussion - the gear in the Leave section, which opens 'Leave Approvers by Department' with one dropdown per department and a Save button.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>Tier 3</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>Otherwise the Owner approves.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr"/>
-      <c r="B20" s="16" t="inlineStr"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="17" t="inlineStr"/>
-      <c r="B21" s="18" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr"/>
+      <c r="B21" s="16" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="17" t="inlineStr"/>
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>WHAT THE LIVE DATA SHOWS</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr"/>
-      <c r="B22" s="16" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr"/>
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>Measured against the dev workspace on 2026-09-12, not assumed:</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>Members</t>
-        </is>
-      </c>
-      <c r="B23" s="16" t="inlineStr">
-        <is>
-          <t>12 team members in the workspace.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>Tier 1 used</t>
+          <t>Members</t>
         </is>
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>1 member has a Reporting Manager set (sai, finance).</t>
+          <t>12 team members in the workspace.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>Tier 2 used</t>
+          <t>Tier 1 used</t>
         </is>
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>0. The tenant leave_approvers mapping is EMPTY - every department reads 'Owner (default)'.</t>
+          <t>1 member has a Reporting Manager set (sai, finance).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>Tier 3 used</t>
+          <t>Tier 2 used</t>
         </is>
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>11 of 12 members fall through to the Owner, Rajesh Sharma.</t>
+          <t>0. The tenant leave_approvers mapping is EMPTY - every department reads 'Owner (default)'.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
+          <t>Tier 3 used</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>11 of 12 members fall through to the Owner, Rajesh Sharma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B27" s="16" t="inlineStr">
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>The Settings screen currently decides leave for NOBODY. It configures a tier that no request reaches.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="15" t="inlineStr"/>
-      <c r="B28" s="16" t="inlineStr"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="17" t="inlineStr"/>
-      <c r="B29" s="18" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr"/>
+      <c r="B29" s="16" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="17" t="inlineStr"/>
+      <c r="B30" s="18" t="inlineStr">
         <is>
           <t>WHAT THE THREE PIECES ARE</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="15" t="inlineStr"/>
-      <c r="B30" s="16" t="inlineStr">
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="15" t="inlineStr"/>
+      <c r="B31" s="16" t="inlineStr">
         <is>
           <t>They are three layers of one feature. Removing one without the others leaves either a screen that cannot save or an endpoint nothing calls.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
-        <is>
-          <t>The gear</t>
-        </is>
-      </c>
-      <c r="B31" s="16" t="inlineStr">
-        <is>
-          <t>The small round icon beside the My Leave / Approvals tabs. It is the only way into the screen. pages/Leave.js:500-510.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>The panel</t>
+          <t>The gear</t>
         </is>
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>'Leave Approvers by Department' - a dropdown per department plus a Save approvers button. pages/Leave.js:387-417.</t>
+          <t>The small round icon beside the My Leave / Approvals tabs. It is the only way into the screen. pages/Leave.js:500-510.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="15" t="inlineStr">
         <is>
+          <t>The panel</t>
+        </is>
+      </c>
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>'Leave Approvers by Department' - a dropdown per department plus a Save approvers button. pages/Leave.js:387-417.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
           <t>The endpoint</t>
         </is>
       </c>
-      <c r="B33" s="16" t="inlineStr">
+      <c r="B34" s="16" t="inlineStr">
         <is>
           <t>PATCH /tenant/leave-approvers, which writes the leave_approvers field on the tenant record. routers/calendar.py:24.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="15" t="inlineStr"/>
-      <c r="B34" s="16" t="inlineStr"/>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="17" t="inlineStr"/>
-      <c r="B35" s="18" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr"/>
+      <c r="B35" s="16" t="inlineStr"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="17" t="inlineStr"/>
+      <c r="B36" s="18" t="inlineStr">
         <is>
           <t>OPTION A - DELETE TIER 2  (the current recommendation)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="15" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>What changes</t>
         </is>
       </c>
-      <c r="B36" s="16" t="inlineStr">
+      <c r="B37" s="16" t="inlineStr">
         <is>
           <t>Remove the gear, the panel and the endpoint. Approval becomes: reporting manager, else owner.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="15" t="inlineStr">
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>Effect today</t>
         </is>
       </c>
-      <c r="B37" s="16" t="inlineStr">
+      <c r="B38" s="16" t="inlineStr">
         <is>
           <t>NONE. Every one of the 12 members resolves to exactly the same approver before and after, because nothing uses tier 2.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="45" customHeight="1">
-      <c r="A38" s="15" t="inlineStr">
+    <row r="39" ht="45" customHeight="1">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>Argument for</t>
         </is>
       </c>
-      <c r="B38" s="16" t="inlineStr">
+      <c r="B39" s="16" t="inlineStr">
         <is>
           <t>The approver is already chosen once, in Team, when the person is added. A second screen expressing the same decision in different words - and silently losing to the first one - mostly creates the chance for the two to disagree with the org chart.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="15" t="inlineStr"/>
-      <c r="B39" s="16" t="inlineStr"/>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="17" t="inlineStr"/>
-      <c r="B40" s="18" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr"/>
+      <c r="B40" s="16" t="inlineStr"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="17" t="inlineStr"/>
+      <c r="B41" s="18" t="inlineStr">
         <is>
           <t>OPTION B - KEEP TIER 2</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="15" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
         <is>
           <t>What it buys</t>
         </is>
       </c>
-      <c r="B41" s="16" t="inlineStr">
+      <c r="B42" s="16" t="inlineStr">
         <is>
           <t>One place to say 'all Sales leave goes to Priya' without making Priya anyone's reporting manager.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="15" t="inlineStr">
-        <is>
-          <t>Cost of A</t>
-        </is>
-      </c>
-      <c r="B42" s="16" t="inlineStr">
-        <is>
-          <t>To get that same outcome after deleting, Priya would have to be set as the reporting manager of each Sales person individually, in Team.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="15" t="inlineStr">
         <is>
+          <t>Cost of A</t>
+        </is>
+      </c>
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>To get that same outcome after deleting, Priya would have to be set as the reporting manager of each Sales person individually, in Team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
           <t>If kept</t>
         </is>
       </c>
-      <c r="B43" s="16" t="inlineStr">
+      <c r="B44" s="16" t="inlineStr">
         <is>
           <t>Then the fix is not to move it into Settings but to make it visible - today it is hidden behind an unlabelled gear inside a work surface, which is why it has stayed empty.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="15" t="inlineStr"/>
-      <c r="B44" s="16" t="inlineStr"/>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="17" t="inlineStr"/>
-      <c r="B45" s="18" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="15" t="inlineStr"/>
+      <c r="B45" s="16" t="inlineStr"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="17" t="inlineStr"/>
+      <c r="B46" s="18" t="inlineStr">
         <is>
           <t>THE ONE QUESTION THAT DECIDES IT</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="15" t="inlineStr"/>
-      <c r="B46" s="16" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="15" t="inlineStr"/>
+      <c r="B47" s="16" t="inlineStr">
         <is>
           <t>Is 'who approves your leave' always the same person as 'who you report to'?</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="15" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="B47" s="16" t="inlineStr">
+      <c r="B48" s="16" t="inlineStr">
         <is>
           <t>They are always the same -&gt; Option A. Tier 2 is pure duplication.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B48" s="16" t="inlineStr">
-        <is>
-          <t>They can differ - for example a department lead signs off leave while people report to a project manager -&gt; Option B, and the work is to surface the screen properly rather than hide it.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="15" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>They can differ - for example a department lead signs off leave while people report to a project manager -&gt; Option B, and the work is to surface the screen properly rather than hide it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
           <t>Read</t>
         </is>
       </c>
-      <c r="B49" s="16" t="inlineStr">
+      <c r="B50" s="16" t="inlineStr">
         <is>
           <t>For an SME the answer is usually yes, which is why A is the standing recommendation - but this is a business call, not a technical one, which is why it is parked rather than filed as a defect.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="15" t="inlineStr"/>
-      <c r="B50" s="16" t="inlineStr"/>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="17" t="inlineStr"/>
-      <c r="B51" s="18" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="15" t="inlineStr"/>
+      <c r="B51" s="16" t="inlineStr"/>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="17" t="inlineStr"/>
+      <c r="B52" s="18" t="inlineStr">
         <is>
           <t>IF OPTION A IS CHOSEN, THE WORK IS</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B52" s="16" t="inlineStr">
-        <is>
-          <t>Delete the gear and the settings tab from pages/Leave.js (:500-510).</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>Delete the LeaveApproverConfig block from pages/Leave.js (:387-417).</t>
+          <t>Delete the gear and the settings tab from pages/Leave.js (:500-510).</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="15" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>Delete the LeaveApproverConfig block from pages/Leave.js (:387-417).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="15" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B54" s="16" t="inlineStr">
+      <c r="B55" s="16" t="inlineStr">
         <is>
           <t>Delete PATCH /tenant/leave-approvers from routers/calendar.py (:24) and the LeaveApproverMapInput model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B55" s="16" t="inlineStr">
-        <is>
-          <t>Drop the tier-2 lookup from _resolve_leave_approver in services/leave.py, leaving reporting manager then owner.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="15" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B56" s="16" t="inlineStr">
         <is>
-          <t>Leave the leave_approvers field on existing tenant records alone, or clear it in the migration - it is empty in practice either way.</t>
+          <t>Drop the tier-2 lookup from _resolve_leave_approver in services/leave.py, leaving reporting manager then owner.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="15" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B57" s="16" t="inlineStr">
         <is>
-          <t>Make sure Team makes the consequence visible: the Reporting Manager dropdown should say that this person also approves their leave, since after this change that is the only place the decision is made.</t>
+          <t>Leave the leave_approvers field on existing tenant records alone, or clear it in the migration - it is empty in practice either way.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="15" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>Make sure Team makes the consequence visible: the Reporting Manager dropdown should say that this person also approves their leave, since after this change that is the only place the decision is made.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="15" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B58" s="16" t="inlineStr">
+      <c r="B59" s="16" t="inlineStr">
         <is>
           <t>This depends on ASK-6. If Leave moves into Team first, the gear disappears with it and steps 1 and 2 become part of that move rather than separate work.</t>
         </is>

</xml_diff>

<commit_message>
Ask section: My Work All Tasks gets a Person filter and a complete filter row (ASK-24)
Founder request, tracked for traction. Person filter (people, Me,
Unassigned, Teams), Pending Approval and Overdue in Status, the missing
Priority dropdown, combined counts, Clear filters, URL-kept filters and
the same four filters on the phone.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_UI_Bug_Report.xlsx
+++ b/docs/DecisionOS_UI_Bug_Report.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bug Log'!$A$1:$Q$89</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Coverage'!$A$1:$J$283</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Verified Non-Issues'!$A$1:$E$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Action List'!$A$1:$K$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Action List'!$A$1:$K$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22458,7 +22458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K112"/>
+  <dimension ref="A1:K113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23825,12 +23825,12 @@
     <row r="25" ht="82" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>MW-08</t>
+          <t>ASK-24</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>UI audit</t>
+          <t>Founder review</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -23840,35 +23840,46 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Task card - Update / Escalate</t>
+          <t>All Tasks: add a Person filter and complete the filter row (options + UI)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Bug fix</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
+          <t>Change request</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Restyle that one button to the segmented-control treatment the rest of the toolbar moved to in the same commit (kr-pressed / kr-pop, as the priority bands use), or simply restore the two constants. Then stop the class recurring: craco narrows ESLint to react-hooks rules only, which drops eslint-config-react-app's no-undef - the rule that would have failed the build on this exact line.</t>
+          <t>Founder request 2026-09-13, tracked here for traction. On My Work &gt; All Tasks (desktop and phone):
+(1) PERSON filter - a new 'Person: All' dropdown between Department and Status, same pill as the others. Shown only on All Tasks (on My Tasks every card is yours). Options, each with an open-task count: 'All people'; 'Me'; every person who holds work in the list, busiest first, with their role under the name (e.g. Priya Nair - Sales); 'Unassigned'; and a 'Teams' group for tasks given to a role with no person (the cards' 'Sales team' line). Names come from /users, already loaded as members. With more than 8 people, a type-to-search box sits at the top of the menu.
+(2) COMPLETE STATUS OPTIONS - add 'Pending Approval' (status blocked - the grey chip on most cards, which cannot be filtered today) and 'Overdue' (the orange chip; a lens like Completed). Order: All statuses, Not Started, In Progress, Waiting, Pending Approval, Under Review, Overdue, Completed. Show counts like Department does.
+(3) PRIORITY dropdown - the ASK-13 comment says Priority was added, but only Department and Status render. Add 'Priority: All / High / Medium / Low' with counts.
+(4) FILTERS COMBINE - Department x Person x Priority x Status apply together, and every count in every menu reflects the OTHER active filters (today Department counts ignore Status).
+(5) FILTER UI - a filter that is not 'All' shows as pressed (kr-pressed) so the reader can see the list is narrowed; a 'Clear filters' text button appears at the end of the row only when one or more is set; when nothing matches, show 'No tasks match these filters' with Clear, not the 'Tasks appear here once decisions are approved' empty state; filters live in the URL (?person=&amp;dept=&amp;priority=&amp;status=) so they survive a refresh and a Team or Desk link can open one person's tasks; changing a filter clears bulk selection (it resets only on scope/tab/view today); with Person set, cards drop the assignee line, as KM-30 drops the status chip.
+(6) PHONE (ASK-22) - the filter circle on the phone opens the same four filters (a bottom sheet with four sections, or grouped menu sections), and the caption row names what is active, e.g. 'Priya Nair - Overdue'.
+ACCEPTANCE: as owner on All Tasks, pick Priya Nair -&gt; only her cards, and the trigger count equals the cards shown; add Status Overdue -&gt; only her overdue cards; Unassigned and a Team entry work; refresh keeps the filters; Clear resets all four; My Tasks hides Person; the same on a 390px phone; Sales / Production (no All Tasks) never see Person.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>The app CRASHES. A ReferenceError is thrown while rendering the form, the form never appears, and the whole React tree unmounts - the page is gone, not just the form. Recovery needs a reload. The work trail, hand-off and escalation flow is therefore completely unusable.</t>
+          <t>With 131 tasks under 'Department: All 131', the owner cannot see one person's load - who is overdue, what is waiting on whom - without reading the name line on every card. The two chips that fill the screen, Pending Approval and Overdue, are not filter options at all, and the Priority filter the code comments promise is missing. This is the owner's daily review of the team.</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:147 (UpdateForm); constants removed in 5fb96f2; lint narrowed at craco.config.js:74</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr"/>
+          <t>pages/MyWork.js:2042-2075 (FilterDropdown), :2150-2157 (STATUS_FILTER_OPTIONS), :2216 (statusFilter), :2240 (selection reset), :2251-2262 (scope, /users members), :2308-2343 (list filtering), :2403-2410 (departmentOptions, mobile tabs), :2514-2530 (phone filter menu), :2756-2781 (desktop filter row), :2802-2811 (empty state), :100-122 (STATUS_LABEL, isOverdue); routers/team.py:130 (/users)</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>ASK-13, ASK-22, MW-19, KM-30</t>
+        </is>
+      </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
           <t>To do</t>
@@ -23878,7 +23889,7 @@
     <row r="26" ht="82" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>MW-20</t>
+          <t>MW-08</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -23893,7 +23904,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Task drawer - every click inside closes it</t>
+          <t>Task card - Update / Escalate</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -23908,17 +23919,17 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Stop propagation at the drawer boundary: onClick={(e) =&gt; e.stopPropagation()} and onKeyDown={(e) =&gt; e.stopPropagation()} on SheetContent. Or, better, render the Sheet as a SIBLING of the card root rather than a child, so the drawer is outside the clickable element in the component tree. Also guard the root handler with e.currentTarget.contains(e.target) - that is a DOM check, which a portal click fails. Add the five-click test to the verify script.</t>
+          <t>Restyle that one button to the segmented-control treatment the rest of the toolbar moved to in the same commit (kr-pressed / kr-pop, as the priority bands use), or simply restore the two constants. Then stop the class recurring: craco narrows ESLint to react-hooks rules only, which drops eslint-config-react-app's no-undef - the rule that would have failed the build on this exact line.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Every click closes it, on both viewports - 10 of 10. The drawer is now the only place a task can be worked (status, progress, Complete, Attach, Log update, hand off), so none of that is usable. On mobile the status pill tap fired its PATCH before the drawer shut, so the action happens but the user is thrown back to the list without seeing it. Likely also (from the code, not testable while the form cannot be opened): pressing Space or Enter in any drawer field hits the card's onKeyDown, which calls preventDefault and toggles the drawer - so a user could not type a space in an update note.</t>
+          <t>The app CRASHES. A ReferenceError is thrown while rendering the form, the form never appears, and the whole React tree unmounts - the page is gone, not just the form. Recovery needs a reload. The work trail, hand-off and escalation flow is therefore completely unusable.</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:1242-1255 (card root onClick / onKeyDown), the &lt;Sheet&gt; rendered inside the same component (~:1360)</t>
+          <t>pages/MyWork.js:147 (UpdateForm); constants removed in 5fb96f2; lint narrowed at craco.config.js:74</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
@@ -23931,7 +23942,7 @@
     <row r="27" ht="82" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>MW-09</t>
+          <t>MW-20</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -23946,7 +23957,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Task card - 'Log update or hand off' (mobile)</t>
+          <t>Task drawer - every click inside closes it</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -23954,24 +23965,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Wire it to the same handler its desktop counterpart uses so it opens UpdateForm - and fix MW-08 first, or the newly working button will simply crash the page instead of doing nothing.</t>
+          <t>Stop propagation at the drawer boundary: onClick={(e) =&gt; e.stopPropagation()} and onKeyDown={(e) =&gt; e.stopPropagation()} on SheetContent. Or, better, render the Sheet as a SIBLING of the card root rather than a child, so the drawer is outside the clickable element in the component tree. Also guard the root handler with e.currentTarget.contains(e.target) - that is a DOM check, which a portal click fails. Add the five-click test to the verify script.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Nothing happens at all - no form, no navigation, no error. The button is inert. Combined with MW-08 on desktop, there is no working way to log a task update or hand a task off on either viewport.</t>
+          <t>Every click closes it, on both viewports - 10 of 10. The drawer is now the only place a task can be worked (status, progress, Complete, Attach, Log update, hand off), so none of that is usable. On mobile the status pill tap fired its PATCH before the drawer shut, so the action happens but the user is thrown back to the list without seeing it. Likely also (from the code, not testable while the form cannot be opened): pressing Space or Enter in any drawer field hits the card's onKeyDown, which calls preventDefault and toggles the drawer - so a user could not type a space in an update note.</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:1496-1505 (log-update-m button, no onClick)</t>
+          <t>pages/MyWork.js:1242-1255 (card root onClick / onKeyDown), the &lt;Sheet&gt; rendered inside the same component (~:1360)</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
@@ -23984,7 +23995,7 @@
     <row r="28" ht="82" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>MW-10</t>
+          <t>MW-09</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -23994,12 +24005,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Application shell</t>
+          <t>Task card - 'Log update or hand off' (mobile)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -24014,17 +24025,17 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Add an error boundary around the routed page area - it should show a short apology, a Reload action, and report the error - so a single broken component costs one panel rather than the whole product. Worth a second boundary around the app shell as a backstop.</t>
+          <t>Wire it to the same handler its desktop counterpart uses so it opens UpdateForm - and fix MW-08 first, or the newly working button will simply crash the page instead of doing nothing.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>One component throwing takes down the entire application. After the MW-08 crash the React root is left with no children, so the user is looking at a blank page with no message and no recovery except a manual reload. Any future render error anywhere will behave the same way.</t>
+          <t>Nothing happens at all - no form, no navigation, no error. The button is inert. Combined with MW-08 on desktop, there is no working way to log a task update or hand a task off on either viewport.</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/App.js (route tree) and components/Layout.js (shell)</t>
+          <t>pages/MyWork.js:1496-1505 (log-update-m button, no onClick)</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
@@ -24037,7 +24048,7 @@
     <row r="29" ht="82" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>MW-01</t>
+          <t>MW-10</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -24047,12 +24058,12 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Task card - status control</t>
+          <t>Application shell</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -24067,17 +24078,17 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Write the PATCH response straight into the cache instead of trusting the refetch: qc.setQueryData(['tasks', mine], rows =&gt; rows.map(r =&gt; r.id === t.id ? data : r)) using the object the PATCH already returns, then invalidate. That is the standard React Query update-from-response pattern and removes the race entirely. If the refetch must stay authoritative, the list read needs read-your-writes consistency instead.</t>
+          <t>Add an error boundary around the routed page area - it should show a short apology, a Reload action, and report the error - so a single broken component costs one panel rather than the whole product. Worth a second boundary around the app shell as a backstop.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>The save succeeds (PATCH returns 200 with the new status) and a success toast appears, but the card keeps showing the PREVIOUS status. The list refetch that follows returns the pre-change value, which overwrites the UI. The correct status only appears after a full page reload. Reproduced 8 out of 8 attempts; mobile pills stay unpressed the same way. The progress percentage behaves identically: setting 50% stores 50 on the server while the card still reads 0 until reloaded.</t>
+          <t>One component throwing takes down the entire application. After the MW-08 crash the React root is left with no children, so the user is looking at a blank page with no message and no recovery except a manual reload. Any future render error anywhere will behave the same way.</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:1127 setStatus / 1134 setProgress; refresh() at 2102</t>
+          <t>frontend/src/App.js (route tree) and components/Layout.js (shell)</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
@@ -24090,7 +24101,7 @@
     <row r="30" ht="82" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>MW-02</t>
+          <t>MW-01</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -24105,7 +24116,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Task card - detail dialog</t>
+          <t>Task card - status control</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -24120,17 +24131,17 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Give the card a way in: an overflow / more menu on the summary row, or make the title open details, calling setDetailOpen(true). If the detail dialog is genuinely retired, delete the component and move the Delete action onto the inline expanded card instead - either way a task must be deletable.</t>
+          <t>Write the PATCH response straight into the cache instead of trusting the refetch: qc.setQueryData(['tasks', mine], rows =&gt; rows.map(r =&gt; r.id === t.id ? data : r)) using the object the PATCH already returns, then invalidate. That is the standard React Query update-from-response pattern and removes the race entirely. If the refetch must stay authoritative, the list read needs read-your-writes consistency instead.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>There is NO delete control anywhere in My Work, on either viewport, and the task detail dialog never opens. The dialog and its Delete button exist in the code but are unreachable, so the proof gallery, the source-reference panel and the AI insight panel are all dead UI too.</t>
+          <t>The save succeeds (PATCH returns 200 with the new status) and a success toast appears, but the card keeps showing the PREVIOUS status. The list refetch that follows returns the pre-change value, which overwrites the UI. The correct status only appears after a full page reload. Reproduced 8 out of 8 attempts; mobile pills stay unpressed the same way. The progress percentage behaves identically: setting 50% stores 50 on the server while the card still reads 0 until reloaded.</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:986 (state), 1837 (render), 737-890 (the dialog + delete)</t>
+          <t>pages/MyWork.js:1127 setStatus / 1134 setProgress; refresh() at 2102</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
@@ -24143,7 +24154,7 @@
     <row r="31" ht="82" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>MW-21</t>
+          <t>MW-02</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -24158,7 +24169,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Task - Delete</t>
+          <t>Task card - detail dialog</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -24173,17 +24184,17 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Put 'Delete task' in the drawer - a quiet destructive button at the foot of the drawer, keeping the existing confirm step - or restore a 'View details' entry. Owner-only, as it was.</t>
+          <t>Give the card a way in: an overflow / more menu on the summary row, or make the title open details, calling setDetailOpen(true). If the detail dialog is genuinely retired, delete the component and move the Delete action onto the inline expanded card instead - either way a task must be deletable.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>There is no way to delete a task. The detail dialog still contains 'Delete task' with its confirmation, but nothing opens that dialog any more. Its only entry point was 'View details' in the card's ••• menu, and 98b43f4 removed that menu on the reasoning that 'the drawer already exposes every detail action' - but the drawer has no Delete.</t>
+          <t>There is NO delete control anywhere in My Work, on either viewport, and the task detail dialog never opens. The dialog and its Delete button exist in the code but are unreachable, so the proof gallery, the source-reference panel and the AI insight panel are all dead UI too.</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:782-940 (TaskDetailDialog + delete), :1074 and :1941 (detailOpen with no opener)</t>
+          <t>pages/MyWork.js:986 (state), 1837 (render), 737-890 (the dialog + delete)</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
@@ -24196,7 +24207,7 @@
     <row r="32" ht="82" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>MW-15</t>
+          <t>MW-21</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -24211,7 +24222,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Task drawer - close (mobile)</t>
+          <t>Task - Delete</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -24226,17 +24237,17 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Below sm, put the close INSIDE the drawer header (a 44px X at the right of the sticky title bar, or a back chevron at its left) and keep the protruding tab for sm and up: e.g. 'right-3 top-3 sm:left-0 sm:right-auto sm:-translate-x-full'. Alternatively leave a strip of scrim on phones (w-[92%]) so tapping outside works. Either way, test on a phone width before shipping a change to the drawer frame.</t>
+          <t>Put 'Delete task' in the drawer - a quiet destructive button at the foot of the drawer, keeping the existing confirm step - or restore a 'View details' entry. Owner-only, as it was.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>There is no way to close it. The drawer is w-full, so it covers the whole screen and there is no scrim left to tap. The new left-edge close tab sits at x=-43, entirely off-screen. The stock Radix close is at top-right but the sticky title bar paints over it - only a sliver of its focus ring peeks out. Escape closes it, but phones have no Escape key. Browser Back does not close the drawer either: it leaves My Work for the previous route. A phone user who opens a task is stuck.</t>
+          <t>There is no way to delete a task. The detail dialog still contains 'Delete task' with its confirmation, but nothing opens that dialog any more. Its only entry point was 'View details' in the card's ••• menu, and 98b43f4 removed that menu on the reasoning that 'the drawer already exposes every detail action' - but the drawer has no Delete.</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:1427-1441 (SheetContent w-full + SheetClose -translate-x-full)</t>
+          <t>pages/MyWork.js:782-940 (TaskDetailDialog + delete), :1074 and :1941 (detailOpen with no opener)</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
@@ -24249,7 +24260,7 @@
     <row r="33" ht="82" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>MW-16</t>
+          <t>MW-15</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -24264,7 +24275,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Task drawer - 'Log update or hand off' (mobile)</t>
+          <t>Task drawer - close (mobile)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -24279,17 +24290,17 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Render TaskTrail (or at least its UpdateForm) outside the lg-gated body, shared by both layouts, or mount a second instance inside the mobile body. Add the MW-09 check to the verify script so the next drawer change cannot regress it silently.</t>
+          <t>Below sm, put the close INSIDE the drawer header (a 44px X at the right of the sticky title bar, or a back chevron at its left) and keep the protruding tab for sm and up: e.g. 'right-3 top-3 sm:left-0 sm:right-auto sm:-translate-x-full'. Alternatively leave a strip of scrim on phones (w-[92%]) so tapping outside works. Either way, test on a phone width before shipping a change to the drawer frame.</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Nothing appears. The button is visible and tappable, and the form IS mounted - but inside the desktop body, which is display:none below lg. This is MW-09 back: the one control that records what happened is inert on phones again. Desktop is unaffected (form opens, no crash).</t>
+          <t>There is no way to close it. The drawer is w-full, so it covers the whole screen and there is no scrim left to tap. The new left-edge close tab sits at x=-43, entirely off-screen. The stock Radix close is at top-right but the sticky title bar paints over it - only a sliver of its focus ring peeks out. Escape closes it, but phones have no Escape key. Browser Back does not close the drawer either: it leaves My Work for the previous route. A phone user who opens a task is stuck.</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:1658-1662 (mobile trigger), :1679 (desktop body 'hidden lg:block'), :1960 (the only &lt;TaskTrail&gt;)</t>
+          <t>pages/MyWork.js:1427-1441 (SheetContent w-full + SheetClose -translate-x-full)</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
@@ -24302,7 +24313,7 @@
     <row r="34" ht="82" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>CR-04</t>
+          <t>MW-16</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -24312,12 +24323,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Add contact menu (mobile)</t>
+          <t>Task drawer - 'Log update or hand off' (mobile)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -24332,17 +24343,17 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Give the popover collision-aware placement so it flips and clamps inside the viewport, or on mobile present the same three choices as a bottom sheet -- the pattern the app already uses elsewhere for phone menus.</t>
+          <t>Render TaskTrail (or at least its UpdateForm) outside the lg-gated body, shared by both layouts, or mount a second instance inside the mobile body. Add the MW-09 check to the verify script so the next drawer change cannot regress it silently.</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Four fifths of the menu is off-screen. It opens anchored to the + button and runs off the right edge, so all the user sees is a 55px strip carrying three anonymous icons -- every label is cut off. 'New Buyer', 'New Supplier' and 'Import from spreadsheet' are all invisible, so adding a contact on a phone means guessing which icon to press.</t>
+          <t>Nothing appears. The button is visible and tappable, and the form IS mounted - but inside the desktop body, which is display:none below lg. This is MW-09 back: the one control that records what happened is inert on phones again. Desktop is unaffected (form opens, no crash).</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:405-480 (crm-add-menu popover)</t>
+          <t>pages/MyWork.js:1658-1662 (mobile trigger), :1679 (desktop body 'hidden lg:block'), :1960 (the only &lt;TaskTrail&gt;)</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
@@ -24355,7 +24366,7 @@
     <row r="35" ht="82" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>CR-05</t>
+          <t>CR-04</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -24370,7 +24381,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Filter button (mobile)</t>
+          <t>Add contact menu (mobile)</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -24385,17 +24396,17 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Wire it to a sheet or popover containing the status filter and sort that desktop shows inline. Both controls already exist and only need somewhere to be shown.</t>
+          <t>Give the popover collision-aware placement so it flips and clamps inside the viewport, or on mobile present the same three choices as a bottom sheet -- the pattern the app already uses elsewhere for phone menus.</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Nothing happens at all. Not a single thing changes -- same text, same element count, no dialog, no menu, no sheet. Meanwhile the status filter and the sort control both exist in the DOM at zero size, so on a phone there is no way to filter by status or change the sort order.</t>
+          <t>Four fifths of the menu is off-screen. It opens anchored to the + button and runs off the right edge, so all the user sees is a 55px strip carrying three anonymous icons -- every label is cut off. 'New Buyer', 'New Supplier' and 'Import from spreadsheet' are all invisible, so adding a contact on a phone means guessing which icon to press.</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:739 (crm-mobile-filter); the controls it should reveal are at :858 (crm-status-filter) and :869 (crm-sort)</t>
+          <t>pages/CRM.js:405-480 (crm-add-menu popover)</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
@@ -24408,7 +24419,7 @@
     <row r="36" ht="82" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>OP-01</t>
+          <t>CR-05</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -24418,12 +24429,12 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Team execution panel</t>
+          <t>Filter button (mobile)</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -24438,17 +24449,17 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Decide which is true and make them agree. A rolling window is the more useful of the two -- an operating score should recover when the business recovers -- so filter each query to the last 30 days and keep the caption. If all-time is deliberate, the caption has to say so.</t>
+          <t>Wire it to a sheet or popover containing the status filter and sort that desktop shows inline. Both controls already exist and only need somewhere to be shown.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>The panel says 'Last 30 days - open anyone to see their full ops'. The service applies no date filter anywhere: tasks, decisions, invoices and the per-employee leaderboard are all queried for the whole tenant with no window at all. So an owner reads a colleague's score believing it reflects the last month, when it carries every task since the workspace opened -- somebody who was slow in August can never recover from it, and somebody who has improved this month does not show it.</t>
+          <t>Nothing happens at all. Not a single thing changes -- same text, same element count, no dialog, no menu, no sheet. Meanwhile the status filter and the sort control both exist in the DOM at zero size, so on a phone there is no way to filter by status or change the sort order.</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>services/operating_score.py (all queries); the caption is in pages/OperatingScore.js, team-execution section</t>
+          <t>pages/CRM.js:739 (crm-mobile-filter); the controls it should reveal are at :858 (crm-status-filter) and :869 (crm-sort)</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
@@ -24461,7 +24472,7 @@
     <row r="37" ht="82" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>OP-02</t>
+          <t>OP-01</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -24476,7 +24487,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>'Do these first' on mobile</t>
+          <t>Team execution panel</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -24491,17 +24502,17 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>On mobile the band should flow with the page rather than being pinned, so the score, the actions and the team list scroll as one column. If it must stay pinned, it needs to collapse to a handle the user can pull up.</t>
+          <t>Decide which is true and make them agree. A rolling window is the more useful of the two -- an operating score should recover when the business recovers -- so filter each query to the last 30 days and keep the caption. If all-time is deliberate, the caption has to say so.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>It is 90 per cent hidden. 'Do these first' occupies y=425 to 710, and a fixed black 'Team execution' band is pinned from y=454 to the bottom of the screen -- 374px, 46 per cent of the viewport -- covering 256 of its 285px. Scrolling does not help: the document itself does not scroll (scrollHeight equals clientHeight), and the element that does scroll is the dark band, not the page. So the three actions the page exists to recommend are permanently reduced to one visible line.</t>
+          <t>The panel says 'Last 30 days - open anyone to see their full ops'. The service applies no date filter anywhere: tasks, decisions, invoices and the per-employee leaderboard are all queried for the whole tenant with no window at all. So an owner reads a colleague's score believing it reflects the last month, when it carries every task since the workspace opened -- somebody who was slow in August can never recover from it, and somebody who has improved this month does not show it.</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>pages/OperatingScore.js (kr-dark-band team-execution section)</t>
+          <t>services/operating_score.py (all queries); the caption is in pages/OperatingScore.js, team-execution section</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
@@ -24514,7 +24525,7 @@
     <row r="38" ht="82" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>OP-03</t>
+          <t>OP-02</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -24529,7 +24540,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Operating score model</t>
+          <t>'Do these first' on mobile</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -24544,17 +24555,17 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Score each leg as a bounded rate rather than a penalty subtracted from a constant, so the number always has somewhere to move. Where a leg really is at the floor, say 'below floor' rather than printing a 0 that looks like an empty metric. See ASK-19 for the wider redesign.</t>
+          <t>On mobile the band should flow with the page rather than being pinned, so the score, the actions and the team list scroll as one column. If it must stay pinned, it needs to collapse to a handle the user can pull up.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Two of the four legs are pinned at the floor and carry no information. Execution reads 0 and Responsiveness reads 0. Responsiveness actually computes to -296 before clamping (100 - 16 complaints x 12 - 68 overdue x 3), so it would take closing 8 complaints AND clearing 33 overdue tasks before the number moves off zero by a single point. The page's own advice is 'Close 16 open complaints' -- doing all of that would leave the score exactly where it is. The owner gets no gradient at precisely the moment they most need one.</t>
+          <t>It is 90 per cent hidden. 'Do these first' occupies y=425 to 710, and a fixed black 'Team execution' band is pinned from y=454 to the bottom of the screen -- 374px, 46 per cent of the viewport -- covering 256 of its 285px. Scrolling does not help: the document itself does not scroll (scrollHeight equals clientHeight), and the element that does scroll is the dark band, not the page. So the three actions the page exists to recommend are permanently reduced to one visible line.</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>services/operating_score.py:_score_execution and the responsiveness expression in _company_operating_view</t>
+          <t>pages/OperatingScore.js (kr-dark-band team-execution section)</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
@@ -24567,7 +24578,7 @@
     <row r="39" ht="82" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>OP-10</t>
+          <t>OP-03</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -24582,7 +24593,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Ops page when the request fails</t>
+          <t>Operating score model</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -24597,17 +24608,17 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Read isError and error from the query and render a message: 403 -&gt; 'Only the owner can view another person's operating page', 404 -&gt; 'This person is no longer on the team', otherwise 'Couldn't load'. Each with a link to /operating-score. WorkCoach.js:36-57 is the pattern to copy. Also set retry: false for 4xx so the error shows at once.</t>
+          <t>Score each leg as a bounded rate rather than a penalty subtracted from a constant, so the number always has somewhere to move. Where a leg really is at the floor, say 'below floor' rather than printing a 0 that looks like an empty metric. See ASK-19 for the wider redesign.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>The loading skeleton stays on screen forever, with aria-busy=true and no text at all. The API answered in milliseconds - 404 'Team member not found' for the owner, 403 for the three other roles - but the page never shows it. The user cannot tell a slow page from a broken link or a refused one, and there is no way back except the browser. Any stale shared link (a person who has left, a link forwarded to a teammate) lands here.</t>
+          <t>Two of the four legs are pinned at the floor and carry no information. Execution reads 0 and Responsiveness reads 0. Responsiveness actually computes to -296 before clamping (100 - 16 complaints x 12 - 68 overdue x 3), so it would take closing 8 complaints AND clearing 33 overdue tasks before the number moves off zero by a single point. The page's own advice is 'Close 16 open complaints' -- doing all of that would leave the score exactly where it is. The owner gets no gradient at precisely the moment they most need one.</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>pages/OperatingScore.js:85-92 (useQuery + the skeleton fallback); pages/WorkCoach.js:36-57 (the working pattern)</t>
+          <t>services/operating_score.py:_score_execution and the responsiveness expression in _company_operating_view</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
@@ -24620,7 +24631,7 @@
     <row r="40" ht="82" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>CR-10</t>
+          <t>OP-10</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -24630,12 +24641,12 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Contact list when loading fails</t>
+          <t>Ops page when the request fails</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -24650,17 +24661,17 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Read isError from the query and render 'Couldn't load your contacts' with a Retry that calls refetch(). Show '-' rather than 0 in the scope chips while loading or failed. Same fix pattern as OP-10 - worth one shared &lt;QueryError&gt; component.</t>
+          <t>Read isError and error from the query and render a message: 403 -&gt; 'Only the owner can view another person's operating page', 404 -&gt; 'This person is no longer on the team', otherwise 'Couldn't load'. Each with a link to /operating-score. WorkCoach.js:36-57 is the pattern to copy. Also set retry: false for 4xx so the error shows at once.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>The loading skeleton stays forever. On desktop the chips read 'Buyers 0' and 'Suppliers 0' above six blank placeholder cards, so an owner with a flaky connection sees what looks like a CRM with no customers, still loading. On mobile it is the same skeleton with nothing else. No toast, no message, no retry. The same fault as OP-10 on Ops.</t>
+          <t>The loading skeleton stays on screen forever, with aria-busy=true and no text at all. The API answered in milliseconds - 404 'Team member not found' for the owner, 403 for the three other roles - but the page never shows it. The user cannot tell a slow page from a broken link or a refused one, and there is no way back except the browser. Any stale shared link (a person who has left, a link forwarded to a teammate) lands here.</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:524-527 (contacts useQuery), scope-count chips :819-835</t>
+          <t>pages/OperatingScore.js:85-92 (useQuery + the skeleton fallback); pages/WorkCoach.js:36-57 (the working pattern)</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
@@ -24673,7 +24684,7 @@
     <row r="41" ht="82" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>FN-01</t>
+          <t>CR-10</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -24683,12 +24694,12 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Every money figure</t>
+          <t>Contact list when loading fails</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -24703,17 +24714,17 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Delete the private fmt() and import inr from lib/format. The helper already exists and already does the right thing, so this is an import swap rather than a rewrite. Worth a lint rule banning Intl.NumberFormat with a currency style outside lib/format.js.</t>
+          <t>Read isError from the query and render 'Couldn't load your contacts' with a Retry that calls refetch(). Show '-' rather than 0 in the scope chips while loading or failed. Same fix pattern as OP-10 - worth one shared &lt;QueryError&gt; component.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Finance renders 2685000 as Rs 2,685,000 -- Western thousands grouping. Indian convention is Rs 26,85,000. Every tile is affected: Asset Value shows Rs 4,085,000 for what an Indian owner reads as Rs 40,85,000. Worse than being consistently wrong, it is inconsistent: the AI panels ON THE SAME PAGE correctly say 'Rs 7.49L' and 'Rs 13.18 L', and CRM cards elsewhere show 'Rs 4,00,000'. And because the locale is left undefined, the grouping follows each viewer's browser -- the same figure renders differently for different people.</t>
+          <t>The loading skeleton stays forever. On desktop the chips read 'Buyers 0' and 'Suppliers 0' above six blank placeholder cards, so an owner with a flaky connection sees what looks like a CRM with no customers, still loading. On mobile it is the same skeleton with nothing else. No toast, no message, no retry. The same fault as OP-10 on Ops.</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:61-64 (private fmt); lib/format.js:19-30 (inr, and the rule it states)</t>
+          <t>pages/CRM.js:524-527 (contacts useQuery), scope-count chips :819-835</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
@@ -24726,7 +24737,7 @@
     <row r="42" ht="82" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>FN-02</t>
+          <t>FN-01</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -24741,7 +24752,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Net profit hero (mobile)</t>
+          <t>Every money figure</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -24756,17 +24767,17 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Either compute a monthly net and show that, or drop the chip. The backend already buckets by month for expenses, so half the machinery exists -- it needs the revenue side to match (see FN-03).</t>
+          <t>Delete the private fmt() and import inr from lib/format. The helper already exists and already does the right thing, so this is an import swap rather than a rewrite. Worth a lint rule banning Intl.NumberFormat with a currency style outside lib/format.js.</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>It is the all-time figure. The hero shows Rs 738,034 beneath a chip reading 'This month', and 738034 is exactly net_profit from the API, which is computed with no date filter over records spanning June to August. So an owner glancing at their phone reads a lifetime number as a monthly one -- and on a money screen that is the kind of mistake that gets acted on.</t>
+          <t>Finance renders 2685000 as Rs 2,685,000 -- Western thousands grouping. Indian convention is Rs 26,85,000. Every tile is affected: Asset Value shows Rs 4,085,000 for what an Indian owner reads as Rs 40,85,000. Worse than being consistently wrong, it is inconsistent: the AI panels ON THE SAME PAGE correctly say 'Rs 7.49L' and 'Rs 13.18 L', and CRM cards elsewhere show 'Rs 4,00,000'. And because the locale is left undefined, the grouping follows each viewer's browser -- the same figure renders differently for different people.</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1005 (net), :1042 ('This month' chip), :1048 (the value)</t>
+          <t>pages/Ledger.js:61-64 (private fmt); lib/format.js:19-30 (inr, and the rule it states)</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr"/>
@@ -24779,7 +24790,7 @@
     <row r="43" ht="82" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>FN-03</t>
+          <t>FN-02</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -24794,7 +24805,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Revenue and Net profit trend badges (mobile)</t>
+          <t>Net profit hero (mobile)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -24809,17 +24820,17 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Have ledger_summary return revenue and net per month alongside expenses, and bind each trend to its own series. Until then the honest move is to hide the badges rather than show a number that means something else -- and drop the ?? fallback, which is what let this ship silently.</t>
+          <t>Either compute a monthly net and show that, or drop the chip. The backend already buckets by month for expenses, so half the machinery exists -- it needs the revenue side to match (see FN-03).</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Both trend badges are computed from EXPENSES. The Revenue tile reads 'Rs 2,685,000, down 22.1%' -- but that 22.1% is the month-on-month fall in SPENDING, from Rs 10,77,500 in July to Rs 8,39,469 in August. Revenue did not fall; costs did, which is usually good news being reported in red as bad. The Net profit trend is the same number from the same series.</t>
+          <t>It is the all-time figure. The hero shows Rs 738,034 beneath a chip reading 'This month', and 738034 is exactly net_profit from the API, which is computed with no date filter over records spanning June to August. So an owner glancing at their phone reads a lifetime number as a monthly one -- and on a money screen that is the kind of mistake that gets acted on.</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1009-1015 (months, netPoints, netTrend), :1061 (revenue trend); routers/ledger.py:1237-1245 (by_month is expenses only)</t>
+          <t>pages/Ledger.js:1005 (net), :1042 ('This month' chip), :1048 (the value)</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
@@ -24832,7 +24843,7 @@
     <row r="44" ht="82" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>FN-06</t>
+          <t>FN-03</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -24847,7 +24858,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Delete on expenses, invoices and payments</t>
+          <t>Revenue and Net profit trend badges (mobile)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -24862,17 +24873,17 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Put a confirm step in del() and delRevenue(): an AlertDialog naming the record and amount ('Delete invoice SBT/25-26/0431 for Rs 2,85,000?'). Alternatively delete optimistically with an Undo toast and commit after a few seconds. Either way, one tap must not be final.</t>
+          <t>Have ledger_summary return revenue and net per month alongside expenses, and bind each trend to its own series. Until then the honest move is to hide the badges rather than show a number that means something else -- and drop the ?? fallback, which is what let this ship silently.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>One tap sends the DELETE straight away. No confirmation dialog, no 'are you sure', no undo toast - for all three record types, both viewports, both roles. The trash icon is a 36px target at the end of each row, so a stray tap while scrolling a phone ledger deletes a real invoice or payment and silently changes Revenue, Received and Net profit. (The harness blocked every DELETE, so nothing was removed.)</t>
+          <t>Both trend badges are computed from EXPENSES. The Revenue tile reads 'Rs 2,685,000, down 22.1%' -- but that 22.1% is the month-on-month fall in SPENDING, from Rs 10,77,500 in July to Rs 8,39,469 in August. Revenue did not fall; costs did, which is usually good news being reported in red as bad. The Net profit trend is the same number from the same series.</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1541-1549 (del, delRevenue); :886 and :912 (revenue invoice/payment trash); :1264 (expense trash)</t>
+          <t>pages/Ledger.js:1009-1015 (months, netPoints, netTrend), :1061 (revenue trend); routers/ledger.py:1237-1245 (by_month is expenses only)</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
@@ -24885,7 +24896,7 @@
     <row r="45" ht="82" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>FN-07</t>
+          <t>FN-06</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -24900,7 +24911,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Finance for Sales and Production</t>
+          <t>Delete on expenses, invoices and payments</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -24915,17 +24926,17 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Decide what data_input-only users should get. If it is capture only, show them the capture bar and Inbox with a line such as 'You can upload bills here; totals are visible to Finance and the Owner', and hide the money tabs. If they should not be here at all, drop data_input from the route and nav perms. In both cases handle 403 in the page (see FN-09).</t>
+          <t>Put a confirm step in del() and delRevenue(): an AlertDialog naming the record and amount ('Delete invoice SBT/25-26/0431 for Rs 2,85,000?'). Alternatively delete optimistically with an Undo toast and commit after a few seconds. Either way, one tap must not be final.</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Both roles see Finance in the nav and the Money dock and can open it - then every ledger request is refused (6 x 403). The Overview sits on 'Loading...' forever. Revenue, Expenses, Assets and Inventory each show their empty state ('No expenses yet...'), telling the user the company has no money records rather than that they are not allowed to see them. Only the capture bar works. So the page misinforms rather than refuses.</t>
+          <t>One tap sends the DELETE straight away. No confirmation dialog, no 'are you sure', no undo toast - for all three record types, both viewports, both roles. The trash icon is a 36px target at the end of each row, so a stray tap while scrolling a phone ledger deletes a real invoice or payment and silently changes Revenue, Received and Net profit. (The harness blocked every DELETE, so nothing was removed.)</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>App.js:237 (route perms); components/Layout.js:79 (nav perms); routers/ledger.py:619-625 (require_ledger); pages/Ledger.js:1522-1527 (queries without isError), :1641-1642 (Loading...)</t>
+          <t>pages/Ledger.js:1541-1549 (del, delRevenue); :886 and :912 (revenue invoice/payment trash); :1264 (expense trash)</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
@@ -24938,7 +24949,7 @@
     <row r="46" ht="82" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>FN-08</t>
+          <t>FN-07</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -24953,7 +24964,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Adding records on a phone</t>
+          <t>Finance for Sales and Production</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -24968,17 +24979,17 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Render the per-tab Add button on mobile too (drop hidden lg:block, or add a mobile placement), and have the tile open AddExpenseDialog directly through state rather than clicking a DOM node by testid.</t>
+          <t>Decide what data_input-only users should get. If it is capture only, show them the capture bar and Inbox with a line such as 'You can upload bills here; totals are visible to Finance and the Owner', and hide the money tabs. If they should not be here at all, drop data_input from the route and nav perms. In both cases handle 403 in the page (see FN-09).</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>There is no way to add a record manually on a phone. The four Add buttons (Add income / expense / asset / inventory) are rendered but hidden below lg. The 'Add expense' tile in 'Simplify your finances' does nothing on any tab: it looks for an element that does not exist. Upload and scan still work, so a cash expense with no bill cannot be recorded from the phone at all.</t>
+          <t>Both roles see Finance in the nav and the Money dock and can open it - then every ledger request is refused (6 x 403). The Overview sits on 'Loading...' forever. Revenue, Expenses, Assets and Inventory each show their empty state ('No expenses yet...'), telling the user the company has no money records rather than that they are not allowed to see them. Only the capture bar works. So the page misinforms rather than refuses.</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1422-1429 (tile + querySelector), :1630 ('hidden lg:block' addBtn), :1551-1557 (addBtn per tab)</t>
+          <t>App.js:237 (route perms); components/Layout.js:79 (nav perms); routers/ledger.py:619-625 (require_ledger); pages/Ledger.js:1522-1527 (queries without isError), :1641-1642 (Loading...)</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
@@ -24991,7 +25002,7 @@
     <row r="47" ht="82" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>DX-01</t>
+          <t>FN-08</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -25001,12 +25012,12 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Ask Dex - money questions</t>
+          <t>Adding records on a phone</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -25021,17 +25032,17 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Only apply keywords as a record filter when they look like an entity reference (a customer, vendor or invoice number that exists in the tenant); otherwise ignore them for aggregation intents. At minimum add owe/owes/owed/receivable(s)/payable(s)/dues to _KW_STOP. And when an aggregation over a finance entity returns 0 rows while the collection is non-empty, re-run without keywords rather than answer 'zero'.</t>
+          <t>Render the per-tab Add button on mobile too (drop hidden lg:block, or add a mobile placement), and have the tile open AddExpenseDialog directly through state rather than clicking a DOM node by testid.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Dex answered, in bold, 'zero invoices, zero billed amount, and zero outstanding balance - the receivables table is empty', with three KPI tiles reading Invoices 0 / Billed Rs 0 / Outstanding Rs 0, suggested the data 'hasn't been synced', and cited 8 unrelated sources (test tasks, a dispatch, resolved complaints). The ledger holds Rs 26,85,000 billed and Rs 7,49,000 outstanding. An owner asking the most basic money question is told, confidently, that nobody owes them anything.</t>
+          <t>There is no way to add a record manually on a phone. The four Add buttons (Add income / expense / asset / inventory) are rendered but hidden below lg. The 'Add expense' tile in 'Simplify your finances' does nothing on any tab: it looks for an element that does not exist. Upload and scan still work, so a cash expense with no bill cannot be recorded from the phone at all.</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>routers/brain.py:172-187 (_KW_STOP, _rx), :294-299 (invoices retrieval), :836-843</t>
+          <t>pages/Ledger.js:1422-1429 (tile + querySelector), :1630 ('hidden lg:block' addBtn), :1551-1557 (addBtn per tab)</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr"/>
@@ -25044,7 +25055,7 @@
     <row r="48" ht="82" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>DX-02</t>
+          <t>DX-01</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -25059,7 +25070,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Ask Dex - 'What needs my attention today?'</t>
+          <t>Ask Dex - money questions</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -25074,17 +25085,17 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Treat 'what needs my attention' as a composite intent served from the Desk's own counters (needs_decision, on_fire, overdue, receivables) rather than a single-entity list; or map it to status overdue|in_progress|todo with no date window. Add it to the planner guardrails in _refine_plan, since it is Dex's first suggested question.</t>
+          <t>Only apply keywords as a record filter when they look like an entity reference (a customer, vendor or invoice number that exists in the tenant); otherwise ignore them for aggregation intents. At minimum add owe/owes/owed/receivable(s)/payable(s)/dues to _KW_STOP. And when an aggregation over a finance entity returns 0 rows while the collection is non-empty, re-run without keywords rather than answer 'zero'.</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>'Good news - there are no open or overdue tasks requiring your attention right now', followed by a list of things already completed. One question later, 'Which tasks are overdue?' answered 'All 34 matching tasks are overdue'. The page's headline suggestion gives the owner false reassurance.</t>
+          <t>Dex answered, in bold, 'zero invoices, zero billed amount, and zero outstanding balance - the receivables table is empty', with three KPI tiles reading Invoices 0 / Billed Rs 0 / Outstanding Rs 0, suggested the data 'hasn't been synced', and cited 8 unrelated sources (test tasks, a dispatch, resolved complaints). The ledger holds Rs 26,85,000 billed and Rs 7,49,000 outstanding. An owner asking the most basic money question is told, confidently, that nobody owes them anything.</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>routers/brain.py:127-141 (_plan), :144+ (_refine_plan), :463-478 (_compute_tasks filters); pages/Brain.js suggestions</t>
+          <t>routers/brain.py:172-187 (_KW_STOP, _rx), :294-299 (invoices retrieval), :836-843</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
@@ -25097,7 +25108,7 @@
     <row r="49" ht="82" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>DD-01</t>
+          <t>DX-02</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -25107,12 +25118,12 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Decision Desk</t>
+          <t>Dex</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>/decisions/:id - missing or not yours</t>
+          <t>Ask Dex - 'What needs my attention today?'</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -25127,17 +25138,17 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Give the error branch a 'Back to Decision Desk' button (and the same close control). Branch the copy on status: 403 -&gt; no access, 404 -&gt; 'This decision no longer exists', otherwise 'Couldn't load - Retry'.</t>
+          <t>Treat 'what needs my attention' as a composite intent served from the Desk's own counters (needs_decision, on_fire, overdue, receivables) rather than a single-entity list; or map it to status overdue|in_progress|todo with no date window. Add it to the planner guardrails in _refine_plan, since it is Dex's first suggested question.</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Full-screen 'Access restricted - You don't have access to this decision.' with no Close, no Back and no link. Escape and outside taps are deliberately ignored on the page variant, so the user is trapped until they find the browser Back button. The message is also wrong for a missing decision (the API said 404 'Not found') and for a network error. Decisions are opened from notifications and pasted links, so this is where stale links land.</t>
+          <t>'Good news - there are no open or overdue tasks requiring your attention right now', followed by a list of things already completed. One question later, 'Which tasks are overdue?' answered 'All 34 matching tasks are overdue'. The page's headline suggestion gives the owner false reassurance.</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>components/DecisionDialog.js:188-218 (error branch, page variant handlers)</t>
+          <t>routers/brain.py:127-141 (_plan), :144+ (_refine_plan), :463-478 (_compute_tasks filters); pages/Brain.js suggestions</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr"/>
@@ -25150,7 +25161,7 @@
     <row r="50" ht="82" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>DD-02</t>
+          <t>DD-01</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -25165,7 +25176,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Desk board when loading fails</t>
+          <t>/decisions/:id - missing or not yours</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -25180,17 +25191,17 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Check isError on the board queries; render 'Couldn't load your desk - Retry' and keep counts as '-' rather than 0. Same shared &lt;QueryError&gt; as OP-10 / CR-10 / FN-09.</t>
+          <t>Give the error branch a 'Back to Decision Desk' button (and the same close control). Branch the copy on status: 403 -&gt; no access, 404 -&gt; 'This decision no longer exists', otherwise 'Couldn't load - Retry'.</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>It says 'Nothing waiting on you' with Needs your decision 0, On fire 0, Due today 0, Important 0. The real counts at the time were 53 decisions and 58 on fire. An owner on a weak connection is told the desk is clear.</t>
+          <t>Full-screen 'Access restricted - You don't have access to this decision.' with no Close, no Back and no link. Escape and outside taps are deliberately ignored on the page variant, so the user is trapped until they find the browser Back button. The message is also wrong for a missing decision (the API said 404 'Not found') and for a network error. Decisions are opened from notifications and pasted links, so this is where stale links land.</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>pages/Desk.js:284-292 (boardQs + zero counters)</t>
+          <t>components/DecisionDialog.js:188-218 (error branch, page variant handlers)</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
@@ -25203,7 +25214,7 @@
     <row r="51" ht="82" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>MW-03</t>
+          <t>DD-02</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -25213,12 +25224,12 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Decision Desk</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Header - global search (Cmd+K)</t>
+          <t>Desk board when loading fails</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -25226,24 +25237,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Inside CommandDialog, wrap a DialogTitle (and a DialogDescription) in the VisuallyHidden primitive so the dialog is named for assistive tech without changing the visual design.</t>
+          <t>Check isError on the board queries; render 'Couldn't load your desk - Retry' and keep counts as '-' rather than 0. Same shared &lt;QueryError&gt; as OP-10 / CR-10 / FN-09.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>The dialog exposes aria-labelledby pointing at an element id that does not exist, so it is announced with no name. Radix logs an error every time it opens. Reproduces on My Work and on Finance, so it affects every screen.</t>
+          <t>It says 'Nothing waiting on you' with Needs your decision 0, On fire 0, Due today 0, Important 0. The real counts at the time were 53 decisions and 58 on fire. An owner on a weak connection is told the desk is clear.</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>components/ui/command.jsx:19 (used at components/Layout.js:599)</t>
+          <t>pages/Desk.js:284-292 (boardQs + zero counters)</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
@@ -25256,7 +25267,7 @@
     <row r="52" ht="82" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>MW-04</t>
+          <t>MW-03</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -25271,7 +25282,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Dex FAB picker (mobile)</t>
+          <t>Header - global search (Cmd+K)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -25286,17 +25297,17 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Close the picker on Escape - either a keydown listener while picker is open, or render it inside a Radix DismissableLayer / Popover so dismissal, focus trapping and aria come from the same primitive the other sheets already use.</t>
+          <t>Inside CommandDialog, wrap a DialogTitle (and a DialogDescription) in the VisuallyHidden primitive so the dialog is named for assistive tech without changing the visual design.</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Escape does nothing - the menu stays open and its full-screen scrim keeps blocking the page underneath. Only a pointer tap outside closes it. There is also no focus trap, so keyboard focus walks behind the open menu.</t>
+          <t>The dialog exposes aria-labelledby pointing at an element id that does not exist, so it is announced with no name. Radix logs an error every time it opens. Reproduces on My Work and on Finance, so it affects every screen.</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>components/mobile/DexFab.jsx:70-82</t>
+          <t>components/ui/command.jsx:19 (used at components/Layout.js:599)</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
@@ -25309,7 +25320,7 @@
     <row r="53" ht="82" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>MW-11</t>
+          <t>MW-04</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -25319,12 +25330,12 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Toolbar in the Leave / Workflows views</t>
+          <t>Dex FAB picker (mobile)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -25339,17 +25350,17 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Render the task-scope controls only while view === 'mywork'. Leave the view toggle itself (Workflows / Leave) in place, since that is how you get back. If a scope control must stay, it should not silently change view - that side effect is what makes it feel broken.</t>
+          <t>Close the picker on Escape - either a keydown listener while picker is open, or render it inside a Radix DismissableLayer / Popover so dismissal, focus trapping and aria come from the same primitive the other sheets already use.</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Four task-only controls stay visible in both views - New Task, My Tasks, All Tasks and AI Priority - none of which mean anything for leave or for pipelines. Worse, pressing My Tasks, All Tasks or AI Priority silently throws you back to the task list, losing the view you were in with no warning. In the Leave view 'New Task' is also the largest, darkest button on screen, and it creates a task, not a leave request.</t>
+          <t>Escape does nothing - the menu stays open and its full-screen scrim keeps blocking the page underneath. Only a pointer tap outside closes it. There is also no focus trap, so keyboard focus walks behind the open menu.</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:2429-2515 (mywork-controls / work-view-toggle); handlers at 2442, 2448, 2463</t>
+          <t>components/mobile/DexFab.jsx:70-82</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
@@ -25362,7 +25373,7 @@
     <row r="54" ht="82" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>MW-12</t>
+          <t>MW-11</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -25377,7 +25388,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Leave and Workflows entry points</t>
+          <t>Toolbar in the Leave / Workflows views</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -25392,17 +25403,17 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Pick one home per feature and use it on both viewports. Given Leave already has its own route and its own mobile tile, the cheaper and more consistent direction is to make the standalone page the home on desktop too - see the note on MW-11 about how little of Leave actually belongs in My Work.</t>
+          <t>Render the task-scope controls only while view === 'mywork'. Leave the view toggle itself (Workflows / Leave) in place, since that is how you get back. If a scope control must stay, it should not silently change view - that side effect is what makes it feel broken.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Neither toggle is reachable on mobile - both are in the DOM but hidden, so from My Work there is no way into Leave or Workflows on a phone. They are reachable, but from somewhere else entirely: the 'More' panel lists them as their own destinations. So the same two features are sub-views of My Work on desktop and separate destinations on mobile.</t>
+          <t>Four task-only controls stay visible in both views - New Task, My Tasks, All Tasks and AI Priority - none of which mean anything for leave or for pipelines. Worse, pressing My Tasks, All Tasks or AI Priority silently throws you back to the task list, losing the view you were in with no warning. In the Leave view 'New Task' is also the largest, darkest button on screen, and it creates a task, not a leave request.</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:2476 (work-view-toggle); components/mobile/AllAppsPanel.jsx</t>
+          <t>pages/MyWork.js:2429-2515 (mywork-controls / work-view-toggle); handlers at 2442, 2448, 2463</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
@@ -25415,7 +25426,7 @@
     <row r="55" ht="82" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>MW-17</t>
+          <t>MW-12</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -25430,7 +25441,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Task drawer - two close buttons, invisible focus</t>
+          <t>Leave and Workflows entry points</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -25445,17 +25456,17 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Give SheetContent a hideClose prop (default false, so other sheets are unchanged) and pass it here; set onOpenAutoFocus to focus the title or the close tab. That also resolves which close MW-15 should keep.</t>
+          <t>Pick one home per feature and use it on both viewports. Given Leave already has its own route and its own mobile tile, the cheaper and more consistent direction is to make the standalone page the home on desktop too - see the note on MW-11 about how little of Leave actually belongs in My Work.</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Every drawer carries TWO close buttons: the new 'Close task' tab and the stock shadcn 'Close' that SheetContent always renders. The stock one is covered by the sticky title bar, yet Radix focuses it on open - so keyboard focus starts on a control nobody can see, and a screen reader announces 'Close' and 'Close task' as two separate buttons.</t>
+          <t>Neither toggle is reachable on mobile - both are in the DOM but hidden, so from My Work there is no way into Leave or Workflows on a phone. They are reachable, but from somewhere else entirely: the 'More' panel lists them as their own destinations. So the same two features are sub-views of My Work on desktop and separate destinations on mobile.</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>components/ui/sheet.jsx:46-58; pages/MyWork.js:1427-1445</t>
+          <t>pages/MyWork.js:2476 (work-view-toggle); components/mobile/AllAppsPanel.jsx</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr"/>
@@ -25468,7 +25479,7 @@
     <row r="56" ht="82" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>MW-18</t>
+          <t>MW-17</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -25478,12 +25489,12 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Application shell at wide widths</t>
+          <t>Task drawer - two close buttons, invisible focus</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -25498,17 +25509,17 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Restore the cap in Layout and lift it only where wanted: give My Work its own page-level wrapper (or a data-wide flag the shell reads). If wider is wanted everywhere, cap at ~1600px rather than none, and constrain the Finance tiles and AI brief rows internally.</t>
+          <t>Give SheetContent a hideClose prop (default false, so other sheets are unchanged) and pass it here; set onOpenAutoFocus to focus the title or the close tab. That also resolves which close MW-15 should keep.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>The cap was removed in the shared Layout, so EVERY page now runs edge-to-edge. On Finance each KPI tile is ~610px wide with its value at the far left and its arrow ~550px away; the Capture bar is 1,856px wide holding three small buttons; AI brief rows put the 'Urgent' tag ~1,700px from the sentence it qualifies. On Team each member card is ~610px wide with the name and '6 permissions' at opposite ends. Nothing overflows - it just reads as sparse and makes the eye travel.</t>
+          <t>Every drawer carries TWO close buttons: the new 'Close task' tab and the stock shadcn 'Close' that SheetContent always renders. The stock one is covered by the sticky title bar, yet Radix focuses it on open - so keyboard focus starts on a control nobody can see, and a screen reader announces 'Close' and 'Close task' as two separate buttons.</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>components/Layout.js:634 (app-shell className)</t>
+          <t>components/ui/sheet.jsx:46-58; pages/MyWork.js:1427-1445</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr"/>
@@ -25521,7 +25532,7 @@
     <row r="57" ht="82" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>TM-05</t>
+          <t>MW-18</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -25531,12 +25542,12 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Member profile - ACCESS block</t>
+          <t>Application shell at wide widths</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -25551,17 +25562,17 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Gate the whole ACCESS section, not just its button. This is the same change the founder asked for in ASK-13 and ASK-15, so treat them as one piece of work: hide access on the roster, and show the section only to people who hold the permission that governs it.</t>
+          <t>Restore the cap in Layout and lift it only where wanted: give My Work its own page-level wrapper (or a data-wide flag the shell reads). If wider is wanted everywhere, cap at ~1600px rather than none, and constrain the Finance tiles and AI brief rows internally.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Every role can read every other member's complete permission matrix. Production and Finance -- who hold neither team_manage nor people -- can open Priya Nair's card and see '6 permissions', then inside: '6 of 14 areas', the granted chips, and the full denial list naming every area she cannot reach. Only the Edit access BUTTON is gated to the owner; viewing is not gated at all.</t>
+          <t>The cap was removed in the shared Layout, so EVERY page now runs edge-to-edge. On Finance each KPI tile is ~610px wide with its value at the far left and its arrow ~550px away; the Capture bar is 1,856px wide holding three small buttons; AI brief rows put the 'Urgent' tag ~1,700px from the sentence it qualifies. On Team each member card is ~610px wide with the name and '6 permissions' at opposite ends. Nothing overflows - it just reads as sparse and makes the eye travel.</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:411 + :441 (card count), :580-606 (ACCESS block, granted-perms and the denial list)</t>
+          <t>components/Layout.js:634 (app-shell className)</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr"/>
@@ -25574,7 +25585,7 @@
     <row r="58" ht="82" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>TM-06</t>
+          <t>TM-05</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -25589,7 +25600,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Add member - all form fields</t>
+          <t>Member profile - ACCESS block</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -25604,17 +25615,17 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Give all six a real label with htmlFor pointing at the input's id. Keep placeholders for examples ('e.g. 98765 43210'), not for the field name. This is part of the ASK-14 redesign but is worth doing even if that redesign is deferred -- it is a few lines and it is the difference between the form being usable with a screen reader and not.</t>
+          <t>Gate the whole ACCESS section, not just its button. This is the same change the founder asked for in ASK-13 and ASK-15, so treat them as one piece of work: hide access on the roster, and show the section only to people who hold the permission that governs it.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Not one of the six fields has a programmatic label. Name, Email, Temp password and Mobile number are placeholder-only, so the field name disappears the moment anything is typed -- a sighted user who tabs away and back cannot tell which box is which. Role and Reporting Manager LOOK labelled, but their text is not associated with the control, so a screen reader gets nothing from them either.</t>
+          <t>Every role can read every other member's complete permission matrix. Production and Finance -- who hold neither team_manage nor people -- can open Priya Nair's card and see '6 permissions', then inside: '6 of 14 areas', the granted chips, and the full denial list naming every area she cannot reach. Only the Edit access BUTTON is gated to the owner; viewing is not gated at all.</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:120, :121, :129, :132 (placeholder-only), :137-138 and :143-144 (unassociated labels)</t>
+          <t>pages/Team.js:411 + :441 (card count), :580-606 (ACCESS block, granted-perms and the denial list)</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr"/>
@@ -25627,7 +25638,7 @@
     <row r="59" ht="82" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>CR-02</t>
+          <t>TM-06</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -25637,12 +25648,12 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Add contact dialog - all fields</t>
+          <t>Add member - all form fields</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -25657,17 +25668,17 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Associate a real label with every field here and in Team's Add member (TM-06). Worth doing as one pass over both dialogs rather than twice, and worth adding a lint rule or a test so the next form starts labelled.</t>
+          <t>Give all six a real label with htmlFor pointing at the input's id. Keep placeholders for examples ('e.g. 98765 43210'), not for the field name. This is part of the ASK-14 redesign but is worth doing even if that redesign is deferred -- it is a few lines and it is the difference between the form being usable with a screen reader and not.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>None of the six fields has a label of any kind - the dialog contains no label elements at all. Name, Company, Phone and Email are placeholder-only, and the two selects have nothing naming them. This is the same defect as TM-06 in Team, in a different dialog, which makes it a pattern across the app rather than a one-off.</t>
+          <t>Not one of the six fields has a programmatic label. Name, Email, Temp password and Mobile number are placeholder-only, so the field name disappears the moment anything is typed -- a sighted user who tabs away and back cannot tell which box is which. Role and Reporting Manager LOOK labelled, but their text is not associated with the control, so a screen reader gets nothing from them either.</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:282 (crm-contact-name), :313 (lifecycle), and the four unlabelled inputs between them</t>
+          <t>pages/Team.js:120, :121, :129, :132 (placeholder-only), :137-138 and :143-144 (unassociated labels)</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr"/>
@@ -25680,7 +25691,7 @@
     <row r="60" ht="82" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>CR-06</t>
+          <t>CR-02</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -25695,7 +25706,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Contact cards (mobile)</t>
+          <t>Add contact dialog - all fields</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -25710,17 +25721,17 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Go single column under about 480px, matching Team. If two columns are wanted on larger phones, drop the company line and the touched line to keep the name whole.</t>
+          <t>Associate a real label with every field here and in Team's Add member (TM-06). Worth doing as one pass over both dialogs rather than twice, and worth adding a lint rule or a test so the next form starts labelled.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>The grid stays two columns on a 375px screen, giving each card 161px. Eight text nodes truncate as a result, including the customer names themselves -- 'Krishna Garments Pvt Ltd' needs 144px and gets 114, 'Anand Fabrics' needs 88 and gets 76. Supporting lines like '6 open complaints' and 'Touched 29 days ago' wrap onto two lines, and the card heights go ragged. Team's roster drops to a single column on the same screen and reads cleanly, so the app already has the better answer.</t>
+          <t>None of the six fields has a label of any kind - the dialog contains no label elements at all. Name, Company, Phone and Email are placeholder-only, and the two selects have nothing naming them. This is the same defect as TM-06 in Team, in a different dialog, which makes it a pattern across the app rather than a one-off.</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:940-1050 (contact card grid)</t>
+          <t>pages/CRM.js:282 (crm-contact-name), :313 (lifecycle), and the four unlabelled inputs between them</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr"/>
@@ -25733,7 +25744,7 @@
     <row r="61" ht="82" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>CR-08</t>
+          <t>CR-06</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -25748,7 +25759,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Contact profile (mobile) - In progress list</t>
+          <t>Contact cards (mobile)</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -25763,17 +25774,17 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Guard on the value, not on the humaniser: render the human date when there is one, the raw date only when the value exists but will not parse, and nothing at all when there is no date. Worth grepping for the same `|| \`... ${value}\`` shape elsewhere -- this pattern fails the same way wherever it appears.</t>
+          <t>Go single column under about 480px, matching Team. If two columns are wanted on larger phones, drop the company line and the touched line to keep the name whole.</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>The literal word 'undefined' is printed to the user: two rows read 'Due undefined - Rs 1' and 'Due undefined - Rs 6,00,000'. It is the kind of thing a customer screenshots.</t>
+          <t>The grid stays two columns on a 375px screen, giving each card 161px. Eight text nodes truncate as a result, including the customer names themselves -- 'Krishna Garments Pvt Ltd' needs 144px and gets 114, 'Anand Fabrics' needs 88 and gets 76. Supporting lines like '6 open complaints' and 'Touched 29 days ago' wrap onto two lines, and the card heights go ragged. Team's roster drops to a single column on the same screen and reads cleanly, so the app already has the better answer.</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>pages/mobile/ContactProfileMobile.jsx:215 (fallback), :24 (humanDate)</t>
+          <t>pages/CRM.js:940-1050 (contact card grid)</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr"/>
@@ -25786,7 +25797,7 @@
     <row r="62" ht="82" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>OP-04</t>
+          <t>CR-08</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -25796,12 +25807,12 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>'Sales' category</t>
+          <t>Contact profile (mobile) - In progress list</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -25816,17 +25827,17 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Rename it to what it measures -- Decision velocity, or Approvals -- which is a genuinely good metric for a decision OS. If a real Sales leg is wanted, invoices already carry the data for revenue this period against last.</t>
+          <t>Guard on the value, not on the humaniser: render the human date when there is one, the raw date only when the value exists but will not parse, and nothing at all when there is no date. Worth grepping for the same `|| \`... ${value}\`` shape elsewhere -- this pattern fails the same way wherever it appears.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>It is the share of DECISIONS that have been approved -- approved/total x 100 -- and contains no revenue, no orders, no pipeline and no customer. On live data it reads 22 because 17 of 77 decisions are approved. An owner could sell nothing all month and lift 'Sales' by approving decisions, or have a record month and watch it fall because approvals are backed up. The number is real and useful; the label is the wrong one.</t>
+          <t>The literal word 'undefined' is printed to the user: two rows read 'Due undefined - Rs 1' and 'Due undefined - Rs 6,00,000'. It is the kind of thing a customer screenshots.</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>services/operating_score.py:_score_sales</t>
+          <t>pages/mobile/ContactProfileMobile.jsx:215 (fallback), :24 (humanDate)</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr"/>
@@ -25839,7 +25850,7 @@
     <row r="63" ht="82" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>OP-05</t>
+          <t>OP-04</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -25854,7 +25865,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Operating score model</t>
+          <t>'Sales' category</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -25869,17 +25880,17 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Pick one home for lateness. Execution is the natural one; Responsiveness should be about complaints and reply time, which is what its name promises.</t>
+          <t>Rename it to what it measures -- Decision velocity, or Approvals -- which is a genuinely good metric for a decision OS. If a real Sales leg is wanted, invoices already carry the data for revenue this period against last.</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>One overdue task is charged twice: it raises the overdue ratio inside Execution (x40 of the ratio) and is also subtracted directly from Responsiveness (x3 per task). Those two legs are 35 and 20 per cent of the overall score, so lateness quietly drives 55 per cent of it. On the live tenant that is -20.9 on one leg and -204 on the other.</t>
+          <t>It is the share of DECISIONS that have been approved -- approved/total x 100 -- and contains no revenue, no orders, no pipeline and no customer. On live data it reads 22 because 17 of 77 decisions are approved. An owner could sell nothing all month and lift 'Sales' by approving decisions, or have a record month and watch it fall because approvals are backed up. The number is real and useful; the label is the wrong one.</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>services/operating_score.py:_score_execution and _company_operating_view</t>
+          <t>services/operating_score.py:_score_sales</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr"/>
@@ -25892,7 +25903,7 @@
     <row r="64" ht="82" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>OP-06</t>
+          <t>OP-05</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -25922,17 +25933,17 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Express each as a rate against the relevant denominator -- complaints per active customer, overdue as a share of open work, overdue invoices as a share of open invoices -- so the score means the same thing at any size.</t>
+          <t>Pick one home for lateness. Execution is the natural one; Responsiveness should be about complaints and reply time, which is what its name promises.</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Three penalties are absolute rather than proportional: complaints x12, overdue x3, overdue invoices x5. A five-person shop with 9 open complaints scores 0 on Responsiveness; so does a 500-person company with 9. As a tenant grows, the score falls for reasons that have nothing to do with how well it is run, and the metric stops being comparable with its own past.</t>
+          <t>One overdue task is charged twice: it raises the overdue ratio inside Execution (x40 of the ratio) and is also subtracted directly from Responsiveness (x3 per task). Those two legs are 35 and 20 per cent of the overall score, so lateness quietly drives 55 per cent of it. On the live tenant that is -20.9 on one leg and -204 on the other.</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>services/operating_score.py:_company_operating_view</t>
+          <t>services/operating_score.py:_score_execution and _company_operating_view</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr"/>
@@ -25945,7 +25956,7 @@
     <row r="65" ht="82" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>OP-09</t>
+          <t>OP-06</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -25960,7 +25971,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>'View all' links and the formula panel (mobile)</t>
+          <t>Operating score model</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -25975,17 +25986,17 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Fixing OP-02 -- letting the page scroll as one column on mobile -- makes the formula panel reachable on its own. The View all links still need to grow to 24px minimum and to sit clear of the Dex button's safe area.</t>
+          <t>Express each as a rate against the relevant denominator -- complaints per active customer, overdue as a share of open work, overdue invoices as a share of open invoices -- so the score means the same thing at any size.</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Three problems, all downstream of the page not scrolling on mobile. The two 'View all' links measure 61x20, under the 24px minimum, and the first of them is physically covered by the floating Dex button. The 'How is this calculated' formula panel sits at y=1153 on an 812px screen and cannot be reached at all, so the one place that explains where the score comes from is invisible on a phone -- which matters more than usual here, given two of the four legs read 0.</t>
+          <t>Three penalties are absolute rather than proportional: complaints x12, overdue x3, overdue invoices x5. A five-person shop with 9 open complaints scores 0 on Responsiveness; so does a 500-person company with 9. As a tenant grows, the score falls for reasons that have nothing to do with how well it is run, and the metric stops being comparable with its own past.</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>pages/OperatingScore.js (View all links, operating-formula-toggle)</t>
+          <t>services/operating_score.py:_company_operating_view</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr"/>
@@ -25998,7 +26009,7 @@
     <row r="66" ht="82" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>OP-11</t>
+          <t>OP-09</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -26013,7 +26024,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Personal (self) view - bottom band (mobile)</t>
+          <t>'View all' links and the formula panel (mobile)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -26028,17 +26039,17 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Keep KM-33 for the owner view. In the self view, drop the kr-dark-band class (or add a variant that stays in the scroll flow) and show the peer ranking as an ordinary line or card above the open work. If a pinned sheet is wanted here, it needs content worth pinning and bottom padding that clears the dock.</t>
+          <t>Fixing OP-02 -- letting the page scroll as one column on mobile -- makes the formula panel reachable on its own. The View all links still need to grow to 24px minimum and to sit clear of the Dex button's safe area.</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>A 176px near-black band is pinned to the bottom of every non-owner's phone screen - over a fifth of the viewport - and it holds ONE sentence: 'Among your sales peers you are ranked 2 of 7.' That sentence sits behind the floating dock, so it is only partly readable, and the band does not move when the page scrolls. It reads as a black rendering fault rather than a panel.</t>
+          <t>Three problems, all downstream of the page not scrolling on mobile. The two 'View all' links measure 61x20, under the 24px minimum, and the first of them is physically covered by the floating Dex button. The 'How is this calculated' formula panel sits at y=1153 on an 812px screen and cannot be reached at all, so the one place that explains where the score comes from is invisible on a phone -- which matters more than usual here, given two of the four legs read 0.</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>pages/OperatingScore.js (operating-self-band section); index.css:2171-2190 (.kr-dark-band fixed below lg, KM-33)</t>
+          <t>pages/OperatingScore.js (View all links, operating-formula-toggle)</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr"/>
@@ -26051,7 +26062,7 @@
     <row r="67" ht="82" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>OP-12</t>
+          <t>OP-11</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -26066,7 +26077,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>AI Work Coach - entry point</t>
+          <t>Personal (self) view - bottom band (mobile)</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -26081,17 +26092,17 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Add 'AI coach' next to 'Back to company' in the view-as banner (owner coaching a teammate), and 'My AI coach' on the self view and in the More panel. If the coach is being retired, remove the route and its endpoints instead of leaving it reachable only by URL.</t>
+          <t>Keep KM-33 for the owner view. In the self view, drop the kr-dark-band class (or add a variant that stays in the scroll flow) and show the peer ranking as an ordinary line or card above the open work. If a pinned sheet is wanted here, it needs content worth pinning and bottom padding that clears the dock.</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Nothing in the app links to the AI Work Coach. It still works - it loads for all four roles, the owner can open a teammate's coach, the permission message is right - but the only way in is typing /coach. On 2026-09-12 the Ops employee card opened the coach (plan item D3); it now opens that person's Ops page instead, which removed the last route in. Two of the four demo seats already have coaching generated on 29 Aug, so this is a feature people used.</t>
+          <t>A 176px near-black band is pinned to the bottom of every non-owner's phone screen - over a fifth of the viewport - and it holds ONE sentence: 'Among your sales peers you are ranked 2 of 7.' That sentence sits behind the floating dock, so it is only partly readable, and the band does not move when the page scrolls. It reads as a black rendering fault rather than a panel.</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>App.js:228 (/coach route); pages/OperatingScore.js:931 (employee card link); pages/OperatingScore.js:119-141 (ViewAsBanner)</t>
+          <t>pages/OperatingScore.js (operating-self-band section); index.css:2171-2190 (.kr-dark-band fixed below lg, KM-33)</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr"/>
@@ -26104,7 +26115,7 @@
     <row r="68" ht="82" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>CR-11</t>
+          <t>OP-12</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -26114,12 +26125,12 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Contact profile when loading fails</t>
+          <t>AI Work Coach - entry point</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -26134,17 +26145,17 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Split the branch: if error has no response (network) or a 5xx, say 'Couldn't load this contact' with Retry; keep the 'isn't here' copy for a 404 or an empty body.</t>
+          <t>Add 'AI coach' next to 'Back to company' in the view-as banner (owner coaching a teammate), and 'My AI coach' on the self view and in the More panel. If the coach is being retired, remove the route and its endpoints instead of leaving it reachable only by URL.</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>The page says 'That contact isn't here. It may have been merged or removed.' The customer exists; only the request failed. An owner reading this on a weak phone signal is told a real customer has been deleted or merged.</t>
+          <t>Nothing in the app links to the AI Work Coach. It still works - it loads for all four roles, the owner can open a teammate's coach, the permission message is right - but the only way in is typing /coach. On 2026-09-12 the Ops employee card opened the coach (plan item D3); it now opens that person's Ops page instead, which removed the last route in. Two of the four demo seats already have coaching generated on 29 Aug, so this is a feature people used.</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>pages/ContactProfile.js:151-160; pages/mobile/ContactProfileMobile.jsx:85-99</t>
+          <t>App.js:228 (/coach route); pages/OperatingScore.js:931 (employee card link); pages/OperatingScore.js:119-141 (ViewAsBanner)</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr"/>
@@ -26157,7 +26168,7 @@
     <row r="69" ht="82" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>CR-12</t>
+          <t>CR-11</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -26172,7 +26183,7 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>GET /api/crm/outstanding</t>
+          <t>Contact profile when loading fails</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -26187,17 +26198,17 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Gate it with require_perm('people') (it only feeds the CRM grid) or require_perm('finance') to match the profile endpoint.</t>
+          <t>Split the branch: if error has no response (network) or a 5xx, say 'Couldn't load this contact' with Retry; keep the 'isn't here' copy for a 404 or an empty body.</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>GET /api/contacts and GET /api/contacts/&lt;id&gt;/profile correctly refuse Sales with 403 - but GET /api/crm/outstanding answers 200 with every customer's receivables, payables, invoice count and days overdue. The keys are contact ids rather than names, so it is not a full leak on its own, but it hands money data to roles the rest of the app deliberately keeps out of finance.</t>
+          <t>The page says 'That contact isn't here. It may have been merged or removed.' The customer exists; only the request failed. An owner reading this on a weak phone signal is told a real customer has been deleted or merged.</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>routers/crm.py:37-38 (outstanding_by_contact, Depends(get_current_user))</t>
+          <t>pages/ContactProfile.js:151-160; pages/mobile/ContactProfileMobile.jsx:85-99</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr"/>
@@ -26210,7 +26221,7 @@
     <row r="70" ht="82" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>FN-04</t>
+          <t>CR-12</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -26220,12 +26231,12 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>'Net profit' tile</t>
+          <t>GET /api/crm/outstanding</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -26240,17 +26251,17 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Rename to something the formula actually supports -- 'Billed minus spend', or 'Gross margin (billed)' -- or compute a real net that accounts for COGS and inventory. The former is a one-line change and stops the page overclaiming.</t>
+          <t>Gate it with require_perm('people') (it only feeds the CRM grid) or require_perm('finance') to match the profile endpoint.</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>It is revenue BILLED minus ALL recorded expenses, including expenses not yet paid. It subtracts no cost of goods and no inventory movement, and ignores assets entirely -- Rs 40,85,000 of them. On live data it reports Rs 7,38,034, where the cash-basis figure is Rs 6,44,500, a gap of Rs 93,534. The arithmetic is right; the name is doing more work than the formula can support.</t>
+          <t>GET /api/contacts and GET /api/contacts/&lt;id&gt;/profile correctly refuse Sales with 403 - but GET /api/crm/outstanding answers 200 with every customer's receivables, payables, invoice count and days overdue. The keys are contact ids rather than names, so it is not a full leak on its own, but it hands money data to roles the rest of the app deliberately keeps out of finance.</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>routers/ledger.py:1257 (net_profit); pages/Ledger.js:566-573 (the tile)</t>
+          <t>routers/crm.py:37-38 (outstanding_by_contact, Depends(get_current_user))</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr"/>
@@ -26263,7 +26274,7 @@
     <row r="71" ht="82" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>FN-05</t>
+          <t>FN-04</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -26278,7 +26289,7 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>All figures</t>
+          <t>'Net profit' tile</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -26293,17 +26304,17 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Accept a period parameter (this month, this quarter, this FY -- the Indian financial year matters here) and filter each query by it, defaulting to the current month. That single change also gives FN-02 and FN-03 the data they are currently faking.</t>
+          <t>Rename to something the formula actually supports -- 'Billed minus spend', or 'Gross margin (billed)' -- or compute a real net that accounts for COGS and inventory. The former is a one-line change and stops the page overclaiming.</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Every figure is all-time and there is no way to change that. Expenses, invoices, payments, assets and inventory are each queried for the whole tenant with no window and capped at 5000 records. So the page can tell an owner what they have billed since the company started, but not what they billed this month -- which is the question a finance screen is opened to answer. It is also why FN-02's 'This month' chip has nothing to bind to.</t>
+          <t>It is revenue BILLED minus ALL recorded expenses, including expenses not yet paid. It subtracts no cost of goods and no inventory movement, and ignores assets entirely -- Rs 40,85,000 of them. On live data it reports Rs 7,38,034, where the cash-basis figure is Rs 6,44,500, a gap of Rs 93,534. The arithmetic is right; the name is doing more work than the formula can support.</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>routers/ledger.py:1223-1262 (ledger_summary)</t>
+          <t>routers/ledger.py:1257 (net_profit); pages/Ledger.js:566-573 (the tile)</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr"/>
@@ -26316,7 +26327,7 @@
     <row r="72" ht="82" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>FN-09</t>
+          <t>FN-05</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -26331,7 +26342,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Finance when a request fails</t>
+          <t>All figures</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -26346,17 +26357,17 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Check isError on each query and render 'Couldn't load &lt;tab&gt;' with Retry (403: 'You don't have access to the ledger'). One shared &lt;QueryError&gt; would serve this, OP-10 and CR-10.</t>
+          <t>Accept a period parameter (this month, this quarter, this FY -- the Indian financial year matters here) and filter each query by it, defaulting to the current month. That single change also gives FN-02 and FN-03 the data they are currently faking.</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Summary fails: the Overview says 'Loading...' indefinitely. Expenses fails: the Expenses tab shows 'No expenses yet - approved purchase bills and payments show up here automatically, or add one manually', directly under an AI panel that is still analysing those same expenses. An owner on a bad connection is told their books are empty. The same missing branch is behind FN-07.</t>
+          <t>Every figure is all-time and there is no way to change that. Expenses, invoices, payments, assets and inventory are each queried for the whole tenant with no window and capped at 5000 records. So the page can tell an owner what they have billed since the company started, but not what they billed this month -- which is the question a finance screen is opened to answer. It is also why FN-02's 'This month' chip has nothing to bind to.</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1522-1527, :1641-1642, :1657-1659</t>
+          <t>routers/ledger.py:1223-1262 (ledger_summary)</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr"/>
@@ -26369,7 +26380,7 @@
     <row r="73" ht="82" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>MW-22</t>
+          <t>FN-09</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -26379,12 +26390,12 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Task card - bulk-select checkbox (mobile)</t>
+          <t>Finance when a request fails</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -26399,17 +26410,17 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Give the checkbox a 44x44 hit area again (a padded label around it, or a transparent ::before), and keep stopPropagation on that area so it never opens the drawer.</t>
+          <t>Check isError on each query and render 'Couldn't load &lt;tab&gt;' with Retry (403: 'You don't have access to the ledger'). One shared &lt;QueryError&gt; would serve this, OP-10 and CR-10.</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>The checkbox is now 16x16 inside a 16x22 label - nothing larger is clickable. A tap 10px off in any direction lands on the card, and since 78d01df the whole card opens the task drawer. So on a phone, trying to select tasks for a bulk action frequently opens a task instead. 12 checkboxes on the first screen, all the same.</t>
+          <t>Summary fails: the Overview says 'Loading...' indefinitely. Expenses fails: the Expenses tab shows 'No expenses yet - approved purchase bills and payments show up here automatically, or add one manually', directly under an AI panel that is still analysing those same expenses. An owner on a bad connection is told their books are empty. The same missing branch is behind FN-07.</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js (task card summary - bulk-select checkbox, top-left)</t>
+          <t>pages/Ledger.js:1522-1527, :1641-1642, :1657-1659</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr"/>
@@ -26422,7 +26433,7 @@
     <row r="74" ht="82" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>GL-01</t>
+          <t>MW-22</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -26432,12 +26443,12 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Desktop header - notification bell</t>
+          <t>Task card - bulk-select checkbox (mobile)</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -26452,17 +26463,17 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Move Bellicon to module scope (a real component that takes notif/unread/bellCount as props), or render the Popover JSX inline rather than through an inner component. The same applies to any other component declared inside Layout.</t>
+          <t>Give the checkbox a 44x44 hit area again (a padded label around it, or a transparent ::before), and keep stopPropagation on that area so it never opens the drawer.</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>On Decision Desk, My Work and Team the dropdown opens and then closes on its own about 0.4s later, dropping focus to &lt;body&gt;; nothing was clicked in between. On Finance it stays open. So on the desktop's most-used pages a user clicks the bell, sees a flash, and cannot read or open a notification. (The phone bell works.)</t>
+          <t>The checkbox is now 16x16 inside a 16x22 label - nothing larger is clickable. A tap 10px off in any direction lands on the card, and since 78d01df the whole card opens the task drawer. So on a phone, trying to select tasks for a bulk action frequently opens a task instead. 12 checkboxes on the first screen, all the same.</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>components/Layout.js:366-424 (Bellicon inside Layout)</t>
+          <t>pages/MyWork.js (task card summary - bulk-select checkbox, top-left)</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr"/>
@@ -26475,7 +26486,7 @@
     <row r="75" ht="82" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>GL-02</t>
+          <t>GL-01</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -26490,7 +26501,7 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Mobile More panel - non-owners</t>
+          <t>Desktop header - notification bell</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -26505,17 +26516,17 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Align the tile filters with the routes: show Ops to everyone (it already renders a self view), Team to everyone (read-only for non-managers), and Settings to everyone (profile + security for non-owners).</t>
+          <t>Move Bellicon to module scope (a real component that takes notif/unread/bellCount as props), or render the Popover JSX inline rather than through an inner component. The same applies to any other component declared inside Layout.</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>On a phone, Sales, Production and Finance see only two tiles: Workflows and Leave. They cannot reach Ops, Team or Settings, although all three routes open for them and the desktop nav shows them Ops and Team. Ops was deliberately opened to every role so staff see their own metrics (App.js:222-226) - on mobile that view is unreachable.</t>
+          <t>On Decision Desk, My Work and Team the dropdown opens and then closes on its own about 0.4s later, dropping focus to &lt;body&gt;; nothing was clicked in between. On Finance it stays open. So on the desktop's most-used pages a user clicks the bell, sees a flash, and cannot read or open a notification. (The phone bell works.)</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>components/mobile/AllAppsPanel.jsx:70-83 and :127 (tile filters)</t>
+          <t>components/Layout.js:366-424 (Bellicon inside Layout)</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr"/>
@@ -26528,7 +26539,7 @@
     <row r="76" ht="82" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>DD-03</t>
+          <t>GL-02</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -26538,12 +26549,12 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Decision Desk</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Money tiles for Sales / Production</t>
+          <t>Mobile More panel - non-owners</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -26558,17 +26569,17 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Render money tiles only when hasPerm(user,'finance') || hasPerm(user,'ledger'); otherwise show the role's own tiles.</t>
+          <t>Align the tile filters with the routes: show Ops to everyone (it already renders a self view), Team to everyone (read-only for non-managers), and Settings to everyone (profile + security for non-owners).</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>'Net profit' and 'Spend, this month' show '...' forever - their data (ledger summary) is refused with 403 - while 'To collect (overdue) Rs 7.5 L' is shown to these roles, a customer-receivables figure they have no finance permission for. Tapping the money tiles leads to the empty Finance page of FN-07.</t>
+          <t>On a phone, Sales, Production and Finance see only two tiles: Workflows and Leave. They cannot reach Ops, Team or Settings, although all three routes open for them and the desktop nav shows them Ops and Team. Ops was deliberately opened to every role so staff see their own metrics (App.js:222-226) - on mobile that view is unreachable.</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>pages/Desk.js:563-661 (KPI tiles), pages/desk/useDeskMetrics.js</t>
+          <t>components/mobile/AllAppsPanel.jsx:70-83 and :127 (tile filters)</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr"/>
@@ -26581,7 +26592,7 @@
     <row r="77" ht="82" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>CL-01</t>
+          <t>DD-03</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -26591,12 +26602,12 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Decision Desk</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Notifications, People, Journal, Calendar when loading fails</t>
+          <t>Money tiles for Sales / Production</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -26611,17 +26622,17 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>One shared &lt;QueryError onRetry&gt; used wherever a query's data drives the page; branch 403 vs other errors. Fixing it once fixes OP-10, CR-10, FN-09, DD-02 and this.</t>
+          <t>Render money tiles only when hasPerm(user,'finance') || hasPerm(user,'ledger'); otherwise show the role's own tiles.</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Notifications says 'You're all caught up.' People says 'Members 0 - No team members yet.' Calendar shows every filter at 0. Journal shows only its header and nothing below. None says anything failed. With OP-10, CR-10, FN-09 and DD-02 this is the same fault on nine surfaces.</t>
+          <t>'Net profit' and 'Spend, this month' show '...' forever - their data (ledger summary) is refused with 403 - while 'To collect (overdue) Rs 7.5 L' is shown to these roles, a customer-receivables figure they have no finance permission for. Tapping the money tiles leads to the empty Finance page of FN-07.</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>pages/Notifications.js:14, pages/People.js:47-53, pages/Journal.js:185, pages/Calendar.js:62</t>
+          <t>pages/Desk.js:563-661 (KPI tiles), pages/desk/useDeskMetrics.js</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr"/>
@@ -26634,7 +26645,7 @@
     <row r="78" ht="82" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>CL-02</t>
+          <t>CL-01</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -26644,12 +26655,12 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Calendar events</t>
+          <t>Notifications, People, Journal, Calendar when loading fails</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -26664,17 +26675,17 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Wrap each event in a Link to its source (task -&gt; /my-work?task=, decision -&gt; /decisions/, invoice -&gt; /finance?tab=revenue, leave -&gt; /team).</t>
+          <t>One shared &lt;QueryError onRetry&gt; used wherever a query's data drives the page; branch 403 vs other errors. Fixing it once fixes OP-10, CR-10, FN-09, DD-02 and this.</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Nothing happens. Events are plain &lt;div&gt;s with no link or handler, so the calendar shows 'Vendor Call - Next Monday - Overdue' but the user cannot get from it to the task to act on it.</t>
+          <t>Notifications says 'You're all caught up.' People says 'Members 0 - No team members yet.' Calendar shows every filter at 0. Journal shows only its header and nothing below. None says anything failed. With OP-10, CR-10, FN-09 and DD-02 this is the same fault on nine surfaces.</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>pages/Calendar.js:233 (cal-event)</t>
+          <t>pages/Notifications.js:14, pages/People.js:47-53, pages/Journal.js:185, pages/Calendar.js:62</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr"/>
@@ -26687,7 +26698,7 @@
     <row r="79" ht="82" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>MW-13</t>
+          <t>CL-02</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -26697,12 +26708,12 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Workflows view - pipeline cards</t>
+          <t>Calendar events</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -26710,24 +26721,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F79" s="8" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="F79" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Give each an aria-label that names its card, e.g. 'Delete card: Dispatch 100 sales items today'. The card title is already to hand where the button is rendered.</t>
+          <t>Wrap each event in a Link to its source (task -&gt; /my-work?task=, decision -&gt; /decisions/, invoice -&gt; /finance?tab=revenue, leave -&gt; /team).</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Five separate buttons are all named exactly 'Delete card', and two are both named 'Advance to Delivered'. Sighted users tell them apart by which card they sit on; a screen-reader user hears the same phrase five times with nothing to say which shipment is about to be deleted. Deletion is the most destructive action in the view, which is what lifts this above cosmetic.</t>
+          <t>Nothing happens. Events are plain &lt;div&gt;s with no link or handler, so the calendar shows 'Vendor Call - Next Monday - Overdue' but the user cannot get from it to the task to act on it.</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>pages/Workflows.js (delete-workflow-* and advance-workflow-* buttons)</t>
+          <t>pages/Calendar.js:233 (cal-event)</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr"/>
@@ -26740,7 +26751,7 @@
     <row r="80" ht="82" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>MW-19</t>
+          <t>MW-13</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -26755,7 +26766,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Department filter dropdown</t>
+          <t>Workflows view - pipeline cards</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -26770,17 +26781,17 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Filter options to count &gt; 0 (keep All), or render zero-count ones disabled; move Completed into the Status dropdown.</t>
+          <t>Give each an aria-label that names its card, e.g. 'Delete card: Dispatch 100 sales items today'. The card title is already to hand where the button is rendered.</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Three problems. (1) 'Completed 7' is listed as a Department - it is a state, and the Status dropdown beside it is where it belongs. (2) Six of the nine options read 0 (Sales 0, Production 0, Quality Control 0, Inventory 0, Finance 0, HR 0) - the old chip strip hid empty categories on a founder ask (U7-05.9). (3) Picking an empty one is silently undone: the trigger still reads 'Department: All 26' and nothing tells the user why.</t>
+          <t>Five separate buttons are all named exactly 'Delete card', and two are both named 'Advance to Delivered'. Sighted users tell them apart by which card they sit on; a screen-reader user hears the same phrase five times with nothing to say which shipment is about to be deleted. Deletion is the most destructive action in the view, which is what lifts this above cosmetic.</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:2042-2075 (FilterDropdown), :2735-2743 (Department options), :2288-2298 (snap-back effect)</t>
+          <t>pages/Workflows.js (delete-workflow-* and advance-workflow-* buttons)</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr"/>
@@ -26793,7 +26804,7 @@
     <row r="81" ht="82" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>TM-01</t>
+          <t>MW-19</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -26803,12 +26814,12 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Add member - login method toggle</t>
+          <t>Department filter dropdown</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -26823,17 +26834,17 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Add aria-pressed to both buttons, and wrap them in a role='group' with an accessible label such as 'Login method' - matching the permission grid immediately below it.</t>
+          <t>Filter options to count &gt; 0 (keep All), or render zero-count ones disabled; move Completed into the Status dropdown.</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Neither half carries aria-pressed. The selection is conveyed only by a class swap (kr-pressed against kr-pop), so a sighted user sees which method is active and a screen-reader user hears two identical unlabelled buttons. Choosing between a password and an OTP decides how that person will sign in for good, so it is worth announcing.</t>
+          <t>Three problems. (1) 'Completed 7' is listed as a Department - it is a state, and the Status dropdown beside it is where it belongs. (2) Six of the nine options read 0 (Sales 0, Production 0, Quality Control 0, Inventory 0, Finance 0, HR 0) - the old chip strip hid empty categories on a founder ask (U7-05.9). (3) Picking an empty one is silently undone: the trigger still reads 'Department: All 26' and nothing tells the user why.</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:122-127 (login-method-toggle); the pattern to copy is at :165</t>
+          <t>pages/MyWork.js:2042-2075 (FilterDropdown), :2735-2743 (Department options), :2288-2298 (snap-back effect)</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr"/>
@@ -26846,7 +26857,7 @@
     <row r="82" ht="82" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>TM-07</t>
+          <t>TM-01</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -26861,7 +26872,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Member profile dialog - closing</t>
+          <t>Add member - login method toggle</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -26876,17 +26887,17 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Keep the Dialog mounted with open={!!u} and render only its content conditionally, so Radix's own focus return runs; or remember the opening card and focus it in onCloseAutoFocus.</t>
+          <t>Add aria-pressed to both buttons, and wrap them in a role='group' with an accessible label such as 'Login method' - matching the permission grid immediately below it.</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Focus drops to &lt;body&gt;. A keyboard or screen-reader user who opens the fifth card and closes it is thrown back to the top of the page and has to Tab through the header, search and every earlier card to get back. On a 12-person roster that is a nuisance; on the larger teams the search box is built for, it makes the roster hard to work through.</t>
+          <t>Neither half carries aria-pressed. The selection is conveyed only by a class swap (kr-pressed against kr-pop), so a sighted user sees which method is active and a screen-reader user hears two identical unlabelled buttons. Choosing between a password and an OTP decides how that person will sign in for good, so it is worth announcing.</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:450 (onOpen sets profileUser), :541-542 (openChange, 'if (!u) return null')</t>
+          <t>pages/Team.js:122-127 (login-method-toggle); the pattern to copy is at :165</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr"/>
@@ -26899,7 +26910,7 @@
     <row r="83" ht="82" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>TM-08</t>
+          <t>TM-07</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -26909,12 +26920,12 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Default close button on every dialog</t>
+          <t>Member profile dialog - closing</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -26929,17 +26940,17 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Give the default close a hit area: 'grid h-8 w-8 place-items-center' around the icon (32px), keeping the icon at 16px. One change fixes every dialog at once.</t>
+          <t>Keep the Dialog mounted with open={!!u} and render only its content conditionally, so Radix's own focus return runs; or remember the opening card and focus it in onCloseAutoFocus.</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>On desktop the close X is 16x16px - the bare icon with no padding. On mobile the same control measures 44x44, so the fault is desktop-only. It comes from the shared dialog component, so it applies to every dialog that keeps the default close: Add member, Edit access, the invite link modal, and the rest of the app's dialogs that use it. The Team profile dialog avoids it by hiding the default and drawing its own 36px close.</t>
+          <t>Focus drops to &lt;body&gt;. A keyboard or screen-reader user who opens the fifth card and closes it is thrown back to the top of the page and has to Tab through the header, search and every earlier card to get back. On a 12-person roster that is a nuisance; on the larger teams the search box is built for, it makes the roster hard to work through.</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>components/ui/dialog.jsx:37-41</t>
+          <t>pages/Team.js:450 (onOpen sets profileUser), :541-542 (openChange, 'if (!u) return null')</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr"/>
@@ -26952,7 +26963,7 @@
     <row r="84" ht="82" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>CR-01</t>
+          <t>TM-08</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -26962,12 +26973,12 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Scope chips (Buyers / Suppliers)</t>
+          <t>Default close button on every dialog</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -26982,17 +26993,17 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Add aria-pressed to the desktop chips, mirroring the mobile pair, and give the row a role='group' with a label. Same family as TM-01.</t>
+          <t>Give the default close a hit area: 'grid h-8 w-8 place-items-center' around the icon (32px), keeping the icon at 16px. One change fixes every dialog at once.</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>The desktop chips carry no aria-pressed at all, while the mobile twins of the same control set it correctly (true on Buyers, false on Suppliers). So the identical control is announced properly on a phone and not on a laptop. The filtering itself is correct - Buyers shows 11, Suppliers shows 6, and switching back restores 11.</t>
+          <t>On desktop the close X is 16x16px - the bare icon with no padding. On mobile the same control measures 44x44, so the fault is desktop-only. It comes from the shared dialog component, so it applies to every dialog that keeps the default close: Add member, Edit access, the invite link modal, and the rest of the app's dialogs that use it. The Team profile dialog avoids it by hiding the default and drawing its own 36px close.</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:819-836 (crm-scope-chips, desktop); the correct pattern is at :794-805 (crm-scope-mobile)</t>
+          <t>components/ui/dialog.jsx:37-41</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr"/>
@@ -27005,7 +27016,7 @@
     <row r="85" ht="82" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>CR-07</t>
+          <t>CR-01</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -27020,7 +27031,7 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Contact profile - Log activity</t>
+          <t>Scope chips (Buyers / Suppliers)</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -27035,17 +27046,17 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Repaint Log with the standard primary, and check the contact profile's background against the list it is reached from -- a detail page changing ground colour makes the two feel like separate apps.</t>
+          <t>Add aria-pressed to the desktop chips, mirroring the mobile pair, and give the row a role='group' with a label. Same family as TM-01.</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>The Log button on the contact profile is indigo, rgb(55,58,205), while every other primary action in the app -- Add contact, Add member, Complete, Approve -- is the near-black ink colour. Contrast is fine at 7.93:1; the problem is that it reads as a different product for a moment. The contact profile also sits on a strong amber gradient while the CRM list it came from is neutral grey, which compounds the shift.</t>
+          <t>The desktop chips carry no aria-pressed at all, while the mobile twins of the same control set it correctly (true on Buyers, false on Suppliers). So the identical control is announced properly on a phone and not on a laptop. The filtering itself is correct - Buyers shows 11, Suppliers shows 6, and switching back restores 11.</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>pages/ContactProfile.js (Log button and page background)</t>
+          <t>pages/CRM.js:819-836 (crm-scope-chips, desktop); the correct pattern is at :794-805 (crm-scope-mobile)</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr"/>
@@ -27058,7 +27069,7 @@
     <row r="86" ht="82" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>OP-07</t>
+          <t>CR-07</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -27068,12 +27079,12 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Operating score - empty workspace</t>
+          <t>Contact profile - Log activity</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -27088,17 +27099,17 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Keep the neutral internal default if it helps the maths, but let the UI show 'not enough data yet' rather than a score, using the enough_data flag that is already computed and sent.</t>
+          <t>Repaint Log with the standard primary, and check the contact profile's background against the list it is reached from -- a detail page changing ground colour makes the two feel like separate apps.</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Completion, approval rate and collection rate each fall back to 0.7 when there is nothing to divide by, so a brand-new tenant that has done nothing at all scores about 70 out of 100 and is told it is doing reasonably well. There is an enough_data flag in the payload, so the page can already tell the difference -- the default just makes the number look earned.</t>
+          <t>The Log button on the contact profile is indigo, rgb(55,58,205), while every other primary action in the app -- Add contact, Add member, Complete, Approve -- is the near-black ink colour. Contrast is fine at 7.93:1; the problem is that it reads as a different product for a moment. The contact profile also sits on a strong amber gradient while the CRM list it came from is neutral grey, which compounds the shift.</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>services/operating_score.py (the 0.7 defaults, enough_data)</t>
+          <t>pages/ContactProfile.js (Log button and page background)</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr"/>
@@ -27111,7 +27122,7 @@
     <row r="87" ht="82" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>OP-08</t>
+          <t>OP-07</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -27126,7 +27137,7 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Category cards</t>
+          <t>Operating score - empty workspace</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -27141,17 +27152,17 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Give a floored score its own treatment -- a filled track in the warning colour, or an explicit 'at floor' marker -- so it reads as a measured bad result rather than an absent one.</t>
+          <t>Keep the neutral internal default if it helps the maths, but let the UI show 'not enough data yet' rather than a score, using the enough_data flag that is already computed and sent.</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Execution and Responsiveness both render '0 / 100' above a completely empty progress bar, which is pixel-identical to how an unmeasured category would look. Two of the four cards on the page therefore read as 'nothing here' when they actually mean 'this is as bad as it gets'.</t>
+          <t>Completion, approval rate and collection rate each fall back to 0.7 when there is nothing to divide by, so a brand-new tenant that has done nothing at all scores about 70 out of 100 and is told it is doing reasonably well. There is an enough_data flag in the payload, so the page can already tell the difference -- the default just makes the number look earned.</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>pages/OperatingScore.js (category card progress track)</t>
+          <t>services/operating_score.py (the 0.7 defaults, enough_data)</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr"/>
@@ -27164,7 +27175,7 @@
     <row r="88" ht="82" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>OP-13</t>
+          <t>OP-08</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -27179,7 +27190,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>'Back to company' and 'See all' links</t>
+          <t>Category cards</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -27194,17 +27205,17 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Give both links py-1.5 (or min-h-6 with inline-flex items-center) so the hit area reaches 24px without changing the look. Fix with OP-09 in one pass.</t>
+          <t>Give a floored score its own treatment -- a filled track in the warning colour, or an explicit 'at floor' marker -- so it reads as a measured bad result rather than an absent one.</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>'Back to company' in the view-as banner is 109x16 on desktop and 117x20 on mobile - and it is the only way out of view-as mode other than the browser. 'See all' above 'Your open work' is 52x16 on desktop and 55x20 on mobile, on every non-owner's page. Same pattern as the 'View all' links in OP-09, on two screens OP-09 did not cover.</t>
+          <t>Execution and Responsiveness both render '0 / 100' above a completely empty progress bar, which is pixel-identical to how an unmeasured category would look. Two of the four cards on the page therefore read as 'nothing here' when they actually mean 'this is as bad as it gets'.</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>pages/OperatingScore.js:133-139 (Back to company); the 'See all' link in the self view's open-work header</t>
+          <t>pages/OperatingScore.js (category card progress track)</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr"/>
@@ -27217,7 +27228,7 @@
     <row r="89" ht="82" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>OP-14</t>
+          <t>OP-13</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -27232,7 +27243,7 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>AI Work Coach - error page</t>
+          <t>'Back to company' and 'See all' links</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -27247,17 +27258,17 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Branch the title too: 403 -&gt; 'Not allowed', 404 -&gt; 'Person not found', otherwise 'Couldn't load coaching'.</t>
+          <t>Give both links py-1.5 (or min-h-6 with inline-flex items-center) so the hit area reaches 24px without changing the look. Fix with OP-09 in one pass.</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>The page is titled 'Access denied' while its body says 'Couldn't load coaching - Something went wrong.' Nothing was denied: the owner may view anyone's coach, and the API answered 404 'Employee not found'. The title blames permissions for a missing person.</t>
+          <t>'Back to company' in the view-as banner is 109x16 on desktop and 117x20 on mobile - and it is the only way out of view-as mode other than the browser. 'See all' above 'Your open work' is 52x16 on desktop and 55x20 on mobile, on every non-owner's page. Same pattern as the 'View all' links in OP-09, on two screens OP-09 did not cover.</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>pages/WorkCoach.js:36-57</t>
+          <t>pages/OperatingScore.js:133-139 (Back to company); the 'See all' link in the self view's open-work header</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr"/>
@@ -27270,7 +27281,7 @@
     <row r="90" ht="82" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>CR-09</t>
+          <t>OP-14</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -27280,12 +27291,12 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Contact profile (mobile) - Score with AI</t>
+          <t>AI Work Coach - error page</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -27300,17 +27311,17 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Add a 'Score with AI' action to the mobile profile's action row, reusing the same POST /contacts/{id}/rescore mutation - or record that scoring is desktop-only by design.</t>
+          <t>Branch the title too: 403 -&gt; 'Not allowed', 404 -&gt; 'Person not found', otherwise 'Couldn't load coaching'.</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Desktop has 'Score with AI' (and 'Re-score'); its failure path works - 'Could not score right now', label restored. The mobile contact profile has no scoring control at all, only a read-only 'Health nn/100' row, so the score cannot be refreshed from a phone.</t>
+          <t>The page is titled 'Access denied' while its body says 'Couldn't load coaching - Something went wrong.' Nothing was denied: the owner may view anyone's coach, and the API answered 404 'Employee not found'. The title blames permissions for a missing person.</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>pages/ContactProfile.js:134-137 + :250-273 (desktop); pages/mobile/ContactProfileMobile.jsx:254 (Health row only)</t>
+          <t>pages/WorkCoach.js:36-57</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr"/>
@@ -27323,7 +27334,7 @@
     <row r="91" ht="82" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>CR-13</t>
+          <t>CR-09</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -27338,7 +27349,7 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Decision Desk 'Complaints' tile -&gt; /crm</t>
+          <t>Contact profile (mobile) - Score with AI</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -27353,17 +27364,17 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Only set the link when hasPerm(user, 'people'); otherwise render the tile as plain (non-link) or point it at a view the role can open.</t>
+          <t>Add a 'Score with AI' action to the mobile profile's action row, reusing the same POST /contacts/{id}/rescore mutation - or record that scoring is desktop-only by design.</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>CRM itself is correctly hidden and a direct visit shows Access Denied - but the 'Complaints' KPI tile on Decision Desk links to /crm for all three roles, on desktop and mobile. Tapping the number lands on 'ACCESS DENIED'. It is the most prominent link on their home screen to a page they are not allowed to see.</t>
+          <t>Desktop has 'Score with AI' (and 'Re-score'); its failure path works - 'Could not score right now', label restored. The mobile contact profile has no scoring control at all, only a read-only 'Health nn/100' row, so the score cannot be refreshed from a phone.</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>pages/Desk.js:569-572 (mobile tile), :614-617 (desktop tile)</t>
+          <t>pages/ContactProfile.js:134-137 + :250-273 (desktop); pages/mobile/ContactProfileMobile.jsx:254 (Health row only)</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr"/>
@@ -27376,7 +27387,7 @@
     <row r="92" ht="82" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>CR-14</t>
+          <t>CR-13</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -27391,7 +27402,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Contact profile - 'Back to CRM' (desktop)</t>
+          <t>Decision Desk 'Complaints' tile -&gt; /crm</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -27406,17 +27417,17 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>py-1 or min-h-6 on the back link.</t>
+          <t>Only set the link when hasPerm(user, 'people'); otherwise render the tile as plain (non-link) or point it at a view the role can open.</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>'Back to CRM' is 103x20 - the only other interactive element under 24px on the page. The mobile 'Back to people' is fine.</t>
+          <t>CRM itself is correctly hidden and a direct visit shows Access Denied - but the 'Complaints' KPI tile on Decision Desk links to /crm for all three roles, on desktop and mobile. Tapping the number lands on 'ACCESS DENIED'. It is the most prominent link on their home screen to a page they are not allowed to see.</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>pages/ContactProfile.js:205 (profile-back)</t>
+          <t>pages/Desk.js:569-572 (mobile tile), :614-617 (desktop tile)</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr"/>
@@ -27429,7 +27440,7 @@
     <row r="93" ht="82" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>FN-10</t>
+          <t>CR-14</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -27439,12 +27450,12 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Mobile capture card - 'Export' tile</t>
+          <t>Contact profile - 'Back to CRM' (desktop)</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -27459,17 +27470,17 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Rename it 'Import - CSV, Excel' with an upload icon. If export is wanted, build it as a separate action.</t>
+          <t>py-1 or min-h-6 on the back link.</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>The fourth tile reads 'Export - CSV, Excel' but is a file picker that UPLOADS a spreadsheet to /ingest/csv. An owner wanting to download their books for the accountant taps it and gets a file-open dialog. Desktop labels the same control correctly as 'CSV / Excel' under Capture. There is no export anywhere on the page.</t>
+          <t>'Back to CRM' is 103x20 - the only other interactive element under 24px on the page. The mobile 'Back to people' is fine.</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1430-1437</t>
+          <t>pages/ContactProfile.js:205 (profile-back)</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr"/>
@@ -27482,7 +27493,7 @@
     <row r="94" ht="82" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>FN-11</t>
+          <t>FN-10</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -27497,7 +27508,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Mobile overview - 'View all 3+ action items'</t>
+          <t>Mobile capture card - 'Export' tile</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -27512,17 +27523,17 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>py-1 on the link.</t>
+          <t>Rename it 'Import - CSV, Excel' with an upload icon. If export is wanted, build it as a separate action.</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>'View all 3+ action items' is 322x20 - wide but under 24px tall. It works (opens the Revenue tab).</t>
+          <t>The fourth tile reads 'Export - CSV, Excel' but is a file picker that UPLOADS a spreadsheet to /ingest/csv. An owner wanting to download their books for the accountant taps it and gets a file-open dialog. Desktop labels the same control correctly as 'CSV / Excel' under Capture. There is no export anywhere on the page.</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:1075 (ledger-mobile-viewall)</t>
+          <t>pages/Ledger.js:1430-1437</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr"/>
@@ -27535,7 +27546,7 @@
     <row r="95" ht="82" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>MW-05</t>
+          <t>FN-11</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -27545,12 +27556,12 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Task list - bento grid</t>
+          <t>Mobile overview - 'View all 3+ action items'</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -27565,17 +27576,17 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Make the button a column flex container and pin content to the top - add 'flex flex-col justify-start' to its className. Verified live in the browser: all three titles then start at 17px.</t>
+          <t>py-1 on the link.</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Titles in one row start at different heights - the spread was 39px, 17px, 11px and 17px across the first four rows. A short title sinks toward the middle of its card while a long one starts at the top, so the row reads as ragged. The checkboxes stay aligned, which makes it more obvious.</t>
+          <t>'View all 3+ action items' is 322x20 - wide but under 24px tall. It works (opens the Revenue tab).</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:1181 (the task-summary button className)</t>
+          <t>pages/Ledger.js:1075 (ledger-mobile-viewall)</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr"/>
@@ -27588,7 +27599,7 @@
     <row r="96" ht="82" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>FN-12</t>
+          <t>MW-05</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -27598,12 +27609,12 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Ask AI about your expenses - answer</t>
+          <t>Task list - bento grid</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -27618,17 +27629,17 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Render the answer through the same markdown renderer Dex uses (or strip ** server-side).</t>
+          <t>Make the button a column flex container and pin content to the top - add 'flex flex-col justify-start' to its className. Verified live in the browser: all three titles then start at 17px.</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>The answer is correct - Surat Spinners, Rs 4,80,000, matching the data - but it is shown with literal markdown: '**Surat Spinners**' and '**Rs 4,80,000**', asterisks visible.</t>
+          <t>Titles in one row start at different heights - the spread was 39px, 17px, 11px and 17px across the first four rows. A short title sinks toward the middle of its card while a long one starts at the top, so the row reads as ragged. The checkboxes stay aligned, which makes it more obvious.</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>pages/Ledger.js:539 (ai-answer)</t>
+          <t>pages/MyWork.js:1181 (the task-summary button className)</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr"/>
@@ -27641,7 +27652,7 @@
     <row r="97" ht="82" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>FN-13</t>
+          <t>FN-12</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -27656,7 +27667,7 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Capture - extraction review</t>
+          <t>Ask AI about your expenses - answer</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -27671,17 +27682,17 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Carry invoice date, GSTIN (and GST amount) and line items through to review; flag bills whose date or due date is more than ~12 months old before 'File it'.</t>
+          <t>Render the answer through the same markdown renderer Dex uses (or strip ** server-side).</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Good overall, in 31.9s at 92% confidence: supplier Service TEST 123 with phone and email, number X33, amount 27,625, due 2018-03-01, booked as Inventory, and a 'Pay vendor bill' follow-up task. But the invoice DATE, the supplier GSTIN and the line items are not captured, and nothing warns that the bill fell due eight years ago - filing it would add an overdue payable dated 2018 without comment.</t>
+          <t>The answer is correct - Surat Spinners, Rs 4,80,000, matching the data - but it is shown with literal markdown: '**Surat Spinners**' and '**Rs 4,80,000**', asterisks visible.</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>pages/finance/ReviewPanel.js; services/ingestion.py (ai_extract_document)</t>
+          <t>pages/Ledger.js:539 (ai-answer)</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr"/>
@@ -27694,7 +27705,7 @@
     <row r="98" ht="82" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>GL-03</t>
+          <t>FN-13</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -27704,12 +27715,12 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>/login while signed in</t>
+          <t>Capture - extraction review</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -27724,17 +27735,17 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>If the auth context has a user, &lt;Navigate to='/app' replace/&gt; (the same hand-off Home already uses).</t>
+          <t>Carry invoice date, GSTIN (and GST amount) and line items through to review; flag bills whose date or due date is more than ~12 months old before 'File it'.</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>The sign-in form is shown again. A user following an old bookmark or a 'Sign in' link sees a login screen while already logged in.</t>
+          <t>Good overall, in 31.9s at 92% confidence: supplier Service TEST 123 with phone and email, number X33, amount 27,625, due 2018-03-01, booked as Inventory, and a 'Pay vendor bill' follow-up task. But the invoice DATE, the supplier GSTIN and the line items are not captured, and nothing warns that the bill fell due eight years ago - filing it would add an overdue payable dated 2018 without comment.</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>pages/Login.js (component top)</t>
+          <t>pages/finance/ReviewPanel.js; services/ingestion.py (ai_extract_document)</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr"/>
@@ -27747,7 +27758,7 @@
     <row r="99" ht="82" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>DD-04</t>
+          <t>GL-03</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -27757,12 +27768,12 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Decision Desk</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Company / You switch (mobile)</t>
+          <t>/login while signed in</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -27777,17 +27788,17 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Show the joined pill pair above the score below lg.</t>
+          <t>If the auth context has a user, &lt;Navigate to='/app' replace/&gt; (the same hand-off Home already uses).</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Both copies of the Company / You pills are in the DOM but invisible at phone width, so the phone only ever shows the company score.</t>
+          <t>The sign-in form is shown again. A user following an old bookmark or a 'Sign in' link sees a login screen while already logged in.</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>pages/Desk.js:426 and :470 (scope pill placements)</t>
+          <t>pages/Login.js (component top)</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr"/>
@@ -27800,7 +27811,7 @@
     <row r="100" ht="82" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>DD-05</t>
+          <t>DD-04</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -27815,7 +27826,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Decision review - note mic</t>
+          <t>Company / You switch (mobile)</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -27830,17 +27841,17 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Wire it to the same capture Dex uses, or remove the mic and its helper line until it is.</t>
+          <t>Show the joined pill pair above the score below lg.</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>It only shows a toast: 'Voice capture is available from the Dex panel'. The button and the helper line invite an action the page does not do.</t>
+          <t>Both copies of the Company / You pills are in the DOM but invisible at phone width, so the phone only ever shows the company score.</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>components/DecisionDialog.js:421-445</t>
+          <t>pages/Desk.js:426 and :470 (scope pill placements)</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr"/>
@@ -27853,7 +27864,7 @@
     <row r="101" ht="82" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>CL-03</t>
+          <t>DD-05</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -27863,12 +27874,12 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Decision Desk</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Mark all read</t>
+          <t>Decision review - note mic</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -27883,17 +27894,17 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>toast.error('Couldn't mark notifications read') in onError.</t>
+          <t>Wire it to the same capture Dex uses, or remove the mic and its helper line until it is.</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Nothing happens and nothing is said - no toast, the unread dots stay - so the user cannot tell whether it worked.</t>
+          <t>It only shows a toast: 'Voice capture is available from the Dex panel'. The button and the helper line invite an action the page does not do.</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>pages/Notifications.js:17-21</t>
+          <t>components/DecisionDialog.js:421-445</t>
         </is>
       </c>
       <c r="J101" s="2" t="inlineStr"/>
@@ -27906,7 +27917,7 @@
     <row r="102" ht="82" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>CL-04</t>
+          <t>CL-03</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -27916,12 +27927,12 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Operations tab - add links</t>
+          <t>Mark all read</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -27936,17 +27947,17 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>py-1 / min-h-6 on both.</t>
+          <t>toast.error('Couldn't mark notifications read') in onError.</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>'Add operational task' (149x20) and 'Add approval rule' (131x20) are under 24px.</t>
+          <t>Nothing happens and nothing is said - no toast, the unread dots stay - so the user cannot tell whether it worked.</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>pages/Settings.js (OperatingModelEditor add buttons)</t>
+          <t>pages/Notifications.js:17-21</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr"/>
@@ -27959,7 +27970,7 @@
     <row r="103" ht="82" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>AU-01</t>
+          <t>CL-04</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -27969,12 +27980,12 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Sign-in</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Login, sign-up and admin fields</t>
+          <t>Operations tab - add links</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
@@ -27989,17 +28000,17 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>Add labels (visually hidden where the design has none). Same fix as TM-06.</t>
+          <t>py-1 / min-h-6 on both.</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Login email and password, the sign-up company name, and the admin email and password have no associated label or aria-label. The admin screen shows the words EMAIL and PASSWORD but they are not tied to the inputs.</t>
+          <t>'Add operational task' (149x20) and 'Add approval rule' (131x20) are under 24px.</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>pages/Login.js:298-299, pages/Signup.js (basics), pages/admin/AdminLogin.js:44-57</t>
+          <t>pages/Settings.js (OperatingModelEditor add buttons)</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr"/>
@@ -28012,7 +28023,7 @@
     <row r="104" ht="82" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>AU-02</t>
+          <t>AU-01</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -28027,7 +28038,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Mobile OTP - phone number</t>
+          <t>Login, sign-up and admin fields</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -28042,17 +28053,17 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>Require 10 digits (after stripping +91 / spaces) before enabling Send, and say 'Enter a 10-digit mobile number'.</t>
+          <t>Add labels (visually hidden where the design has none). Same fix as TM-06.</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>The 3-digit number is sent to the server; with no provider reachable the user only sees 'Something went wrong. Please try again.', which does not tell them the number is wrong.</t>
+          <t>Login email and password, the sign-up company name, and the admin email and password have no associated label or aria-label. The admin screen shows the words EMAIL and PASSWORD but they are not tied to the inputs.</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>pages/Login.js:179-190, :317</t>
+          <t>pages/Login.js:298-299, pages/Signup.js (basics), pages/admin/AdminLogin.js:44-57</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr"/>
@@ -28065,7 +28076,7 @@
     <row r="105" ht="82" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>AU-03</t>
+          <t>AU-02</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -28080,7 +28091,7 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Login - header links (desktop)</t>
+          <t>Mobile OTP - phone number</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
@@ -28095,17 +28106,17 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>py-1 on both links.</t>
+          <t>Require 10 digits (after stripping +91 / spaces) before enabling Send, and say 'Enter a 10-digit mobile number'.</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>The 'DecisionOS' logo link is 91x21 and 'Need a workspace? Register' is 194x20.</t>
+          <t>The 3-digit number is sent to the server; with no provider reachable the user only sees 'Something went wrong. Please try again.', which does not tell them the number is wrong.</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>pages/Login.js:241-246</t>
+          <t>pages/Login.js:179-190, :317</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr"/>
@@ -28118,7 +28129,7 @@
     <row r="106" ht="82" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>MW-14</t>
+          <t>AU-03</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -28128,12 +28139,12 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Sign-in</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Page heading in the Leave / Workflows views</t>
+          <t>Login - header links (desktop)</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -28141,24 +28152,24 @@
           <t>Bug fix</t>
         </is>
       </c>
-      <c r="F106" s="9" t="inlineStr">
-        <is>
-          <t>Nit</t>
+      <c r="F106" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Swap the heading with the view - 'Leave' or 'Workflows' - or append the view name. Only worth doing if the views stay inside My Work at all; see MW-12.</t>
+          <t>py-1 on both links.</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>The heading stays 'My Work' with the eyebrow 'YOUR DAY, SIMPLIFIED' even when the body is entirely leave requests or delivery pipelines. Nothing above the fold says which of the three views is active except the small toggle pill.</t>
+          <t>The 'DecisionOS' logo link is 91x21 and 'Need a workspace? Register' is 194x20.</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js (page header, above the view switch at 2527)</t>
+          <t>pages/Login.js:241-246</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr"/>
@@ -28171,7 +28182,7 @@
     <row r="107" ht="82" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>CR-03</t>
+          <t>MW-14</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -28181,12 +28192,12 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Add contact dialog - dismiss controls</t>
+          <t>Page heading in the Leave / Workflows views</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -28201,17 +28212,17 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>Pick one convention for the whole app - most products keep the X and drop the Cancel, or keep Cancel on destructive-ish forms only - and apply it to both this dialog and TM-04.</t>
+          <t>Swap the heading with the view - 'Leave' or 'Workflows' - or append the view name. Only worth doing if the views stay inside My Work at all; see MW-12.</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>Two: a 'Cancel' button beside Add contact, and a separate 'Close' X. Team's profile dialog has the same duplication (TM-04), so it is worth settling once for the app rather than per dialog.</t>
+          <t>The heading stays 'My Work' with the eyebrow 'YOUR DAY, SIMPLIFIED' even when the body is entirely leave requests or delivery pipelines. Nothing above the fold says which of the three views is active except the small toggle pill.</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>pages/CRM.js:242-365 (crm-contact-dialog footer)</t>
+          <t>pages/MyWork.js (page header, above the view switch at 2527)</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr"/>
@@ -28224,7 +28235,7 @@
     <row r="108" ht="82" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>TM-02</t>
+          <t>CR-03</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -28234,12 +28245,12 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Owner section grid</t>
+          <t>Add contact dialog - dismiss controls</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -28254,17 +28265,17 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>Either let a single-card group span the row, or give the owner its own treatment at the top of the page - it is a different kind of row from a department, and looks like one.</t>
+          <t>Pick one convention for the whole app - most products keep the X and drop the Cancel, or keep Cancel on destructive-ish forms only - and apply it to both this dialog and TM-04.</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>The Owner group uses the same three-column grid as every other role but will almost always hold exactly one card, so 874px of a 1336px row is blank. It reads as a rendering fault rather than a deliberate space.</t>
+          <t>Two: a 'Cancel' button beside Add contact, and a separate 'Close' X. Team's profile dialog has the same duplication (TM-04), so it is worth settling once for the app rather than per dialog.</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:366 (team-cards-&lt;role&gt; grid)</t>
+          <t>pages/CRM.js:242-365 (crm-contact-dialog footer)</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr"/>
@@ -28277,7 +28288,7 @@
     <row r="109" ht="82" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>TM-03</t>
+          <t>TM-02</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
@@ -28292,7 +28303,7 @@
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Member cards</t>
+          <t>Owner section grid</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
@@ -28307,17 +28318,17 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>Put the reporting line on the card - one line, 'Reports to Sunita Rao' - and consider replacing the bare count with the two or three areas that distinguish this person, keeping the full list in the dialog. Cheapest alternative: soften the eyebrow so it stops promising what the list does not show.</t>
+          <t>Either let a single-card group span the row, or give the owner its own treatment at the top of the page - it is a different kind of row from a department, and looks like one.</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>The cards show name, email, status and a permission COUNT. The reporting line is absent entirely, and access is reduced to a number that says nothing about what the person can reach. Both exist one click deeper - the profile dialog reads 'REPORTS TO Sunita Rao' and '13 of 14 areas' with the areas listed - so the data is there and simply is not surfaced where the page says it will be.</t>
+          <t>The Owner group uses the same three-column grid as every other role but will almost always hold exactly one card, so 874px of a 1336px row is blank. It reads as a rendering fault rather than a deliberate space.</t>
         </is>
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:417-450 (member card); manager already resolved at :475</t>
+          <t>pages/Team.js:366 (team-cards-&lt;role&gt; grid)</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr"/>
@@ -28330,7 +28341,7 @@
     <row r="110" ht="82" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>TM-04</t>
+          <t>TM-03</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -28345,7 +28356,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Member profile dialog</t>
+          <t>Member cards</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -28360,17 +28371,17 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>Keep one. If the custom 36px control is the intended one, hide the primitive's default close for this dialog.</t>
+          <t>Put the reporting line on the card - one line, 'Reports to Sunita Rao' - and consider replacing the bare count with the two or three areas that distinguish this person, keeping the full list in the dialog. Cheapest alternative: soften the eyebrow so it stops promising what the list does not show.</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>Two separate visible buttons are both named exactly 'Close'. A screen-reader user tabbing the dialog meets the same name twice with nothing to separate them.</t>
+          <t>The cards show name, email, status and a permission COUNT. The reporting line is absent entirely, and access is reduced to a number that says nothing about what the person can reach. Both exist one click deeper - the profile dialog reads 'REPORTS TO Sunita Rao' and '13 of 14 areas' with the areas listed - so the data is there and simply is not surfaced where the page says it will be.</t>
         </is>
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>pages/Team.js:497-535 (profile dialog header)</t>
+          <t>pages/Team.js:417-450 (member card); manager already resolved at :475</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr"/>
@@ -28383,7 +28394,7 @@
     <row r="111" ht="82" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>MW-06</t>
+          <t>TM-04</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -28393,12 +28404,12 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Category tab bar</t>
+          <t>Member profile dialog</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
@@ -28413,17 +28424,17 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>While the tasks query is loading, render a dash or omit the count, matching the skeleton treatment already used for the cards below.</t>
+          <t>Keep one. If the custom 36px control is the intended one, hide the primitive's default close for this dialog.</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>The tab reads 'All 0' for the whole fetch, which states a count of zero rather than an unknown one. The card skeletons underneath are correct, so the count is the only misleading element.</t>
+          <t>Two separate visible buttons are both named exactly 'Close'. A screen-reader user tabbing the dialog meets the same name twice with nothing to separate them.</t>
         </is>
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>pages/MyWork.js:2556-2566 (work-tabs counts)</t>
+          <t>pages/Team.js:497-535 (profile dialog header)</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr"/>
@@ -28436,58 +28447,111 @@
     <row r="112" ht="82" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
         <is>
+          <t>MW-06</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>UI audit</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>My Work</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Category tab bar</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>Bug fix</t>
+        </is>
+      </c>
+      <c r="F112" s="9" t="inlineStr">
+        <is>
+          <t>Nit</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>While the tasks query is loading, render a dash or omit the count, matching the skeleton treatment already used for the cards below.</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>The tab reads 'All 0' for the whole fetch, which states a count of zero rather than an unknown one. The card skeletons underneath are correct, so the count is the only misleading element.</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>pages/MyWork.js:2556-2566 (work-tabs counts)</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr"/>
+      <c r="K112" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="82" customHeight="1">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
           <t>MW-07</t>
         </is>
       </c>
-      <c r="B112" s="2" t="inlineStr">
+      <c r="B113" s="2" t="inlineStr">
         <is>
           <t>UI audit</t>
         </is>
       </c>
-      <c r="C112" s="2" t="inlineStr">
+      <c r="C113" s="2" t="inlineStr">
         <is>
           <t>My Work</t>
         </is>
       </c>
-      <c r="D112" s="2" t="inlineStr">
+      <c r="D113" s="2" t="inlineStr">
         <is>
           <t>Task card - Complete (evidence required)</t>
         </is>
       </c>
-      <c r="E112" s="2" t="inlineStr">
+      <c r="E113" s="2" t="inlineStr">
         <is>
           <t>By design</t>
         </is>
       </c>
-      <c r="F112" s="9" t="inlineStr">
+      <c r="F113" s="9" t="inlineStr">
         <is>
           <t>Nit</t>
         </is>
       </c>
-      <c r="G112" s="2" t="inlineStr">
+      <c r="G113" s="2" t="inlineStr">
         <is>
           <t>Optional polish only: disable Complete while proof is missing and put the reason in a tooltip or helper line, so the constraint is visible before the click rather than after it. Current behaviour is safe and correct.</t>
         </is>
       </c>
-      <c r="H112" s="2" t="inlineStr">
+      <c r="H113" s="2" t="inlineStr">
         <is>
           <t>Completion IS correctly blocked - the task stays in the active list and an explanatory toast appears. The only nit is that the button looks available and only explains itself after it is pressed.</t>
         </is>
       </c>
-      <c r="I112" s="2" t="inlineStr">
+      <c r="I113" s="2" t="inlineStr">
         <is>
           <t>pages/MyWork.js:1107-1119</t>
         </is>
       </c>
-      <c r="J112" s="2" t="inlineStr"/>
-      <c r="K112" s="4" t="inlineStr">
+      <c r="J113" s="2" t="inlineStr"/>
+      <c r="K113" s="4" t="inlineStr">
         <is>
           <t>Not a defect</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K112"/>
+  <autoFilter ref="A1:K113"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
ASK-24: My Work All Tasks gets a Person filter and a complete filter row
- Person filter on All Tasks: Me, people busiest first with role, Unassigned,
  team queues; search past 8 people; shared names carry the email handle
- Status gains Pending Approval and Overdue; Priority dropdown added
- One predicate for list and counts, so every menu reflects the others
- Active filters render pressed; Clear filters; "No tasks match" empty state
- Person / Priority / Status kept in the URL; Desk ?filter= links and a saved
  Completed tab convert to the visible Status filter; ?task= clears filters
- Phone: filter pill opens a bottom sheet with all four, caption names them

Acceptance: backend/scripts/ux_person_filter_0913.py - 33/33 pass (owner
desktop + phone, Sales), writes blocked. Tracker: ASK-24 Fixed, T-690..T-699.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_UI_Bug_Report.xlsx
+++ b/docs/DecisionOS_UI_Bug_Report.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bug Log'!$A$1:$Q$89</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Coverage'!$A$1:$J$283</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Coverage'!$A$1:$J$293</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Verified Non-Issues'!$A$1:$E$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Action List'!$A$1:$K$113</definedName>
   </definedNames>
@@ -8116,7 +8116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J283"/>
+  <dimension ref="A1:J293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21586,17 +21586,17 @@
     <row r="273" ht="82" customHeight="1">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>T-680</t>
+          <t>T-690</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>LIVE - receivables question</t>
+          <t>All Tasks - filter row</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -21611,44 +21611,44 @@
       </c>
       <c r="F273" s="2" t="inlineStr">
         <is>
-          <t>Dex answers how much customers owe with the ledger's figure</t>
+          <t>All Tasks shows Department, Person, Priority, Status; My Tasks hides Person</t>
         </is>
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H273" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H273" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>Said zero invoices / Rs 0 outstanding; ledger has Rs 7,49,000 outstanding (17.0s)</t>
+          <t>Row shows all four with counts (131); My Tasks shows three (25)</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
         <is>
-          <t>DX-01</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="274" ht="82" customHeight="1">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>T-681</t>
+          <t>T-691</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>LIVE - what needs my attention</t>
+          <t>All Tasks - Person filter</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
@@ -21663,44 +21663,44 @@
       </c>
       <c r="F274" s="2" t="inlineStr">
         <is>
-          <t>Dex surfaces the overdue work and pending decisions</t>
+          <t>Picking a person shows only their tasks, count matches the API</t>
         </is>
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H274" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H274" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>Said nothing open or overdue; owner has 24 open / 6 overdue (24.1s)</t>
+          <t>Priya Nair: 29 cards = trigger 29 = API 29; URL ?person=; name line hidden on cards; menu has Me, people busiest first with role, Unassigned (6), Production team (5); no duplicate rows</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
         <is>
-          <t>DX-02</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="275" ht="82" customHeight="1">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>T-682</t>
+          <t>T-692</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>LIVE - global search hand-off</t>
+          <t>All Tasks - Status options</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -21715,12 +21715,12 @@
       </c>
       <c r="F275" s="2" t="inlineStr">
         <is>
-          <t>A question from global search is answered on arrival</t>
+          <t>Pending Approval, Overdue and Completed are filterable with correct counts</t>
         </is>
       </c>
       <c r="G275" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H275" s="4" t="inlineStr">
@@ -21730,25 +21730,29 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>'Which tasks are overdue?' answered on /brain?q= with a task list (17.5s)</t>
-        </is>
-      </c>
-      <c r="J275" s="2" t="inlineStr"/>
+          <t>Pending Approval 40, Overdue 68, Completed 17, Not Started 78 - all equal the API</t>
+        </is>
+      </c>
+      <c r="J275" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="276" ht="82" customHeight="1">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>T-683</t>
+          <t>T-693</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>LIVE - coach refresh</t>
+          <t>All Tasks - Priority filter</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -21763,12 +21767,12 @@
       </c>
       <c r="F276" s="2" t="inlineStr">
         <is>
-          <t>Generate coaching produces a review grounded in the stats</t>
+          <t>Priority dropdown exists and narrows</t>
         </is>
       </c>
       <c r="G276" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H276" s="4" t="inlineStr">
@@ -21778,25 +21782,29 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>TEST_member: 'AI coach updated' in 8.7s; strengths / improvements reference the 13 actionable tasks and plan use</t>
-        </is>
-      </c>
-      <c r="J276" s="2" t="inlineStr"/>
+          <t>High 66 / Medium 53 / Low 12; Priya x Overdue x High = 16 = API</t>
+        </is>
+      </c>
+      <c r="J276" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="277" ht="82" customHeight="1">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>T-684</t>
+          <t>T-694</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Score with AI</t>
+          <t>All Tasks - combined counts</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -21811,12 +21819,12 @@
       </c>
       <c r="F277" s="2" t="inlineStr">
         <is>
-          <t>Rescore updates the relationship card sensibly</t>
+          <t>Each menu's counts reflect the other active filters</t>
         </is>
       </c>
       <c r="G277" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H277" s="4" t="inlineStr">
@@ -21826,25 +21834,29 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>E2E Test Co: 'Relationship scored by AI' in 7.8s; Relationship 12 / Risk 78, reason cites 4 open complaints and no billing - matches the record</t>
-        </is>
-      </c>
-      <c r="J277" s="2" t="inlineStr"/>
+          <t>With Priya + Overdue, Department 'All' reads 20 = cards = API</t>
+        </is>
+      </c>
+      <c r="J277" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="278" ht="82" customHeight="1">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>T-685</t>
+          <t>T-695</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>LIVE - AI analysis refresh</t>
+          <t>All Tasks - refresh, Clear, no match</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -21859,12 +21871,12 @@
       </c>
       <c r="F278" s="2" t="inlineStr">
         <is>
-          <t>Refresh produces an analysis grounded in the ledger</t>
+          <t>Filters survive refresh; Clear resets; empty result explains itself</t>
         </is>
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H278" s="4" t="inlineStr">
@@ -21874,25 +21886,29 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>'Analysis refreshed' in 20.6s; Rs 6.6L outstanding (ledger 6,55,466), Surat Spinners Rs 4.8L unpaid 33 days (correct), duplicates flagged</t>
-        </is>
-      </c>
-      <c r="J278" s="2" t="inlineStr"/>
+          <t>Reload keeps 16 cards + URL; Clear -&gt; 131, URL clean; Priya x Under Review -&gt; 'No tasks match these filters' with Clear</t>
+        </is>
+      </c>
+      <c r="J278" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="279" ht="82" customHeight="1">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>T-686</t>
+          <t>T-696</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Ask AI</t>
+          <t>All Tasks - person search, links</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -21907,44 +21923,44 @@
       </c>
       <c r="F279" s="2" t="inlineStr">
         <is>
-          <t>The answer is correct and readable</t>
+          <t>Search narrows the menu; Desk overdue link and task deep link behave</t>
         </is>
       </c>
       <c r="G279" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H279" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H279" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>Correct (Surat Spinners Rs 4,80,000, 7.3s) but literal ** markdown shown</t>
+          <t>'pri' -&gt; Priya Nair only; ?filter=overdue -&gt; Status: Overdue 68; ?task= with filters set clears them and shows the card</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
         <is>
-          <t>FN-12</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="280" ht="82" customHeight="1">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>T-688</t>
+          <t>T-697</t>
         </is>
       </c>
       <c r="B280" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>LIVE - owner on a phone</t>
+          <t>Phone - filter sheet</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -21959,12 +21975,12 @@
       </c>
       <c r="F280" s="2" t="inlineStr">
         <is>
-          <t>Dex answers on mobile and the answer fits the screen</t>
+          <t>The phone reaches all four filters and sees what is active</t>
         </is>
       </c>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H280" s="4" t="inlineStr">
@@ -21974,45 +21990,49 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>'53 decisions pending approval across 77' - correct; 17.6s; no overflow</t>
-        </is>
-      </c>
-      <c r="J280" s="2" t="inlineStr"/>
+          <t>Sheet with Department / Person / Priority / Status; Priya + Overdue -&gt; 'Show 20 tasks' = 20 cards; caption 'Showing Priya Nair - Overdue' with Clear; buttons 44px, reachable; no overflow</t>
+        </is>
+      </c>
+      <c r="J280" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="281" ht="82" customHeight="1">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>T-689</t>
+          <t>T-698</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Sales asks money questions</t>
+          <t>Phone - My Tasks / Status without AI</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Mobile 390x844</t>
         </is>
       </c>
       <c r="E281" s="2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F281" s="2" t="inlineStr">
         <is>
-          <t>Dex refuses finance answers to a role the finance API refuses</t>
+          <t>Person hidden on My Tasks; a Status filter is visible even with AI priority off</t>
         </is>
       </c>
       <c r="G281" s="2" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H281" s="4" t="inlineStr">
@@ -22022,113 +22042,613 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>Receivables and profit questions both refused ('You do not have permission to access financial...'), 5.8s / 1.6s; no figures leaked</t>
-        </is>
-      </c>
-      <c r="J281" s="2" t="inlineStr"/>
+          <t>Sheet on My Tasks has no Person; ?status=overdue shows the caption</t>
+        </is>
+      </c>
+      <c r="J281" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="282" ht="82" customHeight="1">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>T-687</t>
+          <t>T-699</t>
         </is>
       </c>
       <c r="B282" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>LIVE - bill extraction</t>
+          <t>Sales - no Person filter</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Desktop + Mobile</t>
         </is>
       </c>
       <c r="E282" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F282" s="2" t="inlineStr">
         <is>
-          <t>A GST bill is extracted into a reviewable record with the key fields</t>
+          <t>Roles without All Tasks never see Person; ?person= is ignored</t>
         </is>
       </c>
       <c r="G282" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H282" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="H282" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>Party, number, amount, due date, category and follow-up correct (31.9s, 92%); date, GSTIN, items missing; no stale-date warning. Left in review, not filed</t>
+          <t>Desktop row has no Person; phone sheet has no Person; ?person=anyone ignored, own 29 cards</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
         <is>
-          <t>FN-13</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="283" ht="82" customHeight="1">
       <c r="A283" s="2" t="inlineStr">
         <is>
+          <t>T-680</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - receivables question</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E283" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F283" s="2" t="inlineStr">
+        <is>
+          <t>Dex answers how much customers owe with the ledger's figure</t>
+        </is>
+      </c>
+      <c r="G283" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H283" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I283" s="2" t="inlineStr">
+        <is>
+          <t>Said zero invoices / Rs 0 outstanding; ledger has Rs 7,49,000 outstanding (17.0s)</t>
+        </is>
+      </c>
+      <c r="J283" s="2" t="inlineStr">
+        <is>
+          <t>DX-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="284" ht="82" customHeight="1">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>T-681</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - what needs my attention</t>
+        </is>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E284" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F284" s="2" t="inlineStr">
+        <is>
+          <t>Dex surfaces the overdue work and pending decisions</t>
+        </is>
+      </c>
+      <c r="G284" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H284" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I284" s="2" t="inlineStr">
+        <is>
+          <t>Said nothing open or overdue; owner has 24 open / 6 overdue (24.1s)</t>
+        </is>
+      </c>
+      <c r="J284" s="2" t="inlineStr">
+        <is>
+          <t>DX-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="285" ht="82" customHeight="1">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>T-682</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - global search hand-off</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E285" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F285" s="2" t="inlineStr">
+        <is>
+          <t>A question from global search is answered on arrival</t>
+        </is>
+      </c>
+      <c r="G285" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H285" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I285" s="2" t="inlineStr">
+        <is>
+          <t>'Which tasks are overdue?' answered on /brain?q= with a task list (17.5s)</t>
+        </is>
+      </c>
+      <c r="J285" s="2" t="inlineStr"/>
+    </row>
+    <row r="286" ht="82" customHeight="1">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>T-683</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - coach refresh</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E286" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>Generate coaching produces a review grounded in the stats</t>
+        </is>
+      </c>
+      <c r="G286" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H286" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I286" s="2" t="inlineStr">
+        <is>
+          <t>TEST_member: 'AI coach updated' in 8.7s; strengths / improvements reference the 13 actionable tasks and plan use</t>
+        </is>
+      </c>
+      <c r="J286" s="2" t="inlineStr"/>
+    </row>
+    <row r="287" ht="82" customHeight="1">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>T-684</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Score with AI</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E287" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F287" s="2" t="inlineStr">
+        <is>
+          <t>Rescore updates the relationship card sensibly</t>
+        </is>
+      </c>
+      <c r="G287" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H287" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I287" s="2" t="inlineStr">
+        <is>
+          <t>E2E Test Co: 'Relationship scored by AI' in 7.8s; Relationship 12 / Risk 78, reason cites 4 open complaints and no billing - matches the record</t>
+        </is>
+      </c>
+      <c r="J287" s="2" t="inlineStr"/>
+    </row>
+    <row r="288" ht="82" customHeight="1">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>T-685</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - AI analysis refresh</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E288" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F288" s="2" t="inlineStr">
+        <is>
+          <t>Refresh produces an analysis grounded in the ledger</t>
+        </is>
+      </c>
+      <c r="G288" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H288" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I288" s="2" t="inlineStr">
+        <is>
+          <t>'Analysis refreshed' in 20.6s; Rs 6.6L outstanding (ledger 6,55,466), Surat Spinners Rs 4.8L unpaid 33 days (correct), duplicates flagged</t>
+        </is>
+      </c>
+      <c r="J288" s="2" t="inlineStr"/>
+    </row>
+    <row r="289" ht="82" customHeight="1">
+      <c r="A289" s="2" t="inlineStr">
+        <is>
+          <t>T-686</t>
+        </is>
+      </c>
+      <c r="B289" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Ask AI</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F289" s="2" t="inlineStr">
+        <is>
+          <t>The answer is correct and readable</t>
+        </is>
+      </c>
+      <c r="G289" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H289" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I289" s="2" t="inlineStr">
+        <is>
+          <t>Correct (Surat Spinners Rs 4,80,000, 7.3s) but literal ** markdown shown</t>
+        </is>
+      </c>
+      <c r="J289" s="2" t="inlineStr">
+        <is>
+          <t>FN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="290" ht="82" customHeight="1">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>T-688</t>
+        </is>
+      </c>
+      <c r="B290" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - owner on a phone</t>
+        </is>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>Mobile 390x844</t>
+        </is>
+      </c>
+      <c r="E290" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F290" s="2" t="inlineStr">
+        <is>
+          <t>Dex answers on mobile and the answer fits the screen</t>
+        </is>
+      </c>
+      <c r="G290" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H290" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I290" s="2" t="inlineStr">
+        <is>
+          <t>'53 decisions pending approval across 77' - correct; 17.6s; no overflow</t>
+        </is>
+      </c>
+      <c r="J290" s="2" t="inlineStr"/>
+    </row>
+    <row r="291" ht="82" customHeight="1">
+      <c r="A291" s="2" t="inlineStr">
+        <is>
+          <t>T-689</t>
+        </is>
+      </c>
+      <c r="B291" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C291" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Sales asks money questions</t>
+        </is>
+      </c>
+      <c r="D291" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E291" s="2" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="F291" s="2" t="inlineStr">
+        <is>
+          <t>Dex refuses finance answers to a role the finance API refuses</t>
+        </is>
+      </c>
+      <c r="G291" s="2" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="H291" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I291" s="2" t="inlineStr">
+        <is>
+          <t>Receivables and profit questions both refused ('You do not have permission to access financial...'), 5.8s / 1.6s; no figures leaked</t>
+        </is>
+      </c>
+      <c r="J291" s="2" t="inlineStr"/>
+    </row>
+    <row r="292" ht="82" customHeight="1">
+      <c r="A292" s="2" t="inlineStr">
+        <is>
+          <t>T-687</t>
+        </is>
+      </c>
+      <c r="B292" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C292" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - bill extraction</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E292" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F292" s="2" t="inlineStr">
+        <is>
+          <t>A GST bill is extracted into a reviewable record with the key fields</t>
+        </is>
+      </c>
+      <c r="G292" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H292" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I292" s="2" t="inlineStr">
+        <is>
+          <t>Party, number, amount, due date, category and follow-up correct (31.9s, 92%); date, GSTIN, items missing; no stale-date warning. Left in review, not filed</t>
+        </is>
+      </c>
+      <c r="J292" s="2" t="inlineStr">
+        <is>
+          <t>FN-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="293" ht="82" customHeight="1">
+      <c r="A293" s="2" t="inlineStr">
+        <is>
           <t>T-676</t>
         </is>
       </c>
-      <c r="B283" s="2" t="inlineStr">
+      <c r="B293" s="2" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="C283" s="2" t="inlineStr">
+      <c r="C293" s="2" t="inlineStr">
         <is>
           <t>Admin portal gating</t>
         </is>
       </c>
-      <c r="D283" s="2" t="inlineStr">
+      <c r="D293" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="E283" s="2" t="inlineStr">
+      <c r="E293" s="2" t="inlineStr">
         <is>
           <t>Signed out / Owner</t>
         </is>
       </c>
-      <c r="F283" s="2" t="inlineStr">
+      <c r="F293" s="2" t="inlineStr">
         <is>
           <t>Only platform admins reach the portal</t>
         </is>
       </c>
-      <c r="G283" s="2" t="inlineStr">
+      <c r="G293" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="H283" s="4" t="inlineStr">
+      <c r="H293" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I283" s="2" t="inlineStr">
+      <c r="I293" s="2" t="inlineStr">
         <is>
           <t>Signed out and tenant owner both get the admin sign-in; /admin/me 401; deep link /admin/tenants too</t>
         </is>
       </c>
-      <c r="J283" s="2" t="inlineStr"/>
+      <c r="J293" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J283"/>
+  <autoFilter ref="A1:J293"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23855,7 +24375,8 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Founder request 2026-09-13, tracked here for traction. On My Work &gt; All Tasks (desktop and phone):
+          <t>BUILT 2026-09-13 - pages/MyWork.js; acceptance 33/33 PASS on desktop 1440 + phone 390, owner and Sales, writes blocked (backend/scripts/ux_person_filter_0913.py, .audit-artifacts/ask24_person_filter/). Notes on the build: Department stays in the saved per-user prefs rather than the URL (it already persisted there); a saved Completed tab and the Desk ?filter=overdue|completed links now convert to the visible Status filter; people who share a display name carry their email handle so the menu can tell them apart; opening a task by link clears filters that would hide it; dismissing AI priority no longer clears Status.
+Founder request 2026-09-13, tracked here for traction. On My Work &gt; All Tasks (desktop and phone):
 (1) PERSON filter - a new 'Person: All' dropdown between Department and Status, same pill as the others. Shown only on All Tasks (on My Tasks every card is yours). Options, each with an open-task count: 'All people'; 'Me'; every person who holds work in the list, busiest first, with their role under the name (e.g. Priya Nair - Sales); 'Unassigned'; and a 'Teams' group for tasks given to a role with no person (the cards' 'Sales team' line). Names come from /users, already loaded as members. With more than 8 people, a type-to-search box sits at the top of the menu.
 (2) COMPLETE STATUS OPTIONS - add 'Pending Approval' (status blocked - the grey chip on most cards, which cannot be filtered today) and 'Overdue' (the orange chip; a lens like Completed). Order: All statuses, Not Started, In Progress, Waiting, Pending Approval, Under Review, Overdue, Completed. Show counts like Department does.
 (3) PRIORITY dropdown - the ASK-13 comment says Priority was added, but only Department and Status render. Add 'Priority: All / High / Medium / Low' with counts.
@@ -23880,9 +24401,9 @@
           <t>ASK-13, ASK-22, MW-19, KM-30</t>
         </is>
       </c>
-      <c r="K25" s="7" t="inlineStr">
-        <is>
-          <t>To do</t>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -29587,7 +30108,7 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>282 (191 pass, 89 fail, 0 blocked, 2 not run)</t>
+          <t>292 (201 pass, 89 fail, 0 blocked, 2 not run)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
My Work: remove the Priority filter (founder call)
The AI-priority view already splits tasks into High / Medium / Low, so the
filter row is back to Department, Person, Status on desktop and in the phone
sheet. Links made while it existed can carry ?priority=; it is ignored on
read and stripped by Clear filters.

Acceptance re-run: backend/scripts/ux_person_filter_0913.py - all pass, with
checks that the filter is gone and a stale ?priority= link does not narrow.
Tracker: ASK-24 note, T-690/T-693/T-695/T-697 updated.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_UI_Bug_Report.xlsx
+++ b/docs/DecisionOS_UI_Bug_Report.xlsx
@@ -21611,7 +21611,7 @@
       </c>
       <c r="F273" s="2" t="inlineStr">
         <is>
-          <t>All Tasks shows Department, Person, Priority, Status; My Tasks hides Person</t>
+          <t>All Tasks shows Department, Person, Status; My Tasks hides Person</t>
         </is>
       </c>
       <c r="G273" s="2" t="inlineStr">
@@ -21626,7 +21626,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>Row shows all four with counts (131); My Tasks shows three (25)</t>
+          <t>Row shows all three with counts (131); My Tasks shows two (25)</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -21752,12 +21752,12 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - Priority filter</t>
+          <t>All Tasks - Priority filter removed</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Desktop + Mobile</t>
         </is>
       </c>
       <c r="E276" s="2" t="inlineStr">
@@ -21767,7 +21767,7 @@
       </c>
       <c r="F276" s="2" t="inlineStr">
         <is>
-          <t>Priority dropdown exists and narrows</t>
+          <t>No Priority filter (founder call 2026-09-13); an old ?priority= link does not narrow the list</t>
         </is>
       </c>
       <c r="G276" s="2" t="inlineStr">
@@ -21782,7 +21782,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>High 66 / Medium 53 / Low 12; Priya x Overdue x High = 16 = API</t>
+          <t>No Priority dropdown on desktop, no Priority chips in the phone sheet; ?person=Priya&amp;status=overdue&amp;priority=high shows the same 20 as without it</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -21886,7 +21886,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>Reload keeps 16 cards + URL; Clear -&gt; 131, URL clean; Priya x Under Review -&gt; 'No tasks match these filters' with Clear</t>
+          <t>Reload keeps 20 cards + URL; Clear -&gt; 131, URL clean; Priya x Under Review -&gt; 'No tasks match these filters' with Clear</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21975,7 +21975,7 @@
       </c>
       <c r="F280" s="2" t="inlineStr">
         <is>
-          <t>The phone reaches all four filters and sees what is active</t>
+          <t>The phone reaches every filter and sees what is active</t>
         </is>
       </c>
       <c r="G280" s="2" t="inlineStr">
@@ -21990,7 +21990,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>Sheet with Department / Person / Priority / Status; Priya + Overdue -&gt; 'Show 20 tasks' = 20 cards; caption 'Showing Priya Nair - Overdue' with Clear; buttons 44px, reachable; no overflow</t>
+          <t>Sheet with Department / Person / Status; Priya + Overdue -&gt; 'Show 20 tasks' = 20 cards; caption 'Showing Priya Nair - Overdue' with Clear; buttons 44px, reachable; no overflow</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -24375,7 +24375,8 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>BUILT 2026-09-13 - pages/MyWork.js; acceptance 33/33 PASS on desktop 1440 + phone 390, owner and Sales, writes blocked (backend/scripts/ux_person_filter_0913.py, .audit-artifacts/ask24_person_filter/). Notes on the build: Department stays in the saved per-user prefs rather than the URL (it already persisted there); a saved Completed tab and the Desk ?filter=overdue|completed links now convert to the visible Status filter; people who share a display name carry their email handle so the menu can tell them apart; opening a task by link clears filters that would hide it; dismissing AI priority no longer clears Status.
+          <t>UPDATE 2026-09-13: the Priority filter was REMOVED on a founder call after it shipped - the AI-priority view already splits tasks into High / Medium / Low, so the row is Department, Person, Status. Old ?priority= links are ignored.
+BUILT 2026-09-13 - pages/MyWork.js; acceptance 33/33 PASS on desktop 1440 + phone 390, owner and Sales, writes blocked (backend/scripts/ux_person_filter_0913.py, .audit-artifacts/ask24_person_filter/). Notes on the build: Department stays in the saved per-user prefs rather than the URL (it already persisted there); a saved Completed tab and the Desk ?filter=overdue|completed links now convert to the visible Status filter; people who share a display name carry their email handle so the menu can tell them apart; opening a task by link clears filters that would hide it; dismissing AI priority no longer clears Status.
 Founder request 2026-09-13, tracked here for traction. On My Work &gt; All Tasks (desktop and phone):
 (1) PERSON filter - a new 'Person: All' dropdown between Department and Status, same pill as the others. Shown only on All Tasks (on My Tasks every card is yours). Options, each with an open-task count: 'All people'; 'Me'; every person who holds work in the list, busiest first, with their role under the name (e.g. Priya Nair - Sales); 'Unassigned'; and a 'Teams' group for tasks given to a role with no person (the cards' 'Sales team' line). Names come from /users, already loaded as members. With more than 8 people, a type-to-search box sits at the top of the menu.
 (2) COMPLETE STATUS OPTIONS - add 'Pending Approval' (status blocked - the grey chip on most cards, which cannot be filtered today) and 'Overdue' (the orange chip; a lens like Completed). Order: All statuses, Not Started, In Progress, Waiting, Pending Approval, Under Review, Overdue, Completed. Show counts like Department does.

</xml_diff>

<commit_message>
Tracker: ASK-28 TK-01 Asked by me built; T-708..T-716; ASK-27..31 number clash noted
ASK-28 records TK-01 as built (20/20 acceptance + 13 unit tests) and what
is not proven live. Adds coverage T-708..T-716. Notes that commit 5096520
labels its drawer / timeline work ASK-27..ASK-31, which collides with the
workbook's ASK-27 (Desk redesign), ASK-28 (task views), ASK-29 (New Task form).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_UI_Bug_Report.xlsx
+++ b/docs/DecisionOS_UI_Bug_Report.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bug Log'!$A$1:$Q$89</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Coverage'!$A$1:$J$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Coverage'!$A$1:$J$310</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Verified Non-Issues'!$A$1:$E$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Action List'!$A$1:$K$118</definedName>
   </definedNames>
@@ -8116,7 +8116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J301"/>
+  <dimension ref="A1:J310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21586,7 +21586,7 @@
     <row r="273" ht="82" customHeight="1">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>T-700</t>
+          <t>T-708</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
@@ -21596,7 +21596,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>New Task - quick part</t>
+          <t>Asked by me - switcher</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -21606,17 +21606,17 @@
       </c>
       <c r="E273" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Owner + Sales</t>
         </is>
       </c>
       <c r="F273" s="2" t="inlineStr">
         <is>
-          <t>Only title, Department, Assign to and Due show before More options</t>
+          <t>Asked by me sits in the view switcher for every role</t>
         </is>
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H273" s="4" t="inlineStr">
@@ -21626,19 +21626,19 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>Visible: Task title, Department, Assign to, Due; Operational category and Supporting employee gone</t>
+          <t>Owner: My Tasks | Asked by me | All Tasks | Workflows; Sales sees it too</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="274" ht="82" customHeight="1">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>T-701</t>
+          <t>T-709</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
@@ -21648,7 +21648,7 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>New Task - More options</t>
+          <t>Asked by me - the rule</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
@@ -21663,12 +21663,12 @@
       </c>
       <c r="F274" s="2" t="inlineStr">
         <is>
-          <t>Priority, helpers, description, time, result, approval, proof, files wait under More; closed section says how many are set</t>
+          <t>Only tasks I created that are not mine to do</t>
         </is>
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H274" s="4" t="inlineStr">
@@ -21678,19 +21678,19 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>Collapsed by default; '5 set' after choosing priority, helper, time, approval, proof</t>
+          <t>GET /tasks?view=asked: 60 tasks, 0 break the rule; 53 open = 53 cards</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="275" ht="82" customHeight="1">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>T-702</t>
+          <t>T-710</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
@@ -21700,7 +21700,7 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>New Task - title required</t>
+          <t>Asked by me - filters</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -21715,12 +21715,12 @@
       </c>
       <c r="F275" s="2" t="inlineStr">
         <is>
-          <t>Create without a title shows an inline error and sends nothing</t>
+          <t>Person (without Me) and Status narrow the list with matching counts</t>
         </is>
       </c>
       <c r="G275" s="2" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H275" s="4" t="inlineStr">
@@ -21730,19 +21730,19 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>'Give the task a title' under the field; clears on typing; no request</t>
+          <t>Person -&gt; 9 cards = API 9; Status Overdue 13 = 13 cards</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="276" ht="82" customHeight="1">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>T-703</t>
+          <t>T-711</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
@@ -21752,7 +21752,7 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>New Task - Assign to</t>
+          <t>Asked by me - URL and default</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -21767,12 +21767,12 @@
       </c>
       <c r="F276" s="2" t="inlineStr">
         <is>
-          <t>One control lists people and teams; a team explains where it goes</t>
+          <t>View survives refresh, other views clear it, plain /my-work does not reopen on it</t>
         </is>
       </c>
       <c r="G276" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H276" s="4" t="inlineStr">
@@ -21782,19 +21782,19 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>12 people + Sales, Production, Finance teams; hint 'Goes to whoever in Sales has the least open work'</t>
+          <t>?view=asked kept on reload; My Tasks clears it; not saved as default</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="277" ht="82" customHeight="1">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>T-704</t>
+          <t>T-712</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
@@ -21804,7 +21804,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>New Task - due presets</t>
+          <t>Asked by me - AI priority</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -21819,12 +21819,12 @@
       </c>
       <c r="F277" s="2" t="inlineStr">
         <is>
-          <t>Today / Tomorrow / In a week set the date without a picker</t>
+          <t>AI priority is not offered on other people's work</t>
         </is>
       </c>
       <c r="G277" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H277" s="4" t="inlineStr">
@@ -21834,19 +21834,19 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>Tomorrow -&gt; 'Due Tue 15 Sept'; Today -&gt; due_date = today, no time</t>
+          <t>AI toggle hidden on Asked by me</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="278" ht="82" customHeight="1">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>T-705</t>
+          <t>T-713</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">
@@ -21856,7 +21856,7 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>New Task - payload (person)</t>
+          <t>Asked by me - empty</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -21866,17 +21866,17 @@
       </c>
       <c r="E278" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F278" s="2" t="inlineStr">
         <is>
-          <t>The form sends exactly what was chosen and nothing removed</t>
+          <t>Someone who has asked for nothing sees an explanation, not the decisions text</t>
         </is>
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Empty state</t>
         </is>
       </c>
       <c r="H278" s="4" t="inlineStr">
@@ -21886,19 +21886,19 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>task_type sales, lead + 1 helper, high, tomorrow 16:30, approval (anyone), proof; no op_category / support_id</t>
+          <t>'Nothing you've asked for is open - Tasks you create for other people show up here, with their live status.'</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="279" ht="82" customHeight="1">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>T-706</t>
+          <t>T-714</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
@@ -21908,7 +21908,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>New Task - payload (team)</t>
+          <t>Asked by me - requester note</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -21918,17 +21918,17 @@
       </c>
       <c r="E279" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales (mocked list)</t>
         </is>
       </c>
       <c r="F279" s="2" t="inlineStr">
         <is>
-          <t>A team task sends the role, no person and no helpers</t>
+          <t>The person who asked can leave a note but not hand off or escalate</t>
         </is>
       </c>
       <c r="G279" s="2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="H279" s="4" t="inlineStr">
@@ -21938,19 +21938,19 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>assignee_role sales, assignee_id null, co_assignee_ids [], due today</t>
+          <t>Update form offers only Log note; server allows a note from the creator (unit-tested)</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="280" ht="82" customHeight="1">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>T-707</t>
+          <t>T-716</t>
         </is>
       </c>
       <c r="B280" s="2" t="inlineStr">
@@ -21960,7 +21960,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>New Task - after create</t>
+          <t>Asked by me - requester drawer</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -21970,17 +21970,17 @@
       </c>
       <c r="E280" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales (mocked list)</t>
         </is>
       </c>
       <c r="F280" s="2" t="inlineStr">
         <is>
-          <t>Dialog closes, reopens empty with More collapsed, My Work still renders</t>
+          <t>The person who asked sees progress and a note box, not the doer's status, plan, complete or attach controls</t>
         </is>
       </c>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t>Flow</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="H280" s="4" t="inlineStr">
@@ -21990,19 +21990,19 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>Closed; reopened clean; 25 cards; no page errors</t>
+          <t>Status, Complete, Attach, Reopen hidden; hint 'You asked for this task, so &lt;doer&gt; does the work. Leave a note below to follow up.'</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="281" ht="82" customHeight="1">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>T-690</t>
+          <t>T-715</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
@@ -22012,12 +22012,12 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - filter row</t>
+          <t>Asked by me - phone link</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Mobile 390x844</t>
         </is>
       </c>
       <c r="E281" s="2" t="inlineStr">
@@ -22027,12 +22027,12 @@
       </c>
       <c r="F281" s="2" t="inlineStr">
         <is>
-          <t>All Tasks shows Department, Person, Status; My Tasks hides Person</t>
+          <t>A link to Asked by me on a phone shows that list, not My Tasks</t>
         </is>
       </c>
       <c r="G281" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H281" s="4" t="inlineStr">
@@ -22042,19 +22042,19 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>Row shows all three with counts (131); My Tasks shows two (25)</t>
+          <t>53 / 53 cards; My Tasks not pressed; no overflow</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="282" ht="82" customHeight="1">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>T-691</t>
+          <t>T-700</t>
         </is>
       </c>
       <c r="B282" s="2" t="inlineStr">
@@ -22064,7 +22064,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - Person filter</t>
+          <t>New Task - quick part</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -22079,12 +22079,12 @@
       </c>
       <c r="F282" s="2" t="inlineStr">
         <is>
-          <t>Picking a person shows only their tasks, count matches the API</t>
+          <t>Only title, Department, Assign to and Due show before More options</t>
         </is>
       </c>
       <c r="G282" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H282" s="4" t="inlineStr">
@@ -22094,19 +22094,19 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>Priya Nair: 29 cards = trigger 29 = API 29; URL ?person=; name line hidden on cards; menu has Me, people busiest first with role, Unassigned (6), Production team (5); no duplicate rows</t>
+          <t>Visible: Task title, Department, Assign to, Due; Operational category and Supporting employee gone</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="283" ht="82" customHeight="1">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>T-692</t>
+          <t>T-701</t>
         </is>
       </c>
       <c r="B283" s="2" t="inlineStr">
@@ -22116,7 +22116,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - Status options</t>
+          <t>New Task - More options</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -22131,12 +22131,12 @@
       </c>
       <c r="F283" s="2" t="inlineStr">
         <is>
-          <t>Pending Approval, Overdue and Completed are filterable with correct counts</t>
+          <t>Priority, helpers, description, time, result, approval, proof, files wait under More; closed section says how many are set</t>
         </is>
       </c>
       <c r="G283" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H283" s="4" t="inlineStr">
@@ -22146,19 +22146,19 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>Pending Approval 40, Overdue 68, Completed 17, Not Started 78 - all equal the API</t>
+          <t>Collapsed by default; '5 set' after choosing priority, helper, time, approval, proof</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="284" ht="82" customHeight="1">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>T-693</t>
+          <t>T-702</t>
         </is>
       </c>
       <c r="B284" s="2" t="inlineStr">
@@ -22168,12 +22168,12 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - Priority filter removed</t>
+          <t>New Task - title required</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>Desktop + Mobile</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E284" s="2" t="inlineStr">
@@ -22183,12 +22183,12 @@
       </c>
       <c r="F284" s="2" t="inlineStr">
         <is>
-          <t>No Priority filter (founder call 2026-09-13); an old ?priority= link does not narrow the list</t>
+          <t>Create without a title shows an inline error and sends nothing</t>
         </is>
       </c>
       <c r="G284" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="H284" s="4" t="inlineStr">
@@ -22198,19 +22198,19 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>No Priority dropdown on desktop, no Priority chips in the phone sheet; ?person=Priya&amp;status=overdue&amp;priority=high shows the same 20 as without it</t>
+          <t>'Give the task a title' under the field; clears on typing; no request</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="285" ht="82" customHeight="1">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>T-694</t>
+          <t>T-703</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
@@ -22220,7 +22220,7 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - combined counts</t>
+          <t>New Task - Assign to</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -22235,12 +22235,12 @@
       </c>
       <c r="F285" s="2" t="inlineStr">
         <is>
-          <t>Each menu's counts reflect the other active filters</t>
+          <t>One control lists people and teams; a team explains where it goes</t>
         </is>
       </c>
       <c r="G285" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H285" s="4" t="inlineStr">
@@ -22250,19 +22250,19 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>With Priya + Overdue, Department 'All' reads 20 = cards = API</t>
+          <t>12 people + Sales, Production, Finance teams; hint 'Goes to whoever in Sales has the least open work'</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="286" ht="82" customHeight="1">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>T-695</t>
+          <t>T-704</t>
         </is>
       </c>
       <c r="B286" s="2" t="inlineStr">
@@ -22272,7 +22272,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - refresh, Clear, no match</t>
+          <t>New Task - due presets</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -22287,12 +22287,12 @@
       </c>
       <c r="F286" s="2" t="inlineStr">
         <is>
-          <t>Filters survive refresh; Clear resets; empty result explains itself</t>
+          <t>Today / Tomorrow / In a week set the date without a picker</t>
         </is>
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H286" s="4" t="inlineStr">
@@ -22302,19 +22302,19 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>Reload keeps 20 cards + URL; Clear -&gt; 131, URL clean; Priya x Under Review -&gt; 'No tasks match these filters' with Clear</t>
+          <t>Tomorrow -&gt; 'Due Tue 15 Sept'; Today -&gt; due_date = today, no time</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="287" ht="82" customHeight="1">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>T-696</t>
+          <t>T-705</t>
         </is>
       </c>
       <c r="B287" s="2" t="inlineStr">
@@ -22324,7 +22324,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - person search, links</t>
+          <t>New Task - payload (person)</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -22339,12 +22339,12 @@
       </c>
       <c r="F287" s="2" t="inlineStr">
         <is>
-          <t>Search narrows the menu; Desk overdue link and task deep link behave</t>
+          <t>The form sends exactly what was chosen and nothing removed</t>
         </is>
       </c>
       <c r="G287" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H287" s="4" t="inlineStr">
@@ -22354,19 +22354,19 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>'pri' -&gt; Priya Nair only; ?filter=overdue -&gt; Status: Overdue 68; ?task= with filters set clears them and shows the card</t>
+          <t>task_type sales, lead + 1 helper, high, tomorrow 16:30, approval (anyone), proof; no op_category / support_id</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="288" ht="82" customHeight="1">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>T-697</t>
+          <t>T-706</t>
         </is>
       </c>
       <c r="B288" s="2" t="inlineStr">
@@ -22376,12 +22376,12 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>Phone - filter sheet</t>
+          <t>New Task - payload (team)</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
         <is>
-          <t>Mobile 390x844</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E288" s="2" t="inlineStr">
@@ -22391,12 +22391,12 @@
       </c>
       <c r="F288" s="2" t="inlineStr">
         <is>
-          <t>The phone reaches every filter and sees what is active</t>
+          <t>A team task sends the role, no person and no helpers</t>
         </is>
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H288" s="4" t="inlineStr">
@@ -22406,19 +22406,19 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>Sheet with Department / Person / Status; Priya + Overdue -&gt; 'Show 20 tasks' = 20 cards; caption 'Showing Priya Nair - Overdue' with Clear; buttons 44px, reachable; no overflow</t>
+          <t>assignee_role sales, assignee_id null, co_assignee_ids [], due today</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="289" ht="82" customHeight="1">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>T-698</t>
+          <t>T-707</t>
         </is>
       </c>
       <c r="B289" s="2" t="inlineStr">
@@ -22428,12 +22428,12 @@
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>Phone - My Tasks / Status without AI</t>
+          <t>New Task - after create</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
         <is>
-          <t>Mobile 390x844</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E289" s="2" t="inlineStr">
@@ -22443,12 +22443,12 @@
       </c>
       <c r="F289" s="2" t="inlineStr">
         <is>
-          <t>Person hidden on My Tasks; a Status filter is visible even with AI priority off</t>
+          <t>Dialog closes, reopens empty with More collapsed, My Work still renders</t>
         </is>
       </c>
       <c r="G289" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H289" s="4" t="inlineStr">
@@ -22458,19 +22458,19 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>Sheet on My Tasks has no Person; ?status=overdue shows the caption</t>
+          <t>Closed; reopened clean; 25 cards; no page errors</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="290" ht="82" customHeight="1">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>T-699</t>
+          <t>T-690</t>
         </is>
       </c>
       <c r="B290" s="2" t="inlineStr">
@@ -22480,27 +22480,27 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>Sales - no Person filter</t>
+          <t>All Tasks - filter row</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
         <is>
-          <t>Desktop + Mobile</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E290" s="2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F290" s="2" t="inlineStr">
         <is>
-          <t>Roles without All Tasks never see Person; ?person= is ignored</t>
+          <t>All Tasks shows Department, Person, Status; My Tasks hides Person</t>
         </is>
       </c>
       <c r="G290" s="2" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H290" s="4" t="inlineStr">
@@ -22510,7 +22510,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>Desktop row has no Person; phone sheet has no Person; ?person=anyone ignored, own 29 cards</t>
+          <t>Row shows all three with counts (131); My Tasks shows two (25)</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
@@ -22522,17 +22522,17 @@
     <row r="291" ht="82" customHeight="1">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>T-680</t>
+          <t>T-691</t>
         </is>
       </c>
       <c r="B291" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>LIVE - receivables question</t>
+          <t>All Tasks - Person filter</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -22547,44 +22547,44 @@
       </c>
       <c r="F291" s="2" t="inlineStr">
         <is>
-          <t>Dex answers how much customers owe with the ledger's figure</t>
+          <t>Picking a person shows only their tasks, count matches the API</t>
         </is>
       </c>
       <c r="G291" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H291" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H291" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>Said zero invoices / Rs 0 outstanding; ledger has Rs 7,49,000 outstanding (17.0s)</t>
+          <t>Priya Nair: 29 cards = trigger 29 = API 29; URL ?person=; name line hidden on cards; menu has Me, people busiest first with role, Unassigned (6), Production team (5); no duplicate rows</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
         <is>
-          <t>DX-01</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="292" ht="82" customHeight="1">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>T-681</t>
+          <t>T-692</t>
         </is>
       </c>
       <c r="B292" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>LIVE - what needs my attention</t>
+          <t>All Tasks - Status options</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -22599,49 +22599,49 @@
       </c>
       <c r="F292" s="2" t="inlineStr">
         <is>
-          <t>Dex surfaces the overdue work and pending decisions</t>
+          <t>Pending Approval, Overdue and Completed are filterable with correct counts</t>
         </is>
       </c>
       <c r="G292" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H292" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H292" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>Said nothing open or overdue; owner has 24 open / 6 overdue (24.1s)</t>
+          <t>Pending Approval 40, Overdue 68, Completed 17, Not Started 78 - all equal the API</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
         <is>
-          <t>DX-02</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="293" ht="82" customHeight="1">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>T-682</t>
+          <t>T-693</t>
         </is>
       </c>
       <c r="B293" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>LIVE - global search hand-off</t>
+          <t>All Tasks - Priority filter removed</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Desktop + Mobile</t>
         </is>
       </c>
       <c r="E293" s="2" t="inlineStr">
@@ -22651,12 +22651,12 @@
       </c>
       <c r="F293" s="2" t="inlineStr">
         <is>
-          <t>A question from global search is answered on arrival</t>
+          <t>No Priority filter (founder call 2026-09-13); an old ?priority= link does not narrow the list</t>
         </is>
       </c>
       <c r="G293" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H293" s="4" t="inlineStr">
@@ -22666,25 +22666,29 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>'Which tasks are overdue?' answered on /brain?q= with a task list (17.5s)</t>
-        </is>
-      </c>
-      <c r="J293" s="2" t="inlineStr"/>
+          <t>No Priority dropdown on desktop, no Priority chips in the phone sheet; ?person=Priya&amp;status=overdue&amp;priority=high shows the same 20 as without it</t>
+        </is>
+      </c>
+      <c r="J293" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="294" ht="82" customHeight="1">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>T-683</t>
+          <t>T-694</t>
         </is>
       </c>
       <c r="B294" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>LIVE - coach refresh</t>
+          <t>All Tasks - combined counts</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
@@ -22699,12 +22703,12 @@
       </c>
       <c r="F294" s="2" t="inlineStr">
         <is>
-          <t>Generate coaching produces a review grounded in the stats</t>
+          <t>Each menu's counts reflect the other active filters</t>
         </is>
       </c>
       <c r="G294" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H294" s="4" t="inlineStr">
@@ -22714,25 +22718,29 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>TEST_member: 'AI coach updated' in 8.7s; strengths / improvements reference the 13 actionable tasks and plan use</t>
-        </is>
-      </c>
-      <c r="J294" s="2" t="inlineStr"/>
+          <t>With Priya + Overdue, Department 'All' reads 20 = cards = API</t>
+        </is>
+      </c>
+      <c r="J294" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="295" ht="82" customHeight="1">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>T-684</t>
+          <t>T-695</t>
         </is>
       </c>
       <c r="B295" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Score with AI</t>
+          <t>All Tasks - refresh, Clear, no match</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -22747,12 +22755,12 @@
       </c>
       <c r="F295" s="2" t="inlineStr">
         <is>
-          <t>Rescore updates the relationship card sensibly</t>
+          <t>Filters survive refresh; Clear resets; empty result explains itself</t>
         </is>
       </c>
       <c r="G295" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H295" s="4" t="inlineStr">
@@ -22762,25 +22770,29 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>E2E Test Co: 'Relationship scored by AI' in 7.8s; Relationship 12 / Risk 78, reason cites 4 open complaints and no billing - matches the record</t>
-        </is>
-      </c>
-      <c r="J295" s="2" t="inlineStr"/>
+          <t>Reload keeps 20 cards + URL; Clear -&gt; 131, URL clean; Priya x Under Review -&gt; 'No tasks match these filters' with Clear</t>
+        </is>
+      </c>
+      <c r="J295" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="296" ht="82" customHeight="1">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>T-685</t>
+          <t>T-696</t>
         </is>
       </c>
       <c r="B296" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>LIVE - AI analysis refresh</t>
+          <t>All Tasks - person search, links</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -22795,12 +22807,12 @@
       </c>
       <c r="F296" s="2" t="inlineStr">
         <is>
-          <t>Refresh produces an analysis grounded in the ledger</t>
+          <t>Search narrows the menu; Desk overdue link and task deep link behave</t>
         </is>
       </c>
       <c r="G296" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H296" s="4" t="inlineStr">
@@ -22810,30 +22822,34 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>'Analysis refreshed' in 20.6s; Rs 6.6L outstanding (ledger 6,55,466), Surat Spinners Rs 4.8L unpaid 33 days (correct), duplicates flagged</t>
-        </is>
-      </c>
-      <c r="J296" s="2" t="inlineStr"/>
+          <t>'pri' -&gt; Priya Nair only; ?filter=overdue -&gt; Status: Overdue 68; ?task= with filters set clears them and shows the card</t>
+        </is>
+      </c>
+      <c r="J296" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="297" ht="82" customHeight="1">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>T-686</t>
+          <t>T-697</t>
         </is>
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Ask AI</t>
+          <t>Phone - filter sheet</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Mobile 390x844</t>
         </is>
       </c>
       <c r="E297" s="2" t="inlineStr">
@@ -22843,44 +22859,44 @@
       </c>
       <c r="F297" s="2" t="inlineStr">
         <is>
-          <t>The answer is correct and readable</t>
+          <t>The phone reaches every filter and sees what is active</t>
         </is>
       </c>
       <c r="G297" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H297" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H297" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>Correct (Surat Spinners Rs 4,80,000, 7.3s) but literal ** markdown shown</t>
+          <t>Sheet with Department / Person / Status; Priya + Overdue -&gt; 'Show 20 tasks' = 20 cards; caption 'Showing Priya Nair - Overdue' with Clear; buttons 44px, reachable; no overflow</t>
         </is>
       </c>
       <c r="J297" s="2" t="inlineStr">
         <is>
-          <t>FN-12</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="298" ht="82" customHeight="1">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>T-688</t>
+          <t>T-698</t>
         </is>
       </c>
       <c r="B298" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>LIVE - owner on a phone</t>
+          <t>Phone - My Tasks / Status without AI</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -22895,12 +22911,12 @@
       </c>
       <c r="F298" s="2" t="inlineStr">
         <is>
-          <t>Dex answers on mobile and the answer fits the screen</t>
+          <t>Person hidden on My Tasks; a Status filter is visible even with AI priority off</t>
         </is>
       </c>
       <c r="G298" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H298" s="4" t="inlineStr">
@@ -22910,30 +22926,34 @@
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>'53 decisions pending approval across 77' - correct; 17.6s; no overflow</t>
-        </is>
-      </c>
-      <c r="J298" s="2" t="inlineStr"/>
+          <t>Sheet on My Tasks has no Person; ?status=overdue shows the caption</t>
+        </is>
+      </c>
+      <c r="J298" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="299" ht="82" customHeight="1">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>T-689</t>
+          <t>T-699</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Sales asks money questions</t>
+          <t>Sales - no Person filter</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Desktop + Mobile</t>
         </is>
       </c>
       <c r="E299" s="2" t="inlineStr">
@@ -22943,7 +22963,7 @@
       </c>
       <c r="F299" s="2" t="inlineStr">
         <is>
-          <t>Dex refuses finance answers to a role the finance API refuses</t>
+          <t>Roles without All Tasks never see Person; ?person= is ignored</t>
         </is>
       </c>
       <c r="G299" s="2" t="inlineStr">
@@ -22958,25 +22978,29 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>Receivables and profit questions both refused ('You do not have permission to access financial...'), 5.8s / 1.6s; no figures leaked</t>
-        </is>
-      </c>
-      <c r="J299" s="2" t="inlineStr"/>
+          <t>Desktop row has no Person; phone sheet has no Person; ?person=anyone ignored, own 29 cards</t>
+        </is>
+      </c>
+      <c r="J299" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="300" ht="82" customHeight="1">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>T-687</t>
+          <t>T-680</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Dex</t>
         </is>
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>LIVE - bill extraction</t>
+          <t>LIVE - receivables question</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
@@ -22991,7 +23015,7 @@
       </c>
       <c r="F300" s="2" t="inlineStr">
         <is>
-          <t>A GST bill is extracted into a reviewable record with the key fields</t>
+          <t>Dex answers how much customers owe with the ledger's figure</t>
         </is>
       </c>
       <c r="G300" s="2" t="inlineStr">
@@ -23006,65 +23030,509 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>Party, number, amount, due date, category and follow-up correct (31.9s, 92%); date, GSTIN, items missing; no stale-date warning. Left in review, not filed</t>
+          <t>Said zero invoices / Rs 0 outstanding; ledger has Rs 7,49,000 outstanding (17.0s)</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
         <is>
-          <t>FN-13</t>
+          <t>DX-01</t>
         </is>
       </c>
     </row>
     <row r="301" ht="82" customHeight="1">
       <c r="A301" s="2" t="inlineStr">
         <is>
+          <t>T-681</t>
+        </is>
+      </c>
+      <c r="B301" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C301" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - what needs my attention</t>
+        </is>
+      </c>
+      <c r="D301" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E301" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F301" s="2" t="inlineStr">
+        <is>
+          <t>Dex surfaces the overdue work and pending decisions</t>
+        </is>
+      </c>
+      <c r="G301" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H301" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I301" s="2" t="inlineStr">
+        <is>
+          <t>Said nothing open or overdue; owner has 24 open / 6 overdue (24.1s)</t>
+        </is>
+      </c>
+      <c r="J301" s="2" t="inlineStr">
+        <is>
+          <t>DX-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="302" ht="82" customHeight="1">
+      <c r="A302" s="2" t="inlineStr">
+        <is>
+          <t>T-682</t>
+        </is>
+      </c>
+      <c r="B302" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C302" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - global search hand-off</t>
+        </is>
+      </c>
+      <c r="D302" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E302" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F302" s="2" t="inlineStr">
+        <is>
+          <t>A question from global search is answered on arrival</t>
+        </is>
+      </c>
+      <c r="G302" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H302" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I302" s="2" t="inlineStr">
+        <is>
+          <t>'Which tasks are overdue?' answered on /brain?q= with a task list (17.5s)</t>
+        </is>
+      </c>
+      <c r="J302" s="2" t="inlineStr"/>
+    </row>
+    <row r="303" ht="82" customHeight="1">
+      <c r="A303" s="2" t="inlineStr">
+        <is>
+          <t>T-683</t>
+        </is>
+      </c>
+      <c r="B303" s="2" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="C303" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - coach refresh</t>
+        </is>
+      </c>
+      <c r="D303" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E303" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F303" s="2" t="inlineStr">
+        <is>
+          <t>Generate coaching produces a review grounded in the stats</t>
+        </is>
+      </c>
+      <c r="G303" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H303" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I303" s="2" t="inlineStr">
+        <is>
+          <t>TEST_member: 'AI coach updated' in 8.7s; strengths / improvements reference the 13 actionable tasks and plan use</t>
+        </is>
+      </c>
+      <c r="J303" s="2" t="inlineStr"/>
+    </row>
+    <row r="304" ht="82" customHeight="1">
+      <c r="A304" s="2" t="inlineStr">
+        <is>
+          <t>T-684</t>
+        </is>
+      </c>
+      <c r="B304" s="2" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C304" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Score with AI</t>
+        </is>
+      </c>
+      <c r="D304" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E304" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F304" s="2" t="inlineStr">
+        <is>
+          <t>Rescore updates the relationship card sensibly</t>
+        </is>
+      </c>
+      <c r="G304" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H304" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I304" s="2" t="inlineStr">
+        <is>
+          <t>E2E Test Co: 'Relationship scored by AI' in 7.8s; Relationship 12 / Risk 78, reason cites 4 open complaints and no billing - matches the record</t>
+        </is>
+      </c>
+      <c r="J304" s="2" t="inlineStr"/>
+    </row>
+    <row r="305" ht="82" customHeight="1">
+      <c r="A305" s="2" t="inlineStr">
+        <is>
+          <t>T-685</t>
+        </is>
+      </c>
+      <c r="B305" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C305" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - AI analysis refresh</t>
+        </is>
+      </c>
+      <c r="D305" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E305" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F305" s="2" t="inlineStr">
+        <is>
+          <t>Refresh produces an analysis grounded in the ledger</t>
+        </is>
+      </c>
+      <c r="G305" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H305" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I305" s="2" t="inlineStr">
+        <is>
+          <t>'Analysis refreshed' in 20.6s; Rs 6.6L outstanding (ledger 6,55,466), Surat Spinners Rs 4.8L unpaid 33 days (correct), duplicates flagged</t>
+        </is>
+      </c>
+      <c r="J305" s="2" t="inlineStr"/>
+    </row>
+    <row r="306" ht="82" customHeight="1">
+      <c r="A306" s="2" t="inlineStr">
+        <is>
+          <t>T-686</t>
+        </is>
+      </c>
+      <c r="B306" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C306" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Ask AI</t>
+        </is>
+      </c>
+      <c r="D306" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E306" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F306" s="2" t="inlineStr">
+        <is>
+          <t>The answer is correct and readable</t>
+        </is>
+      </c>
+      <c r="G306" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H306" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I306" s="2" t="inlineStr">
+        <is>
+          <t>Correct (Surat Spinners Rs 4,80,000, 7.3s) but literal ** markdown shown</t>
+        </is>
+      </c>
+      <c r="J306" s="2" t="inlineStr">
+        <is>
+          <t>FN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="307" ht="82" customHeight="1">
+      <c r="A307" s="2" t="inlineStr">
+        <is>
+          <t>T-688</t>
+        </is>
+      </c>
+      <c r="B307" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C307" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - owner on a phone</t>
+        </is>
+      </c>
+      <c r="D307" s="2" t="inlineStr">
+        <is>
+          <t>Mobile 390x844</t>
+        </is>
+      </c>
+      <c r="E307" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F307" s="2" t="inlineStr">
+        <is>
+          <t>Dex answers on mobile and the answer fits the screen</t>
+        </is>
+      </c>
+      <c r="G307" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H307" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I307" s="2" t="inlineStr">
+        <is>
+          <t>'53 decisions pending approval across 77' - correct; 17.6s; no overflow</t>
+        </is>
+      </c>
+      <c r="J307" s="2" t="inlineStr"/>
+    </row>
+    <row r="308" ht="82" customHeight="1">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>T-689</t>
+        </is>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C308" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Sales asks money questions</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E308" s="2" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="F308" s="2" t="inlineStr">
+        <is>
+          <t>Dex refuses finance answers to a role the finance API refuses</t>
+        </is>
+      </c>
+      <c r="G308" s="2" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="H308" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I308" s="2" t="inlineStr">
+        <is>
+          <t>Receivables and profit questions both refused ('You do not have permission to access financial...'), 5.8s / 1.6s; no figures leaked</t>
+        </is>
+      </c>
+      <c r="J308" s="2" t="inlineStr"/>
+    </row>
+    <row r="309" ht="82" customHeight="1">
+      <c r="A309" s="2" t="inlineStr">
+        <is>
+          <t>T-687</t>
+        </is>
+      </c>
+      <c r="B309" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C309" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - bill extraction</t>
+        </is>
+      </c>
+      <c r="D309" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E309" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F309" s="2" t="inlineStr">
+        <is>
+          <t>A GST bill is extracted into a reviewable record with the key fields</t>
+        </is>
+      </c>
+      <c r="G309" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H309" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I309" s="2" t="inlineStr">
+        <is>
+          <t>Party, number, amount, due date, category and follow-up correct (31.9s, 92%); date, GSTIN, items missing; no stale-date warning. Left in review, not filed</t>
+        </is>
+      </c>
+      <c r="J309" s="2" t="inlineStr">
+        <is>
+          <t>FN-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="310" ht="82" customHeight="1">
+      <c r="A310" s="2" t="inlineStr">
+        <is>
           <t>T-676</t>
         </is>
       </c>
-      <c r="B301" s="2" t="inlineStr">
+      <c r="B310" s="2" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="C301" s="2" t="inlineStr">
+      <c r="C310" s="2" t="inlineStr">
         <is>
           <t>Admin portal gating</t>
         </is>
       </c>
-      <c r="D301" s="2" t="inlineStr">
+      <c r="D310" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="E301" s="2" t="inlineStr">
+      <c r="E310" s="2" t="inlineStr">
         <is>
           <t>Signed out / Owner</t>
         </is>
       </c>
-      <c r="F301" s="2" t="inlineStr">
+      <c r="F310" s="2" t="inlineStr">
         <is>
           <t>Only platform admins reach the portal</t>
         </is>
       </c>
-      <c r="G301" s="2" t="inlineStr">
+      <c r="G310" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="H301" s="4" t="inlineStr">
+      <c r="H310" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I301" s="2" t="inlineStr">
+      <c r="I310" s="2" t="inlineStr">
         <is>
           <t>Signed out and tenant owner both get the admin sign-in; /admin/me 401; deep link /admin/tenants too</t>
         </is>
       </c>
-      <c r="J301" s="2" t="inlineStr"/>
+      <c r="J310" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J301"/>
+  <autoFilter ref="A1:J310"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -25028,7 +25496,8 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Plan: docs/TASK_MANAGEMENT_PLAN.md Phase 1; checklist: https://claude.ai/code/artifact/53a2b23e-66a5-4eeb-bfb3-52a87ce08043. TK-01 Asked by me (tasks I created for others). TK-02 Waiting for my approval (named approver, or anyone with approvals when none is named). TK-03 My team (doer or helper reports to me, via reporting_manager_id). TK-04 /my-work?task= opens the task even when it is not in the current view.</t>
+          <t>PROGRESS 2026-09-14 - TK-01 Asked by me BUILT (desktop): GET /tasks?view=asked (created by me, not mine to do: I am neither the doer nor a helper); My Work switcher gets Asked by me (owner: My Tasks | Asked by me | All Tasks; staff: My Work | Asked by me), kept in the URL (?view=asked) and never saved as the default; Department, Person (no Me option) and Status filters work on it; AI priority is off there; its own empty state; the person who asked can leave a note on the task (server + form), hand-off and escalate stay with the doer; a phone link lands on the list. Acceptance 20/20 (backend/scripts/ux_task_asked_0914.py, writes blocked) + 13 unit tests (backend/tests/test_task_view_asked.py). NOT proven live: a non-owner creating a task and then seeing it - no non-owner in the demo company has created one, and creating one writes to the production database; the note-only form was checked with a mocked list. TK-02..TK-04 still to do.
+Plan: docs/TASK_MANAGEMENT_PLAN.md Phase 1; checklist: https://claude.ai/code/artifact/53a2b23e-66a5-4eeb-bfb3-52a87ce08043. TK-01 Asked by me (tasks I created for others). TK-02 Waiting for my approval (named approver, or anyone with approvals when none is named). TK-03 My team (doer or helper reports to me, via reporting_manager_id). TK-04 /my-work?task= opens the task even when it is not in the current view.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -29785,7 +30254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:B61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -29867,490 +30336,502 @@
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
         <is>
+          <t>ASK clash 14 Sep</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Commit 5096520 (task drawer rebuilt, activity timeline, grayscale My Work) and its code comments say ASK-27..ASK-31, but this workbook already uses ASK-27 = Decision Desk redesign, ASK-28 = task views, ASK-29 = New Task form (9b88efc). Those comments do NOT refer to these rows. The drawer/timeline work has no row of its own yet; give it the next free number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Still happening. Later commits label ASK-18 (Workflows well), ASK-19 (card summary), ASK-20 (My Work scroll) and ASK-21 (New Task dialog) from the other list. In this workbook ASK-18 is the CRM In-progress list, ASK-19 the operating score KPIs, and ASK-20 / ASK-21 / ASK-22 are the three root causes from the full audit (load errors, permission map, phone parity). Match commits to this sheet by content, not by number.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="16" t="inlineStr"/>
-      <c r="B10" s="17" t="inlineStr"/>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="13" t="inlineStr"/>
-      <c r="B11" s="14" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr"/>
+      <c r="B11" s="17" t="inlineStr"/>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="13" t="inlineStr"/>
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Leave approvals: who approves, and is the Settings screen needed?</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="13" t="inlineStr"/>
-      <c r="B12" s="15" t="inlineStr">
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="13" t="inlineStr"/>
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>Raised 2026-09-12 by Yogesh - Owner. Status: DEFERRED, Yogesh deciding. Relates to ASK-8. Nothing is to be built from this note until that call is made.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr"/>
-      <c r="B13" s="17" t="inlineStr"/>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="18" t="inlineStr"/>
-      <c r="B14" s="19" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr"/>
+      <c r="B14" s="17" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="18" t="inlineStr"/>
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>THE QUESTION</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="16" t="inlineStr"/>
-      <c r="B15" s="17" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="16" t="inlineStr"/>
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Leave approval is mostly done by either the owner or a manager. The approver is already chosen when a team member is added. So does the 'Leave Approvers by Department' settings screen need to exist at all?</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr"/>
-      <c r="B16" s="17" t="inlineStr"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="18" t="inlineStr"/>
-      <c r="B17" s="19" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr"/>
+      <c r="B17" s="17" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="18" t="inlineStr"/>
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>HOW APPROVAL IS DECIDED TODAY</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="16" t="inlineStr"/>
-      <c r="B18" s="17" t="inlineStr">
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="16" t="inlineStr"/>
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>When someone requests leave the system asks three questions IN ORDER and stops at the first that answers. The code is services/leave.py, _resolve_leave_approver.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>Tier 1</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>Does this person have a Reporting Manager? If yes, that manager approves. The Reporting Manager is chosen in Team when the member is added or edited (pages/Team.js:144, the member-manager-select dropdown; stored as reporting_manager_id).</t>
         </is>
       </c>
     </row>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Does this person have a Reporting Manager? If yes, that manager approves. The Reporting Manager is chosen in Team when the member is added or edited (pages/Team.js:144, the member-manager-select dropdown; stored as reporting_manager_id).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="B20" s="17" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>Otherwise: is there a department rule for their role? If yes, that person approves. THIS IS THE SETTINGS SCREEN under discussion - the gear in the Leave section, which opens 'Leave Approvers by Department' with one dropdown per department and a Save button.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>Tier 3</t>
         </is>
       </c>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>Otherwise the Owner approves.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr"/>
-      <c r="B22" s="17" t="inlineStr"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="18" t="inlineStr"/>
-      <c r="B23" s="19" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr"/>
+      <c r="B23" s="17" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="18" t="inlineStr"/>
+      <c r="B24" s="19" t="inlineStr">
         <is>
           <t>WHAT THE LIVE DATA SHOWS</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="16" t="inlineStr"/>
-      <c r="B24" s="17" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr"/>
+      <c r="B25" s="17" t="inlineStr">
         <is>
           <t>Measured against the dev workspace on 2026-09-12, not assumed:</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t>Members</t>
-        </is>
-      </c>
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>12 team members in the workspace.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
         <is>
-          <t>Tier 1 used</t>
+          <t>Members</t>
         </is>
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>1 member has a Reporting Manager set (sai, finance).</t>
+          <t>12 team members in the workspace.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>Tier 2 used</t>
+          <t>Tier 1 used</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>0. The tenant leave_approvers mapping is EMPTY - every department reads 'Owner (default)'.</t>
+          <t>1 member has a Reporting Manager set (sai, finance).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>Tier 3 used</t>
+          <t>Tier 2 used</t>
         </is>
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>11 of 12 members fall through to the Owner, Rajesh Sharma.</t>
+          <t>0. The tenant leave_approvers mapping is EMPTY - every department reads 'Owner (default)'.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
         <is>
+          <t>Tier 3 used</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>11 of 12 members fall through to the Owner, Rajesh Sharma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>The Settings screen currently decides leave for NOBODY. It configures a tier that no request reaches.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="16" t="inlineStr"/>
-      <c r="B30" s="17" t="inlineStr"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="18" t="inlineStr"/>
-      <c r="B31" s="19" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr"/>
+      <c r="B31" s="17" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="18" t="inlineStr"/>
+      <c r="B32" s="19" t="inlineStr">
         <is>
           <t>WHAT THE THREE PIECES ARE</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="16" t="inlineStr"/>
-      <c r="B32" s="17" t="inlineStr">
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="16" t="inlineStr"/>
+      <c r="B33" s="17" t="inlineStr">
         <is>
           <t>They are three layers of one feature. Removing one without the others leaves either a screen that cannot save or an endpoint nothing calls.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="16" t="inlineStr">
-        <is>
-          <t>The gear</t>
-        </is>
-      </c>
-      <c r="B33" s="17" t="inlineStr">
-        <is>
-          <t>The small round icon beside the My Leave / Approvals tabs. It is the only way into the screen. pages/Leave.js:500-510.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="16" t="inlineStr">
         <is>
-          <t>The panel</t>
+          <t>The gear</t>
         </is>
       </c>
       <c r="B34" s="17" t="inlineStr">
         <is>
-          <t>'Leave Approvers by Department' - a dropdown per department plus a Save approvers button. pages/Leave.js:387-417.</t>
+          <t>The small round icon beside the My Leave / Approvals tabs. It is the only way into the screen. pages/Leave.js:500-510.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="16" t="inlineStr">
         <is>
+          <t>The panel</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>'Leave Approvers by Department' - a dropdown per department plus a Save approvers button. pages/Leave.js:387-417.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
           <t>The endpoint</t>
         </is>
       </c>
-      <c r="B35" s="17" t="inlineStr">
+      <c r="B36" s="17" t="inlineStr">
         <is>
           <t>PATCH /tenant/leave-approvers, which writes the leave_approvers field on the tenant record. routers/calendar.py:24.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="16" t="inlineStr"/>
-      <c r="B36" s="17" t="inlineStr"/>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="18" t="inlineStr"/>
-      <c r="B37" s="19" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr"/>
+      <c r="B37" s="17" t="inlineStr"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="18" t="inlineStr"/>
+      <c r="B38" s="19" t="inlineStr">
         <is>
           <t>OPTION A - DELETE TIER 2  (the current recommendation)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
         <is>
           <t>What changes</t>
         </is>
       </c>
-      <c r="B38" s="17" t="inlineStr">
+      <c r="B39" s="17" t="inlineStr">
         <is>
           <t>Remove the gear, the panel and the endpoint. Approval becomes: reporting manager, else owner.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="16" t="inlineStr">
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t>Effect today</t>
         </is>
       </c>
-      <c r="B39" s="17" t="inlineStr">
+      <c r="B40" s="17" t="inlineStr">
         <is>
           <t>NONE. Every one of the 12 members resolves to exactly the same approver before and after, because nothing uses tier 2.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="45" customHeight="1">
-      <c r="A40" s="16" t="inlineStr">
+    <row r="41" ht="45" customHeight="1">
+      <c r="A41" s="16" t="inlineStr">
         <is>
           <t>Argument for</t>
         </is>
       </c>
-      <c r="B40" s="17" t="inlineStr">
+      <c r="B41" s="17" t="inlineStr">
         <is>
           <t>The approver is already chosen once, in Team, when the person is added. A second screen expressing the same decision in different words - and silently losing to the first one - mostly creates the chance for the two to disagree with the org chart.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="16" t="inlineStr"/>
-      <c r="B41" s="17" t="inlineStr"/>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="18" t="inlineStr"/>
-      <c r="B42" s="19" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr"/>
+      <c r="B42" s="17" t="inlineStr"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="18" t="inlineStr"/>
+      <c r="B43" s="19" t="inlineStr">
         <is>
           <t>OPTION B - KEEP TIER 2</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="16" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t>What it buys</t>
         </is>
       </c>
-      <c r="B43" s="17" t="inlineStr">
+      <c r="B44" s="17" t="inlineStr">
         <is>
           <t>One place to say 'all Sales leave goes to Priya' without making Priya anyone's reporting manager.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="16" t="inlineStr">
-        <is>
-          <t>Cost of A</t>
-        </is>
-      </c>
-      <c r="B44" s="17" t="inlineStr">
-        <is>
-          <t>To get that same outcome after deleting, Priya would have to be set as the reporting manager of each Sales person individually, in Team.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="16" t="inlineStr">
         <is>
+          <t>Cost of A</t>
+        </is>
+      </c>
+      <c r="B45" s="17" t="inlineStr">
+        <is>
+          <t>To get that same outcome after deleting, Priya would have to be set as the reporting manager of each Sales person individually, in Team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
           <t>If kept</t>
         </is>
       </c>
-      <c r="B45" s="17" t="inlineStr">
+      <c r="B46" s="17" t="inlineStr">
         <is>
           <t>Then the fix is not to move it into Settings but to make it visible - today it is hidden behind an unlabelled gear inside a work surface, which is why it has stayed empty.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="16" t="inlineStr"/>
-      <c r="B46" s="17" t="inlineStr"/>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="18" t="inlineStr"/>
-      <c r="B47" s="19" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr"/>
+      <c r="B47" s="17" t="inlineStr"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="18" t="inlineStr"/>
+      <c r="B48" s="19" t="inlineStr">
         <is>
           <t>THE ONE QUESTION THAT DECIDES IT</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="16" t="inlineStr"/>
-      <c r="B48" s="17" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr"/>
+      <c r="B49" s="17" t="inlineStr">
         <is>
           <t>Is 'who approves your leave' always the same person as 'who you report to'?</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="16" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="B49" s="17" t="inlineStr">
+      <c r="B50" s="17" t="inlineStr">
         <is>
           <t>They are always the same -&gt; Option A. Tier 2 is pure duplication.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B50" s="17" t="inlineStr">
-        <is>
-          <t>They can differ - for example a department lead signs off leave while people report to a project manager -&gt; Option B, and the work is to surface the screen properly rather than hide it.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="16" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B51" s="17" t="inlineStr">
+        <is>
+          <t>They can differ - for example a department lead signs off leave while people report to a project manager -&gt; Option B, and the work is to surface the screen properly rather than hide it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="16" t="inlineStr">
+        <is>
           <t>Read</t>
         </is>
       </c>
-      <c r="B51" s="17" t="inlineStr">
+      <c r="B52" s="17" t="inlineStr">
         <is>
           <t>For an SME the answer is usually yes, which is why A is the standing recommendation - but this is a business call, not a technical one, which is why it is parked rather than filed as a defect.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="16" t="inlineStr"/>
-      <c r="B52" s="17" t="inlineStr"/>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="18" t="inlineStr"/>
-      <c r="B53" s="19" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr"/>
+      <c r="B53" s="17" t="inlineStr"/>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="18" t="inlineStr"/>
+      <c r="B54" s="19" t="inlineStr">
         <is>
           <t>IF OPTION A IS CHOSEN, THE WORK IS</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B54" s="17" t="inlineStr">
-        <is>
-          <t>Delete the gear and the settings tab from pages/Leave.js (:500-510).</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B55" s="17" t="inlineStr">
         <is>
-          <t>Delete the LeaveApproverConfig block from pages/Leave.js (:387-417).</t>
+          <t>Delete the gear and the settings tab from pages/Leave.js (:500-510).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B56" s="17" t="inlineStr">
+        <is>
+          <t>Delete the LeaveApproverConfig block from pages/Leave.js (:387-417).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B56" s="17" t="inlineStr">
+      <c r="B57" s="17" t="inlineStr">
         <is>
           <t>Delete PATCH /tenant/leave-approvers from routers/calendar.py (:24) and the LeaveApproverMapInput model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="16" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B57" s="17" t="inlineStr">
-        <is>
-          <t>Drop the tier-2 lookup from _resolve_leave_approver in services/leave.py, leaving reporting manager then owner.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="16" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B58" s="17" t="inlineStr">
         <is>
-          <t>Leave the leave_approvers field on existing tenant records alone, or clear it in the migration - it is empty in practice either way.</t>
+          <t>Drop the tier-2 lookup from _resolve_leave_approver in services/leave.py, leaving reporting manager then owner.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="16" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B59" s="17" t="inlineStr">
         <is>
-          <t>Make sure Team makes the consequence visible: the Reporting Manager dropdown should say that this person also approves their leave, since after this change that is the only place the decision is made.</t>
+          <t>Leave the leave_approvers field on existing tenant records alone, or clear it in the migration - it is empty in practice either way.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="16" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B60" s="17" t="inlineStr">
+        <is>
+          <t>Make sure Team makes the consequence visible: the Reporting Manager dropdown should say that this person also approves their leave, since after this change that is the only place the decision is made.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="16" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B60" s="17" t="inlineStr">
+      <c r="B61" s="17" t="inlineStr">
         <is>
           <t>This depends on ASK-6. If Leave moves into Team first, the gear disappears with it and steps 1 and 2 become part of that move rather than separate work.</t>
         </is>
@@ -30810,7 +31291,7 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>300 (209 pass, 89 fail, 0 blocked, 2 not run)</t>
+          <t>309 (218 pass, 89 fail, 0 blocked, 2 not run)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker fix: builder parses again; workbook rebuilt with ASK-28 TK-02 and T-717..T-725
974b8b2 put apostrophes inside a single-quoted string in the ASK-28 note, so
build_ui_bug_report.py raised SyntaxError and the workbook was never rebuilt.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_UI_Bug_Report.xlsx
+++ b/docs/DecisionOS_UI_Bug_Report.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bug Log'!$A$1:$Q$89</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Coverage'!$A$1:$J$310</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Coverage'!$A$1:$J$319</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Verified Non-Issues'!$A$1:$E$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Action List'!$A$1:$K$118</definedName>
   </definedNames>
@@ -8116,7 +8116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J310"/>
+  <dimension ref="A1:J319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21586,7 +21586,7 @@
     <row r="273" ht="82" customHeight="1">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>T-708</t>
+          <t>T-717</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
@@ -21596,7 +21596,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - switcher</t>
+          <t>Approvals - the rule</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -21606,17 +21606,17 @@
       </c>
       <c r="E273" s="2" t="inlineStr">
         <is>
-          <t>Owner + Sales</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F273" s="2" t="inlineStr">
         <is>
-          <t>Asked by me sits in the view switcher for every role</t>
+          <t>The feed holds only tasks that still need approval and are not finished</t>
         </is>
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>Views</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H273" s="4" t="inlineStr">
@@ -21626,7 +21626,7 @@
       </c>
       <c r="I273" s="2" t="inlineStr">
         <is>
-          <t>Owner: My Tasks | Asked by me | All Tasks | Workflows; Sales sees it too</t>
+          <t>GET /tasks?view=approvals: 7 (6 pending + 1 changes requested), 0 break the rule</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr">
@@ -21638,7 +21638,7 @@
     <row r="274" ht="82" customHeight="1">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>T-709</t>
+          <t>T-718</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
@@ -21648,7 +21648,7 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - the rule</t>
+          <t>Approvals - one button, with count</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
@@ -21663,12 +21663,12 @@
       </c>
       <c r="F274" s="2" t="inlineStr">
         <is>
-          <t>Only tasks I created that are not mine to do</t>
+          <t>One Approvals button in the switcher, showing how many wait</t>
         </is>
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H274" s="4" t="inlineStr">
@@ -21678,7 +21678,7 @@
       </c>
       <c r="I274" s="2" t="inlineStr">
         <is>
-          <t>GET /tasks?view=asked: 60 tasks, 0 break the rule; 53 open = 53 cards</t>
+          <t>My Tasks | Asked by me | All Tasks | Approvals (6) | Workflows; no duplicate</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr">
@@ -21690,7 +21690,7 @@
     <row r="275" ht="82" customHeight="1">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>T-710</t>
+          <t>T-719</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
@@ -21700,7 +21700,7 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - filters</t>
+          <t>Approvals - Tasks tab</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -21715,12 +21715,12 @@
       </c>
       <c r="F275" s="2" t="inlineStr">
         <is>
-          <t>Person (without Me) and Status narrow the list with matching counts</t>
+          <t>The Tasks tab is exactly what waits on me, oldest request first</t>
         </is>
       </c>
       <c r="G275" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H275" s="4" t="inlineStr">
@@ -21730,7 +21730,7 @@
       </c>
       <c r="I275" s="2" t="inlineStr">
         <is>
-          <t>Person -&gt; 9 cards = API 9; Status Overdue 13 = 13 cards</t>
+          <t>6 cards = 6 pending from the server rule; 14 Aug first, 20 Aug last; tab reads Tasks 6</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr">
@@ -21742,7 +21742,7 @@
     <row r="276" ht="82" customHeight="1">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>T-711</t>
+          <t>T-720</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
@@ -21752,7 +21752,7 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - URL and default</t>
+          <t>Approvals - drawer actions</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -21767,7 +21767,7 @@
       </c>
       <c r="F276" s="2" t="inlineStr">
         <is>
-          <t>View survives refresh, other views clear it, plain /my-work does not reopen on it</t>
+          <t>Opening a waiting task offers Approve, Request changes, Ask clarification</t>
         </is>
       </c>
       <c r="G276" s="2" t="inlineStr">
@@ -21782,7 +21782,7 @@
       </c>
       <c r="I276" s="2" t="inlineStr">
         <is>
-          <t>?view=asked kept on reload; My Tasks clears it; not saved as default</t>
+          <t>All three shown; Approve sends POST /tasks/{id}/approve (answered by the test)</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr">
@@ -21794,7 +21794,7 @@
     <row r="277" ht="82" customHeight="1">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>T-712</t>
+          <t>T-721</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
@@ -21804,7 +21804,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - AI priority</t>
+          <t>Approvals - notification link</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -21819,12 +21819,12 @@
       </c>
       <c r="F277" s="2" t="inlineStr">
         <is>
-          <t>AI priority is not offered on other people's work</t>
+          <t>An approval-requested notification opens the task inside Approvals</t>
         </is>
       </c>
       <c r="G277" s="2" t="inlineStr">
         <is>
-          <t>Views</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H277" s="4" t="inlineStr">
@@ -21834,7 +21834,7 @@
       </c>
       <c r="I277" s="2" t="inlineStr">
         <is>
-          <t>AI toggle hidden on Asked by me</t>
+          <t>/my-work?view=approvals&amp;task=&lt;id&gt; shows the Approvals view with the drawer and its approval box</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr">
@@ -21846,17 +21846,17 @@
     <row r="278" ht="82" customHeight="1">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>T-713</t>
+          <t>T-722</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Decision Desk</t>
         </is>
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - empty</t>
+          <t>Task approvals card</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -21866,17 +21866,17 @@
       </c>
       <c r="E278" s="2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F278" s="2" t="inlineStr">
         <is>
-          <t>Someone who has asked for nothing sees an explanation, not the decisions text</t>
+          <t>The Desk card and My Work Approvals count the same thing</t>
         </is>
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>Empty state</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H278" s="4" t="inlineStr">
@@ -21886,7 +21886,7 @@
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>'Nothing you've asked for is open - Tasks you create for other people show up here, with their live status.'</t>
+          <t>Desk card 6 = Approvals 6 (both read /tasks?view=approvals)</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
@@ -21898,7 +21898,7 @@
     <row r="279" ht="82" customHeight="1">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>T-714</t>
+          <t>T-723</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
@@ -21908,7 +21908,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - requester note</t>
+          <t>Approvals - no access</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -21918,12 +21918,12 @@
       </c>
       <c r="E279" s="2" t="inlineStr">
         <is>
-          <t>Sales (mocked list)</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F279" s="2" t="inlineStr">
         <is>
-          <t>The person who asked can leave a note but not hand off or escalate</t>
+          <t>Someone who can approve nothing gets no Approvals button and an empty feed</t>
         </is>
       </c>
       <c r="G279" s="2" t="inlineStr">
@@ -21938,7 +21938,7 @@
       </c>
       <c r="I279" s="2" t="inlineStr">
         <is>
-          <t>Update form offers only Log note; server allows a note from the creator (unit-tested)</t>
+          <t>No button; API returns 0</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr">
@@ -21950,7 +21950,7 @@
     <row r="280" ht="82" customHeight="1">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>T-716</t>
+          <t>T-724</t>
         </is>
       </c>
       <c r="B280" s="2" t="inlineStr">
@@ -21960,7 +21960,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - requester drawer</t>
+          <t>Approvals - named approver</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -21975,7 +21975,7 @@
       </c>
       <c r="F280" s="2" t="inlineStr">
         <is>
-          <t>The person who asked sees progress and a note box, not the doer's status, plan, complete or attach controls</t>
+          <t>A non-owner named as approver, without approval access, sees the view and can approve</t>
         </is>
       </c>
       <c r="G280" s="2" t="inlineStr">
@@ -21990,7 +21990,7 @@
       </c>
       <c r="I280" s="2" t="inlineStr">
         <is>
-          <t>Status, Complete, Attach, Reopen hidden; hint 'You asked for this task, so &lt;doer&gt; does the work. Leave a note below to follow up.'</t>
+          <t>Button with badge 1; card in the Tasks tab; approval box; Approve POST sent (list mocked)</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr">
@@ -22002,7 +22002,7 @@
     <row r="281" ht="82" customHeight="1">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>T-715</t>
+          <t>T-725</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
@@ -22012,7 +22012,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - phone link</t>
+          <t>Approvals - phone link</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -22027,7 +22027,7 @@
       </c>
       <c r="F281" s="2" t="inlineStr">
         <is>
-          <t>A link to Asked by me on a phone shows that list, not My Tasks</t>
+          <t>A link to Approvals on a phone shows the same tasks</t>
         </is>
       </c>
       <c r="G281" s="2" t="inlineStr">
@@ -22042,7 +22042,7 @@
       </c>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>53 / 53 cards; My Tasks not pressed; no overflow</t>
+          <t>6 / 6 cards; no overflow</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr">
@@ -22054,7 +22054,7 @@
     <row r="282" ht="82" customHeight="1">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>T-700</t>
+          <t>T-708</t>
         </is>
       </c>
       <c r="B282" s="2" t="inlineStr">
@@ -22064,7 +22064,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>New Task - quick part</t>
+          <t>Asked by me - switcher</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -22074,17 +22074,17 @@
       </c>
       <c r="E282" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Owner + Sales</t>
         </is>
       </c>
       <c r="F282" s="2" t="inlineStr">
         <is>
-          <t>Only title, Department, Assign to and Due show before More options</t>
+          <t>Asked by me sits in the view switcher for every role</t>
         </is>
       </c>
       <c r="G282" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H282" s="4" t="inlineStr">
@@ -22094,19 +22094,19 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>Visible: Task title, Department, Assign to, Due; Operational category and Supporting employee gone</t>
+          <t>Owner: My Tasks | Asked by me | All Tasks | Workflows; Sales sees it too</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="283" ht="82" customHeight="1">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>T-701</t>
+          <t>T-709</t>
         </is>
       </c>
       <c r="B283" s="2" t="inlineStr">
@@ -22116,7 +22116,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>New Task - More options</t>
+          <t>Asked by me - the rule</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -22131,12 +22131,12 @@
       </c>
       <c r="F283" s="2" t="inlineStr">
         <is>
-          <t>Priority, helpers, description, time, result, approval, proof, files wait under More; closed section says how many are set</t>
+          <t>Only tasks I created that are not mine to do</t>
         </is>
       </c>
       <c r="G283" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H283" s="4" t="inlineStr">
@@ -22146,19 +22146,19 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>Collapsed by default; '5 set' after choosing priority, helper, time, approval, proof</t>
+          <t>GET /tasks?view=asked: 60 tasks, 0 break the rule; 53 open = 53 cards</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="284" ht="82" customHeight="1">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>T-702</t>
+          <t>T-710</t>
         </is>
       </c>
       <c r="B284" s="2" t="inlineStr">
@@ -22168,7 +22168,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>New Task - title required</t>
+          <t>Asked by me - filters</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -22183,12 +22183,12 @@
       </c>
       <c r="F284" s="2" t="inlineStr">
         <is>
-          <t>Create without a title shows an inline error and sends nothing</t>
+          <t>Person (without Me) and Status narrow the list with matching counts</t>
         </is>
       </c>
       <c r="G284" s="2" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H284" s="4" t="inlineStr">
@@ -22198,19 +22198,19 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>'Give the task a title' under the field; clears on typing; no request</t>
+          <t>Person -&gt; 9 cards = API 9; Status Overdue 13 = 13 cards</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="285" ht="82" customHeight="1">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>T-703</t>
+          <t>T-711</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
@@ -22220,7 +22220,7 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>New Task - Assign to</t>
+          <t>Asked by me - URL and default</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -22235,12 +22235,12 @@
       </c>
       <c r="F285" s="2" t="inlineStr">
         <is>
-          <t>One control lists people and teams; a team explains where it goes</t>
+          <t>View survives refresh, other views clear it, plain /my-work does not reopen on it</t>
         </is>
       </c>
       <c r="G285" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H285" s="4" t="inlineStr">
@@ -22250,19 +22250,19 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>12 people + Sales, Production, Finance teams; hint 'Goes to whoever in Sales has the least open work'</t>
+          <t>?view=asked kept on reload; My Tasks clears it; not saved as default</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="286" ht="82" customHeight="1">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>T-704</t>
+          <t>T-712</t>
         </is>
       </c>
       <c r="B286" s="2" t="inlineStr">
@@ -22272,7 +22272,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>New Task - due presets</t>
+          <t>Asked by me - AI priority</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -22287,12 +22287,12 @@
       </c>
       <c r="F286" s="2" t="inlineStr">
         <is>
-          <t>Today / Tomorrow / In a week set the date without a picker</t>
+          <t>AI priority is not offered on other people's work</t>
         </is>
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H286" s="4" t="inlineStr">
@@ -22302,19 +22302,19 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>Tomorrow -&gt; 'Due Tue 15 Sept'; Today -&gt; due_date = today, no time</t>
+          <t>AI toggle hidden on Asked by me</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="287" ht="82" customHeight="1">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>T-705</t>
+          <t>T-713</t>
         </is>
       </c>
       <c r="B287" s="2" t="inlineStr">
@@ -22324,7 +22324,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>New Task - payload (person)</t>
+          <t>Asked by me - empty</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -22334,17 +22334,17 @@
       </c>
       <c r="E287" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F287" s="2" t="inlineStr">
         <is>
-          <t>The form sends exactly what was chosen and nothing removed</t>
+          <t>Someone who has asked for nothing sees an explanation, not the decisions text</t>
         </is>
       </c>
       <c r="G287" s="2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Empty state</t>
         </is>
       </c>
       <c r="H287" s="4" t="inlineStr">
@@ -22354,19 +22354,19 @@
       </c>
       <c r="I287" s="2" t="inlineStr">
         <is>
-          <t>task_type sales, lead + 1 helper, high, tomorrow 16:30, approval (anyone), proof; no op_category / support_id</t>
+          <t>'Nothing you've asked for is open - Tasks you create for other people show up here, with their live status.'</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="288" ht="82" customHeight="1">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>T-706</t>
+          <t>T-714</t>
         </is>
       </c>
       <c r="B288" s="2" t="inlineStr">
@@ -22376,7 +22376,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>New Task - payload (team)</t>
+          <t>Asked by me - requester note</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -22386,17 +22386,17 @@
       </c>
       <c r="E288" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales (mocked list)</t>
         </is>
       </c>
       <c r="F288" s="2" t="inlineStr">
         <is>
-          <t>A team task sends the role, no person and no helpers</t>
+          <t>The person who asked can leave a note but not hand off or escalate</t>
         </is>
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="H288" s="4" t="inlineStr">
@@ -22406,19 +22406,19 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>assignee_role sales, assignee_id null, co_assignee_ids [], due today</t>
+          <t>Update form offers only Log note; server allows a note from the creator (unit-tested)</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="289" ht="82" customHeight="1">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>T-707</t>
+          <t>T-716</t>
         </is>
       </c>
       <c r="B289" s="2" t="inlineStr">
@@ -22428,7 +22428,7 @@
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>New Task - after create</t>
+          <t>Asked by me - requester drawer</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
@@ -22438,17 +22438,17 @@
       </c>
       <c r="E289" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales (mocked list)</t>
         </is>
       </c>
       <c r="F289" s="2" t="inlineStr">
         <is>
-          <t>Dialog closes, reopens empty with More collapsed, My Work still renders</t>
+          <t>The person who asked sees progress and a note box, not the doer's status, plan, complete or attach controls</t>
         </is>
       </c>
       <c r="G289" s="2" t="inlineStr">
         <is>
-          <t>Flow</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="H289" s="4" t="inlineStr">
@@ -22458,19 +22458,19 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>Closed; reopened clean; 25 cards; no page errors</t>
+          <t>Status, Complete, Attach, Reopen hidden; hint 'You asked for this task, so &lt;doer&gt; does the work. Leave a note below to follow up.'</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="290" ht="82" customHeight="1">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>T-690</t>
+          <t>T-715</t>
         </is>
       </c>
       <c r="B290" s="2" t="inlineStr">
@@ -22480,12 +22480,12 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - filter row</t>
+          <t>Asked by me - phone link</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Mobile 390x844</t>
         </is>
       </c>
       <c r="E290" s="2" t="inlineStr">
@@ -22495,12 +22495,12 @@
       </c>
       <c r="F290" s="2" t="inlineStr">
         <is>
-          <t>All Tasks shows Department, Person, Status; My Tasks hides Person</t>
+          <t>A link to Asked by me on a phone shows that list, not My Tasks</t>
         </is>
       </c>
       <c r="G290" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H290" s="4" t="inlineStr">
@@ -22510,19 +22510,19 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>Row shows all three with counts (131); My Tasks shows two (25)</t>
+          <t>53 / 53 cards; My Tasks not pressed; no overflow</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="291" ht="82" customHeight="1">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>T-691</t>
+          <t>T-700</t>
         </is>
       </c>
       <c r="B291" s="2" t="inlineStr">
@@ -22532,7 +22532,7 @@
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - Person filter</t>
+          <t>New Task - quick part</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -22547,12 +22547,12 @@
       </c>
       <c r="F291" s="2" t="inlineStr">
         <is>
-          <t>Picking a person shows only their tasks, count matches the API</t>
+          <t>Only title, Department, Assign to and Due show before More options</t>
         </is>
       </c>
       <c r="G291" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H291" s="4" t="inlineStr">
@@ -22562,19 +22562,19 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>Priya Nair: 29 cards = trigger 29 = API 29; URL ?person=; name line hidden on cards; menu has Me, people busiest first with role, Unassigned (6), Production team (5); no duplicate rows</t>
+          <t>Visible: Task title, Department, Assign to, Due; Operational category and Supporting employee gone</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="292" ht="82" customHeight="1">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>T-692</t>
+          <t>T-701</t>
         </is>
       </c>
       <c r="B292" s="2" t="inlineStr">
@@ -22584,7 +22584,7 @@
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - Status options</t>
+          <t>New Task - More options</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -22599,12 +22599,12 @@
       </c>
       <c r="F292" s="2" t="inlineStr">
         <is>
-          <t>Pending Approval, Overdue and Completed are filterable with correct counts</t>
+          <t>Priority, helpers, description, time, result, approval, proof, files wait under More; closed section says how many are set</t>
         </is>
       </c>
       <c r="G292" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H292" s="4" t="inlineStr">
@@ -22614,19 +22614,19 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>Pending Approval 40, Overdue 68, Completed 17, Not Started 78 - all equal the API</t>
+          <t>Collapsed by default; '5 set' after choosing priority, helper, time, approval, proof</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="293" ht="82" customHeight="1">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>T-693</t>
+          <t>T-702</t>
         </is>
       </c>
       <c r="B293" s="2" t="inlineStr">
@@ -22636,12 +22636,12 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - Priority filter removed</t>
+          <t>New Task - title required</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
         <is>
-          <t>Desktop + Mobile</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E293" s="2" t="inlineStr">
@@ -22651,12 +22651,12 @@
       </c>
       <c r="F293" s="2" t="inlineStr">
         <is>
-          <t>No Priority filter (founder call 2026-09-13); an old ?priority= link does not narrow the list</t>
+          <t>Create without a title shows an inline error and sends nothing</t>
         </is>
       </c>
       <c r="G293" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="H293" s="4" t="inlineStr">
@@ -22666,19 +22666,19 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>No Priority dropdown on desktop, no Priority chips in the phone sheet; ?person=Priya&amp;status=overdue&amp;priority=high shows the same 20 as without it</t>
+          <t>'Give the task a title' under the field; clears on typing; no request</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="294" ht="82" customHeight="1">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>T-694</t>
+          <t>T-703</t>
         </is>
       </c>
       <c r="B294" s="2" t="inlineStr">
@@ -22688,7 +22688,7 @@
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - combined counts</t>
+          <t>New Task - Assign to</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
@@ -22703,12 +22703,12 @@
       </c>
       <c r="F294" s="2" t="inlineStr">
         <is>
-          <t>Each menu's counts reflect the other active filters</t>
+          <t>One control lists people and teams; a team explains where it goes</t>
         </is>
       </c>
       <c r="G294" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H294" s="4" t="inlineStr">
@@ -22718,19 +22718,19 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>With Priya + Overdue, Department 'All' reads 20 = cards = API</t>
+          <t>12 people + Sales, Production, Finance teams; hint 'Goes to whoever in Sales has the least open work'</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="295" ht="82" customHeight="1">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>T-695</t>
+          <t>T-704</t>
         </is>
       </c>
       <c r="B295" s="2" t="inlineStr">
@@ -22740,7 +22740,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - refresh, Clear, no match</t>
+          <t>New Task - due presets</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -22755,12 +22755,12 @@
       </c>
       <c r="F295" s="2" t="inlineStr">
         <is>
-          <t>Filters survive refresh; Clear resets; empty result explains itself</t>
+          <t>Today / Tomorrow / In a week set the date without a picker</t>
         </is>
       </c>
       <c r="G295" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H295" s="4" t="inlineStr">
@@ -22770,19 +22770,19 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>Reload keeps 20 cards + URL; Clear -&gt; 131, URL clean; Priya x Under Review -&gt; 'No tasks match these filters' with Clear</t>
+          <t>Tomorrow -&gt; 'Due Tue 15 Sept'; Today -&gt; due_date = today, no time</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="296" ht="82" customHeight="1">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>T-696</t>
+          <t>T-705</t>
         </is>
       </c>
       <c r="B296" s="2" t="inlineStr">
@@ -22792,7 +22792,7 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - person search, links</t>
+          <t>New Task - payload (person)</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -22807,12 +22807,12 @@
       </c>
       <c r="F296" s="2" t="inlineStr">
         <is>
-          <t>Search narrows the menu; Desk overdue link and task deep link behave</t>
+          <t>The form sends exactly what was chosen and nothing removed</t>
         </is>
       </c>
       <c r="G296" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H296" s="4" t="inlineStr">
@@ -22822,19 +22822,19 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>'pri' -&gt; Priya Nair only; ?filter=overdue -&gt; Status: Overdue 68; ?task= with filters set clears them and shows the card</t>
+          <t>task_type sales, lead + 1 helper, high, tomorrow 16:30, approval (anyone), proof; no op_category / support_id</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="297" ht="82" customHeight="1">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>T-697</t>
+          <t>T-706</t>
         </is>
       </c>
       <c r="B297" s="2" t="inlineStr">
@@ -22844,12 +22844,12 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>Phone - filter sheet</t>
+          <t>New Task - payload (team)</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
         <is>
-          <t>Mobile 390x844</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E297" s="2" t="inlineStr">
@@ -22859,12 +22859,12 @@
       </c>
       <c r="F297" s="2" t="inlineStr">
         <is>
-          <t>The phone reaches every filter and sees what is active</t>
+          <t>A team task sends the role, no person and no helpers</t>
         </is>
       </c>
       <c r="G297" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H297" s="4" t="inlineStr">
@@ -22874,19 +22874,19 @@
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>Sheet with Department / Person / Status; Priya + Overdue -&gt; 'Show 20 tasks' = 20 cards; caption 'Showing Priya Nair - Overdue' with Clear; buttons 44px, reachable; no overflow</t>
+          <t>assignee_role sales, assignee_id null, co_assignee_ids [], due today</t>
         </is>
       </c>
       <c r="J297" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="298" ht="82" customHeight="1">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>T-698</t>
+          <t>T-707</t>
         </is>
       </c>
       <c r="B298" s="2" t="inlineStr">
@@ -22896,12 +22896,12 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>Phone - My Tasks / Status without AI</t>
+          <t>New Task - after create</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
         <is>
-          <t>Mobile 390x844</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E298" s="2" t="inlineStr">
@@ -22911,12 +22911,12 @@
       </c>
       <c r="F298" s="2" t="inlineStr">
         <is>
-          <t>Person hidden on My Tasks; a Status filter is visible even with AI priority off</t>
+          <t>Dialog closes, reopens empty with More collapsed, My Work still renders</t>
         </is>
       </c>
       <c r="G298" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H298" s="4" t="inlineStr">
@@ -22926,19 +22926,19 @@
       </c>
       <c r="I298" s="2" t="inlineStr">
         <is>
-          <t>Sheet on My Tasks has no Person; ?status=overdue shows the caption</t>
+          <t>Closed; reopened clean; 25 cards; no page errors</t>
         </is>
       </c>
       <c r="J298" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="299" ht="82" customHeight="1">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>T-699</t>
+          <t>T-690</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
@@ -22948,27 +22948,27 @@
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>Sales - no Person filter</t>
+          <t>All Tasks - filter row</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
         <is>
-          <t>Desktop + Mobile</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E299" s="2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F299" s="2" t="inlineStr">
         <is>
-          <t>Roles without All Tasks never see Person; ?person= is ignored</t>
+          <t>All Tasks shows Department, Person, Status; My Tasks hides Person</t>
         </is>
       </c>
       <c r="G299" s="2" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H299" s="4" t="inlineStr">
@@ -22978,7 +22978,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>Desktop row has no Person; phone sheet has no Person; ?person=anyone ignored, own 29 cards</t>
+          <t>Row shows all three with counts (131); My Tasks shows two (25)</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr">
@@ -22990,17 +22990,17 @@
     <row r="300" ht="82" customHeight="1">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>T-680</t>
+          <t>T-691</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>LIVE - receivables question</t>
+          <t>All Tasks - Person filter</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
@@ -23015,44 +23015,44 @@
       </c>
       <c r="F300" s="2" t="inlineStr">
         <is>
-          <t>Dex answers how much customers owe with the ledger's figure</t>
+          <t>Picking a person shows only their tasks, count matches the API</t>
         </is>
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H300" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H300" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>Said zero invoices / Rs 0 outstanding; ledger has Rs 7,49,000 outstanding (17.0s)</t>
+          <t>Priya Nair: 29 cards = trigger 29 = API 29; URL ?person=; name line hidden on cards; menu has Me, people busiest first with role, Unassigned (6), Production team (5); no duplicate rows</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
         <is>
-          <t>DX-01</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="301" ht="82" customHeight="1">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>T-681</t>
+          <t>T-692</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>LIVE - what needs my attention</t>
+          <t>All Tasks - Status options</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -23067,49 +23067,49 @@
       </c>
       <c r="F301" s="2" t="inlineStr">
         <is>
-          <t>Dex surfaces the overdue work and pending decisions</t>
+          <t>Pending Approval, Overdue and Completed are filterable with correct counts</t>
         </is>
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H301" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H301" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>Said nothing open or overdue; owner has 24 open / 6 overdue (24.1s)</t>
+          <t>Pending Approval 40, Overdue 68, Completed 17, Not Started 78 - all equal the API</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
         <is>
-          <t>DX-02</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="302" ht="82" customHeight="1">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>T-682</t>
+          <t>T-693</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>LIVE - global search hand-off</t>
+          <t>All Tasks - Priority filter removed</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Desktop + Mobile</t>
         </is>
       </c>
       <c r="E302" s="2" t="inlineStr">
@@ -23119,12 +23119,12 @@
       </c>
       <c r="F302" s="2" t="inlineStr">
         <is>
-          <t>A question from global search is answered on arrival</t>
+          <t>No Priority filter (founder call 2026-09-13); an old ?priority= link does not narrow the list</t>
         </is>
       </c>
       <c r="G302" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H302" s="4" t="inlineStr">
@@ -23134,25 +23134,29 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>'Which tasks are overdue?' answered on /brain?q= with a task list (17.5s)</t>
-        </is>
-      </c>
-      <c r="J302" s="2" t="inlineStr"/>
+          <t>No Priority dropdown on desktop, no Priority chips in the phone sheet; ?person=Priya&amp;status=overdue&amp;priority=high shows the same 20 as without it</t>
+        </is>
+      </c>
+      <c r="J302" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="303" ht="82" customHeight="1">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>T-683</t>
+          <t>T-694</t>
         </is>
       </c>
       <c r="B303" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>LIVE - coach refresh</t>
+          <t>All Tasks - combined counts</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
@@ -23167,12 +23171,12 @@
       </c>
       <c r="F303" s="2" t="inlineStr">
         <is>
-          <t>Generate coaching produces a review grounded in the stats</t>
+          <t>Each menu's counts reflect the other active filters</t>
         </is>
       </c>
       <c r="G303" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H303" s="4" t="inlineStr">
@@ -23182,25 +23186,29 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>TEST_member: 'AI coach updated' in 8.7s; strengths / improvements reference the 13 actionable tasks and plan use</t>
-        </is>
-      </c>
-      <c r="J303" s="2" t="inlineStr"/>
+          <t>With Priya + Overdue, Department 'All' reads 20 = cards = API</t>
+        </is>
+      </c>
+      <c r="J303" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="304" ht="82" customHeight="1">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>T-684</t>
+          <t>T-695</t>
         </is>
       </c>
       <c r="B304" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Score with AI</t>
+          <t>All Tasks - refresh, Clear, no match</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
@@ -23215,12 +23223,12 @@
       </c>
       <c r="F304" s="2" t="inlineStr">
         <is>
-          <t>Rescore updates the relationship card sensibly</t>
+          <t>Filters survive refresh; Clear resets; empty result explains itself</t>
         </is>
       </c>
       <c r="G304" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H304" s="4" t="inlineStr">
@@ -23230,25 +23238,29 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>E2E Test Co: 'Relationship scored by AI' in 7.8s; Relationship 12 / Risk 78, reason cites 4 open complaints and no billing - matches the record</t>
-        </is>
-      </c>
-      <c r="J304" s="2" t="inlineStr"/>
+          <t>Reload keeps 20 cards + URL; Clear -&gt; 131, URL clean; Priya x Under Review -&gt; 'No tasks match these filters' with Clear</t>
+        </is>
+      </c>
+      <c r="J304" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="305" ht="82" customHeight="1">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>T-685</t>
+          <t>T-696</t>
         </is>
       </c>
       <c r="B305" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>LIVE - AI analysis refresh</t>
+          <t>All Tasks - person search, links</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
@@ -23263,12 +23275,12 @@
       </c>
       <c r="F305" s="2" t="inlineStr">
         <is>
-          <t>Refresh produces an analysis grounded in the ledger</t>
+          <t>Search narrows the menu; Desk overdue link and task deep link behave</t>
         </is>
       </c>
       <c r="G305" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H305" s="4" t="inlineStr">
@@ -23278,30 +23290,34 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>'Analysis refreshed' in 20.6s; Rs 6.6L outstanding (ledger 6,55,466), Surat Spinners Rs 4.8L unpaid 33 days (correct), duplicates flagged</t>
-        </is>
-      </c>
-      <c r="J305" s="2" t="inlineStr"/>
+          <t>'pri' -&gt; Priya Nair only; ?filter=overdue -&gt; Status: Overdue 68; ?task= with filters set clears them and shows the card</t>
+        </is>
+      </c>
+      <c r="J305" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="306" ht="82" customHeight="1">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>T-686</t>
+          <t>T-697</t>
         </is>
       </c>
       <c r="B306" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Ask AI</t>
+          <t>Phone - filter sheet</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Mobile 390x844</t>
         </is>
       </c>
       <c r="E306" s="2" t="inlineStr">
@@ -23311,44 +23327,44 @@
       </c>
       <c r="F306" s="2" t="inlineStr">
         <is>
-          <t>The answer is correct and readable</t>
+          <t>The phone reaches every filter and sees what is active</t>
         </is>
       </c>
       <c r="G306" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H306" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H306" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>Correct (Surat Spinners Rs 4,80,000, 7.3s) but literal ** markdown shown</t>
+          <t>Sheet with Department / Person / Status; Priya + Overdue -&gt; 'Show 20 tasks' = 20 cards; caption 'Showing Priya Nair - Overdue' with Clear; buttons 44px, reachable; no overflow</t>
         </is>
       </c>
       <c r="J306" s="2" t="inlineStr">
         <is>
-          <t>FN-12</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="307" ht="82" customHeight="1">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>T-688</t>
+          <t>T-698</t>
         </is>
       </c>
       <c r="B307" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>LIVE - owner on a phone</t>
+          <t>Phone - My Tasks / Status without AI</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
@@ -23363,12 +23379,12 @@
       </c>
       <c r="F307" s="2" t="inlineStr">
         <is>
-          <t>Dex answers on mobile and the answer fits the screen</t>
+          <t>Person hidden on My Tasks; a Status filter is visible even with AI priority off</t>
         </is>
       </c>
       <c r="G307" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H307" s="4" t="inlineStr">
@@ -23378,30 +23394,34 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>'53 decisions pending approval across 77' - correct; 17.6s; no overflow</t>
-        </is>
-      </c>
-      <c r="J307" s="2" t="inlineStr"/>
+          <t>Sheet on My Tasks has no Person; ?status=overdue shows the caption</t>
+        </is>
+      </c>
+      <c r="J307" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="308" ht="82" customHeight="1">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>T-689</t>
+          <t>T-699</t>
         </is>
       </c>
       <c r="B308" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Sales asks money questions</t>
+          <t>Sales - no Person filter</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Desktop + Mobile</t>
         </is>
       </c>
       <c r="E308" s="2" t="inlineStr">
@@ -23411,7 +23431,7 @@
       </c>
       <c r="F308" s="2" t="inlineStr">
         <is>
-          <t>Dex refuses finance answers to a role the finance API refuses</t>
+          <t>Roles without All Tasks never see Person; ?person= is ignored</t>
         </is>
       </c>
       <c r="G308" s="2" t="inlineStr">
@@ -23426,25 +23446,29 @@
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>Receivables and profit questions both refused ('You do not have permission to access financial...'), 5.8s / 1.6s; no figures leaked</t>
-        </is>
-      </c>
-      <c r="J308" s="2" t="inlineStr"/>
+          <t>Desktop row has no Person; phone sheet has no Person; ?person=anyone ignored, own 29 cards</t>
+        </is>
+      </c>
+      <c r="J308" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="309" ht="82" customHeight="1">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>T-687</t>
+          <t>T-680</t>
         </is>
       </c>
       <c r="B309" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Dex</t>
         </is>
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>LIVE - bill extraction</t>
+          <t>LIVE - receivables question</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
@@ -23459,7 +23483,7 @@
       </c>
       <c r="F309" s="2" t="inlineStr">
         <is>
-          <t>A GST bill is extracted into a reviewable record with the key fields</t>
+          <t>Dex answers how much customers owe with the ledger's figure</t>
         </is>
       </c>
       <c r="G309" s="2" t="inlineStr">
@@ -23474,65 +23498,509 @@
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>Party, number, amount, due date, category and follow-up correct (31.9s, 92%); date, GSTIN, items missing; no stale-date warning. Left in review, not filed</t>
+          <t>Said zero invoices / Rs 0 outstanding; ledger has Rs 7,49,000 outstanding (17.0s)</t>
         </is>
       </c>
       <c r="J309" s="2" t="inlineStr">
         <is>
-          <t>FN-13</t>
+          <t>DX-01</t>
         </is>
       </c>
     </row>
     <row r="310" ht="82" customHeight="1">
       <c r="A310" s="2" t="inlineStr">
         <is>
+          <t>T-681</t>
+        </is>
+      </c>
+      <c r="B310" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C310" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - what needs my attention</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E310" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F310" s="2" t="inlineStr">
+        <is>
+          <t>Dex surfaces the overdue work and pending decisions</t>
+        </is>
+      </c>
+      <c r="G310" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H310" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I310" s="2" t="inlineStr">
+        <is>
+          <t>Said nothing open or overdue; owner has 24 open / 6 overdue (24.1s)</t>
+        </is>
+      </c>
+      <c r="J310" s="2" t="inlineStr">
+        <is>
+          <t>DX-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="311" ht="82" customHeight="1">
+      <c r="A311" s="2" t="inlineStr">
+        <is>
+          <t>T-682</t>
+        </is>
+      </c>
+      <c r="B311" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C311" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - global search hand-off</t>
+        </is>
+      </c>
+      <c r="D311" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E311" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F311" s="2" t="inlineStr">
+        <is>
+          <t>A question from global search is answered on arrival</t>
+        </is>
+      </c>
+      <c r="G311" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H311" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I311" s="2" t="inlineStr">
+        <is>
+          <t>'Which tasks are overdue?' answered on /brain?q= with a task list (17.5s)</t>
+        </is>
+      </c>
+      <c r="J311" s="2" t="inlineStr"/>
+    </row>
+    <row r="312" ht="82" customHeight="1">
+      <c r="A312" s="2" t="inlineStr">
+        <is>
+          <t>T-683</t>
+        </is>
+      </c>
+      <c r="B312" s="2" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="C312" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - coach refresh</t>
+        </is>
+      </c>
+      <c r="D312" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E312" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F312" s="2" t="inlineStr">
+        <is>
+          <t>Generate coaching produces a review grounded in the stats</t>
+        </is>
+      </c>
+      <c r="G312" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H312" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I312" s="2" t="inlineStr">
+        <is>
+          <t>TEST_member: 'AI coach updated' in 8.7s; strengths / improvements reference the 13 actionable tasks and plan use</t>
+        </is>
+      </c>
+      <c r="J312" s="2" t="inlineStr"/>
+    </row>
+    <row r="313" ht="82" customHeight="1">
+      <c r="A313" s="2" t="inlineStr">
+        <is>
+          <t>T-684</t>
+        </is>
+      </c>
+      <c r="B313" s="2" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C313" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Score with AI</t>
+        </is>
+      </c>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E313" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F313" s="2" t="inlineStr">
+        <is>
+          <t>Rescore updates the relationship card sensibly</t>
+        </is>
+      </c>
+      <c r="G313" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H313" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I313" s="2" t="inlineStr">
+        <is>
+          <t>E2E Test Co: 'Relationship scored by AI' in 7.8s; Relationship 12 / Risk 78, reason cites 4 open complaints and no billing - matches the record</t>
+        </is>
+      </c>
+      <c r="J313" s="2" t="inlineStr"/>
+    </row>
+    <row r="314" ht="82" customHeight="1">
+      <c r="A314" s="2" t="inlineStr">
+        <is>
+          <t>T-685</t>
+        </is>
+      </c>
+      <c r="B314" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C314" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - AI analysis refresh</t>
+        </is>
+      </c>
+      <c r="D314" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E314" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F314" s="2" t="inlineStr">
+        <is>
+          <t>Refresh produces an analysis grounded in the ledger</t>
+        </is>
+      </c>
+      <c r="G314" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H314" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I314" s="2" t="inlineStr">
+        <is>
+          <t>'Analysis refreshed' in 20.6s; Rs 6.6L outstanding (ledger 6,55,466), Surat Spinners Rs 4.8L unpaid 33 days (correct), duplicates flagged</t>
+        </is>
+      </c>
+      <c r="J314" s="2" t="inlineStr"/>
+    </row>
+    <row r="315" ht="82" customHeight="1">
+      <c r="A315" s="2" t="inlineStr">
+        <is>
+          <t>T-686</t>
+        </is>
+      </c>
+      <c r="B315" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C315" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Ask AI</t>
+        </is>
+      </c>
+      <c r="D315" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E315" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F315" s="2" t="inlineStr">
+        <is>
+          <t>The answer is correct and readable</t>
+        </is>
+      </c>
+      <c r="G315" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H315" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I315" s="2" t="inlineStr">
+        <is>
+          <t>Correct (Surat Spinners Rs 4,80,000, 7.3s) but literal ** markdown shown</t>
+        </is>
+      </c>
+      <c r="J315" s="2" t="inlineStr">
+        <is>
+          <t>FN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="316" ht="82" customHeight="1">
+      <c r="A316" s="2" t="inlineStr">
+        <is>
+          <t>T-688</t>
+        </is>
+      </c>
+      <c r="B316" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C316" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - owner on a phone</t>
+        </is>
+      </c>
+      <c r="D316" s="2" t="inlineStr">
+        <is>
+          <t>Mobile 390x844</t>
+        </is>
+      </c>
+      <c r="E316" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F316" s="2" t="inlineStr">
+        <is>
+          <t>Dex answers on mobile and the answer fits the screen</t>
+        </is>
+      </c>
+      <c r="G316" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H316" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I316" s="2" t="inlineStr">
+        <is>
+          <t>'53 decisions pending approval across 77' - correct; 17.6s; no overflow</t>
+        </is>
+      </c>
+      <c r="J316" s="2" t="inlineStr"/>
+    </row>
+    <row r="317" ht="82" customHeight="1">
+      <c r="A317" s="2" t="inlineStr">
+        <is>
+          <t>T-689</t>
+        </is>
+      </c>
+      <c r="B317" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C317" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Sales asks money questions</t>
+        </is>
+      </c>
+      <c r="D317" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E317" s="2" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="F317" s="2" t="inlineStr">
+        <is>
+          <t>Dex refuses finance answers to a role the finance API refuses</t>
+        </is>
+      </c>
+      <c r="G317" s="2" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="H317" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I317" s="2" t="inlineStr">
+        <is>
+          <t>Receivables and profit questions both refused ('You do not have permission to access financial...'), 5.8s / 1.6s; no figures leaked</t>
+        </is>
+      </c>
+      <c r="J317" s="2" t="inlineStr"/>
+    </row>
+    <row r="318" ht="82" customHeight="1">
+      <c r="A318" s="2" t="inlineStr">
+        <is>
+          <t>T-687</t>
+        </is>
+      </c>
+      <c r="B318" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C318" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - bill extraction</t>
+        </is>
+      </c>
+      <c r="D318" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E318" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F318" s="2" t="inlineStr">
+        <is>
+          <t>A GST bill is extracted into a reviewable record with the key fields</t>
+        </is>
+      </c>
+      <c r="G318" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H318" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I318" s="2" t="inlineStr">
+        <is>
+          <t>Party, number, amount, due date, category and follow-up correct (31.9s, 92%); date, GSTIN, items missing; no stale-date warning. Left in review, not filed</t>
+        </is>
+      </c>
+      <c r="J318" s="2" t="inlineStr">
+        <is>
+          <t>FN-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="319" ht="82" customHeight="1">
+      <c r="A319" s="2" t="inlineStr">
+        <is>
           <t>T-676</t>
         </is>
       </c>
-      <c r="B310" s="2" t="inlineStr">
+      <c r="B319" s="2" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="C310" s="2" t="inlineStr">
+      <c r="C319" s="2" t="inlineStr">
         <is>
           <t>Admin portal gating</t>
         </is>
       </c>
-      <c r="D310" s="2" t="inlineStr">
+      <c r="D319" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="E310" s="2" t="inlineStr">
+      <c r="E319" s="2" t="inlineStr">
         <is>
           <t>Signed out / Owner</t>
         </is>
       </c>
-      <c r="F310" s="2" t="inlineStr">
+      <c r="F319" s="2" t="inlineStr">
         <is>
           <t>Only platform admins reach the portal</t>
         </is>
       </c>
-      <c r="G310" s="2" t="inlineStr">
+      <c r="G319" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="H310" s="4" t="inlineStr">
+      <c r="H319" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I310" s="2" t="inlineStr">
+      <c r="I319" s="2" t="inlineStr">
         <is>
           <t>Signed out and tenant owner both get the admin sign-in; /admin/me 401; deep link /admin/tenants too</t>
         </is>
       </c>
-      <c r="J310" s="2" t="inlineStr"/>
+      <c r="J319" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J310"/>
+  <autoFilter ref="A1:J319"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -25496,7 +25964,8 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>PROGRESS 2026-09-14 - TK-01 Asked by me BUILT (desktop): GET /tasks?view=asked (created by me, not mine to do: I am neither the doer nor a helper); My Work switcher gets Asked by me (owner: My Tasks | Asked by me | All Tasks; staff: My Work | Asked by me), kept in the URL (?view=asked) and never saved as the default; Department, Person (no Me option) and Status filters work on it; AI priority is off there; its own empty state; the person who asked can leave a note on the task (server + form), hand-off and escalate stay with the doer; a phone link lands on the list. Acceptance 20/20 (backend/scripts/ux_task_asked_0914.py, writes blocked) + 13 unit tests (backend/tests/test_task_view_asked.py). NOT proven live: a non-owner creating a task and then seeing it - no non-owner in the demo company has created one, and creating one writes to the production database; the note-only form was checked with a mocked list. TK-02..TK-04 still to do.
+          <t>PROGRESS 2026-09-14 - TK-02 Waiting for my approval BUILT (desktop), merged into the Approvals view that 3c23e49 added to My Work: GET /tasks?view=approvals (approval required, not approved, not finished; owner sees all, a named approver sees tasks naming them, an Approve Tasks holder also sees tasks naming nobody - the same rule as _can_approve_task) now feeds the Tasks tab of that view AND the Task approvals card on the Desk (both read /tasks?mine=false before, which for a non-owner is their own lane only, so a named approver outside it saw nothing). The Approvals button carries the pending count and also shows for a named approver without approval access; list is oldest first; the approval-requested notification opens /my-work?view=approvals&amp;task=&lt;id&gt; inside Approvals. Acceptance 21/21 (backend/scripts/ux_task_approvals_0914.py, writes blocked, Approve answered by the script) + 8 unit tests (backend/tests/test_task_view_approvals.py). NOT proven live: a non-owner approver approving a real task - no demo user holds approval access or is named on a task, so that path was checked with a mocked list.
+PROGRESS 2026-09-14 - TK-01 Asked by me BUILT (desktop): GET /tasks?view=asked (created by me, not mine to do: I am neither the doer nor a helper); My Work switcher gets Asked by me (owner: My Tasks | Asked by me | All Tasks; staff: My Work | Asked by me), kept in the URL (?view=asked) and never saved as the default; Department, Person (no Me option) and Status filters work on it; AI priority is off there; its own empty state; the person who asked can leave a note on the task (server + form), hand-off and escalate stay with the doer; a phone link lands on the list. Acceptance 20/20 (backend/scripts/ux_task_asked_0914.py, writes blocked) + 13 unit tests (backend/tests/test_task_view_asked.py). NOT proven live: a non-owner creating a task and then seeing it - no non-owner in the demo company has created one, and creating one writes to the production database; the note-only form was checked with a mocked list. TK-02..TK-04 still to do.
 Plan: docs/TASK_MANAGEMENT_PLAN.md Phase 1; checklist: https://claude.ai/code/artifact/53a2b23e-66a5-4eeb-bfb3-52a87ce08043. TK-01 Asked by me (tasks I created for others). TK-02 Waiting for my approval (named approver, or anyone with approvals when none is named). TK-03 My team (doer or helper reports to me, via reporting_manager_id). TK-04 /my-work?task= opens the task even when it is not in the current view.</t>
         </is>
       </c>
@@ -30254,7 +30723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -30333,505 +30802,517 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t>ASK clash 14 Sep</t>
+          <t>ASK clash 14 Sep (2)</t>
         </is>
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>Commit 5096520 (task drawer rebuilt, activity timeline, grayscale My Work) and its code comments say ASK-27..ASK-31, but this workbook already uses ASK-27 = Decision Desk redesign, ASK-28 = task views, ASK-29 = New Task form (9b88efc). Those comments do NOT refer to these rows. The drawer/timeline work has no row of its own yet; give it the next free number.</t>
+          <t>Commit 3c23e49 (Decision Desk redesign + Approvals inside My Work) says ASK-25, but this workbook uses ASK-25 for the My Work cards + photos (513b9f0). The Desk redesign is ASK-27 here; the Approvals view it added is where ASK-28 TK-02 now lives.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
+          <t>ASK clash 14 Sep</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Commit 5096520 (task drawer rebuilt, activity timeline, grayscale My Work) and its code comments say ASK-27..ASK-31, but this workbook already uses ASK-27 = Decision Desk redesign, ASK-28 = task views, ASK-29 = New Task form (9b88efc). Those comments do NOT refer to these rows. The drawer/timeline work has no row of its own yet; give it the next free number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Still happening. Later commits label ASK-18 (Workflows well), ASK-19 (card summary), ASK-20 (My Work scroll) and ASK-21 (New Task dialog) from the other list. In this workbook ASK-18 is the CRM In-progress list, ASK-19 the operating score KPIs, and ASK-20 / ASK-21 / ASK-22 are the three root causes from the full audit (load errors, permission map, phone parity). Match commits to this sheet by content, not by number.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="16" t="inlineStr"/>
-      <c r="B11" s="17" t="inlineStr"/>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="13" t="inlineStr"/>
-      <c r="B12" s="14" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr"/>
+      <c r="B12" s="17" t="inlineStr"/>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="13" t="inlineStr"/>
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>Leave approvals: who approves, and is the Settings screen needed?</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="13" t="inlineStr"/>
-      <c r="B13" s="15" t="inlineStr">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="13" t="inlineStr"/>
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Raised 2026-09-12 by Yogesh - Owner. Status: DEFERRED, Yogesh deciding. Relates to ASK-8. Nothing is to be built from this note until that call is made.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="16" t="inlineStr"/>
-      <c r="B14" s="17" t="inlineStr"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="18" t="inlineStr"/>
-      <c r="B15" s="19" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr"/>
+      <c r="B15" s="17" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="18" t="inlineStr"/>
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>THE QUESTION</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="16" t="inlineStr"/>
-      <c r="B16" s="17" t="inlineStr">
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="16" t="inlineStr"/>
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Leave approval is mostly done by either the owner or a manager. The approver is already chosen when a team member is added. So does the 'Leave Approvers by Department' settings screen need to exist at all?</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr"/>
-      <c r="B17" s="17" t="inlineStr"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="18" t="inlineStr"/>
-      <c r="B18" s="19" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr"/>
+      <c r="B18" s="17" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="18" t="inlineStr"/>
+      <c r="B19" s="19" t="inlineStr">
         <is>
           <t>HOW APPROVAL IS DECIDED TODAY</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="16" t="inlineStr"/>
-      <c r="B19" s="17" t="inlineStr">
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="16" t="inlineStr"/>
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>When someone requests leave the system asks three questions IN ORDER and stops at the first that answers. The code is services/leave.py, _resolve_leave_approver.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>Tier 1</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>Does this person have a Reporting Manager? If yes, that manager approves. The Reporting Manager is chosen in Team when the member is added or edited (pages/Team.js:144, the member-manager-select dropdown; stored as reporting_manager_id).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Does this person have a Reporting Manager? If yes, that manager approves. The Reporting Manager is chosen in Team when the member is added or edited (pages/Team.js:144, the member-manager-select dropdown; stored as reporting_manager_id).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>Otherwise: is there a department rule for their role? If yes, that person approves. THIS IS THE SETTINGS SCREEN under discussion - the gear in the Leave section, which opens 'Leave Approvers by Department' with one dropdown per department and a Save button.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>Tier 3</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>Otherwise the Owner approves.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="16" t="inlineStr"/>
-      <c r="B23" s="17" t="inlineStr"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="18" t="inlineStr"/>
-      <c r="B24" s="19" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr"/>
+      <c r="B24" s="17" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="18" t="inlineStr"/>
+      <c r="B25" s="19" t="inlineStr">
         <is>
           <t>WHAT THE LIVE DATA SHOWS</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="16" t="inlineStr"/>
-      <c r="B25" s="17" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr"/>
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>Measured against the dev workspace on 2026-09-12, not assumed:</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="16" t="inlineStr">
-        <is>
-          <t>Members</t>
-        </is>
-      </c>
-      <c r="B26" s="17" t="inlineStr">
-        <is>
-          <t>12 team members in the workspace.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>Tier 1 used</t>
+          <t>Members</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>1 member has a Reporting Manager set (sai, finance).</t>
+          <t>12 team members in the workspace.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>Tier 2 used</t>
+          <t>Tier 1 used</t>
         </is>
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>0. The tenant leave_approvers mapping is EMPTY - every department reads 'Owner (default)'.</t>
+          <t>1 member has a Reporting Manager set (sai, finance).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>Tier 3 used</t>
+          <t>Tier 2 used</t>
         </is>
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>11 of 12 members fall through to the Owner, Rajesh Sharma.</t>
+          <t>0. The tenant leave_approvers mapping is EMPTY - every department reads 'Owner (default)'.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="16" t="inlineStr">
         <is>
+          <t>Tier 3 used</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>11 of 12 members fall through to the Owner, Rajesh Sharma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B30" s="17" t="inlineStr">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>The Settings screen currently decides leave for NOBODY. It configures a tier that no request reaches.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="16" t="inlineStr"/>
-      <c r="B31" s="17" t="inlineStr"/>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="18" t="inlineStr"/>
-      <c r="B32" s="19" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr"/>
+      <c r="B32" s="17" t="inlineStr"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="18" t="inlineStr"/>
+      <c r="B33" s="19" t="inlineStr">
         <is>
           <t>WHAT THE THREE PIECES ARE</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="16" t="inlineStr"/>
-      <c r="B33" s="17" t="inlineStr">
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="16" t="inlineStr"/>
+      <c r="B34" s="17" t="inlineStr">
         <is>
           <t>They are three layers of one feature. Removing one without the others leaves either a screen that cannot save or an endpoint nothing calls.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t>The gear</t>
-        </is>
-      </c>
-      <c r="B34" s="17" t="inlineStr">
-        <is>
-          <t>The small round icon beside the My Leave / Approvals tabs. It is the only way into the screen. pages/Leave.js:500-510.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="16" t="inlineStr">
         <is>
-          <t>The panel</t>
+          <t>The gear</t>
         </is>
       </c>
       <c r="B35" s="17" t="inlineStr">
         <is>
-          <t>'Leave Approvers by Department' - a dropdown per department plus a Save approvers button. pages/Leave.js:387-417.</t>
+          <t>The small round icon beside the My Leave / Approvals tabs. It is the only way into the screen. pages/Leave.js:500-510.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="16" t="inlineStr">
         <is>
+          <t>The panel</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>'Leave Approvers by Department' - a dropdown per department plus a Save approvers button. pages/Leave.js:387-417.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
           <t>The endpoint</t>
         </is>
       </c>
-      <c r="B36" s="17" t="inlineStr">
+      <c r="B37" s="17" t="inlineStr">
         <is>
           <t>PATCH /tenant/leave-approvers, which writes the leave_approvers field on the tenant record. routers/calendar.py:24.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="16" t="inlineStr"/>
-      <c r="B37" s="17" t="inlineStr"/>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="18" t="inlineStr"/>
-      <c r="B38" s="19" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr"/>
+      <c r="B38" s="17" t="inlineStr"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="18" t="inlineStr"/>
+      <c r="B39" s="19" t="inlineStr">
         <is>
           <t>OPTION A - DELETE TIER 2  (the current recommendation)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="16" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t>What changes</t>
         </is>
       </c>
-      <c r="B39" s="17" t="inlineStr">
+      <c r="B40" s="17" t="inlineStr">
         <is>
           <t>Remove the gear, the panel and the endpoint. Approval becomes: reporting manager, else owner.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="16" t="inlineStr">
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="16" t="inlineStr">
         <is>
           <t>Effect today</t>
         </is>
       </c>
-      <c r="B40" s="17" t="inlineStr">
+      <c r="B41" s="17" t="inlineStr">
         <is>
           <t>NONE. Every one of the 12 members resolves to exactly the same approver before and after, because nothing uses tier 2.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="45" customHeight="1">
-      <c r="A41" s="16" t="inlineStr">
+    <row r="42" ht="45" customHeight="1">
+      <c r="A42" s="16" t="inlineStr">
         <is>
           <t>Argument for</t>
         </is>
       </c>
-      <c r="B41" s="17" t="inlineStr">
+      <c r="B42" s="17" t="inlineStr">
         <is>
           <t>The approver is already chosen once, in Team, when the person is added. A second screen expressing the same decision in different words - and silently losing to the first one - mostly creates the chance for the two to disagree with the org chart.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="16" t="inlineStr"/>
-      <c r="B42" s="17" t="inlineStr"/>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="18" t="inlineStr"/>
-      <c r="B43" s="19" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr"/>
+      <c r="B43" s="17" t="inlineStr"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="18" t="inlineStr"/>
+      <c r="B44" s="19" t="inlineStr">
         <is>
           <t>OPTION B - KEEP TIER 2</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="16" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t>What it buys</t>
         </is>
       </c>
-      <c r="B44" s="17" t="inlineStr">
+      <c r="B45" s="17" t="inlineStr">
         <is>
           <t>One place to say 'all Sales leave goes to Priya' without making Priya anyone's reporting manager.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="16" t="inlineStr">
-        <is>
-          <t>Cost of A</t>
-        </is>
-      </c>
-      <c r="B45" s="17" t="inlineStr">
-        <is>
-          <t>To get that same outcome after deleting, Priya would have to be set as the reporting manager of each Sales person individually, in Team.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="16" t="inlineStr">
         <is>
+          <t>Cost of A</t>
+        </is>
+      </c>
+      <c r="B46" s="17" t="inlineStr">
+        <is>
+          <t>To get that same outcome after deleting, Priya would have to be set as the reporting manager of each Sales person individually, in Team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
           <t>If kept</t>
         </is>
       </c>
-      <c r="B46" s="17" t="inlineStr">
+      <c r="B47" s="17" t="inlineStr">
         <is>
           <t>Then the fix is not to move it into Settings but to make it visible - today it is hidden behind an unlabelled gear inside a work surface, which is why it has stayed empty.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="16" t="inlineStr"/>
-      <c r="B47" s="17" t="inlineStr"/>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="18" t="inlineStr"/>
-      <c r="B48" s="19" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr"/>
+      <c r="B48" s="17" t="inlineStr"/>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="18" t="inlineStr"/>
+      <c r="B49" s="19" t="inlineStr">
         <is>
           <t>THE ONE QUESTION THAT DECIDES IT</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="16" t="inlineStr"/>
-      <c r="B49" s="17" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr"/>
+      <c r="B50" s="17" t="inlineStr">
         <is>
           <t>Is 'who approves your leave' always the same person as 'who you report to'?</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="16" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="B50" s="17" t="inlineStr">
+      <c r="B51" s="17" t="inlineStr">
         <is>
           <t>They are always the same -&gt; Option A. Tier 2 is pure duplication.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B51" s="17" t="inlineStr">
-        <is>
-          <t>They can differ - for example a department lead signs off leave while people report to a project manager -&gt; Option B, and the work is to surface the screen properly rather than hide it.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="16" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>They can differ - for example a department lead signs off leave while people report to a project manager -&gt; Option B, and the work is to surface the screen properly rather than hide it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
           <t>Read</t>
         </is>
       </c>
-      <c r="B52" s="17" t="inlineStr">
+      <c r="B53" s="17" t="inlineStr">
         <is>
           <t>For an SME the answer is usually yes, which is why A is the standing recommendation - but this is a business call, not a technical one, which is why it is parked rather than filed as a defect.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="16" t="inlineStr"/>
-      <c r="B53" s="17" t="inlineStr"/>
-    </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="18" t="inlineStr"/>
-      <c r="B54" s="19" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="16" t="inlineStr"/>
+      <c r="B54" s="17" t="inlineStr"/>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="18" t="inlineStr"/>
+      <c r="B55" s="19" t="inlineStr">
         <is>
           <t>IF OPTION A IS CHOSEN, THE WORK IS</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B55" s="17" t="inlineStr">
-        <is>
-          <t>Delete the gear and the settings tab from pages/Leave.js (:500-510).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B56" s="17" t="inlineStr">
         <is>
-          <t>Delete the LeaveApproverConfig block from pages/Leave.js (:387-417).</t>
+          <t>Delete the gear and the settings tab from pages/Leave.js (:500-510).</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B57" s="17" t="inlineStr">
+        <is>
+          <t>Delete the LeaveApproverConfig block from pages/Leave.js (:387-417).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="16" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B57" s="17" t="inlineStr">
+      <c r="B58" s="17" t="inlineStr">
         <is>
           <t>Delete PATCH /tenant/leave-approvers from routers/calendar.py (:24) and the LeaveApproverMapInput model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="16" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B58" s="17" t="inlineStr">
-        <is>
-          <t>Drop the tier-2 lookup from _resolve_leave_approver in services/leave.py, leaving reporting manager then owner.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="16" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B59" s="17" t="inlineStr">
         <is>
-          <t>Leave the leave_approvers field on existing tenant records alone, or clear it in the migration - it is empty in practice either way.</t>
+          <t>Drop the tier-2 lookup from _resolve_leave_approver in services/leave.py, leaving reporting manager then owner.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="16" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B60" s="17" t="inlineStr">
         <is>
-          <t>Make sure Team makes the consequence visible: the Reporting Manager dropdown should say that this person also approves their leave, since after this change that is the only place the decision is made.</t>
+          <t>Leave the leave_approvers field on existing tenant records alone, or clear it in the migration - it is empty in practice either way.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="16" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B61" s="17" t="inlineStr">
+        <is>
+          <t>Make sure Team makes the consequence visible: the Reporting Manager dropdown should say that this person also approves their leave, since after this change that is the only place the decision is made.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="30" customHeight="1">
+      <c r="A62" s="16" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B61" s="17" t="inlineStr">
+      <c r="B62" s="17" t="inlineStr">
         <is>
           <t>This depends on ASK-6. If Leave moves into Team first, the gear disappears with it and steps 1 and 2 become part of that move rather than separate work.</t>
         </is>
@@ -31291,7 +31772,7 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>309 (218 pass, 89 fail, 0 blocked, 2 not run)</t>
+          <t>318 (227 pass, 89 fail, 0 blocked, 2 not run)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: ASK-28 TK-04 links always land; T-745..T-756; acceptance scripts kept green on the merged glass page
- Tracker: TK-04 progress (before/after, 23/23 on real data with writes
  blocked, run after rebasing onto 0eaa411 and afc6136) and coverage
  T-745..T-756.
- Scripts, for the merged page: settle() waits for real content (first cards
  arrive ~3.5 s after load); the person filter waits for the card count to
  move and hold after Clear (~1 s, traced); asked accepts ?view=mine; the
  approval-stage and New Task form scripts follow 0eaa411 (no More options
  row -> n/a; GlassSelect dropdowns driven by option testids).
- Re-runs on the merged page: links 23/23, asked 20/20, approvals 21/21,
  team 21/21, approval stage 19/19, person filter 33/33, New Task form 13/13
  + 3 n/a.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_UI_Bug_Report.xlsx
+++ b/docs/DecisionOS_UI_Bug_Report.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bug Log'!$A$1:$Q$89</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Coverage'!$A$1:$J$338</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Coverage'!$A$1:$J$350</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Verified Non-Issues'!$A$1:$E$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Action List'!$A$1:$K$118</definedName>
   </definedNames>
@@ -8116,7 +8116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J338"/>
+  <dimension ref="A1:J350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23042,7 +23042,7 @@
     <row r="301" ht="82" customHeight="1">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>T-708</t>
+          <t>T-745</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
@@ -23052,7 +23052,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - switcher</t>
+          <t>Task link - not in the list</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -23062,17 +23062,17 @@
       </c>
       <c r="E301" s="2" t="inlineStr">
         <is>
-          <t>Owner + Sales</t>
+          <t>Finance (manager of sai)</t>
         </is>
       </c>
       <c r="F301" s="2" t="inlineStr">
         <is>
-          <t>Asked by me sits in the view switcher for every role</t>
+          <t>A link to a task the person may open but that is not in their list opens its drawer</t>
         </is>
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>Views</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H301" s="4" t="inlineStr">
@@ -23082,7 +23082,7 @@
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>Owner: My Tasks | Asked by me | All Tasks | Workflows; Sales sees it too</t>
+          <t>sai task from Sunita My Tasks: drawer opens, no card in the list (was: nothing)</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr">
@@ -23094,7 +23094,7 @@
     <row r="302" ht="82" customHeight="1">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>T-709</t>
+          <t>T-746</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
@@ -23104,7 +23104,7 @@
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - the rule</t>
+          <t>Task link - finished task</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
@@ -23114,17 +23114,17 @@
       </c>
       <c r="E302" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Finance (manager)</t>
         </is>
       </c>
       <c r="F302" s="2" t="inlineStr">
         <is>
-          <t>Only tasks I created that are not mine to do</t>
+          <t>A link to a finished task opens it</t>
         </is>
       </c>
       <c r="G302" s="2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H302" s="4" t="inlineStr">
@@ -23134,7 +23134,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>GET /tasks?view=asked: 60 tasks, 0 break the rule; 53 open = 53 cards</t>
+          <t>Completed task of sai opens (was: nothing)</t>
         </is>
       </c>
       <c r="J302" s="2" t="inlineStr">
@@ -23146,7 +23146,7 @@
     <row r="303" ht="82" customHeight="1">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>T-710</t>
+          <t>T-747</t>
         </is>
       </c>
       <c r="B303" s="2" t="inlineStr">
@@ -23156,7 +23156,7 @@
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - filters</t>
+          <t>Task link - while on My Work</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
@@ -23166,17 +23166,17 @@
       </c>
       <c r="E303" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Finance (manager)</t>
         </is>
       </c>
       <c r="F303" s="2" t="inlineStr">
         <is>
-          <t>Person (without Me) and Status narrow the list with matching counts</t>
+          <t>A task link followed while My Work is already open opens the task</t>
         </is>
       </c>
       <c r="G303" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H303" s="4" t="inlineStr">
@@ -23186,7 +23186,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>Person -&gt; 9 cards = API 9; Status Overdue 13 = 13 cards</t>
+          <t>In-app navigation to ?task= opens the drawer (was: nothing)</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -23198,7 +23198,7 @@
     <row r="304" ht="82" customHeight="1">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>T-711</t>
+          <t>T-748</t>
         </is>
       </c>
       <c r="B304" s="2" t="inlineStr">
@@ -23208,7 +23208,7 @@
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - URL and default</t>
+          <t>Task link - older focus form</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
@@ -23218,12 +23218,12 @@
       </c>
       <c r="E304" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Finance (manager)</t>
         </is>
       </c>
       <c r="F304" s="2" t="inlineStr">
         <is>
-          <t>View survives refresh, other views clear it, plain /my-work does not reopen on it</t>
+          <t>?focus=task:&lt;id&gt; links from the Brief and phone screens open the task</t>
         </is>
       </c>
       <c r="G304" s="2" t="inlineStr">
@@ -23238,7 +23238,7 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>?view=asked kept on reload; My Tasks clears it; not saved as default</t>
+          <t>Drawer opens; link cleared on close (was: ignored)</t>
         </is>
       </c>
       <c r="J304" s="2" t="inlineStr">
@@ -23250,7 +23250,7 @@
     <row r="305" ht="82" customHeight="1">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>T-712</t>
+          <t>T-749</t>
         </is>
       </c>
       <c r="B305" s="2" t="inlineStr">
@@ -23260,7 +23260,7 @@
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - AI priority</t>
+          <t>Task link - closing</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
@@ -23270,17 +23270,17 @@
       </c>
       <c r="E305" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Finance (manager)</t>
         </is>
       </c>
       <c r="F305" s="2" t="inlineStr">
         <is>
-          <t>AI priority is not offered on other people's work</t>
+          <t>Closing the drawer takes the link out of the address; refresh keeps it closed</t>
         </is>
       </c>
       <c r="G305" s="2" t="inlineStr">
         <is>
-          <t>Views</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H305" s="4" t="inlineStr">
@@ -23290,7 +23290,7 @@
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>AI toggle hidden on Asked by me</t>
+          <t>url {} after Escape and after reload</t>
         </is>
       </c>
       <c r="J305" s="2" t="inlineStr">
@@ -23302,7 +23302,7 @@
     <row r="306" ht="82" customHeight="1">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>T-713</t>
+          <t>T-750</t>
         </is>
       </c>
       <c r="B306" s="2" t="inlineStr">
@@ -23312,7 +23312,7 @@
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - empty</t>
+          <t>Task link - inside My team</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
@@ -23322,17 +23322,17 @@
       </c>
       <c r="E306" s="2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance (manager)</t>
         </is>
       </c>
       <c r="F306" s="2" t="inlineStr">
         <is>
-          <t>Someone who has asked for nothing sees an explanation, not the decisions text</t>
+          <t>When the task is in the list, the list card opens (no stand-in)</t>
         </is>
       </c>
       <c r="G306" s="2" t="inlineStr">
         <is>
-          <t>Empty state</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H306" s="4" t="inlineStr">
@@ -23342,7 +23342,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>'Nothing you've asked for is open - Tasks you create for other people show up here, with their live status.'</t>
+          <t>?view=team&amp;task=&lt;id&gt;: My team pressed, card drawer</t>
         </is>
       </c>
       <c r="J306" s="2" t="inlineStr">
@@ -23354,7 +23354,7 @@
     <row r="307" ht="82" customHeight="1">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>T-714</t>
+          <t>T-751</t>
         </is>
       </c>
       <c r="B307" s="2" t="inlineStr">
@@ -23364,7 +23364,7 @@
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - requester note</t>
+          <t>Task link - missing task</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
@@ -23374,17 +23374,17 @@
       </c>
       <c r="E307" s="2" t="inlineStr">
         <is>
-          <t>Sales (mocked list)</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F307" s="2" t="inlineStr">
         <is>
-          <t>The person who asked can leave a note but not hand off or escalate</t>
+          <t>A link to a task that no longer exists says so and can be dismissed</t>
         </is>
       </c>
       <c r="G307" s="2" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Errors</t>
         </is>
       </c>
       <c r="H307" s="4" t="inlineStr">
@@ -23394,7 +23394,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>Update form offers only Log note; server allows a note from the creator (unit-tested)</t>
+          <t>This task no longer exists + Dismiss clears the link (was: Access restricted)</t>
         </is>
       </c>
       <c r="J307" s="2" t="inlineStr">
@@ -23406,7 +23406,7 @@
     <row r="308" ht="82" customHeight="1">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>T-716</t>
+          <t>T-752</t>
         </is>
       </c>
       <c r="B308" s="2" t="inlineStr">
@@ -23416,7 +23416,7 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - requester drawer</t>
+          <t>Task link - no access</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -23426,12 +23426,12 @@
       </c>
       <c r="E308" s="2" t="inlineStr">
         <is>
-          <t>Sales (mocked list)</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="F308" s="2" t="inlineStr">
         <is>
-          <t>The person who asked sees progress and a note box, not the doer's status, plan, complete or attach controls</t>
+          <t>A link to a task the person may not open says Access restricted and opens nothing</t>
         </is>
       </c>
       <c r="G308" s="2" t="inlineStr">
@@ -23446,7 +23446,7 @@
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>Status, Complete, Attach, Reopen hidden; hint 'You asked for this task, so &lt;doer&gt; does the work. Leave a note below to follow up.'</t>
+          <t>API 403; banner reason denied; no drawer</t>
         </is>
       </c>
       <c r="J308" s="2" t="inlineStr">
@@ -23458,7 +23458,7 @@
     <row r="309" ht="82" customHeight="1">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>T-715</t>
+          <t>T-753</t>
         </is>
       </c>
       <c r="B309" s="2" t="inlineStr">
@@ -23468,12 +23468,12 @@
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - phone link</t>
+          <t>View survives refresh</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
         <is>
-          <t>Mobile 390x844</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E309" s="2" t="inlineStr">
@@ -23483,7 +23483,7 @@
       </c>
       <c r="F309" s="2" t="inlineStr">
         <is>
-          <t>A link to Asked by me on a phone shows that list, not My Tasks</t>
+          <t>The chosen view is in the address and survives refresh</t>
         </is>
       </c>
       <c r="G309" s="2" t="inlineStr">
@@ -23498,7 +23498,7 @@
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>53 / 53 cards; My Tasks not pressed; no overflow</t>
+          <t>Workflows: ?view=workflows, still Workflows after reload (was: My Tasks)</t>
         </is>
       </c>
       <c r="J309" s="2" t="inlineStr">
@@ -23510,7 +23510,7 @@
     <row r="310" ht="82" customHeight="1">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>T-700</t>
+          <t>T-754</t>
         </is>
       </c>
       <c r="B310" s="2" t="inlineStr">
@@ -23520,7 +23520,7 @@
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>New Task - quick part</t>
+          <t>Back and Forward</t>
         </is>
       </c>
       <c r="D310" s="2" t="inlineStr">
@@ -23535,12 +23535,12 @@
       </c>
       <c r="F310" s="2" t="inlineStr">
         <is>
-          <t>Only title, Department, Assign to and Due show before More options</t>
+          <t>Back and Forward move between the views visited</t>
         </is>
       </c>
       <c r="G310" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H310" s="4" t="inlineStr">
@@ -23550,19 +23550,19 @@
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>Visible: Task title, Department, Assign to, Due; Operational category and Supporting employee gone</t>
+          <t>My Tasks &gt; Asked &gt; All; Back Asked, Back My Tasks, Forward Asked (was: Back left the page)</t>
         </is>
       </c>
       <c r="J310" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="311" ht="82" customHeight="1">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>T-701</t>
+          <t>T-755</t>
         </is>
       </c>
       <c r="B311" s="2" t="inlineStr">
@@ -23572,7 +23572,7 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>New Task - More options</t>
+          <t>View links</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
@@ -23587,12 +23587,12 @@
       </c>
       <c r="F311" s="2" t="inlineStr">
         <is>
-          <t>Priority, helpers, description, time, result, approval, proof, files wait under More; closed section says how many are set</t>
+          <t>?view=all and ?view=approvals land on those views</t>
         </is>
       </c>
       <c r="G311" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H311" s="4" t="inlineStr">
@@ -23602,19 +23602,19 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>Collapsed by default; '5 set' after choosing priority, helper, time, approval, proof</t>
+          <t>All Tasks pressed; Approvals hub shown</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="312" ht="82" customHeight="1">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>T-702</t>
+          <t>T-756</t>
         </is>
       </c>
       <c r="B312" s="2" t="inlineStr">
@@ -23624,27 +23624,27 @@
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>New Task - title required</t>
+          <t>Task link - phone</t>
         </is>
       </c>
       <c r="D312" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Mobile 390x844</t>
         </is>
       </c>
       <c r="E312" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Finance (manager)</t>
         </is>
       </c>
       <c r="F312" s="2" t="inlineStr">
         <is>
-          <t>Create without a title shows an inline error and sends nothing</t>
+          <t>A task link not in the list opens on a phone</t>
         </is>
       </c>
       <c r="G312" s="2" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H312" s="4" t="inlineStr">
@@ -23654,19 +23654,19 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>'Give the task a title' under the field; clears on typing; no request</t>
+          <t>Drawer opens; no overflow</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="313" ht="82" customHeight="1">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>T-703</t>
+          <t>T-708</t>
         </is>
       </c>
       <c r="B313" s="2" t="inlineStr">
@@ -23676,7 +23676,7 @@
       </c>
       <c r="C313" s="2" t="inlineStr">
         <is>
-          <t>New Task - Assign to</t>
+          <t>Asked by me - switcher</t>
         </is>
       </c>
       <c r="D313" s="2" t="inlineStr">
@@ -23686,17 +23686,17 @@
       </c>
       <c r="E313" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Owner + Sales</t>
         </is>
       </c>
       <c r="F313" s="2" t="inlineStr">
         <is>
-          <t>One control lists people and teams; a team explains where it goes</t>
+          <t>Asked by me sits in the view switcher for every role</t>
         </is>
       </c>
       <c r="G313" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H313" s="4" t="inlineStr">
@@ -23706,19 +23706,19 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>12 people + Sales, Production, Finance teams; hint 'Goes to whoever in Sales has the least open work'</t>
+          <t>Owner: My Tasks | Asked by me | All Tasks | Workflows; Sales sees it too</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="314" ht="82" customHeight="1">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>T-704</t>
+          <t>T-709</t>
         </is>
       </c>
       <c r="B314" s="2" t="inlineStr">
@@ -23728,7 +23728,7 @@
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>New Task - due presets</t>
+          <t>Asked by me - the rule</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
@@ -23743,12 +23743,12 @@
       </c>
       <c r="F314" s="2" t="inlineStr">
         <is>
-          <t>Today / Tomorrow / In a week set the date without a picker</t>
+          <t>Only tasks I created that are not mine to do</t>
         </is>
       </c>
       <c r="G314" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H314" s="4" t="inlineStr">
@@ -23758,19 +23758,19 @@
       </c>
       <c r="I314" s="2" t="inlineStr">
         <is>
-          <t>Tomorrow -&gt; 'Due Tue 15 Sept'; Today -&gt; due_date = today, no time</t>
+          <t>GET /tasks?view=asked: 60 tasks, 0 break the rule; 53 open = 53 cards</t>
         </is>
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="315" ht="82" customHeight="1">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>T-705</t>
+          <t>T-710</t>
         </is>
       </c>
       <c r="B315" s="2" t="inlineStr">
@@ -23780,7 +23780,7 @@
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>New Task - payload (person)</t>
+          <t>Asked by me - filters</t>
         </is>
       </c>
       <c r="D315" s="2" t="inlineStr">
@@ -23795,12 +23795,12 @@
       </c>
       <c r="F315" s="2" t="inlineStr">
         <is>
-          <t>The form sends exactly what was chosen and nothing removed</t>
+          <t>Person (without Me) and Status narrow the list with matching counts</t>
         </is>
       </c>
       <c r="G315" s="2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H315" s="4" t="inlineStr">
@@ -23810,19 +23810,19 @@
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>task_type sales, lead + 1 helper, high, tomorrow 16:30, approval (anyone), proof; no op_category / support_id</t>
+          <t>Person -&gt; 9 cards = API 9; Status Overdue 13 = 13 cards</t>
         </is>
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="316" ht="82" customHeight="1">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>T-706</t>
+          <t>T-711</t>
         </is>
       </c>
       <c r="B316" s="2" t="inlineStr">
@@ -23832,7 +23832,7 @@
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>New Task - payload (team)</t>
+          <t>Asked by me - URL and default</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr">
@@ -23847,12 +23847,12 @@
       </c>
       <c r="F316" s="2" t="inlineStr">
         <is>
-          <t>A team task sends the role, no person and no helpers</t>
+          <t>View survives refresh, other views clear it, plain /my-work does not reopen on it</t>
         </is>
       </c>
       <c r="G316" s="2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H316" s="4" t="inlineStr">
@@ -23862,19 +23862,19 @@
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>assignee_role sales, assignee_id null, co_assignee_ids [], due today</t>
+          <t>?view=asked kept on reload; My Tasks clears it; not saved as default</t>
         </is>
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="317" ht="82" customHeight="1">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>T-707</t>
+          <t>T-712</t>
         </is>
       </c>
       <c r="B317" s="2" t="inlineStr">
@@ -23884,7 +23884,7 @@
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>New Task - after create</t>
+          <t>Asked by me - AI priority</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
@@ -23899,12 +23899,12 @@
       </c>
       <c r="F317" s="2" t="inlineStr">
         <is>
-          <t>Dialog closes, reopens empty with More collapsed, My Work still renders</t>
+          <t>AI priority is not offered on other people's work</t>
         </is>
       </c>
       <c r="G317" s="2" t="inlineStr">
         <is>
-          <t>Flow</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H317" s="4" t="inlineStr">
@@ -23914,19 +23914,19 @@
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>Closed; reopened clean; 25 cards; no page errors</t>
+          <t>AI toggle hidden on Asked by me</t>
         </is>
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="318" ht="82" customHeight="1">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>T-690</t>
+          <t>T-713</t>
         </is>
       </c>
       <c r="B318" s="2" t="inlineStr">
@@ -23936,7 +23936,7 @@
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - filter row</t>
+          <t>Asked by me - empty</t>
         </is>
       </c>
       <c r="D318" s="2" t="inlineStr">
@@ -23946,17 +23946,17 @@
       </c>
       <c r="E318" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F318" s="2" t="inlineStr">
         <is>
-          <t>All Tasks shows Department, Person, Status; My Tasks hides Person</t>
+          <t>Someone who has asked for nothing sees an explanation, not the decisions text</t>
         </is>
       </c>
       <c r="G318" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Empty state</t>
         </is>
       </c>
       <c r="H318" s="4" t="inlineStr">
@@ -23966,19 +23966,19 @@
       </c>
       <c r="I318" s="2" t="inlineStr">
         <is>
-          <t>Row shows all three with counts (131); My Tasks shows two (25)</t>
+          <t>'Nothing you've asked for is open - Tasks you create for other people show up here, with their live status.'</t>
         </is>
       </c>
       <c r="J318" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="319" ht="82" customHeight="1">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>T-691</t>
+          <t>T-714</t>
         </is>
       </c>
       <c r="B319" s="2" t="inlineStr">
@@ -23988,7 +23988,7 @@
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - Person filter</t>
+          <t>Asked by me - requester note</t>
         </is>
       </c>
       <c r="D319" s="2" t="inlineStr">
@@ -23998,17 +23998,17 @@
       </c>
       <c r="E319" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales (mocked list)</t>
         </is>
       </c>
       <c r="F319" s="2" t="inlineStr">
         <is>
-          <t>Picking a person shows only their tasks, count matches the API</t>
+          <t>The person who asked can leave a note but not hand off or escalate</t>
         </is>
       </c>
       <c r="G319" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="H319" s="4" t="inlineStr">
@@ -24018,19 +24018,19 @@
       </c>
       <c r="I319" s="2" t="inlineStr">
         <is>
-          <t>Priya Nair: 29 cards = trigger 29 = API 29; URL ?person=; name line hidden on cards; menu has Me, people busiest first with role, Unassigned (6), Production team (5); no duplicate rows</t>
+          <t>Update form offers only Log note; server allows a note from the creator (unit-tested)</t>
         </is>
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="320" ht="82" customHeight="1">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>T-692</t>
+          <t>T-716</t>
         </is>
       </c>
       <c r="B320" s="2" t="inlineStr">
@@ -24040,7 +24040,7 @@
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - Status options</t>
+          <t>Asked by me - requester drawer</t>
         </is>
       </c>
       <c r="D320" s="2" t="inlineStr">
@@ -24050,17 +24050,17 @@
       </c>
       <c r="E320" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales (mocked list)</t>
         </is>
       </c>
       <c r="F320" s="2" t="inlineStr">
         <is>
-          <t>Pending Approval, Overdue and Completed are filterable with correct counts</t>
+          <t>The person who asked sees progress and a note box, not the doer's status, plan, complete or attach controls</t>
         </is>
       </c>
       <c r="G320" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="H320" s="4" t="inlineStr">
@@ -24070,19 +24070,19 @@
       </c>
       <c r="I320" s="2" t="inlineStr">
         <is>
-          <t>Pending Approval 40, Overdue 68, Completed 17, Not Started 78 - all equal the API</t>
+          <t>Status, Complete, Attach, Reopen hidden; hint 'You asked for this task, so &lt;doer&gt; does the work. Leave a note below to follow up.'</t>
         </is>
       </c>
       <c r="J320" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="321" ht="82" customHeight="1">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>T-693</t>
+          <t>T-715</t>
         </is>
       </c>
       <c r="B321" s="2" t="inlineStr">
@@ -24092,12 +24092,12 @@
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - Priority filter removed</t>
+          <t>Asked by me - phone link</t>
         </is>
       </c>
       <c r="D321" s="2" t="inlineStr">
         <is>
-          <t>Desktop + Mobile</t>
+          <t>Mobile 390x844</t>
         </is>
       </c>
       <c r="E321" s="2" t="inlineStr">
@@ -24107,12 +24107,12 @@
       </c>
       <c r="F321" s="2" t="inlineStr">
         <is>
-          <t>No Priority filter (founder call 2026-09-13); an old ?priority= link does not narrow the list</t>
+          <t>A link to Asked by me on a phone shows that list, not My Tasks</t>
         </is>
       </c>
       <c r="G321" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H321" s="4" t="inlineStr">
@@ -24122,19 +24122,19 @@
       </c>
       <c r="I321" s="2" t="inlineStr">
         <is>
-          <t>No Priority dropdown on desktop, no Priority chips in the phone sheet; ?person=Priya&amp;status=overdue&amp;priority=high shows the same 20 as without it</t>
+          <t>53 / 53 cards; My Tasks not pressed; no overflow</t>
         </is>
       </c>
       <c r="J321" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="322" ht="82" customHeight="1">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>T-694</t>
+          <t>T-700</t>
         </is>
       </c>
       <c r="B322" s="2" t="inlineStr">
@@ -24144,7 +24144,7 @@
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - combined counts</t>
+          <t>New Task - quick part</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
@@ -24159,12 +24159,12 @@
       </c>
       <c r="F322" s="2" t="inlineStr">
         <is>
-          <t>Each menu's counts reflect the other active filters</t>
+          <t>Only title, Department, Assign to and Due show before More options</t>
         </is>
       </c>
       <c r="G322" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H322" s="4" t="inlineStr">
@@ -24174,19 +24174,19 @@
       </c>
       <c r="I322" s="2" t="inlineStr">
         <is>
-          <t>With Priya + Overdue, Department 'All' reads 20 = cards = API</t>
+          <t>Visible: Task title, Department, Assign to, Due; Operational category and Supporting employee gone</t>
         </is>
       </c>
       <c r="J322" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="323" ht="82" customHeight="1">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>T-695</t>
+          <t>T-701</t>
         </is>
       </c>
       <c r="B323" s="2" t="inlineStr">
@@ -24196,7 +24196,7 @@
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - refresh, Clear, no match</t>
+          <t>New Task - More options</t>
         </is>
       </c>
       <c r="D323" s="2" t="inlineStr">
@@ -24211,12 +24211,12 @@
       </c>
       <c r="F323" s="2" t="inlineStr">
         <is>
-          <t>Filters survive refresh; Clear resets; empty result explains itself</t>
+          <t>Priority, helpers, description, time, result, approval, proof, files wait under More; closed section says how many are set</t>
         </is>
       </c>
       <c r="G323" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H323" s="4" t="inlineStr">
@@ -24226,19 +24226,19 @@
       </c>
       <c r="I323" s="2" t="inlineStr">
         <is>
-          <t>Reload keeps 20 cards + URL; Clear -&gt; 131, URL clean; Priya x Under Review -&gt; 'No tasks match these filters' with Clear</t>
+          <t>Collapsed by default; '5 set' after choosing priority, helper, time, approval, proof</t>
         </is>
       </c>
       <c r="J323" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="324" ht="82" customHeight="1">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>T-696</t>
+          <t>T-702</t>
         </is>
       </c>
       <c r="B324" s="2" t="inlineStr">
@@ -24248,7 +24248,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - person search, links</t>
+          <t>New Task - title required</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -24263,12 +24263,12 @@
       </c>
       <c r="F324" s="2" t="inlineStr">
         <is>
-          <t>Search narrows the menu; Desk overdue link and task deep link behave</t>
+          <t>Create without a title shows an inline error and sends nothing</t>
         </is>
       </c>
       <c r="G324" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="H324" s="4" t="inlineStr">
@@ -24278,19 +24278,19 @@
       </c>
       <c r="I324" s="2" t="inlineStr">
         <is>
-          <t>'pri' -&gt; Priya Nair only; ?filter=overdue -&gt; Status: Overdue 68; ?task= with filters set clears them and shows the card</t>
+          <t>'Give the task a title' under the field; clears on typing; no request</t>
         </is>
       </c>
       <c r="J324" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="325" ht="82" customHeight="1">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>T-697</t>
+          <t>T-703</t>
         </is>
       </c>
       <c r="B325" s="2" t="inlineStr">
@@ -24300,12 +24300,12 @@
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>Phone - filter sheet</t>
+          <t>New Task - Assign to</t>
         </is>
       </c>
       <c r="D325" s="2" t="inlineStr">
         <is>
-          <t>Mobile 390x844</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E325" s="2" t="inlineStr">
@@ -24315,12 +24315,12 @@
       </c>
       <c r="F325" s="2" t="inlineStr">
         <is>
-          <t>The phone reaches every filter and sees what is active</t>
+          <t>One control lists people and teams; a team explains where it goes</t>
         </is>
       </c>
       <c r="G325" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H325" s="4" t="inlineStr">
@@ -24330,19 +24330,19 @@
       </c>
       <c r="I325" s="2" t="inlineStr">
         <is>
-          <t>Sheet with Department / Person / Status; Priya + Overdue -&gt; 'Show 20 tasks' = 20 cards; caption 'Showing Priya Nair - Overdue' with Clear; buttons 44px, reachable; no overflow</t>
+          <t>12 people + Sales, Production, Finance teams; hint 'Goes to whoever in Sales has the least open work'</t>
         </is>
       </c>
       <c r="J325" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="326" ht="82" customHeight="1">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>T-698</t>
+          <t>T-704</t>
         </is>
       </c>
       <c r="B326" s="2" t="inlineStr">
@@ -24352,12 +24352,12 @@
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>Phone - My Tasks / Status without AI</t>
+          <t>New Task - due presets</t>
         </is>
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>Mobile 390x844</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E326" s="2" t="inlineStr">
@@ -24367,12 +24367,12 @@
       </c>
       <c r="F326" s="2" t="inlineStr">
         <is>
-          <t>Person hidden on My Tasks; a Status filter is visible even with AI priority off</t>
+          <t>Today / Tomorrow / In a week set the date without a picker</t>
         </is>
       </c>
       <c r="G326" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H326" s="4" t="inlineStr">
@@ -24382,19 +24382,19 @@
       </c>
       <c r="I326" s="2" t="inlineStr">
         <is>
-          <t>Sheet on My Tasks has no Person; ?status=overdue shows the caption</t>
+          <t>Tomorrow -&gt; 'Due Tue 15 Sept'; Today -&gt; due_date = today, no time</t>
         </is>
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="327" ht="82" customHeight="1">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>T-699</t>
+          <t>T-705</t>
         </is>
       </c>
       <c r="B327" s="2" t="inlineStr">
@@ -24404,27 +24404,27 @@
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>Sales - no Person filter</t>
+          <t>New Task - payload (person)</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
         <is>
-          <t>Desktop + Mobile</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E327" s="2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F327" s="2" t="inlineStr">
         <is>
-          <t>Roles without All Tasks never see Person; ?person= is ignored</t>
+          <t>The form sends exactly what was chosen and nothing removed</t>
         </is>
       </c>
       <c r="G327" s="2" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H327" s="4" t="inlineStr">
@@ -24434,29 +24434,29 @@
       </c>
       <c r="I327" s="2" t="inlineStr">
         <is>
-          <t>Desktop row has no Person; phone sheet has no Person; ?person=anyone ignored, own 29 cards</t>
+          <t>task_type sales, lead + 1 helper, high, tomorrow 16:30, approval (anyone), proof; no op_category / support_id</t>
         </is>
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="328" ht="82" customHeight="1">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>T-680</t>
+          <t>T-706</t>
         </is>
       </c>
       <c r="B328" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>LIVE - receivables question</t>
+          <t>New Task - payload (team)</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr">
@@ -24471,44 +24471,44 @@
       </c>
       <c r="F328" s="2" t="inlineStr">
         <is>
-          <t>Dex answers how much customers owe with the ledger's figure</t>
+          <t>A team task sends the role, no person and no helpers</t>
         </is>
       </c>
       <c r="G328" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H328" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="H328" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I328" s="2" t="inlineStr">
         <is>
-          <t>Said zero invoices / Rs 0 outstanding; ledger has Rs 7,49,000 outstanding (17.0s)</t>
+          <t>assignee_role sales, assignee_id null, co_assignee_ids [], due today</t>
         </is>
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>DX-01</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="329" ht="82" customHeight="1">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>T-681</t>
+          <t>T-707</t>
         </is>
       </c>
       <c r="B329" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>LIVE - what needs my attention</t>
+          <t>New Task - after create</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr">
@@ -24523,44 +24523,44 @@
       </c>
       <c r="F329" s="2" t="inlineStr">
         <is>
-          <t>Dex surfaces the overdue work and pending decisions</t>
+          <t>Dialog closes, reopens empty with More collapsed, My Work still renders</t>
         </is>
       </c>
       <c r="G329" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H329" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="H329" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I329" s="2" t="inlineStr">
         <is>
-          <t>Said nothing open or overdue; owner has 24 open / 6 overdue (24.1s)</t>
+          <t>Closed; reopened clean; 25 cards; no page errors</t>
         </is>
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>DX-02</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="330" ht="82" customHeight="1">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>T-682</t>
+          <t>T-690</t>
         </is>
       </c>
       <c r="B330" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>LIVE - global search hand-off</t>
+          <t>All Tasks - filter row</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
@@ -24575,12 +24575,12 @@
       </c>
       <c r="F330" s="2" t="inlineStr">
         <is>
-          <t>A question from global search is answered on arrival</t>
+          <t>All Tasks shows Department, Person, Status; My Tasks hides Person</t>
         </is>
       </c>
       <c r="G330" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H330" s="4" t="inlineStr">
@@ -24590,25 +24590,29 @@
       </c>
       <c r="I330" s="2" t="inlineStr">
         <is>
-          <t>'Which tasks are overdue?' answered on /brain?q= with a task list (17.5s)</t>
-        </is>
-      </c>
-      <c r="J330" s="2" t="inlineStr"/>
+          <t>Row shows all three with counts (131); My Tasks shows two (25)</t>
+        </is>
+      </c>
+      <c r="J330" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="331" ht="82" customHeight="1">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>T-683</t>
+          <t>T-691</t>
         </is>
       </c>
       <c r="B331" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>LIVE - coach refresh</t>
+          <t>All Tasks - Person filter</t>
         </is>
       </c>
       <c r="D331" s="2" t="inlineStr">
@@ -24623,12 +24627,12 @@
       </c>
       <c r="F331" s="2" t="inlineStr">
         <is>
-          <t>Generate coaching produces a review grounded in the stats</t>
+          <t>Picking a person shows only their tasks, count matches the API</t>
         </is>
       </c>
       <c r="G331" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H331" s="4" t="inlineStr">
@@ -24638,25 +24642,29 @@
       </c>
       <c r="I331" s="2" t="inlineStr">
         <is>
-          <t>TEST_member: 'AI coach updated' in 8.7s; strengths / improvements reference the 13 actionable tasks and plan use</t>
-        </is>
-      </c>
-      <c r="J331" s="2" t="inlineStr"/>
+          <t>Priya Nair: 29 cards = trigger 29 = API 29; URL ?person=; name line hidden on cards; menu has Me, people busiest first with role, Unassigned (6), Production team (5); no duplicate rows</t>
+        </is>
+      </c>
+      <c r="J331" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="332" ht="82" customHeight="1">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>T-684</t>
+          <t>T-692</t>
         </is>
       </c>
       <c r="B332" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Score with AI</t>
+          <t>All Tasks - Status options</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
@@ -24671,12 +24679,12 @@
       </c>
       <c r="F332" s="2" t="inlineStr">
         <is>
-          <t>Rescore updates the relationship card sensibly</t>
+          <t>Pending Approval, Overdue and Completed are filterable with correct counts</t>
         </is>
       </c>
       <c r="G332" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H332" s="4" t="inlineStr">
@@ -24686,30 +24694,34 @@
       </c>
       <c r="I332" s="2" t="inlineStr">
         <is>
-          <t>E2E Test Co: 'Relationship scored by AI' in 7.8s; Relationship 12 / Risk 78, reason cites 4 open complaints and no billing - matches the record</t>
-        </is>
-      </c>
-      <c r="J332" s="2" t="inlineStr"/>
+          <t>Pending Approval 40, Overdue 68, Completed 17, Not Started 78 - all equal the API</t>
+        </is>
+      </c>
+      <c r="J332" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="333" ht="82" customHeight="1">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>T-685</t>
+          <t>T-693</t>
         </is>
       </c>
       <c r="B333" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>LIVE - AI analysis refresh</t>
+          <t>All Tasks - Priority filter removed</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Desktop + Mobile</t>
         </is>
       </c>
       <c r="E333" s="2" t="inlineStr">
@@ -24719,12 +24731,12 @@
       </c>
       <c r="F333" s="2" t="inlineStr">
         <is>
-          <t>Refresh produces an analysis grounded in the ledger</t>
+          <t>No Priority filter (founder call 2026-09-13); an old ?priority= link does not narrow the list</t>
         </is>
       </c>
       <c r="G333" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H333" s="4" t="inlineStr">
@@ -24734,25 +24746,29 @@
       </c>
       <c r="I333" s="2" t="inlineStr">
         <is>
-          <t>'Analysis refreshed' in 20.6s; Rs 6.6L outstanding (ledger 6,55,466), Surat Spinners Rs 4.8L unpaid 33 days (correct), duplicates flagged</t>
-        </is>
-      </c>
-      <c r="J333" s="2" t="inlineStr"/>
+          <t>No Priority dropdown on desktop, no Priority chips in the phone sheet; ?person=Priya&amp;status=overdue&amp;priority=high shows the same 20 as without it</t>
+        </is>
+      </c>
+      <c r="J333" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="334" ht="82" customHeight="1">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>T-686</t>
+          <t>T-694</t>
         </is>
       </c>
       <c r="B334" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Ask AI</t>
+          <t>All Tasks - combined counts</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
@@ -24767,49 +24783,49 @@
       </c>
       <c r="F334" s="2" t="inlineStr">
         <is>
-          <t>The answer is correct and readable</t>
+          <t>Each menu's counts reflect the other active filters</t>
         </is>
       </c>
       <c r="G334" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H334" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H334" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I334" s="2" t="inlineStr">
         <is>
-          <t>Correct (Surat Spinners Rs 4,80,000, 7.3s) but literal ** markdown shown</t>
+          <t>With Priya + Overdue, Department 'All' reads 20 = cards = API</t>
         </is>
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>FN-12</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="335" ht="82" customHeight="1">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>T-688</t>
+          <t>T-695</t>
         </is>
       </c>
       <c r="B335" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>LIVE - owner on a phone</t>
+          <t>All Tasks - refresh, Clear, no match</t>
         </is>
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>Mobile 390x844</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E335" s="2" t="inlineStr">
@@ -24819,12 +24835,12 @@
       </c>
       <c r="F335" s="2" t="inlineStr">
         <is>
-          <t>Dex answers on mobile and the answer fits the screen</t>
+          <t>Filters survive refresh; Clear resets; empty result explains itself</t>
         </is>
       </c>
       <c r="G335" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H335" s="4" t="inlineStr">
@@ -24834,25 +24850,29 @@
       </c>
       <c r="I335" s="2" t="inlineStr">
         <is>
-          <t>'53 decisions pending approval across 77' - correct; 17.6s; no overflow</t>
-        </is>
-      </c>
-      <c r="J335" s="2" t="inlineStr"/>
+          <t>Reload keeps 20 cards + URL; Clear -&gt; 131, URL clean; Priya x Under Review -&gt; 'No tasks match these filters' with Clear</t>
+        </is>
+      </c>
+      <c r="J335" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="336" ht="82" customHeight="1">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>T-689</t>
+          <t>T-696</t>
         </is>
       </c>
       <c r="B336" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Sales asks money questions</t>
+          <t>All Tasks - person search, links</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr">
@@ -24862,17 +24882,17 @@
       </c>
       <c r="E336" s="2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F336" s="2" t="inlineStr">
         <is>
-          <t>Dex refuses finance answers to a role the finance API refuses</t>
+          <t>Search narrows the menu; Desk overdue link and task deep link behave</t>
         </is>
       </c>
       <c r="G336" s="2" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H336" s="4" t="inlineStr">
@@ -24882,30 +24902,34 @@
       </c>
       <c r="I336" s="2" t="inlineStr">
         <is>
-          <t>Receivables and profit questions both refused ('You do not have permission to access financial...'), 5.8s / 1.6s; no figures leaked</t>
-        </is>
-      </c>
-      <c r="J336" s="2" t="inlineStr"/>
+          <t>'pri' -&gt; Priya Nair only; ?filter=overdue -&gt; Status: Overdue 68; ?task= with filters set clears them and shows the card</t>
+        </is>
+      </c>
+      <c r="J336" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="337" ht="82" customHeight="1">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>T-687</t>
+          <t>T-697</t>
         </is>
       </c>
       <c r="B337" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>LIVE - bill extraction</t>
+          <t>Phone - filter sheet</t>
         </is>
       </c>
       <c r="D337" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Mobile 390x844</t>
         </is>
       </c>
       <c r="E337" s="2" t="inlineStr">
@@ -24915,80 +24939,680 @@
       </c>
       <c r="F337" s="2" t="inlineStr">
         <is>
-          <t>A GST bill is extracted into a reviewable record with the key fields</t>
+          <t>The phone reaches every filter and sees what is active</t>
         </is>
       </c>
       <c r="G337" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H337" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H337" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I337" s="2" t="inlineStr">
         <is>
-          <t>Party, number, amount, due date, category and follow-up correct (31.9s, 92%); date, GSTIN, items missing; no stale-date warning. Left in review, not filed</t>
+          <t>Sheet with Department / Person / Status; Priya + Overdue -&gt; 'Show 20 tasks' = 20 cards; caption 'Showing Priya Nair - Overdue' with Clear; buttons 44px, reachable; no overflow</t>
         </is>
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>FN-13</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="338" ht="82" customHeight="1">
       <c r="A338" s="2" t="inlineStr">
         <is>
+          <t>T-698</t>
+        </is>
+      </c>
+      <c r="B338" s="2" t="inlineStr">
+        <is>
+          <t>My Work</t>
+        </is>
+      </c>
+      <c r="C338" s="2" t="inlineStr">
+        <is>
+          <t>Phone - My Tasks / Status without AI</t>
+        </is>
+      </c>
+      <c r="D338" s="2" t="inlineStr">
+        <is>
+          <t>Mobile 390x844</t>
+        </is>
+      </c>
+      <c r="E338" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F338" s="2" t="inlineStr">
+        <is>
+          <t>Person hidden on My Tasks; a Status filter is visible even with AI priority off</t>
+        </is>
+      </c>
+      <c r="G338" s="2" t="inlineStr">
+        <is>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H338" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I338" s="2" t="inlineStr">
+        <is>
+          <t>Sheet on My Tasks has no Person; ?status=overdue shows the caption</t>
+        </is>
+      </c>
+      <c r="J338" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="339" ht="82" customHeight="1">
+      <c r="A339" s="2" t="inlineStr">
+        <is>
+          <t>T-699</t>
+        </is>
+      </c>
+      <c r="B339" s="2" t="inlineStr">
+        <is>
+          <t>My Work</t>
+        </is>
+      </c>
+      <c r="C339" s="2" t="inlineStr">
+        <is>
+          <t>Sales - no Person filter</t>
+        </is>
+      </c>
+      <c r="D339" s="2" t="inlineStr">
+        <is>
+          <t>Desktop + Mobile</t>
+        </is>
+      </c>
+      <c r="E339" s="2" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="F339" s="2" t="inlineStr">
+        <is>
+          <t>Roles without All Tasks never see Person; ?person= is ignored</t>
+        </is>
+      </c>
+      <c r="G339" s="2" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="H339" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I339" s="2" t="inlineStr">
+        <is>
+          <t>Desktop row has no Person; phone sheet has no Person; ?person=anyone ignored, own 29 cards</t>
+        </is>
+      </c>
+      <c r="J339" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="340" ht="82" customHeight="1">
+      <c r="A340" s="2" t="inlineStr">
+        <is>
+          <t>T-680</t>
+        </is>
+      </c>
+      <c r="B340" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C340" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - receivables question</t>
+        </is>
+      </c>
+      <c r="D340" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E340" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F340" s="2" t="inlineStr">
+        <is>
+          <t>Dex answers how much customers owe with the ledger's figure</t>
+        </is>
+      </c>
+      <c r="G340" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H340" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I340" s="2" t="inlineStr">
+        <is>
+          <t>Said zero invoices / Rs 0 outstanding; ledger has Rs 7,49,000 outstanding (17.0s)</t>
+        </is>
+      </c>
+      <c r="J340" s="2" t="inlineStr">
+        <is>
+          <t>DX-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="341" ht="82" customHeight="1">
+      <c r="A341" s="2" t="inlineStr">
+        <is>
+          <t>T-681</t>
+        </is>
+      </c>
+      <c r="B341" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C341" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - what needs my attention</t>
+        </is>
+      </c>
+      <c r="D341" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E341" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F341" s="2" t="inlineStr">
+        <is>
+          <t>Dex surfaces the overdue work and pending decisions</t>
+        </is>
+      </c>
+      <c r="G341" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H341" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I341" s="2" t="inlineStr">
+        <is>
+          <t>Said nothing open or overdue; owner has 24 open / 6 overdue (24.1s)</t>
+        </is>
+      </c>
+      <c r="J341" s="2" t="inlineStr">
+        <is>
+          <t>DX-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="342" ht="82" customHeight="1">
+      <c r="A342" s="2" t="inlineStr">
+        <is>
+          <t>T-682</t>
+        </is>
+      </c>
+      <c r="B342" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C342" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - global search hand-off</t>
+        </is>
+      </c>
+      <c r="D342" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E342" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F342" s="2" t="inlineStr">
+        <is>
+          <t>A question from global search is answered on arrival</t>
+        </is>
+      </c>
+      <c r="G342" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H342" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I342" s="2" t="inlineStr">
+        <is>
+          <t>'Which tasks are overdue?' answered on /brain?q= with a task list (17.5s)</t>
+        </is>
+      </c>
+      <c r="J342" s="2" t="inlineStr"/>
+    </row>
+    <row r="343" ht="82" customHeight="1">
+      <c r="A343" s="2" t="inlineStr">
+        <is>
+          <t>T-683</t>
+        </is>
+      </c>
+      <c r="B343" s="2" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="C343" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - coach refresh</t>
+        </is>
+      </c>
+      <c r="D343" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E343" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F343" s="2" t="inlineStr">
+        <is>
+          <t>Generate coaching produces a review grounded in the stats</t>
+        </is>
+      </c>
+      <c r="G343" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H343" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I343" s="2" t="inlineStr">
+        <is>
+          <t>TEST_member: 'AI coach updated' in 8.7s; strengths / improvements reference the 13 actionable tasks and plan use</t>
+        </is>
+      </c>
+      <c r="J343" s="2" t="inlineStr"/>
+    </row>
+    <row r="344" ht="82" customHeight="1">
+      <c r="A344" s="2" t="inlineStr">
+        <is>
+          <t>T-684</t>
+        </is>
+      </c>
+      <c r="B344" s="2" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C344" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Score with AI</t>
+        </is>
+      </c>
+      <c r="D344" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E344" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F344" s="2" t="inlineStr">
+        <is>
+          <t>Rescore updates the relationship card sensibly</t>
+        </is>
+      </c>
+      <c r="G344" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H344" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I344" s="2" t="inlineStr">
+        <is>
+          <t>E2E Test Co: 'Relationship scored by AI' in 7.8s; Relationship 12 / Risk 78, reason cites 4 open complaints and no billing - matches the record</t>
+        </is>
+      </c>
+      <c r="J344" s="2" t="inlineStr"/>
+    </row>
+    <row r="345" ht="82" customHeight="1">
+      <c r="A345" s="2" t="inlineStr">
+        <is>
+          <t>T-685</t>
+        </is>
+      </c>
+      <c r="B345" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C345" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - AI analysis refresh</t>
+        </is>
+      </c>
+      <c r="D345" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E345" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F345" s="2" t="inlineStr">
+        <is>
+          <t>Refresh produces an analysis grounded in the ledger</t>
+        </is>
+      </c>
+      <c r="G345" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H345" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I345" s="2" t="inlineStr">
+        <is>
+          <t>'Analysis refreshed' in 20.6s; Rs 6.6L outstanding (ledger 6,55,466), Surat Spinners Rs 4.8L unpaid 33 days (correct), duplicates flagged</t>
+        </is>
+      </c>
+      <c r="J345" s="2" t="inlineStr"/>
+    </row>
+    <row r="346" ht="82" customHeight="1">
+      <c r="A346" s="2" t="inlineStr">
+        <is>
+          <t>T-686</t>
+        </is>
+      </c>
+      <c r="B346" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C346" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Ask AI</t>
+        </is>
+      </c>
+      <c r="D346" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E346" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F346" s="2" t="inlineStr">
+        <is>
+          <t>The answer is correct and readable</t>
+        </is>
+      </c>
+      <c r="G346" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H346" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I346" s="2" t="inlineStr">
+        <is>
+          <t>Correct (Surat Spinners Rs 4,80,000, 7.3s) but literal ** markdown shown</t>
+        </is>
+      </c>
+      <c r="J346" s="2" t="inlineStr">
+        <is>
+          <t>FN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="347" ht="82" customHeight="1">
+      <c r="A347" s="2" t="inlineStr">
+        <is>
+          <t>T-688</t>
+        </is>
+      </c>
+      <c r="B347" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C347" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - owner on a phone</t>
+        </is>
+      </c>
+      <c r="D347" s="2" t="inlineStr">
+        <is>
+          <t>Mobile 390x844</t>
+        </is>
+      </c>
+      <c r="E347" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F347" s="2" t="inlineStr">
+        <is>
+          <t>Dex answers on mobile and the answer fits the screen</t>
+        </is>
+      </c>
+      <c r="G347" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H347" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I347" s="2" t="inlineStr">
+        <is>
+          <t>'53 decisions pending approval across 77' - correct; 17.6s; no overflow</t>
+        </is>
+      </c>
+      <c r="J347" s="2" t="inlineStr"/>
+    </row>
+    <row r="348" ht="82" customHeight="1">
+      <c r="A348" s="2" t="inlineStr">
+        <is>
+          <t>T-689</t>
+        </is>
+      </c>
+      <c r="B348" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C348" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Sales asks money questions</t>
+        </is>
+      </c>
+      <c r="D348" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E348" s="2" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="F348" s="2" t="inlineStr">
+        <is>
+          <t>Dex refuses finance answers to a role the finance API refuses</t>
+        </is>
+      </c>
+      <c r="G348" s="2" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="H348" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I348" s="2" t="inlineStr">
+        <is>
+          <t>Receivables and profit questions both refused ('You do not have permission to access financial...'), 5.8s / 1.6s; no figures leaked</t>
+        </is>
+      </c>
+      <c r="J348" s="2" t="inlineStr"/>
+    </row>
+    <row r="349" ht="82" customHeight="1">
+      <c r="A349" s="2" t="inlineStr">
+        <is>
+          <t>T-687</t>
+        </is>
+      </c>
+      <c r="B349" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C349" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - bill extraction</t>
+        </is>
+      </c>
+      <c r="D349" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E349" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F349" s="2" t="inlineStr">
+        <is>
+          <t>A GST bill is extracted into a reviewable record with the key fields</t>
+        </is>
+      </c>
+      <c r="G349" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H349" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I349" s="2" t="inlineStr">
+        <is>
+          <t>Party, number, amount, due date, category and follow-up correct (31.9s, 92%); date, GSTIN, items missing; no stale-date warning. Left in review, not filed</t>
+        </is>
+      </c>
+      <c r="J349" s="2" t="inlineStr">
+        <is>
+          <t>FN-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="350" ht="82" customHeight="1">
+      <c r="A350" s="2" t="inlineStr">
+        <is>
           <t>T-676</t>
         </is>
       </c>
-      <c r="B338" s="2" t="inlineStr">
+      <c r="B350" s="2" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="C338" s="2" t="inlineStr">
+      <c r="C350" s="2" t="inlineStr">
         <is>
           <t>Admin portal gating</t>
         </is>
       </c>
-      <c r="D338" s="2" t="inlineStr">
+      <c r="D350" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="E338" s="2" t="inlineStr">
+      <c r="E350" s="2" t="inlineStr">
         <is>
           <t>Signed out / Owner</t>
         </is>
       </c>
-      <c r="F338" s="2" t="inlineStr">
+      <c r="F350" s="2" t="inlineStr">
         <is>
           <t>Only platform admins reach the portal</t>
         </is>
       </c>
-      <c r="G338" s="2" t="inlineStr">
+      <c r="G350" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="H338" s="4" t="inlineStr">
+      <c r="H350" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I338" s="2" t="inlineStr">
+      <c r="I350" s="2" t="inlineStr">
         <is>
           <t>Signed out and tenant owner both get the admin sign-in; /admin/me 401; deep link /admin/tenants too</t>
         </is>
       </c>
-      <c r="J338" s="2" t="inlineStr"/>
+      <c r="J350" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J338"/>
+  <autoFilter ref="A1:J350"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26952,7 +27576,8 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>PROGRESS 2026-09-14 - TK-03 My team BUILT (desktop, founder call D3: owner keeps All Tasks, managers get My team): a manager is anyone named as a Reporting Manager (Team page field, until now used only for leave). GET /tasks?view=team = tasks whose doer or a helper is one of my direct reports (services/tasks.task_list_query, 9 unit tests, backend/tests/test_task_view_team.py).My Work: My team in the desktop switcher only for a non-owner with reports; kept in the URL (?view=team), not saved as default; Department, Person (lists the team, no Me) and Status filters work; AI priority off; own empty state; a My team link opened by someone without reports lands on My Tasks. The manager can open a report task and its activity (GET /tasks/{id} and /activity now allow the doer or helper manager) and leave a note; if the task is outside the manager department the drawer is note-only (same as Asked by me), inside it the existing department rule still gives full controls. Acceptance 21/21 (backend/scripts/ux_task_team_0914.py, writes blocked, REAL data: Sunita Rao manages sai, 16 tasks; the other-department note-only drawer uses one made-up task) + ux_task_asked_0914 20/20 re-run. Demo data has only one manager, so a manager of several people is covered by unit tests only.
+          <t>PROGRESS 2026-09-14 - TK-04 Links always land BUILT (desktop + phone link; frontend only): BEFORE (baseline, writes blocked) a task link opened only when the task sat in the list on screen - Sunita opening a task of sai (her report, not in her My Tasks) got no drawer, nor for a finished task, nor when already on My Work (a notification clicked from there); ?focus=task:&lt;id&gt; links (Brief blocks, phone) were ignored; a deleted task said Access restricted; Workflows was lost on refresh; Back left My Work instead of returning to the previous view. NOW: ?task=&lt;id&gt; and ?focus=task:&lt;id&gt; open the drawer whatever the view - from the list card when the task is in the list, else drawn from the single-task request; the link opens again when it changes while My Work is open; closing the drawer takes the link out of the address; a missing task says This task no longer exists and a refused one keeps Access restricted, both with Dismiss; every view writes ?view=mine|asked|team|all|approvals|workflows and pushes a history entry, and the page follows Back and Forward; ?view=all and ?view=mine links work. Acceptance 23/23 (backend/scripts/ux_task_links_0914.py, writes blocked, REAL data: Sunita Rao and sai; owner; a production user refused with 403; one phone check), run after rebasing onto 0eaa411 (glass pass) and afc6136 (UI-SCALE). Re-runs on the merged page: ux_task_asked_0914 20/20, ux_task_approvals_0914 21/21, ux_task_team_0914 21/21, ux_task_approval_stage_0914 19/19, ux_person_filter_0913 33/33, ux_newtask_form_0914 13/13 + 3 n/a. Script upkeep in the same push: the merged page draws its first cards about 3.5 s after load and redraws about 1 s after Clear (traced), so settle() in the links, asked and person-filter scripts now waits for real content and the person filter waits for the card count to change and hold; the asked clears-url check accepts view=mine; the approval-stage and New Task form scripts follow 0eaa411 (no More options row: those three checks report n/a; GlassSelect dropdowns are driven by their option testids). Bisect (MyWork.js from afc6136, without TK-04): the person-filter failures showed there too; the one asked failure that did not repeat without TK-04 was a half-loaded page (traced with TK-04: all 53 cards 3.5 s after reload) and passes once the script waits. Traced separately: Clear filters restores all 129 cards about 1 s after the click.
+PROGRESS 2026-09-14 - TK-03 My team BUILT (desktop, founder call D3: owner keeps All Tasks, managers get My team): a manager is anyone named as a Reporting Manager (Team page field, until now used only for leave). GET /tasks?view=team = tasks whose doer or a helper is one of my direct reports (services/tasks.task_list_query, 9 unit tests, backend/tests/test_task_view_team.py).My Work: My team in the desktop switcher only for a non-owner with reports; kept in the URL (?view=team), not saved as default; Department, Person (lists the team, no Me) and Status filters work; AI priority off; own empty state; a My team link opened by someone without reports lands on My Tasks. The manager can open a report task and its activity (GET /tasks/{id} and /activity now allow the doer or helper manager) and leave a note; if the task is outside the manager department the drawer is note-only (same as Asked by me), inside it the existing department rule still gives full controls. Acceptance 21/21 (backend/scripts/ux_task_team_0914.py, writes blocked, REAL data: Sunita Rao manages sai, 16 tasks; the other-department note-only drawer uses one made-up task) + ux_task_asked_0914 20/20 re-run. Demo data has only one manager, so a manager of several people is covered by unit tests only.
 PROGRESS 2026-09-14 - TK-05 Approval moment BUILT (desktop, plan Phase 4, founder call D2): the creator picks when a task is approved - New Task, More options, Needs approval: No / Before work starts / Before it is marked done (stored as approval_stage start or close; older approval tasks count as start). Before work starts is the lock tasks always had. Before it is marked done leaves the work open: Complete (proof still required) moves the task to Under review with approval pending and notifies the approver (Approval needed to close, opens Approvals); Approve closes it and runs the close hooks (workflow advance, Brain record, invoice draft - moved into one helper so both paths share them); Request changes sends it back to In progress with the reason shown to the doer; moving the status back withdraws the request; a person who may approve closes it directly; a checklist reaching 100 percent follows the same rule. GET /tasks?view=approvals holds a before-done task only while it waits, so the Approvals count and the Desk card include both kinds. Cards say Approval to start / Approval to close / Needs approval to close; the approver box and the doer banners say which moment it is. Acceptance 19/19 (backend/scripts/ux_task_approval_stage_0914.py, writes blocked, test tasks made up by the script, real approvals feed read-only) + 17 unit tests (backend/tests/test_task_approval_stage.py); ux_newtask_form_0914 16/16 and ux_task_approvals_0914 21/21 re-run. NOT proven live: saving a before-done task and approving it for real - waits on a test database. Open: the server still does not check that a named approver holds approval access (plan 4.3).
 PROGRESS 2026-09-14 - TK-02 Waiting for my approval BUILT (desktop), merged into the Approvals view that 3c23e49 added to My Work: GET /tasks?view=approvals (approval required, not approved, not finished; owner sees all, a named approver sees tasks naming them, an Approve Tasks holder also sees tasks naming nobody - the same rule as _can_approve_task) now feeds the Tasks tab of that view AND the Task approvals card on the Desk (both read /tasks?mine=false before, which for a non-owner is their own lane only, so a named approver outside it saw nothing). The Approvals button carries the pending count and also shows for a named approver without approval access; list is oldest first; the approval-requested notification opens /my-work?view=approvals&amp;task=&lt;id&gt; inside Approvals. Acceptance 21/21 (backend/scripts/ux_task_approvals_0914.py, writes blocked, Approve answered by the script) + 8 unit tests (backend/tests/test_task_view_approvals.py). NOT proven live: a non-owner approver approving a real task - no demo user holds approval access or is named on a task, so that path was checked with a mocked list.
 PROGRESS 2026-09-14 - TK-01 Asked by me BUILT (desktop): GET /tasks?view=asked (created by me, not mine to do: I am neither the doer nor a helper); My Work switcher gets Asked by me (owner: My Tasks | Asked by me | All Tasks; staff: My Work | Asked by me), kept in the URL (?view=asked) and never saved as the default; Department, Person (no Me option) and Status filters work on it; AI priority is off there; its own empty state; the person who asked can leave a note on the task (server + form), hand-off and escalate stay with the doer; a phone link lands on the list. Acceptance 20/20 (backend/scripts/ux_task_asked_0914.py, writes blocked) + 13 unit tests (backend/tests/test_task_view_asked.py). NOT proven live: a non-owner creating a task and then seeing it - no non-owner in the demo company has created one, and creating one writes to the production database; the note-only form was checked with a mocked list. TK-02..TK-04 still to do.
@@ -32762,7 +33387,7 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>337 (246 pass, 89 fail, 0 blocked, 2 not run)</t>
+          <t>349 (258 pass, 89 fail, 0 blocked, 2 not run)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: ASK-28 TK-06 who is on a task (plan Phase 2); T-768..T-775
Full suite 1426 passed (only the known test_website_intel_ssrf_block_and_fallback failure).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_UI_Bug_Report.xlsx
+++ b/docs/DecisionOS_UI_Bug_Report.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bug Log'!$A$1:$Q$89</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Coverage'!$A$1:$J$361</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Coverage'!$A$1:$J$369</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Verified Non-Issues'!$A$1:$E$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Action List'!$A$1:$K$118</definedName>
   </definedNames>
@@ -8116,7 +8116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J361"/>
+  <dimension ref="A1:J369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -24238,7 +24238,7 @@
     <row r="324" ht="82" customHeight="1">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>T-708</t>
+          <t>T-768</t>
         </is>
       </c>
       <c r="B324" s="2" t="inlineStr">
@@ -24248,7 +24248,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - switcher</t>
+          <t>Drawer - Asked by</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -24258,12 +24258,12 @@
       </c>
       <c r="E324" s="2" t="inlineStr">
         <is>
-          <t>Owner + Sales</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F324" s="2" t="inlineStr">
         <is>
-          <t>Asked by me sits in the view switcher for every role</t>
+          <t>The drawer names who asked for the task</t>
         </is>
       </c>
       <c r="G324" s="2" t="inlineStr">
@@ -24278,7 +24278,7 @@
       </c>
       <c r="I324" s="2" t="inlineStr">
         <is>
-          <t>Owner: My Tasks | Asked by me | All Tasks | Workflows; Sales sees it too</t>
+          <t>Asked by &lt;name&gt;; Asked by You on a task the owner created</t>
         </is>
       </c>
       <c r="J324" s="2" t="inlineStr">
@@ -24290,7 +24290,7 @@
     <row r="325" ht="82" customHeight="1">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>T-709</t>
+          <t>T-769</t>
         </is>
       </c>
       <c r="B325" s="2" t="inlineStr">
@@ -24300,7 +24300,7 @@
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - the rule</t>
+          <t>Drawer - approver and moment</t>
         </is>
       </c>
       <c r="D325" s="2" t="inlineStr">
@@ -24315,12 +24315,12 @@
       </c>
       <c r="F325" s="2" t="inlineStr">
         <is>
-          <t>Only tasks I created that are not mine to do</t>
+          <t>The drawer names the approver and when approval happens</t>
         </is>
       </c>
       <c r="G325" s="2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H325" s="4" t="inlineStr">
@@ -24330,7 +24330,7 @@
       </c>
       <c r="I325" s="2" t="inlineStr">
         <is>
-          <t>GET /tasks?view=asked: 60 tasks, 0 break the rule; 53 open = 53 cards</t>
+          <t>Approval before work starts / before it is marked done: &lt;approver or anyone with approval access&gt;</t>
         </is>
       </c>
       <c r="J325" s="2" t="inlineStr">
@@ -24342,7 +24342,7 @@
     <row r="326" ht="82" customHeight="1">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>T-710</t>
+          <t>T-770</t>
         </is>
       </c>
       <c r="B326" s="2" t="inlineStr">
@@ -24352,7 +24352,7 @@
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - filters</t>
+          <t>Drawer - picked automatically</t>
         </is>
       </c>
       <c r="D326" s="2" t="inlineStr">
@@ -24362,17 +24362,17 @@
       </c>
       <c r="E326" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Owner (made-up task)</t>
         </is>
       </c>
       <c r="F326" s="2" t="inlineStr">
         <is>
-          <t>Person (without Me) and Status narrow the list with matching counts</t>
+          <t>A team task says it went to the member with the fewest open tasks</t>
         </is>
       </c>
       <c r="G326" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H326" s="4" t="inlineStr">
@@ -24382,7 +24382,7 @@
       </c>
       <c r="I326" s="2" t="inlineStr">
         <is>
-          <t>Person -&gt; 9 cards = API 9; Status Overdue 13 = 13 cards</t>
+          <t>Picked automatically: fewest open tasks in Sales; no supporting-employee line</t>
         </is>
       </c>
       <c r="J326" s="2" t="inlineStr">
@@ -24394,7 +24394,7 @@
     <row r="327" ht="82" customHeight="1">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>T-711</t>
+          <t>T-771</t>
         </is>
       </c>
       <c r="B327" s="2" t="inlineStr">
@@ -24404,7 +24404,7 @@
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - URL and default</t>
+          <t>New Task - team toast</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
@@ -24419,12 +24419,12 @@
       </c>
       <c r="F327" s="2" t="inlineStr">
         <is>
-          <t>View survives refresh, other views clear it, plain /my-work does not reopen on it</t>
+          <t>Giving a task to a team says who it went to and why</t>
         </is>
       </c>
       <c r="G327" s="2" t="inlineStr">
         <is>
-          <t>Flow</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H327" s="4" t="inlineStr">
@@ -24434,7 +24434,7 @@
       </c>
       <c r="I327" s="2" t="inlineStr">
         <is>
-          <t>?view=asked kept on reload; My Tasks clears it; not saved as default</t>
+          <t>Assigned to Priya Nair: fewest open tasks in Sales (POST answered by the script); no Supporting employee field</t>
         </is>
       </c>
       <c r="J327" s="2" t="inlineStr">
@@ -24446,7 +24446,7 @@
     <row r="328" ht="82" customHeight="1">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>T-712</t>
+          <t>T-772</t>
         </is>
       </c>
       <c r="B328" s="2" t="inlineStr">
@@ -24456,12 +24456,12 @@
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - AI priority</t>
+          <t>Drawer - people lines on a phone</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Mobile 390x844</t>
         </is>
       </c>
       <c r="E328" s="2" t="inlineStr">
@@ -24471,7 +24471,7 @@
       </c>
       <c r="F328" s="2" t="inlineStr">
         <is>
-          <t>AI priority is not offered on other people's work</t>
+          <t>The people lines fit a phone</t>
         </is>
       </c>
       <c r="G328" s="2" t="inlineStr">
@@ -24486,7 +24486,7 @@
       </c>
       <c r="I328" s="2" t="inlineStr">
         <is>
-          <t>AI toggle hidden on Asked by me</t>
+          <t>Lines shown; no sideways overflow</t>
         </is>
       </c>
       <c r="J328" s="2" t="inlineStr">
@@ -24498,22 +24498,22 @@
     <row r="329" ht="82" customHeight="1">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>T-713</t>
+          <t>T-773</t>
         </is>
       </c>
       <c r="B329" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Tasks API</t>
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - empty</t>
+          <t>Supporting employee removed</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Backend (isolated DB)</t>
         </is>
       </c>
       <c r="E329" s="2" t="inlineStr">
@@ -24523,12 +24523,12 @@
       </c>
       <c r="F329" s="2" t="inlineStr">
         <is>
-          <t>Someone who has asked for nothing sees an explanation, not the decisions text</t>
+          <t>An old app sending support_id still creates the task; the field is not kept and grants no access</t>
         </is>
       </c>
       <c r="G329" s="2" t="inlineStr">
         <is>
-          <t>Empty state</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H329" s="4" t="inlineStr">
@@ -24538,7 +24538,7 @@
       </c>
       <c r="I329" s="2" t="inlineStr">
         <is>
-          <t>'Nothing you've asked for is open - Tasks you create for other people show up here, with their live status.'</t>
+          <t>created; no support_id stored; would-be supporter gets 403</t>
         </is>
       </c>
       <c r="J329" s="2" t="inlineStr">
@@ -24550,37 +24550,37 @@
     <row r="330" ht="82" customHeight="1">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>T-714</t>
+          <t>T-774</t>
         </is>
       </c>
       <c r="B330" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Tasks API</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - requester note</t>
+          <t>Auto-assigned note</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Backend (isolated DB)</t>
         </is>
       </c>
       <c r="E330" s="2" t="inlineStr">
         <is>
-          <t>Sales (mocked list)</t>
+          <t>Sales / Owner</t>
         </is>
       </c>
       <c r="F330" s="2" t="inlineStr">
         <is>
-          <t>The person who asked can leave a note but not hand off or escalate</t>
+          <t>A team task records how it was routed, and a reassign clears it</t>
         </is>
       </c>
       <c r="G330" s="2" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H330" s="4" t="inlineStr">
@@ -24590,7 +24590,7 @@
       </c>
       <c r="I330" s="2" t="inlineStr">
         <is>
-          <t>Update form offers only Log note; server allows a note from the creator (unit-tested)</t>
+          <t>auto_assigned {role operations, fewest_open_tasks}; cleared after PATCH assignee; named doer never auto</t>
         </is>
       </c>
       <c r="J330" s="2" t="inlineStr">
@@ -24602,37 +24602,37 @@
     <row r="331" ht="82" customHeight="1">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>T-716</t>
+          <t>T-775</t>
         </is>
       </c>
       <c r="B331" s="2" t="inlineStr">
         <is>
-          <t>My Work</t>
+          <t>Tasks API</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - requester drawer</t>
+          <t>Helpers get notified</t>
         </is>
       </c>
       <c r="D331" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Backend (isolated DB)</t>
         </is>
       </c>
       <c r="E331" s="2" t="inlineStr">
         <is>
-          <t>Sales (mocked list)</t>
+          <t>Operations lead / Finance helper</t>
         </is>
       </c>
       <c r="F331" s="2" t="inlineStr">
         <is>
-          <t>The person who asked sees progress and a note box, not the doer's status, plan, complete or attach controls</t>
+          <t>A helper hears status changes and overdue reminders like the lead</t>
         </is>
       </c>
       <c r="G331" s="2" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H331" s="4" t="inlineStr">
@@ -24642,7 +24642,7 @@
       </c>
       <c r="I331" s="2" t="inlineStr">
         <is>
-          <t>Status, Complete, Attach, Reopen hidden; hint 'You asked for this task, so &lt;doer&gt; does the work. Leave a note below to follow up.'</t>
+          <t>status change -&gt; helper + asker notified; overdue reminder -&gt; lead + helper</t>
         </is>
       </c>
       <c r="J331" s="2" t="inlineStr">
@@ -24654,7 +24654,7 @@
     <row r="332" ht="82" customHeight="1">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>T-715</t>
+          <t>T-708</t>
         </is>
       </c>
       <c r="B332" s="2" t="inlineStr">
@@ -24664,22 +24664,22 @@
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>Asked by me - phone link</t>
+          <t>Asked by me - switcher</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
         <is>
-          <t>Mobile 390x844</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E332" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Owner + Sales</t>
         </is>
       </c>
       <c r="F332" s="2" t="inlineStr">
         <is>
-          <t>A link to Asked by me on a phone shows that list, not My Tasks</t>
+          <t>Asked by me sits in the view switcher for every role</t>
         </is>
       </c>
       <c r="G332" s="2" t="inlineStr">
@@ -24694,7 +24694,7 @@
       </c>
       <c r="I332" s="2" t="inlineStr">
         <is>
-          <t>53 / 53 cards; My Tasks not pressed; no overflow</t>
+          <t>Owner: My Tasks | Asked by me | All Tasks | Workflows; Sales sees it too</t>
         </is>
       </c>
       <c r="J332" s="2" t="inlineStr">
@@ -24706,7 +24706,7 @@
     <row r="333" ht="82" customHeight="1">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>T-700</t>
+          <t>T-709</t>
         </is>
       </c>
       <c r="B333" s="2" t="inlineStr">
@@ -24716,7 +24716,7 @@
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>New Task - quick part</t>
+          <t>Asked by me - the rule</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr">
@@ -24731,12 +24731,12 @@
       </c>
       <c r="F333" s="2" t="inlineStr">
         <is>
-          <t>Only title, Department, Assign to and Due show before More options</t>
+          <t>Only tasks I created that are not mine to do</t>
         </is>
       </c>
       <c r="G333" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H333" s="4" t="inlineStr">
@@ -24746,19 +24746,19 @@
       </c>
       <c r="I333" s="2" t="inlineStr">
         <is>
-          <t>Visible: Task title, Department, Assign to, Due; Operational category and Supporting employee gone</t>
+          <t>GET /tasks?view=asked: 60 tasks, 0 break the rule; 53 open = 53 cards</t>
         </is>
       </c>
       <c r="J333" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="334" ht="82" customHeight="1">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>T-701</t>
+          <t>T-710</t>
         </is>
       </c>
       <c r="B334" s="2" t="inlineStr">
@@ -24768,7 +24768,7 @@
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>New Task - More options</t>
+          <t>Asked by me - filters</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
@@ -24783,12 +24783,12 @@
       </c>
       <c r="F334" s="2" t="inlineStr">
         <is>
-          <t>Priority, helpers, description, time, result, approval, proof, files wait under More; closed section says how many are set</t>
+          <t>Person (without Me) and Status narrow the list with matching counts</t>
         </is>
       </c>
       <c r="G334" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H334" s="4" t="inlineStr">
@@ -24798,19 +24798,19 @@
       </c>
       <c r="I334" s="2" t="inlineStr">
         <is>
-          <t>Collapsed by default; '5 set' after choosing priority, helper, time, approval, proof</t>
+          <t>Person -&gt; 9 cards = API 9; Status Overdue 13 = 13 cards</t>
         </is>
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="335" ht="82" customHeight="1">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>T-702</t>
+          <t>T-711</t>
         </is>
       </c>
       <c r="B335" s="2" t="inlineStr">
@@ -24820,7 +24820,7 @@
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>New Task - title required</t>
+          <t>Asked by me - URL and default</t>
         </is>
       </c>
       <c r="D335" s="2" t="inlineStr">
@@ -24835,12 +24835,12 @@
       </c>
       <c r="F335" s="2" t="inlineStr">
         <is>
-          <t>Create without a title shows an inline error and sends nothing</t>
+          <t>View survives refresh, other views clear it, plain /my-work does not reopen on it</t>
         </is>
       </c>
       <c r="G335" s="2" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H335" s="4" t="inlineStr">
@@ -24850,19 +24850,19 @@
       </c>
       <c r="I335" s="2" t="inlineStr">
         <is>
-          <t>'Give the task a title' under the field; clears on typing; no request</t>
+          <t>?view=asked kept on reload; My Tasks clears it; not saved as default</t>
         </is>
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="336" ht="82" customHeight="1">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>T-703</t>
+          <t>T-712</t>
         </is>
       </c>
       <c r="B336" s="2" t="inlineStr">
@@ -24872,7 +24872,7 @@
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>New Task - Assign to</t>
+          <t>Asked by me - AI priority</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr">
@@ -24887,12 +24887,12 @@
       </c>
       <c r="F336" s="2" t="inlineStr">
         <is>
-          <t>One control lists people and teams; a team explains where it goes</t>
+          <t>AI priority is not offered on other people's work</t>
         </is>
       </c>
       <c r="G336" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H336" s="4" t="inlineStr">
@@ -24902,19 +24902,19 @@
       </c>
       <c r="I336" s="2" t="inlineStr">
         <is>
-          <t>12 people + Sales, Production, Finance teams; hint 'Goes to whoever in Sales has the least open work'</t>
+          <t>AI toggle hidden on Asked by me</t>
         </is>
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="337" ht="82" customHeight="1">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>T-704</t>
+          <t>T-713</t>
         </is>
       </c>
       <c r="B337" s="2" t="inlineStr">
@@ -24924,7 +24924,7 @@
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>New Task - due presets</t>
+          <t>Asked by me - empty</t>
         </is>
       </c>
       <c r="D337" s="2" t="inlineStr">
@@ -24934,17 +24934,17 @@
       </c>
       <c r="E337" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F337" s="2" t="inlineStr">
         <is>
-          <t>Today / Tomorrow / In a week set the date without a picker</t>
+          <t>Someone who has asked for nothing sees an explanation, not the decisions text</t>
         </is>
       </c>
       <c r="G337" s="2" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Empty state</t>
         </is>
       </c>
       <c r="H337" s="4" t="inlineStr">
@@ -24954,19 +24954,19 @@
       </c>
       <c r="I337" s="2" t="inlineStr">
         <is>
-          <t>Tomorrow -&gt; 'Due Tue 15 Sept'; Today -&gt; due_date = today, no time</t>
+          <t>'Nothing you've asked for is open - Tasks you create for other people show up here, with their live status.'</t>
         </is>
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="338" ht="82" customHeight="1">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>T-705</t>
+          <t>T-714</t>
         </is>
       </c>
       <c r="B338" s="2" t="inlineStr">
@@ -24976,7 +24976,7 @@
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>New Task - payload (person)</t>
+          <t>Asked by me - requester note</t>
         </is>
       </c>
       <c r="D338" s="2" t="inlineStr">
@@ -24986,17 +24986,17 @@
       </c>
       <c r="E338" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales (mocked list)</t>
         </is>
       </c>
       <c r="F338" s="2" t="inlineStr">
         <is>
-          <t>The form sends exactly what was chosen and nothing removed</t>
+          <t>The person who asked can leave a note but not hand off or escalate</t>
         </is>
       </c>
       <c r="G338" s="2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="H338" s="4" t="inlineStr">
@@ -25006,19 +25006,19 @@
       </c>
       <c r="I338" s="2" t="inlineStr">
         <is>
-          <t>task_type sales, lead + 1 helper, high, tomorrow 16:30, approval (anyone), proof; no op_category / support_id</t>
+          <t>Update form offers only Log note; server allows a note from the creator (unit-tested)</t>
         </is>
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="339" ht="82" customHeight="1">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>T-706</t>
+          <t>T-716</t>
         </is>
       </c>
       <c r="B339" s="2" t="inlineStr">
@@ -25028,7 +25028,7 @@
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>New Task - payload (team)</t>
+          <t>Asked by me - requester drawer</t>
         </is>
       </c>
       <c r="D339" s="2" t="inlineStr">
@@ -25038,17 +25038,17 @@
       </c>
       <c r="E339" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales (mocked list)</t>
         </is>
       </c>
       <c r="F339" s="2" t="inlineStr">
         <is>
-          <t>A team task sends the role, no person and no helpers</t>
+          <t>The person who asked sees progress and a note box, not the doer's status, plan, complete or attach controls</t>
         </is>
       </c>
       <c r="G339" s="2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="H339" s="4" t="inlineStr">
@@ -25058,19 +25058,19 @@
       </c>
       <c r="I339" s="2" t="inlineStr">
         <is>
-          <t>assignee_role sales, assignee_id null, co_assignee_ids [], due today</t>
+          <t>Status, Complete, Attach, Reopen hidden; hint 'You asked for this task, so &lt;doer&gt; does the work. Leave a note below to follow up.'</t>
         </is>
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="340" ht="82" customHeight="1">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>T-707</t>
+          <t>T-715</t>
         </is>
       </c>
       <c r="B340" s="2" t="inlineStr">
@@ -25080,12 +25080,12 @@
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>New Task - after create</t>
+          <t>Asked by me - phone link</t>
         </is>
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Mobile 390x844</t>
         </is>
       </c>
       <c r="E340" s="2" t="inlineStr">
@@ -25095,12 +25095,12 @@
       </c>
       <c r="F340" s="2" t="inlineStr">
         <is>
-          <t>Dialog closes, reopens empty with More collapsed, My Work still renders</t>
+          <t>A link to Asked by me on a phone shows that list, not My Tasks</t>
         </is>
       </c>
       <c r="G340" s="2" t="inlineStr">
         <is>
-          <t>Flow</t>
+          <t>Views</t>
         </is>
       </c>
       <c r="H340" s="4" t="inlineStr">
@@ -25110,19 +25110,19 @@
       </c>
       <c r="I340" s="2" t="inlineStr">
         <is>
-          <t>Closed; reopened clean; 25 cards; no page errors</t>
+          <t>53 / 53 cards; My Tasks not pressed; no overflow</t>
         </is>
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>ASK-29</t>
+          <t>ASK-28</t>
         </is>
       </c>
     </row>
     <row r="341" ht="82" customHeight="1">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>T-690</t>
+          <t>T-700</t>
         </is>
       </c>
       <c r="B341" s="2" t="inlineStr">
@@ -25132,7 +25132,7 @@
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - filter row</t>
+          <t>New Task - quick part</t>
         </is>
       </c>
       <c r="D341" s="2" t="inlineStr">
@@ -25147,12 +25147,12 @@
       </c>
       <c r="F341" s="2" t="inlineStr">
         <is>
-          <t>All Tasks shows Department, Person, Status; My Tasks hides Person</t>
+          <t>Only title, Department, Assign to and Due show before More options</t>
         </is>
       </c>
       <c r="G341" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H341" s="4" t="inlineStr">
@@ -25162,19 +25162,19 @@
       </c>
       <c r="I341" s="2" t="inlineStr">
         <is>
-          <t>Row shows all three with counts (131); My Tasks shows two (25)</t>
+          <t>Visible: Task title, Department, Assign to, Due; Operational category and Supporting employee gone</t>
         </is>
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="342" ht="82" customHeight="1">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>T-691</t>
+          <t>T-701</t>
         </is>
       </c>
       <c r="B342" s="2" t="inlineStr">
@@ -25184,7 +25184,7 @@
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - Person filter</t>
+          <t>New Task - More options</t>
         </is>
       </c>
       <c r="D342" s="2" t="inlineStr">
@@ -25199,12 +25199,12 @@
       </c>
       <c r="F342" s="2" t="inlineStr">
         <is>
-          <t>Picking a person shows only their tasks, count matches the API</t>
+          <t>Priority, helpers, description, time, result, approval, proof, files wait under More; closed section says how many are set</t>
         </is>
       </c>
       <c r="G342" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H342" s="4" t="inlineStr">
@@ -25214,19 +25214,19 @@
       </c>
       <c r="I342" s="2" t="inlineStr">
         <is>
-          <t>Priya Nair: 29 cards = trigger 29 = API 29; URL ?person=; name line hidden on cards; menu has Me, people busiest first with role, Unassigned (6), Production team (5); no duplicate rows</t>
+          <t>Collapsed by default; '5 set' after choosing priority, helper, time, approval, proof</t>
         </is>
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="343" ht="82" customHeight="1">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>T-692</t>
+          <t>T-702</t>
         </is>
       </c>
       <c r="B343" s="2" t="inlineStr">
@@ -25236,7 +25236,7 @@
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - Status options</t>
+          <t>New Task - title required</t>
         </is>
       </c>
       <c r="D343" s="2" t="inlineStr">
@@ -25251,12 +25251,12 @@
       </c>
       <c r="F343" s="2" t="inlineStr">
         <is>
-          <t>Pending Approval, Overdue and Completed are filterable with correct counts</t>
+          <t>Create without a title shows an inline error and sends nothing</t>
         </is>
       </c>
       <c r="G343" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="H343" s="4" t="inlineStr">
@@ -25266,19 +25266,19 @@
       </c>
       <c r="I343" s="2" t="inlineStr">
         <is>
-          <t>Pending Approval 40, Overdue 68, Completed 17, Not Started 78 - all equal the API</t>
+          <t>'Give the task a title' under the field; clears on typing; no request</t>
         </is>
       </c>
       <c r="J343" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="344" ht="82" customHeight="1">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>T-693</t>
+          <t>T-703</t>
         </is>
       </c>
       <c r="B344" s="2" t="inlineStr">
@@ -25288,12 +25288,12 @@
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - Priority filter removed</t>
+          <t>New Task - Assign to</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
         <is>
-          <t>Desktop + Mobile</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E344" s="2" t="inlineStr">
@@ -25303,12 +25303,12 @@
       </c>
       <c r="F344" s="2" t="inlineStr">
         <is>
-          <t>No Priority filter (founder call 2026-09-13); an old ?priority= link does not narrow the list</t>
+          <t>One control lists people and teams; a team explains where it goes</t>
         </is>
       </c>
       <c r="G344" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H344" s="4" t="inlineStr">
@@ -25318,19 +25318,19 @@
       </c>
       <c r="I344" s="2" t="inlineStr">
         <is>
-          <t>No Priority dropdown on desktop, no Priority chips in the phone sheet; ?person=Priya&amp;status=overdue&amp;priority=high shows the same 20 as without it</t>
+          <t>12 people + Sales, Production, Finance teams; hint 'Goes to whoever in Sales has the least open work'</t>
         </is>
       </c>
       <c r="J344" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="345" ht="82" customHeight="1">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>T-694</t>
+          <t>T-704</t>
         </is>
       </c>
       <c r="B345" s="2" t="inlineStr">
@@ -25340,7 +25340,7 @@
       </c>
       <c r="C345" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - combined counts</t>
+          <t>New Task - due presets</t>
         </is>
       </c>
       <c r="D345" s="2" t="inlineStr">
@@ -25355,12 +25355,12 @@
       </c>
       <c r="F345" s="2" t="inlineStr">
         <is>
-          <t>Each menu's counts reflect the other active filters</t>
+          <t>Today / Tomorrow / In a week set the date without a picker</t>
         </is>
       </c>
       <c r="G345" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="H345" s="4" t="inlineStr">
@@ -25370,19 +25370,19 @@
       </c>
       <c r="I345" s="2" t="inlineStr">
         <is>
-          <t>With Priya + Overdue, Department 'All' reads 20 = cards = API</t>
+          <t>Tomorrow -&gt; 'Due Tue 15 Sept'; Today -&gt; due_date = today, no time</t>
         </is>
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="346" ht="82" customHeight="1">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>T-695</t>
+          <t>T-705</t>
         </is>
       </c>
       <c r="B346" s="2" t="inlineStr">
@@ -25392,7 +25392,7 @@
       </c>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - refresh, Clear, no match</t>
+          <t>New Task - payload (person)</t>
         </is>
       </c>
       <c r="D346" s="2" t="inlineStr">
@@ -25407,12 +25407,12 @@
       </c>
       <c r="F346" s="2" t="inlineStr">
         <is>
-          <t>Filters survive refresh; Clear resets; empty result explains itself</t>
+          <t>The form sends exactly what was chosen and nothing removed</t>
         </is>
       </c>
       <c r="G346" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H346" s="4" t="inlineStr">
@@ -25422,19 +25422,19 @@
       </c>
       <c r="I346" s="2" t="inlineStr">
         <is>
-          <t>Reload keeps 20 cards + URL; Clear -&gt; 131, URL clean; Priya x Under Review -&gt; 'No tasks match these filters' with Clear</t>
+          <t>task_type sales, lead + 1 helper, high, tomorrow 16:30, approval (anyone), proof; no op_category / support_id</t>
         </is>
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="347" ht="82" customHeight="1">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>T-696</t>
+          <t>T-706</t>
         </is>
       </c>
       <c r="B347" s="2" t="inlineStr">
@@ -25444,7 +25444,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>All Tasks - person search, links</t>
+          <t>New Task - payload (team)</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -25459,12 +25459,12 @@
       </c>
       <c r="F347" s="2" t="inlineStr">
         <is>
-          <t>Search narrows the menu; Desk overdue link and task deep link behave</t>
+          <t>A team task sends the role, no person and no helpers</t>
         </is>
       </c>
       <c r="G347" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="H347" s="4" t="inlineStr">
@@ -25474,19 +25474,19 @@
       </c>
       <c r="I347" s="2" t="inlineStr">
         <is>
-          <t>'pri' -&gt; Priya Nair only; ?filter=overdue -&gt; Status: Overdue 68; ?task= with filters set clears them and shows the card</t>
+          <t>assignee_role sales, assignee_id null, co_assignee_ids [], due today</t>
         </is>
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="348" ht="82" customHeight="1">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>T-697</t>
+          <t>T-707</t>
         </is>
       </c>
       <c r="B348" s="2" t="inlineStr">
@@ -25496,12 +25496,12 @@
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>Phone - filter sheet</t>
+          <t>New Task - after create</t>
         </is>
       </c>
       <c r="D348" s="2" t="inlineStr">
         <is>
-          <t>Mobile 390x844</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E348" s="2" t="inlineStr">
@@ -25511,12 +25511,12 @@
       </c>
       <c r="F348" s="2" t="inlineStr">
         <is>
-          <t>The phone reaches every filter and sees what is active</t>
+          <t>Dialog closes, reopens empty with More collapsed, My Work still renders</t>
         </is>
       </c>
       <c r="G348" s="2" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="H348" s="4" t="inlineStr">
@@ -25526,19 +25526,19 @@
       </c>
       <c r="I348" s="2" t="inlineStr">
         <is>
-          <t>Sheet with Department / Person / Status; Priya + Overdue -&gt; 'Show 20 tasks' = 20 cards; caption 'Showing Priya Nair - Overdue' with Clear; buttons 44px, reachable; no overflow</t>
+          <t>Closed; reopened clean; 25 cards; no page errors</t>
         </is>
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>ASK-24</t>
+          <t>ASK-29</t>
         </is>
       </c>
     </row>
     <row r="349" ht="82" customHeight="1">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>T-698</t>
+          <t>T-690</t>
         </is>
       </c>
       <c r="B349" s="2" t="inlineStr">
@@ -25548,12 +25548,12 @@
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>Phone - My Tasks / Status without AI</t>
+          <t>All Tasks - filter row</t>
         </is>
       </c>
       <c r="D349" s="2" t="inlineStr">
         <is>
-          <t>Mobile 390x844</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E349" s="2" t="inlineStr">
@@ -25563,7 +25563,7 @@
       </c>
       <c r="F349" s="2" t="inlineStr">
         <is>
-          <t>Person hidden on My Tasks; a Status filter is visible even with AI priority off</t>
+          <t>All Tasks shows Department, Person, Status; My Tasks hides Person</t>
         </is>
       </c>
       <c r="G349" s="2" t="inlineStr">
@@ -25578,7 +25578,7 @@
       </c>
       <c r="I349" s="2" t="inlineStr">
         <is>
-          <t>Sheet on My Tasks has no Person; ?status=overdue shows the caption</t>
+          <t>Row shows all three with counts (131); My Tasks shows two (25)</t>
         </is>
       </c>
       <c r="J349" s="2" t="inlineStr">
@@ -25590,7 +25590,7 @@
     <row r="350" ht="82" customHeight="1">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>T-699</t>
+          <t>T-691</t>
         </is>
       </c>
       <c r="B350" s="2" t="inlineStr">
@@ -25600,27 +25600,27 @@
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>Sales - no Person filter</t>
+          <t>All Tasks - Person filter</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
         <is>
-          <t>Desktop + Mobile</t>
+          <t>Desktop 1440x900</t>
         </is>
       </c>
       <c r="E350" s="2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F350" s="2" t="inlineStr">
         <is>
-          <t>Roles without All Tasks never see Person; ?person= is ignored</t>
+          <t>Picking a person shows only their tasks, count matches the API</t>
         </is>
       </c>
       <c r="G350" s="2" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H350" s="4" t="inlineStr">
@@ -25630,7 +25630,7 @@
       </c>
       <c r="I350" s="2" t="inlineStr">
         <is>
-          <t>Desktop row has no Person; phone sheet has no Person; ?person=anyone ignored, own 29 cards</t>
+          <t>Priya Nair: 29 cards = trigger 29 = API 29; URL ?person=; name line hidden on cards; menu has Me, people busiest first with role, Unassigned (6), Production team (5); no duplicate rows</t>
         </is>
       </c>
       <c r="J350" s="2" t="inlineStr">
@@ -25642,17 +25642,17 @@
     <row r="351" ht="82" customHeight="1">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>T-680</t>
+          <t>T-692</t>
         </is>
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>LIVE - receivables question</t>
+          <t>All Tasks - Status options</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
@@ -25667,49 +25667,49 @@
       </c>
       <c r="F351" s="2" t="inlineStr">
         <is>
-          <t>Dex answers how much customers owe with the ledger's figure</t>
+          <t>Pending Approval, Overdue and Completed are filterable with correct counts</t>
         </is>
       </c>
       <c r="G351" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H351" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H351" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I351" s="2" t="inlineStr">
         <is>
-          <t>Said zero invoices / Rs 0 outstanding; ledger has Rs 7,49,000 outstanding (17.0s)</t>
+          <t>Pending Approval 40, Overdue 68, Completed 17, Not Started 78 - all equal the API</t>
         </is>
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>DX-01</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="352" ht="82" customHeight="1">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>T-681</t>
+          <t>T-693</t>
         </is>
       </c>
       <c r="B352" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>LIVE - what needs my attention</t>
+          <t>All Tasks - Priority filter removed</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Desktop + Mobile</t>
         </is>
       </c>
       <c r="E352" s="2" t="inlineStr">
@@ -25719,44 +25719,44 @@
       </c>
       <c r="F352" s="2" t="inlineStr">
         <is>
-          <t>Dex surfaces the overdue work and pending decisions</t>
+          <t>No Priority filter (founder call 2026-09-13); an old ?priority= link does not narrow the list</t>
         </is>
       </c>
       <c r="G352" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H352" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H352" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I352" s="2" t="inlineStr">
         <is>
-          <t>Said nothing open or overdue; owner has 24 open / 6 overdue (24.1s)</t>
+          <t>No Priority dropdown on desktop, no Priority chips in the phone sheet; ?person=Priya&amp;status=overdue&amp;priority=high shows the same 20 as without it</t>
         </is>
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>DX-02</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="353" ht="82" customHeight="1">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>T-682</t>
+          <t>T-694</t>
         </is>
       </c>
       <c r="B353" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>LIVE - global search hand-off</t>
+          <t>All Tasks - combined counts</t>
         </is>
       </c>
       <c r="D353" s="2" t="inlineStr">
@@ -25771,12 +25771,12 @@
       </c>
       <c r="F353" s="2" t="inlineStr">
         <is>
-          <t>A question from global search is answered on arrival</t>
+          <t>Each menu's counts reflect the other active filters</t>
         </is>
       </c>
       <c r="G353" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H353" s="4" t="inlineStr">
@@ -25786,25 +25786,29 @@
       </c>
       <c r="I353" s="2" t="inlineStr">
         <is>
-          <t>'Which tasks are overdue?' answered on /brain?q= with a task list (17.5s)</t>
-        </is>
-      </c>
-      <c r="J353" s="2" t="inlineStr"/>
+          <t>With Priya + Overdue, Department 'All' reads 20 = cards = API</t>
+        </is>
+      </c>
+      <c r="J353" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="354" ht="82" customHeight="1">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>T-683</t>
+          <t>T-695</t>
         </is>
       </c>
       <c r="B354" s="2" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>LIVE - coach refresh</t>
+          <t>All Tasks - refresh, Clear, no match</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
@@ -25819,12 +25823,12 @@
       </c>
       <c r="F354" s="2" t="inlineStr">
         <is>
-          <t>Generate coaching produces a review grounded in the stats</t>
+          <t>Filters survive refresh; Clear resets; empty result explains itself</t>
         </is>
       </c>
       <c r="G354" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H354" s="4" t="inlineStr">
@@ -25834,25 +25838,29 @@
       </c>
       <c r="I354" s="2" t="inlineStr">
         <is>
-          <t>TEST_member: 'AI coach updated' in 8.7s; strengths / improvements reference the 13 actionable tasks and plan use</t>
-        </is>
-      </c>
-      <c r="J354" s="2" t="inlineStr"/>
+          <t>Reload keeps 20 cards + URL; Clear -&gt; 131, URL clean; Priya x Under Review -&gt; 'No tasks match these filters' with Clear</t>
+        </is>
+      </c>
+      <c r="J354" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="355" ht="82" customHeight="1">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>T-684</t>
+          <t>T-696</t>
         </is>
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Score with AI</t>
+          <t>All Tasks - person search, links</t>
         </is>
       </c>
       <c r="D355" s="2" t="inlineStr">
@@ -25867,12 +25875,12 @@
       </c>
       <c r="F355" s="2" t="inlineStr">
         <is>
-          <t>Rescore updates the relationship card sensibly</t>
+          <t>Search narrows the menu; Desk overdue link and task deep link behave</t>
         </is>
       </c>
       <c r="G355" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H355" s="4" t="inlineStr">
@@ -25882,30 +25890,34 @@
       </c>
       <c r="I355" s="2" t="inlineStr">
         <is>
-          <t>E2E Test Co: 'Relationship scored by AI' in 7.8s; Relationship 12 / Risk 78, reason cites 4 open complaints and no billing - matches the record</t>
-        </is>
-      </c>
-      <c r="J355" s="2" t="inlineStr"/>
+          <t>'pri' -&gt; Priya Nair only; ?filter=overdue -&gt; Status: Overdue 68; ?task= with filters set clears them and shows the card</t>
+        </is>
+      </c>
+      <c r="J355" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="356" ht="82" customHeight="1">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>T-685</t>
+          <t>T-697</t>
         </is>
       </c>
       <c r="B356" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>LIVE - AI analysis refresh</t>
+          <t>Phone - filter sheet</t>
         </is>
       </c>
       <c r="D356" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Mobile 390x844</t>
         </is>
       </c>
       <c r="E356" s="2" t="inlineStr">
@@ -25915,12 +25927,12 @@
       </c>
       <c r="F356" s="2" t="inlineStr">
         <is>
-          <t>Refresh produces an analysis grounded in the ledger</t>
+          <t>The phone reaches every filter and sees what is active</t>
         </is>
       </c>
       <c r="G356" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="H356" s="4" t="inlineStr">
@@ -25930,30 +25942,34 @@
       </c>
       <c r="I356" s="2" t="inlineStr">
         <is>
-          <t>'Analysis refreshed' in 20.6s; Rs 6.6L outstanding (ledger 6,55,466), Surat Spinners Rs 4.8L unpaid 33 days (correct), duplicates flagged</t>
-        </is>
-      </c>
-      <c r="J356" s="2" t="inlineStr"/>
+          <t>Sheet with Department / Person / Status; Priya + Overdue -&gt; 'Show 20 tasks' = 20 cards; caption 'Showing Priya Nair - Overdue' with Clear; buttons 44px, reachable; no overflow</t>
+        </is>
+      </c>
+      <c r="J356" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="357" ht="82" customHeight="1">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>T-686</t>
+          <t>T-698</t>
         </is>
       </c>
       <c r="B357" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Ask AI</t>
+          <t>Phone - My Tasks / Status without AI</t>
         </is>
       </c>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>Desktop 1440x900</t>
+          <t>Mobile 390x844</t>
         </is>
       </c>
       <c r="E357" s="2" t="inlineStr">
@@ -25963,64 +25979,64 @@
       </c>
       <c r="F357" s="2" t="inlineStr">
         <is>
-          <t>The answer is correct and readable</t>
+          <t>Person hidden on My Tasks; a Status filter is visible even with AI priority off</t>
         </is>
       </c>
       <c r="G357" s="2" t="inlineStr">
         <is>
-          <t>AI accuracy</t>
-        </is>
-      </c>
-      <c r="H357" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Filters</t>
+        </is>
+      </c>
+      <c r="H357" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I357" s="2" t="inlineStr">
         <is>
-          <t>Correct (Surat Spinners Rs 4,80,000, 7.3s) but literal ** markdown shown</t>
+          <t>Sheet on My Tasks has no Person; ?status=overdue shows the caption</t>
         </is>
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>FN-12</t>
+          <t>ASK-24</t>
         </is>
       </c>
     </row>
     <row r="358" ht="82" customHeight="1">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>T-688</t>
+          <t>T-699</t>
         </is>
       </c>
       <c r="B358" s="2" t="inlineStr">
         <is>
-          <t>Dex</t>
+          <t>My Work</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>LIVE - owner on a phone</t>
+          <t>Sales - no Person filter</t>
         </is>
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>Mobile 390x844</t>
+          <t>Desktop + Mobile</t>
         </is>
       </c>
       <c r="E358" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F358" s="2" t="inlineStr">
         <is>
-          <t>Dex answers on mobile and the answer fits the screen</t>
+          <t>Roles without All Tasks never see Person; ?person= is ignored</t>
         </is>
       </c>
       <c r="G358" s="2" t="inlineStr">
         <is>
-          <t>AI flow</t>
+          <t>Permissions</t>
         </is>
       </c>
       <c r="H358" s="4" t="inlineStr">
@@ -26030,15 +26046,19 @@
       </c>
       <c r="I358" s="2" t="inlineStr">
         <is>
-          <t>'53 decisions pending approval across 77' - correct; 17.6s; no overflow</t>
-        </is>
-      </c>
-      <c r="J358" s="2" t="inlineStr"/>
+          <t>Desktop row has no Person; phone sheet has no Person; ?person=anyone ignored, own 29 cards</t>
+        </is>
+      </c>
+      <c r="J358" s="2" t="inlineStr">
+        <is>
+          <t>ASK-24</t>
+        </is>
+      </c>
     </row>
     <row r="359" ht="82" customHeight="1">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>T-689</t>
+          <t>T-680</t>
         </is>
       </c>
       <c r="B359" s="2" t="inlineStr">
@@ -26048,7 +26068,7 @@
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>LIVE - Sales asks money questions</t>
+          <t>LIVE - receivables question</t>
         </is>
       </c>
       <c r="D359" s="2" t="inlineStr">
@@ -26058,45 +26078,49 @@
       </c>
       <c r="E359" s="2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F359" s="2" t="inlineStr">
         <is>
-          <t>Dex refuses finance answers to a role the finance API refuses</t>
+          <t>Dex answers how much customers owe with the ledger's figure</t>
         </is>
       </c>
       <c r="G359" s="2" t="inlineStr">
         <is>
-          <t>Permissions</t>
-        </is>
-      </c>
-      <c r="H359" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H359" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="I359" s="2" t="inlineStr">
         <is>
-          <t>Receivables and profit questions both refused ('You do not have permission to access financial...'), 5.8s / 1.6s; no figures leaked</t>
-        </is>
-      </c>
-      <c r="J359" s="2" t="inlineStr"/>
+          <t>Said zero invoices / Rs 0 outstanding; ledger has Rs 7,49,000 outstanding (17.0s)</t>
+        </is>
+      </c>
+      <c r="J359" s="2" t="inlineStr">
+        <is>
+          <t>DX-01</t>
+        </is>
+      </c>
     </row>
     <row r="360" ht="82" customHeight="1">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>T-687</t>
+          <t>T-681</t>
         </is>
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Dex</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>LIVE - bill extraction</t>
+          <t>LIVE - what needs my attention</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
@@ -26111,7 +26135,7 @@
       </c>
       <c r="F360" s="2" t="inlineStr">
         <is>
-          <t>A GST bill is extracted into a reviewable record with the key fields</t>
+          <t>Dex surfaces the overdue work and pending decisions</t>
         </is>
       </c>
       <c r="G360" s="2" t="inlineStr">
@@ -26126,65 +26150,457 @@
       </c>
       <c r="I360" s="2" t="inlineStr">
         <is>
-          <t>Party, number, amount, due date, category and follow-up correct (31.9s, 92%); date, GSTIN, items missing; no stale-date warning. Left in review, not filed</t>
+          <t>Said nothing open or overdue; owner has 24 open / 6 overdue (24.1s)</t>
         </is>
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>FN-13</t>
+          <t>DX-02</t>
         </is>
       </c>
     </row>
     <row r="361" ht="82" customHeight="1">
       <c r="A361" s="2" t="inlineStr">
         <is>
+          <t>T-682</t>
+        </is>
+      </c>
+      <c r="B361" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C361" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - global search hand-off</t>
+        </is>
+      </c>
+      <c r="D361" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E361" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F361" s="2" t="inlineStr">
+        <is>
+          <t>A question from global search is answered on arrival</t>
+        </is>
+      </c>
+      <c r="G361" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H361" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I361" s="2" t="inlineStr">
+        <is>
+          <t>'Which tasks are overdue?' answered on /brain?q= with a task list (17.5s)</t>
+        </is>
+      </c>
+      <c r="J361" s="2" t="inlineStr"/>
+    </row>
+    <row r="362" ht="82" customHeight="1">
+      <c r="A362" s="2" t="inlineStr">
+        <is>
+          <t>T-683</t>
+        </is>
+      </c>
+      <c r="B362" s="2" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="C362" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - coach refresh</t>
+        </is>
+      </c>
+      <c r="D362" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E362" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F362" s="2" t="inlineStr">
+        <is>
+          <t>Generate coaching produces a review grounded in the stats</t>
+        </is>
+      </c>
+      <c r="G362" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H362" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I362" s="2" t="inlineStr">
+        <is>
+          <t>TEST_member: 'AI coach updated' in 8.7s; strengths / improvements reference the 13 actionable tasks and plan use</t>
+        </is>
+      </c>
+      <c r="J362" s="2" t="inlineStr"/>
+    </row>
+    <row r="363" ht="82" customHeight="1">
+      <c r="A363" s="2" t="inlineStr">
+        <is>
+          <t>T-684</t>
+        </is>
+      </c>
+      <c r="B363" s="2" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C363" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Score with AI</t>
+        </is>
+      </c>
+      <c r="D363" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E363" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F363" s="2" t="inlineStr">
+        <is>
+          <t>Rescore updates the relationship card sensibly</t>
+        </is>
+      </c>
+      <c r="G363" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H363" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I363" s="2" t="inlineStr">
+        <is>
+          <t>E2E Test Co: 'Relationship scored by AI' in 7.8s; Relationship 12 / Risk 78, reason cites 4 open complaints and no billing - matches the record</t>
+        </is>
+      </c>
+      <c r="J363" s="2" t="inlineStr"/>
+    </row>
+    <row r="364" ht="82" customHeight="1">
+      <c r="A364" s="2" t="inlineStr">
+        <is>
+          <t>T-685</t>
+        </is>
+      </c>
+      <c r="B364" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C364" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - AI analysis refresh</t>
+        </is>
+      </c>
+      <c r="D364" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E364" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F364" s="2" t="inlineStr">
+        <is>
+          <t>Refresh produces an analysis grounded in the ledger</t>
+        </is>
+      </c>
+      <c r="G364" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H364" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I364" s="2" t="inlineStr">
+        <is>
+          <t>'Analysis refreshed' in 20.6s; Rs 6.6L outstanding (ledger 6,55,466), Surat Spinners Rs 4.8L unpaid 33 days (correct), duplicates flagged</t>
+        </is>
+      </c>
+      <c r="J364" s="2" t="inlineStr"/>
+    </row>
+    <row r="365" ht="82" customHeight="1">
+      <c r="A365" s="2" t="inlineStr">
+        <is>
+          <t>T-686</t>
+        </is>
+      </c>
+      <c r="B365" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C365" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Ask AI</t>
+        </is>
+      </c>
+      <c r="D365" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E365" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F365" s="2" t="inlineStr">
+        <is>
+          <t>The answer is correct and readable</t>
+        </is>
+      </c>
+      <c r="G365" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H365" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I365" s="2" t="inlineStr">
+        <is>
+          <t>Correct (Surat Spinners Rs 4,80,000, 7.3s) but literal ** markdown shown</t>
+        </is>
+      </c>
+      <c r="J365" s="2" t="inlineStr">
+        <is>
+          <t>FN-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="366" ht="82" customHeight="1">
+      <c r="A366" s="2" t="inlineStr">
+        <is>
+          <t>T-688</t>
+        </is>
+      </c>
+      <c r="B366" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C366" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - owner on a phone</t>
+        </is>
+      </c>
+      <c r="D366" s="2" t="inlineStr">
+        <is>
+          <t>Mobile 390x844</t>
+        </is>
+      </c>
+      <c r="E366" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F366" s="2" t="inlineStr">
+        <is>
+          <t>Dex answers on mobile and the answer fits the screen</t>
+        </is>
+      </c>
+      <c r="G366" s="2" t="inlineStr">
+        <is>
+          <t>AI flow</t>
+        </is>
+      </c>
+      <c r="H366" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I366" s="2" t="inlineStr">
+        <is>
+          <t>'53 decisions pending approval across 77' - correct; 17.6s; no overflow</t>
+        </is>
+      </c>
+      <c r="J366" s="2" t="inlineStr"/>
+    </row>
+    <row r="367" ht="82" customHeight="1">
+      <c r="A367" s="2" t="inlineStr">
+        <is>
+          <t>T-689</t>
+        </is>
+      </c>
+      <c r="B367" s="2" t="inlineStr">
+        <is>
+          <t>Dex</t>
+        </is>
+      </c>
+      <c r="C367" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - Sales asks money questions</t>
+        </is>
+      </c>
+      <c r="D367" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E367" s="2" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="F367" s="2" t="inlineStr">
+        <is>
+          <t>Dex refuses finance answers to a role the finance API refuses</t>
+        </is>
+      </c>
+      <c r="G367" s="2" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="H367" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I367" s="2" t="inlineStr">
+        <is>
+          <t>Receivables and profit questions both refused ('You do not have permission to access financial...'), 5.8s / 1.6s; no figures leaked</t>
+        </is>
+      </c>
+      <c r="J367" s="2" t="inlineStr"/>
+    </row>
+    <row r="368" ht="82" customHeight="1">
+      <c r="A368" s="2" t="inlineStr">
+        <is>
+          <t>T-687</t>
+        </is>
+      </c>
+      <c r="B368" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C368" s="2" t="inlineStr">
+        <is>
+          <t>LIVE - bill extraction</t>
+        </is>
+      </c>
+      <c r="D368" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1440x900</t>
+        </is>
+      </c>
+      <c r="E368" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F368" s="2" t="inlineStr">
+        <is>
+          <t>A GST bill is extracted into a reviewable record with the key fields</t>
+        </is>
+      </c>
+      <c r="G368" s="2" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+      <c r="H368" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I368" s="2" t="inlineStr">
+        <is>
+          <t>Party, number, amount, due date, category and follow-up correct (31.9s, 92%); date, GSTIN, items missing; no stale-date warning. Left in review, not filed</t>
+        </is>
+      </c>
+      <c r="J368" s="2" t="inlineStr">
+        <is>
+          <t>FN-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="369" ht="82" customHeight="1">
+      <c r="A369" s="2" t="inlineStr">
+        <is>
           <t>T-676</t>
         </is>
       </c>
-      <c r="B361" s="2" t="inlineStr">
+      <c r="B369" s="2" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="C361" s="2" t="inlineStr">
+      <c r="C369" s="2" t="inlineStr">
         <is>
           <t>Admin portal gating</t>
         </is>
       </c>
-      <c r="D361" s="2" t="inlineStr">
+      <c r="D369" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="E361" s="2" t="inlineStr">
+      <c r="E369" s="2" t="inlineStr">
         <is>
           <t>Signed out / Owner</t>
         </is>
       </c>
-      <c r="F361" s="2" t="inlineStr">
+      <c r="F369" s="2" t="inlineStr">
         <is>
           <t>Only platform admins reach the portal</t>
         </is>
       </c>
-      <c r="G361" s="2" t="inlineStr">
+      <c r="G369" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="H361" s="4" t="inlineStr">
+      <c r="H369" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="I361" s="2" t="inlineStr">
+      <c r="I369" s="2" t="inlineStr">
         <is>
           <t>Signed out and tenant owner both get the admin sign-in; /admin/me 401; deep link /admin/tenants too</t>
         </is>
       </c>
-      <c r="J361" s="2" t="inlineStr"/>
+      <c r="J369" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J361"/>
+  <autoFilter ref="A1:J369"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -28148,7 +28564,8 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>PROGRESS 2026-09-14 - REMAINING ITEMS CLOSED: (1) PHONE PASS - My Work had a view switcher on the phone only for the owner (My Tasks | All Tasks); nobody could reach Asked by me, My team or Approvals on a phone. Now one view pill for everyone names the view on screen, carries the approvals waiting count, and opens a sheet of the views that person has (My Tasks, Asked by me, My team for managers, All Tasks for the owner, Approvals for approvers); picks go through ?view= so Back works. New Task was already full-screen on the phone after 0eaa411; the approval choice label Before it is marked done was cut off at 390px and now wraps below lg. Acceptance 21/21 (backend/scripts/ux_task_phone_0914.py: owner, sales, finance manager; writes blocked, New Task POST answered by the script). (2) PLAN 4.3 - a named approver must be able to approve: POST /tasks refuses (400, says who and why) an approver who is not the owner and holds no approvals access through own permissions or the company role settings; someone outside the company is still dropped. (3) REAL SAVES - the journeys the browser could only check with writes blocked now run with real saves in an isolated, dropped test database: backend/tests/test_task_management_e2e.py, 6/6 (Asked by me incl. note-only asker; a non-owner named approver approves before work starts; before done: complete, sign-off request and notification, changes requested, complete again, approve closes, reopen needs sign-off again; approver completing closes directly; 4.3 refusal and role-settings grant; My team see, open, note, refused hand-off). Single-process like the Sprint 12 journeys (skipped under xdist): python -m pytest tests/test_task_management_e2e.py -o addopts= -p no:xdist. (4) OLD AUDIT SCRIPTS - ux_lifecycle_mywork.py and ux_gaps_mywork.py create and delete real tasks, so they now refuse to run unless UX_ALLOW_WRITES=1 (the local database is production), and their selectors follow the current My Work (glass dropdowns via option testids, the progress slider, Status: Completed and ?view=all links instead of the old tabs, the bulk reassign picker); not executed here by design. ux_flow_mywork.py, ux_person_filter_0913.py and ux_task_asked_0914.py use the phone view pill. Re-runs: ux_task_asked_0914 20/20, ux_person_filter_0913 33/33, ux_task_approval_stage_0914 19/19, ux_newtask_form_0914 13/13 + 3 n/a. Full backend suite 1425 passed; failures: the known test_website_intel_ssrf_block_and_fallback and test_thirty_parallel_task_creates_no_lost_writes, which only inserts into its own test database and passed when re-run alone (timing).
+          <t>PROGRESS 2026-09-14 - TK-06 WHO IS ON A TASK BUILT (plan Phase 2, founder call: keep it as simple as possible - a task has a Doer, Helpers, Asked by and an optional Approver). (2.1) Supporting employee removed: no stored task used it (0 of 185, read-only check), so nothing to move; the server no longer saves support_id or lets it open a task or its activity; older app builds that still send it are not refused (the field is ignored); gone from the web drawer and the Flutter New Task form (mobile/lib/screens/work_screen.dart, not built here). (2.2) The drawer people section says Asked by (You when it was you). (2.3) It names the approver and the moment (Approval before work starts / before it is marked done, or anyone with approval access). (2.4) A team task routed to the member with the fewest open tasks stores auto_assigned; New Task says Assigned to Priya: fewest open tasks in Sales; the drawer says Picked automatically: fewest open tasks in Sales; any later reassign clears it. (2.5) Status changes and overdue reminders now reach everyone on the task (approved, changes requested, clarification and comments already did). Acceptance 10/10 (backend/scripts/ux_task_people_0914.py, writes blocked, one made-up task for the auto-assigned drawer, New Task POST answered by the script) + 3 new real-save journeys in backend/tests/test_task_management_e2e.py (9/9 in total: old apps still create and support_id grants nothing; auto_assigned set then cleared on reassign; a helper hears a status change and the overdue reminder). Re-runs: ux_newtask_form_0914 13/13 + 3 n/a, ux_task_team_0914 21/21.
+PROGRESS 2026-09-14 - REMAINING ITEMS CLOSED: (1) PHONE PASS - My Work had a view switcher on the phone only for the owner (My Tasks | All Tasks); nobody could reach Asked by me, My team or Approvals on a phone. Now one view pill for everyone names the view on screen, carries the approvals waiting count, and opens a sheet of the views that person has (My Tasks, Asked by me, My team for managers, All Tasks for the owner, Approvals for approvers); picks go through ?view= so Back works. New Task was already full-screen on the phone after 0eaa411; the approval choice label Before it is marked done was cut off at 390px and now wraps below lg. Acceptance 21/21 (backend/scripts/ux_task_phone_0914.py: owner, sales, finance manager; writes blocked, New Task POST answered by the script). (2) PLAN 4.3 - a named approver must be able to approve: POST /tasks refuses (400, says who and why) an approver who is not the owner and holds no approvals access through own permissions or the company role settings; someone outside the company is still dropped. (3) REAL SAVES - the journeys the browser could only check with writes blocked now run with real saves in an isolated, dropped test database: backend/tests/test_task_management_e2e.py, 6/6 (Asked by me incl. note-only asker; a non-owner named approver approves before work starts; before done: complete, sign-off request and notification, changes requested, complete again, approve closes, reopen needs sign-off again; approver completing closes directly; 4.3 refusal and role-settings grant; My team see, open, note, refused hand-off). Single-process like the Sprint 12 journeys (skipped under xdist): python -m pytest tests/test_task_management_e2e.py -o addopts= -p no:xdist. (4) OLD AUDIT SCRIPTS - ux_lifecycle_mywork.py and ux_gaps_mywork.py create and delete real tasks, so they now refuse to run unless UX_ALLOW_WRITES=1 (the local database is production), and their selectors follow the current My Work (glass dropdowns via option testids, the progress slider, Status: Completed and ?view=all links instead of the old tabs, the bulk reassign picker); not executed here by design. ux_flow_mywork.py, ux_person_filter_0913.py and ux_task_asked_0914.py use the phone view pill. Re-runs: ux_task_asked_0914 20/20, ux_person_filter_0913 33/33, ux_task_approval_stage_0914 19/19, ux_newtask_form_0914 13/13 + 3 n/a. Full backend suite 1425 passed; failures: the known test_website_intel_ssrf_block_and_fallback and test_thirty_parallel_task_creates_no_lost_writes, which only inserts into its own test database and passed when re-run alone (timing).
 PROGRESS 2026-09-14 - TK-04 Links always land BUILT (desktop + phone link; frontend only): BEFORE (baseline, writes blocked) a task link opened only when the task sat in the list on screen - Sunita opening a task of sai (her report, not in her My Tasks) got no drawer, nor for a finished task, nor when already on My Work (a notification clicked from there); ?focus=task:&lt;id&gt; links (Brief blocks, phone) were ignored; a deleted task said Access restricted; Workflows was lost on refresh; Back left My Work instead of returning to the previous view. NOW: ?task=&lt;id&gt; and ?focus=task:&lt;id&gt; open the drawer whatever the view - from the list card when the task is in the list, else drawn from the single-task request; the link opens again when it changes while My Work is open; closing the drawer takes the link out of the address; a missing task says This task no longer exists and a refused one keeps Access restricted, both with Dismiss; every view writes ?view=mine|asked|team|all|approvals|workflows and pushes a history entry, and the page follows Back and Forward; ?view=all and ?view=mine links work. Acceptance 23/23 (backend/scripts/ux_task_links_0914.py, writes blocked, REAL data: Sunita Rao and sai; owner; a production user refused with 403; one phone check), run after rebasing onto 0eaa411 (glass pass) and afc6136 (UI-SCALE). Re-runs on the merged page: ux_task_asked_0914 20/20, ux_task_approvals_0914 21/21, ux_task_team_0914 21/21, ux_task_approval_stage_0914 19/19, ux_person_filter_0913 33/33, ux_newtask_form_0914 13/13 + 3 n/a. Script upkeep in the same push: the merged page draws its first cards about 3.5 s after load and redraws about 1 s after Clear (traced), so settle() in the links, asked and person-filter scripts now waits for real content and the person filter waits for the card count to change and hold; the asked clears-url check accepts view=mine; the approval-stage and New Task form scripts follow 0eaa411 (no More options row: those three checks report n/a; GlassSelect dropdowns are driven by their option testids). Bisect (MyWork.js from afc6136, without TK-04): the person-filter failures showed there too; the one asked failure that did not repeat without TK-04 was a half-loaded page (traced with TK-04: all 53 cards 3.5 s after reload) and passes once the script waits. Traced separately: Clear filters restores all 129 cards about 1 s after the click.
 PROGRESS 2026-09-14 - TK-03 My team BUILT (desktop, founder call D3: owner keeps All Tasks, managers get My team): a manager is anyone named as a Reporting Manager (Team page field, until now used only for leave). GET /tasks?view=team = tasks whose doer or a helper is one of my direct reports (services/tasks.task_list_query, 9 unit tests, backend/tests/test_task_view_team.py).My Work: My team in the desktop switcher only for a non-owner with reports; kept in the URL (?view=team), not saved as default; Department, Person (lists the team, no Me) and Status filters work; AI priority off; own empty state; a My team link opened by someone without reports lands on My Tasks. The manager can open a report task and its activity (GET /tasks/{id} and /activity now allow the doer or helper manager) and leave a note; if the task is outside the manager department the drawer is note-only (same as Asked by me), inside it the existing department rule still gives full controls. Acceptance 21/21 (backend/scripts/ux_task_team_0914.py, writes blocked, REAL data: Sunita Rao manages sai, 16 tasks; the other-department note-only drawer uses one made-up task) + ux_task_asked_0914 20/20 re-run. Demo data has only one manager, so a manager of several people is covered by unit tests only.
 PROGRESS 2026-09-14 - TK-05 Approval moment BUILT (desktop, plan Phase 4, founder call D2): the creator picks when a task is approved - New Task, More options, Needs approval: No / Before work starts / Before it is marked done (stored as approval_stage start or close; older approval tasks count as start). Before work starts is the lock tasks always had. Before it is marked done leaves the work open: Complete (proof still required) moves the task to Under review with approval pending and notifies the approver (Approval needed to close, opens Approvals); Approve closes it and runs the close hooks (workflow advance, Brain record, invoice draft - moved into one helper so both paths share them); Request changes sends it back to In progress with the reason shown to the doer; moving the status back withdraws the request; a person who may approve closes it directly; a checklist reaching 100 percent follows the same rule. GET /tasks?view=approvals holds a before-done task only while it waits, so the Approvals count and the Desk card include both kinds. Cards say Approval to start / Approval to close / Needs approval to close; the approver box and the doer banners say which moment it is. Acceptance 19/19 (backend/scripts/ux_task_approval_stage_0914.py, writes blocked, test tasks made up by the script, real approvals feed read-only) + 17 unit tests (backend/tests/test_task_approval_stage.py); ux_newtask_form_0914 16/16 and ux_task_approvals_0914 21/21 re-run. NOT proven live: saving a before-done task and approving it for real - waits on a test database. Open: the server still does not check that a named approver holds approval access (plan 4.3).
@@ -33960,7 +34377,7 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>360 (269 pass, 89 fail, 0 blocked, 2 not run)</t>
+          <t>368 (277 pass, 89 fail, 0 blocked, 2 not run)</t>
         </is>
       </c>
     </row>

</xml_diff>